<commit_message>
Short & Intraday sorted
</commit_message>
<xml_diff>
--- a/data/short term PAX.xlsx
+++ b/data/short term PAX.xlsx
@@ -530,7 +530,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46150.20833333334</v>
+        <v>46152.20833333334</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
@@ -577,7 +577,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46150.21875</v>
+        <v>46152.21875</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
@@ -624,7 +624,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46150.22916666666</v>
+        <v>46152.22916666666</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -671,7 +671,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46150.23958333334</v>
+        <v>46152.23958333334</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
@@ -718,7 +718,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46150.25</v>
+        <v>46152.25</v>
       </c>
       <c r="B6" t="n">
         <v>27</v>
@@ -765,7 +765,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46150.26041666666</v>
+        <v>46152.26041666666</v>
       </c>
       <c r="B7" t="n">
         <v>82</v>
@@ -812,7 +812,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46150.27083333334</v>
+        <v>46152.27083333334</v>
       </c>
       <c r="B8" t="n">
         <v>180</v>
@@ -859,7 +859,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46150.28125</v>
+        <v>46152.28125</v>
       </c>
       <c r="B9" t="n">
         <v>275</v>
@@ -906,7 +906,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46150.29166666666</v>
+        <v>46152.29166666666</v>
       </c>
       <c r="B10" t="n">
         <v>342</v>
@@ -953,7 +953,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46150.30208333334</v>
+        <v>46152.30208333334</v>
       </c>
       <c r="B11" t="n">
         <v>327</v>
@@ -1000,7 +1000,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46150.3125</v>
+        <v>46152.3125</v>
       </c>
       <c r="B12" t="n">
         <v>386</v>
@@ -1047,7 +1047,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46150.32291666666</v>
+        <v>46152.32291666666</v>
       </c>
       <c r="B13" t="n">
         <v>401</v>
@@ -1094,7 +1094,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46150.33333333334</v>
+        <v>46152.33333333334</v>
       </c>
       <c r="B14" t="n">
         <v>399</v>
@@ -1141,7 +1141,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46150.34375</v>
+        <v>46152.34375</v>
       </c>
       <c r="B15" t="n">
         <v>384</v>
@@ -1188,7 +1188,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46150.35416666666</v>
+        <v>46152.35416666666</v>
       </c>
       <c r="B16" t="n">
         <v>438</v>
@@ -1235,7 +1235,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46150.36458333334</v>
+        <v>46152.36458333334</v>
       </c>
       <c r="B17" t="n">
         <v>433</v>
@@ -1282,7 +1282,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46150.375</v>
+        <v>46152.375</v>
       </c>
       <c r="B18" t="n">
         <v>398</v>
@@ -1329,7 +1329,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46150.38541666666</v>
+        <v>46152.38541666666</v>
       </c>
       <c r="B19" t="n">
         <v>463</v>
@@ -1376,7 +1376,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46150.39583333334</v>
+        <v>46152.39583333334</v>
       </c>
       <c r="B20" t="n">
         <v>422</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46150.40625</v>
+        <v>46152.40625</v>
       </c>
       <c r="B21" t="n">
         <v>448</v>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46150.41666666666</v>
+        <v>46152.41666666666</v>
       </c>
       <c r="B22" t="n">
         <v>603</v>
@@ -1517,7 +1517,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46150.42708333334</v>
+        <v>46152.42708333334</v>
       </c>
       <c r="B23" t="n">
         <v>621</v>
@@ -1564,7 +1564,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46150.4375</v>
+        <v>46152.4375</v>
       </c>
       <c r="B24" t="n">
         <v>521</v>
@@ -1611,7 +1611,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46150.44791666666</v>
+        <v>46152.44791666666</v>
       </c>
       <c r="B25" t="n">
         <v>392</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46150.45833333334</v>
+        <v>46152.45833333334</v>
       </c>
       <c r="B26" t="n">
         <v>358</v>
@@ -1705,7 +1705,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46150.46875</v>
+        <v>46152.46875</v>
       </c>
       <c r="B27" t="n">
         <v>487</v>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46150.47916666666</v>
+        <v>46152.47916666666</v>
       </c>
       <c r="B28" t="n">
         <v>557</v>
@@ -1799,7 +1799,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46150.48958333334</v>
+        <v>46152.48958333334</v>
       </c>
       <c r="B29" t="n">
         <v>565</v>
@@ -1846,7 +1846,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46150.5</v>
+        <v>46152.5</v>
       </c>
       <c r="B30" t="n">
         <v>387</v>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46150.51041666666</v>
+        <v>46152.51041666666</v>
       </c>
       <c r="B31" t="n">
         <v>227</v>
@@ -1940,7 +1940,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46150.52083333334</v>
+        <v>46152.52083333334</v>
       </c>
       <c r="B32" t="n">
         <v>382</v>
@@ -1987,7 +1987,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46150.53125</v>
+        <v>46152.53125</v>
       </c>
       <c r="B33" t="n">
         <v>612</v>
@@ -2034,7 +2034,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46150.54166666666</v>
+        <v>46152.54166666666</v>
       </c>
       <c r="B34" t="n">
         <v>699</v>
@@ -2081,7 +2081,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46150.55208333334</v>
+        <v>46152.55208333334</v>
       </c>
       <c r="B35" t="n">
         <v>627</v>
@@ -2128,7 +2128,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46150.5625</v>
+        <v>46152.5625</v>
       </c>
       <c r="B36" t="n">
         <v>538</v>
@@ -2175,7 +2175,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46150.57291666666</v>
+        <v>46152.57291666666</v>
       </c>
       <c r="B37" t="n">
         <v>464</v>
@@ -2222,7 +2222,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46150.58333333334</v>
+        <v>46152.58333333334</v>
       </c>
       <c r="B38" t="n">
         <v>402</v>
@@ -2269,7 +2269,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46150.59375</v>
+        <v>46152.59375</v>
       </c>
       <c r="B39" t="n">
         <v>262</v>
@@ -2316,7 +2316,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46150.60416666666</v>
+        <v>46152.60416666666</v>
       </c>
       <c r="B40" t="n">
         <v>228</v>
@@ -2363,7 +2363,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46150.61458333334</v>
+        <v>46152.61458333334</v>
       </c>
       <c r="B41" t="n">
         <v>350</v>
@@ -2410,7 +2410,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46150.625</v>
+        <v>46152.625</v>
       </c>
       <c r="B42" t="n">
         <v>506</v>
@@ -2457,7 +2457,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46150.63541666666</v>
+        <v>46152.63541666666</v>
       </c>
       <c r="B43" t="n">
         <v>530</v>
@@ -2504,7 +2504,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46150.64583333334</v>
+        <v>46152.64583333334</v>
       </c>
       <c r="B44" t="n">
         <v>459</v>
@@ -2551,7 +2551,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46150.65625</v>
+        <v>46152.65625</v>
       </c>
       <c r="B45" t="n">
         <v>398</v>
@@ -2598,7 +2598,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46150.66666666666</v>
+        <v>46152.66666666666</v>
       </c>
       <c r="B46" t="n">
         <v>488</v>
@@ -2645,7 +2645,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46150.67708333334</v>
+        <v>46152.67708333334</v>
       </c>
       <c r="B47" t="n">
         <v>532</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46150.6875</v>
+        <v>46152.6875</v>
       </c>
       <c r="B48" t="n">
         <v>716</v>
@@ -2739,7 +2739,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46150.69791666666</v>
+        <v>46152.69791666666</v>
       </c>
       <c r="B49" t="n">
         <v>673</v>
@@ -2786,7 +2786,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46150.70833333334</v>
+        <v>46152.70833333334</v>
       </c>
       <c r="B50" t="n">
         <v>504</v>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46150.71875</v>
+        <v>46152.71875</v>
       </c>
       <c r="B51" t="n">
         <v>616</v>
@@ -2880,7 +2880,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46150.72916666666</v>
+        <v>46152.72916666666</v>
       </c>
       <c r="B52" t="n">
         <v>569</v>
@@ -2927,7 +2927,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46150.73958333334</v>
+        <v>46152.73958333334</v>
       </c>
       <c r="B53" t="n">
         <v>619</v>
@@ -2974,7 +2974,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>46150.75</v>
+        <v>46152.75</v>
       </c>
       <c r="B54" t="n">
         <v>597</v>
@@ -3021,7 +3021,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>46150.76041666666</v>
+        <v>46152.76041666666</v>
       </c>
       <c r="B55" t="n">
         <v>373</v>
@@ -3068,7 +3068,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>46150.77083333334</v>
+        <v>46152.77083333334</v>
       </c>
       <c r="B56" t="n">
         <v>298</v>
@@ -3115,7 +3115,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>46150.78125</v>
+        <v>46152.78125</v>
       </c>
       <c r="B57" t="n">
         <v>325</v>
@@ -3162,7 +3162,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46150.79166666666</v>
+        <v>46152.79166666666</v>
       </c>
       <c r="B58" t="n">
         <v>350</v>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>46150.80208333334</v>
+        <v>46152.80208333334</v>
       </c>
       <c r="B59" t="n">
         <v>373</v>
@@ -3256,7 +3256,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46150.8125</v>
+        <v>46152.8125</v>
       </c>
       <c r="B60" t="n">
         <v>344</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46150.82291666666</v>
+        <v>46152.82291666666</v>
       </c>
       <c r="B61" t="n">
         <v>385</v>
@@ -3350,7 +3350,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>46150.83333333334</v>
+        <v>46152.83333333334</v>
       </c>
       <c r="B62" t="n">
         <v>439</v>
@@ -3397,7 +3397,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>46150.84375</v>
+        <v>46152.84375</v>
       </c>
       <c r="B63" t="n">
         <v>408</v>
@@ -3444,7 +3444,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>46150.85416666666</v>
+        <v>46152.85416666666</v>
       </c>
       <c r="B64" t="n">
         <v>319</v>
@@ -3491,7 +3491,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>46150.86458333334</v>
+        <v>46152.86458333334</v>
       </c>
       <c r="B65" t="n">
         <v>166</v>
@@ -3538,7 +3538,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46150.875</v>
+        <v>46152.875</v>
       </c>
       <c r="B66" t="n">
         <v>29</v>
@@ -3585,7 +3585,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>46150.88541666666</v>
+        <v>46152.88541666666</v>
       </c>
       <c r="B67" t="n">
         <v>61</v>
@@ -3632,7 +3632,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>46150.89583333334</v>
+        <v>46152.89583333334</v>
       </c>
       <c r="B68" t="n">
         <v>107</v>
@@ -3679,7 +3679,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>46150.90625</v>
+        <v>46152.90625</v>
       </c>
       <c r="B69" t="n">
         <v>93</v>
@@ -3726,7 +3726,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>46150.91666666666</v>
+        <v>46152.91666666666</v>
       </c>
       <c r="B70" t="n">
         <v>115</v>
@@ -3773,7 +3773,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>46150.92708333334</v>
+        <v>46152.92708333334</v>
       </c>
       <c r="B71" t="n">
         <v>58</v>
@@ -3820,7 +3820,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>46150.9375</v>
+        <v>46152.9375</v>
       </c>
       <c r="B72" t="n">
         <v>0</v>
@@ -3867,7 +3867,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46150.94791666666</v>
+        <v>46152.94791666666</v>
       </c>
       <c r="B73" t="n">
         <v>0</v>
@@ -3914,7 +3914,7 @@
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>46150.95833333334</v>
+        <v>46152.95833333334</v>
       </c>
       <c r="B74" t="n">
         <v>0</v>
@@ -3961,7 +3961,7 @@
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>46150.96875</v>
+        <v>46152.96875</v>
       </c>
       <c r="B75" t="n">
         <v>0</v>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>46150.97916666666</v>
+        <v>46152.97916666666</v>
       </c>
       <c r="B76" t="n">
         <v>0</v>
@@ -4055,7 +4055,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>46150.98958333334</v>
+        <v>46152.98958333334</v>
       </c>
       <c r="B77" t="n">
         <v>0</v>
@@ -4102,7 +4102,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="B78" t="n">
         <v>0</v>
@@ -4149,7 +4149,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>46151.01041666666</v>
+        <v>46153.01041666666</v>
       </c>
       <c r="B79" t="n">
         <v>10</v>
@@ -4196,7 +4196,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>46151.02083333334</v>
+        <v>46153.02083333334</v>
       </c>
       <c r="B80" t="n">
         <v>28</v>
@@ -4243,7 +4243,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>46151.03125</v>
+        <v>46153.03125</v>
       </c>
       <c r="B81" t="n">
         <v>48</v>
@@ -4290,7 +4290,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>46151.04166666666</v>
+        <v>46153.04166666666</v>
       </c>
       <c r="B82" t="n">
         <v>58</v>
@@ -4337,7 +4337,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>46151.05208333334</v>
+        <v>46153.05208333334</v>
       </c>
       <c r="B83" t="n">
         <v>9</v>
@@ -4384,7 +4384,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46151.0625</v>
+        <v>46153.0625</v>
       </c>
       <c r="B84" t="n">
         <v>0</v>
@@ -4431,7 +4431,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46151.07291666666</v>
+        <v>46153.07291666666</v>
       </c>
       <c r="B85" t="n">
         <v>4</v>
@@ -4478,7 +4478,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>46151.08333333334</v>
+        <v>46153.08333333334</v>
       </c>
       <c r="B86" t="n">
         <v>11</v>
@@ -4525,7 +4525,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46151.09375</v>
+        <v>46153.09375</v>
       </c>
       <c r="B87" t="n">
         <v>20</v>
@@ -4572,7 +4572,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>46151.10416666666</v>
+        <v>46153.10416666666</v>
       </c>
       <c r="B88" t="n">
         <v>33</v>
@@ -4619,7 +4619,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>46151.11458333334</v>
+        <v>46153.11458333334</v>
       </c>
       <c r="B89" t="n">
         <v>17</v>
@@ -4666,7 +4666,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46151.125</v>
+        <v>46153.125</v>
       </c>
       <c r="B90" t="n">
         <v>27</v>
@@ -4713,7 +4713,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46151.13541666666</v>
+        <v>46153.13541666666</v>
       </c>
       <c r="B91" t="n">
         <v>41</v>
@@ -4760,7 +4760,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46151.14583333334</v>
+        <v>46153.14583333334</v>
       </c>
       <c r="B92" t="n">
         <v>75</v>
@@ -4807,7 +4807,7 @@
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>46151.15625</v>
+        <v>46153.15625</v>
       </c>
       <c r="B93" t="n">
         <v>268</v>
@@ -4854,7 +4854,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>46151.16666666666</v>
+        <v>46153.16666666666</v>
       </c>
       <c r="B94" t="n">
         <v>527</v>
@@ -4901,7 +4901,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>46151.17708333334</v>
+        <v>46153.17708333334</v>
       </c>
       <c r="B95" t="n">
         <v>888</v>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46151.1875</v>
+        <v>46153.1875</v>
       </c>
       <c r="B96" t="n">
         <v>1032</v>
@@ -4995,7 +4995,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>46151.19791666666</v>
+        <v>46153.19791666666</v>
       </c>
       <c r="B97" t="n">
         <v>780</v>
@@ -5042,7 +5042,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46151.20833333334</v>
+        <v>46153.20833333334</v>
       </c>
       <c r="B98" t="n">
         <v>847</v>
@@ -5089,7 +5089,7 @@
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>46151.21875</v>
+        <v>46153.21875</v>
       </c>
       <c r="B99" t="n">
         <v>689</v>
@@ -5136,7 +5136,7 @@
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>46151.22916666666</v>
+        <v>46153.22916666666</v>
       </c>
       <c r="B100" t="n">
         <v>660</v>
@@ -5183,7 +5183,7 @@
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>46151.23958333334</v>
+        <v>46153.23958333334</v>
       </c>
       <c r="B101" t="n">
         <v>671</v>
@@ -5230,7 +5230,7 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>46151.25</v>
+        <v>46153.25</v>
       </c>
       <c r="B102" t="n">
         <v>627</v>
@@ -5277,7 +5277,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>46151.26041666666</v>
+        <v>46153.26041666666</v>
       </c>
       <c r="B103" t="n">
         <v>513</v>
@@ -5324,7 +5324,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>46151.27083333334</v>
+        <v>46153.27083333334</v>
       </c>
       <c r="B104" t="n">
         <v>544</v>
@@ -5371,7 +5371,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>46151.28125</v>
+        <v>46153.28125</v>
       </c>
       <c r="B105" t="n">
         <v>417</v>
@@ -5418,7 +5418,7 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>46151.29166666666</v>
+        <v>46153.29166666666</v>
       </c>
       <c r="B106" t="n">
         <v>285</v>
@@ -5465,7 +5465,7 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>46151.30208333334</v>
+        <v>46153.30208333334</v>
       </c>
       <c r="B107" t="n">
         <v>290</v>
@@ -5512,7 +5512,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>46151.3125</v>
+        <v>46153.3125</v>
       </c>
       <c r="B108" t="n">
         <v>323</v>
@@ -5559,7 +5559,7 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>46151.32291666666</v>
+        <v>46153.32291666666</v>
       </c>
       <c r="B109" t="n">
         <v>271</v>
@@ -5606,7 +5606,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>46151.33333333334</v>
+        <v>46153.33333333334</v>
       </c>
       <c r="B110" t="n">
         <v>246</v>
@@ -5653,7 +5653,7 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>46151.34375</v>
+        <v>46153.34375</v>
       </c>
       <c r="B111" t="n">
         <v>287</v>
@@ -5700,7 +5700,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>46151.35416666666</v>
+        <v>46153.35416666666</v>
       </c>
       <c r="B112" t="n">
         <v>275</v>
@@ -5747,7 +5747,7 @@
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>46151.36458333334</v>
+        <v>46153.36458333334</v>
       </c>
       <c r="B113" t="n">
         <v>447</v>
@@ -5794,7 +5794,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>46151.375</v>
+        <v>46153.375</v>
       </c>
       <c r="B114" t="n">
         <v>566</v>
@@ -5841,7 +5841,7 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>46151.38541666666</v>
+        <v>46153.38541666666</v>
       </c>
       <c r="B115" t="n">
         <v>590</v>
@@ -5888,7 +5888,7 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>46151.39583333334</v>
+        <v>46153.39583333334</v>
       </c>
       <c r="B116" t="n">
         <v>558</v>
@@ -5935,7 +5935,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>46151.40625</v>
+        <v>46153.40625</v>
       </c>
       <c r="B117" t="n">
         <v>354</v>
@@ -5982,7 +5982,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>46151.41666666666</v>
+        <v>46153.41666666666</v>
       </c>
       <c r="B118" t="n">
         <v>483</v>
@@ -6029,7 +6029,7 @@
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>46151.42708333334</v>
+        <v>46153.42708333334</v>
       </c>
       <c r="B119" t="n">
         <v>537</v>
@@ -6076,7 +6076,7 @@
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>46151.4375</v>
+        <v>46153.4375</v>
       </c>
       <c r="B120" t="n">
         <v>558</v>
@@ -6123,7 +6123,7 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46151.44791666666</v>
+        <v>46153.44791666666</v>
       </c>
       <c r="B121" t="n">
         <v>570</v>
@@ -6170,7 +6170,7 @@
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46151.45833333334</v>
+        <v>46153.45833333334</v>
       </c>
       <c r="B122" t="n">
         <v>424</v>
@@ -6217,7 +6217,7 @@
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>46151.46875</v>
+        <v>46153.46875</v>
       </c>
       <c r="B123" t="n">
         <v>377</v>
@@ -6264,7 +6264,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>46151.47916666666</v>
+        <v>46153.47916666666</v>
       </c>
       <c r="B124" t="n">
         <v>372</v>
@@ -6311,7 +6311,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>46151.48958333334</v>
+        <v>46153.48958333334</v>
       </c>
       <c r="B125" t="n">
         <v>374</v>
@@ -6358,7 +6358,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46151.5</v>
+        <v>46153.5</v>
       </c>
       <c r="B126" t="n">
         <v>508</v>
@@ -6405,7 +6405,7 @@
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>46151.51041666666</v>
+        <v>46153.51041666666</v>
       </c>
       <c r="B127" t="n">
         <v>482</v>
@@ -6452,7 +6452,7 @@
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>46151.52083333334</v>
+        <v>46153.52083333334</v>
       </c>
       <c r="B128" t="n">
         <v>416</v>
@@ -6499,7 +6499,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46151.53125</v>
+        <v>46153.53125</v>
       </c>
       <c r="B129" t="n">
         <v>498</v>
@@ -6546,7 +6546,7 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>46151.54166666666</v>
+        <v>46153.54166666666</v>
       </c>
       <c r="B130" t="n">
         <v>378</v>
@@ -6593,7 +6593,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>46151.55208333334</v>
+        <v>46153.55208333334</v>
       </c>
       <c r="B131" t="n">
         <v>245</v>
@@ -6640,7 +6640,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>46151.5625</v>
+        <v>46153.5625</v>
       </c>
       <c r="B132" t="n">
         <v>253</v>
@@ -6687,7 +6687,7 @@
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>46151.57291666666</v>
+        <v>46153.57291666666</v>
       </c>
       <c r="B133" t="n">
         <v>302</v>
@@ -6734,7 +6734,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>46151.58333333334</v>
+        <v>46153.58333333334</v>
       </c>
       <c r="B134" t="n">
         <v>405</v>
@@ -6781,7 +6781,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>46151.59375</v>
+        <v>46153.59375</v>
       </c>
       <c r="B135" t="n">
         <v>472</v>
@@ -6828,7 +6828,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46151.60416666666</v>
+        <v>46153.60416666666</v>
       </c>
       <c r="B136" t="n">
         <v>591</v>
@@ -6875,7 +6875,7 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46151.61458333334</v>
+        <v>46153.61458333334</v>
       </c>
       <c r="B137" t="n">
         <v>607</v>
@@ -6922,7 +6922,7 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46151.625</v>
+        <v>46153.625</v>
       </c>
       <c r="B138" t="n">
         <v>441</v>
@@ -6969,7 +6969,7 @@
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46151.63541666666</v>
+        <v>46153.63541666666</v>
       </c>
       <c r="B139" t="n">
         <v>309</v>
@@ -7016,7 +7016,7 @@
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46151.64583333334</v>
+        <v>46153.64583333334</v>
       </c>
       <c r="B140" t="n">
         <v>406</v>
@@ -7063,7 +7063,7 @@
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46151.65625</v>
+        <v>46153.65625</v>
       </c>
       <c r="B141" t="n">
         <v>545</v>
@@ -7110,7 +7110,7 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46151.66666666666</v>
+        <v>46153.66666666666</v>
       </c>
       <c r="B142" t="n">
         <v>659</v>
@@ -7157,7 +7157,7 @@
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46151.67708333334</v>
+        <v>46153.67708333334</v>
       </c>
       <c r="B143" t="n">
         <v>904</v>
@@ -7204,7 +7204,7 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46151.6875</v>
+        <v>46153.6875</v>
       </c>
       <c r="B144" t="n">
         <v>870</v>
@@ -7251,7 +7251,7 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46151.69791666666</v>
+        <v>46153.69791666666</v>
       </c>
       <c r="B145" t="n">
         <v>773</v>
@@ -7298,7 +7298,7 @@
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46151.70833333334</v>
+        <v>46153.70833333334</v>
       </c>
       <c r="B146" t="n">
         <v>654</v>
@@ -7345,7 +7345,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46151.71875</v>
+        <v>46153.71875</v>
       </c>
       <c r="B147" t="n">
         <v>472</v>
@@ -7392,7 +7392,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46151.72916666666</v>
+        <v>46153.72916666666</v>
       </c>
       <c r="B148" t="n">
         <v>483</v>
@@ -7439,7 +7439,7 @@
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46151.73958333334</v>
+        <v>46153.73958333334</v>
       </c>
       <c r="B149" t="n">
         <v>597</v>
@@ -7486,7 +7486,7 @@
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46151.75</v>
+        <v>46153.75</v>
       </c>
       <c r="B150" t="n">
         <v>597</v>
@@ -7533,7 +7533,7 @@
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46151.76041666666</v>
+        <v>46153.76041666666</v>
       </c>
       <c r="B151" t="n">
         <v>569</v>
@@ -7580,7 +7580,7 @@
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46151.77083333334</v>
+        <v>46153.77083333334</v>
       </c>
       <c r="B152" t="n">
         <v>423</v>
@@ -7627,7 +7627,7 @@
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46151.78125</v>
+        <v>46153.78125</v>
       </c>
       <c r="B153" t="n">
         <v>269</v>
@@ -7674,7 +7674,7 @@
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46151.79166666666</v>
+        <v>46153.79166666666</v>
       </c>
       <c r="B154" t="n">
         <v>312</v>
@@ -7721,7 +7721,7 @@
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46151.80208333334</v>
+        <v>46153.80208333334</v>
       </c>
       <c r="B155" t="n">
         <v>557</v>
@@ -7768,7 +7768,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>46151.8125</v>
+        <v>46153.8125</v>
       </c>
       <c r="B156" t="n">
         <v>690</v>
@@ -7815,7 +7815,7 @@
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>46151.82291666666</v>
+        <v>46153.82291666666</v>
       </c>
       <c r="B157" t="n">
         <v>511</v>
@@ -7862,7 +7862,7 @@
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
-        <v>46151.83333333334</v>
+        <v>46153.83333333334</v>
       </c>
       <c r="B158" t="n">
         <v>188</v>
@@ -7909,7 +7909,7 @@
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
-        <v>46151.84375</v>
+        <v>46153.84375</v>
       </c>
       <c r="B159" t="n">
         <v>204</v>
@@ -7956,7 +7956,7 @@
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
-        <v>46151.85416666666</v>
+        <v>46153.85416666666</v>
       </c>
       <c r="B160" t="n">
         <v>287</v>
@@ -8003,7 +8003,7 @@
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
-        <v>46151.86458333334</v>
+        <v>46153.86458333334</v>
       </c>
       <c r="B161" t="n">
         <v>177</v>
@@ -8050,7 +8050,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>46151.875</v>
+        <v>46153.875</v>
       </c>
       <c r="B162" t="n">
         <v>9</v>
@@ -8097,7 +8097,7 @@
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
-        <v>46151.88541666666</v>
+        <v>46153.88541666666</v>
       </c>
       <c r="B163" t="n">
         <v>0</v>
@@ -8144,7 +8144,7 @@
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
-        <v>46151.89583333334</v>
+        <v>46153.89583333334</v>
       </c>
       <c r="B164" t="n">
         <v>0</v>
@@ -8191,7 +8191,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>46151.90625</v>
+        <v>46153.90625</v>
       </c>
       <c r="B165" t="n">
         <v>15</v>
@@ -8238,7 +8238,7 @@
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
-        <v>46151.91666666666</v>
+        <v>46153.91666666666</v>
       </c>
       <c r="B166" t="n">
         <v>69</v>
@@ -8285,7 +8285,7 @@
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
-        <v>46151.92708333334</v>
+        <v>46153.92708333334</v>
       </c>
       <c r="B167" t="n">
         <v>126</v>
@@ -8332,7 +8332,7 @@
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
-        <v>46151.9375</v>
+        <v>46153.9375</v>
       </c>
       <c r="B168" t="n">
         <v>175</v>
@@ -8379,7 +8379,7 @@
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
-        <v>46151.94791666666</v>
+        <v>46153.94791666666</v>
       </c>
       <c r="B169" t="n">
         <v>82</v>
@@ -8426,7 +8426,7 @@
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
-        <v>46151.95833333334</v>
+        <v>46153.95833333334</v>
       </c>
       <c r="B170" t="n">
         <v>0</v>
@@ -8473,7 +8473,7 @@
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
-        <v>46151.96875</v>
+        <v>46153.96875</v>
       </c>
       <c r="B171" t="n">
         <v>0</v>
@@ -8520,7 +8520,7 @@
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
-        <v>46151.97916666666</v>
+        <v>46153.97916666666</v>
       </c>
       <c r="B172" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>46151.98958333334</v>
+        <v>46153.98958333334</v>
       </c>
       <c r="B173" t="n">
         <v>0</v>
@@ -8614,7 +8614,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>46152</v>
+        <v>46154</v>
       </c>
       <c r="B174" t="n">
         <v>0</v>
@@ -8661,7 +8661,7 @@
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
-        <v>46152.01041666666</v>
+        <v>46154.01041666666</v>
       </c>
       <c r="B175" t="n">
         <v>10</v>
@@ -8708,7 +8708,7 @@
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
-        <v>46152.02083333334</v>
+        <v>46154.02083333334</v>
       </c>
       <c r="B176" t="n">
         <v>35</v>
@@ -8755,7 +8755,7 @@
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
-        <v>46152.03125</v>
+        <v>46154.03125</v>
       </c>
       <c r="B177" t="n">
         <v>62</v>
@@ -8802,7 +8802,7 @@
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
-        <v>46152.04166666666</v>
+        <v>46154.04166666666</v>
       </c>
       <c r="B178" t="n">
         <v>80</v>
@@ -8849,7 +8849,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>46152.05208333334</v>
+        <v>46154.05208333334</v>
       </c>
       <c r="B179" t="n">
         <v>27</v>
@@ -8896,7 +8896,7 @@
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
-        <v>46152.0625</v>
+        <v>46154.0625</v>
       </c>
       <c r="B180" t="n">
         <v>0</v>
@@ -8943,7 +8943,7 @@
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
-        <v>46152.07291666666</v>
+        <v>46154.07291666666</v>
       </c>
       <c r="B181" t="n">
         <v>4</v>
@@ -8990,7 +8990,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>46152.08333333334</v>
+        <v>46154.08333333334</v>
       </c>
       <c r="B182" t="n">
         <v>11</v>
@@ -9037,7 +9037,7 @@
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
-        <v>46152.09375</v>
+        <v>46154.09375</v>
       </c>
       <c r="B183" t="n">
         <v>20</v>
@@ -9084,7 +9084,7 @@
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
-        <v>46152.10416666666</v>
+        <v>46154.10416666666</v>
       </c>
       <c r="B184" t="n">
         <v>33</v>
@@ -9131,7 +9131,7 @@
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
-        <v>46152.11458333334</v>
+        <v>46154.11458333334</v>
       </c>
       <c r="B185" t="n">
         <v>17</v>
@@ -9178,7 +9178,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>46152.125</v>
+        <v>46154.125</v>
       </c>
       <c r="B186" t="n">
         <v>19</v>
@@ -9225,7 +9225,7 @@
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
-        <v>46152.13541666666</v>
+        <v>46154.13541666666</v>
       </c>
       <c r="B187" t="n">
         <v>26</v>
@@ -9272,7 +9272,7 @@
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
-        <v>46152.14583333334</v>
+        <v>46154.14583333334</v>
       </c>
       <c r="B188" t="n">
         <v>65</v>
@@ -9319,7 +9319,7 @@
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
-        <v>46152.15625</v>
+        <v>46154.15625</v>
       </c>
       <c r="B189" t="n">
         <v>256</v>
@@ -9366,7 +9366,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>46152.16666666666</v>
+        <v>46154.16666666666</v>
       </c>
       <c r="B190" t="n">
         <v>528</v>
@@ -9413,7 +9413,7 @@
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
-        <v>46152.17708333334</v>
+        <v>46154.17708333334</v>
       </c>
       <c r="B191" t="n">
         <v>850</v>
@@ -9460,7 +9460,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>46152.1875</v>
+        <v>46154.1875</v>
       </c>
       <c r="B192" t="n">
         <v>967</v>
@@ -9507,7 +9507,7 @@
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
-        <v>46152.19791666666</v>
+        <v>46154.19791666666</v>
       </c>
       <c r="B193" t="n">
         <v>755</v>
@@ -9554,7 +9554,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>46152.20833333334</v>
+        <v>46154.20833333334</v>
       </c>
       <c r="B194" t="n">
         <v>800</v>
@@ -9601,7 +9601,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>46152.21875</v>
+        <v>46154.21875</v>
       </c>
       <c r="B195" t="n">
         <v>656</v>
@@ -9648,7 +9648,7 @@
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
-        <v>46152.22916666666</v>
+        <v>46154.22916666666</v>
       </c>
       <c r="B196" t="n">
         <v>515</v>
@@ -9695,7 +9695,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>46152.23958333334</v>
+        <v>46154.23958333334</v>
       </c>
       <c r="B197" t="n">
         <v>474</v>
@@ -9742,7 +9742,7 @@
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
-        <v>46152.25</v>
+        <v>46154.25</v>
       </c>
       <c r="B198" t="n">
         <v>601</v>
@@ -9789,7 +9789,7 @@
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
-        <v>46152.26041666666</v>
+        <v>46154.26041666666</v>
       </c>
       <c r="B199" t="n">
         <v>632</v>
@@ -9836,7 +9836,7 @@
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
-        <v>46152.27083333334</v>
+        <v>46154.27083333334</v>
       </c>
       <c r="B200" t="n">
         <v>592</v>
@@ -9883,7 +9883,7 @@
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
-        <v>46152.28125</v>
+        <v>46154.28125</v>
       </c>
       <c r="B201" t="n">
         <v>493</v>
@@ -9930,7 +9930,7 @@
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
-        <v>46152.29166666666</v>
+        <v>46154.29166666666</v>
       </c>
       <c r="B202" t="n">
         <v>448</v>
@@ -9977,7 +9977,7 @@
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
-        <v>46152.30208333334</v>
+        <v>46154.30208333334</v>
       </c>
       <c r="B203" t="n">
         <v>459</v>
@@ -10024,7 +10024,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>46152.3125</v>
+        <v>46154.3125</v>
       </c>
       <c r="B204" t="n">
         <v>432</v>
@@ -10071,7 +10071,7 @@
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
-        <v>46152.32291666666</v>
+        <v>46154.32291666666</v>
       </c>
       <c r="B205" t="n">
         <v>368</v>
@@ -10118,7 +10118,7 @@
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
-        <v>46152.33333333334</v>
+        <v>46154.33333333334</v>
       </c>
       <c r="B206" t="n">
         <v>320</v>
@@ -10165,7 +10165,7 @@
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
-        <v>46152.34375</v>
+        <v>46154.34375</v>
       </c>
       <c r="B207" t="n">
         <v>237</v>
@@ -10212,7 +10212,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>46152.35416666666</v>
+        <v>46154.35416666666</v>
       </c>
       <c r="B208" t="n">
         <v>262</v>
@@ -10259,7 +10259,7 @@
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">
-        <v>46152.36458333334</v>
+        <v>46154.36458333334</v>
       </c>
       <c r="B209" t="n">
         <v>445</v>
@@ -10306,7 +10306,7 @@
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
-        <v>46152.375</v>
+        <v>46154.375</v>
       </c>
       <c r="B210" t="n">
         <v>627</v>
@@ -10353,7 +10353,7 @@
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
-        <v>46152.38541666666</v>
+        <v>46154.38541666666</v>
       </c>
       <c r="B211" t="n">
         <v>623</v>
@@ -10400,7 +10400,7 @@
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
-        <v>46152.39583333334</v>
+        <v>46154.39583333334</v>
       </c>
       <c r="B212" t="n">
         <v>576</v>
@@ -10447,7 +10447,7 @@
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
-        <v>46152.40625</v>
+        <v>46154.40625</v>
       </c>
       <c r="B213" t="n">
         <v>542</v>
@@ -10494,7 +10494,7 @@
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
-        <v>46152.41666666666</v>
+        <v>46154.41666666666</v>
       </c>
       <c r="B214" t="n">
         <v>484</v>
@@ -10541,7 +10541,7 @@
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
-        <v>46152.42708333334</v>
+        <v>46154.42708333334</v>
       </c>
       <c r="B215" t="n">
         <v>377</v>
@@ -10588,7 +10588,7 @@
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
-        <v>46152.4375</v>
+        <v>46154.4375</v>
       </c>
       <c r="B216" t="n">
         <v>281</v>
@@ -10635,7 +10635,7 @@
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
-        <v>46152.44791666666</v>
+        <v>46154.44791666666</v>
       </c>
       <c r="B217" t="n">
         <v>386</v>
@@ -10682,7 +10682,7 @@
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
-        <v>46152.45833333334</v>
+        <v>46154.45833333334</v>
       </c>
       <c r="B218" t="n">
         <v>548</v>
@@ -10729,7 +10729,7 @@
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
-        <v>46152.46875</v>
+        <v>46154.46875</v>
       </c>
       <c r="B219" t="n">
         <v>620</v>
@@ -10776,7 +10776,7 @@
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
-        <v>46152.47916666666</v>
+        <v>46154.47916666666</v>
       </c>
       <c r="B220" t="n">
         <v>531</v>
@@ -10823,7 +10823,7 @@
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
-        <v>46152.48958333334</v>
+        <v>46154.48958333334</v>
       </c>
       <c r="B221" t="n">
         <v>491</v>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
-        <v>46152.5</v>
+        <v>46154.5</v>
       </c>
       <c r="B222" t="n">
         <v>385</v>
@@ -10917,7 +10917,7 @@
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
-        <v>46152.51041666666</v>
+        <v>46154.51041666666</v>
       </c>
       <c r="B223" t="n">
         <v>397</v>
@@ -10964,7 +10964,7 @@
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
-        <v>46152.52083333334</v>
+        <v>46154.52083333334</v>
       </c>
       <c r="B224" t="n">
         <v>490</v>
@@ -11011,7 +11011,7 @@
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
-        <v>46152.53125</v>
+        <v>46154.53125</v>
       </c>
       <c r="B225" t="n">
         <v>547</v>
@@ -11058,7 +11058,7 @@
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
-        <v>46152.54166666666</v>
+        <v>46154.54166666666</v>
       </c>
       <c r="B226" t="n">
         <v>415</v>
@@ -11105,7 +11105,7 @@
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
-        <v>46152.55208333334</v>
+        <v>46154.55208333334</v>
       </c>
       <c r="B227" t="n">
         <v>228</v>
@@ -11152,7 +11152,7 @@
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
-        <v>46152.5625</v>
+        <v>46154.5625</v>
       </c>
       <c r="B228" t="n">
         <v>309</v>
@@ -11199,7 +11199,7 @@
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
-        <v>46152.57291666666</v>
+        <v>46154.57291666666</v>
       </c>
       <c r="B229" t="n">
         <v>411</v>
@@ -11246,7 +11246,7 @@
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
-        <v>46152.58333333334</v>
+        <v>46154.58333333334</v>
       </c>
       <c r="B230" t="n">
         <v>385</v>
@@ -11293,7 +11293,7 @@
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
-        <v>46152.59375</v>
+        <v>46154.59375</v>
       </c>
       <c r="B231" t="n">
         <v>436</v>
@@ -11340,7 +11340,7 @@
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
-        <v>46152.60416666666</v>
+        <v>46154.60416666666</v>
       </c>
       <c r="B232" t="n">
         <v>446</v>
@@ -11387,7 +11387,7 @@
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
-        <v>46152.61458333334</v>
+        <v>46154.61458333334</v>
       </c>
       <c r="B233" t="n">
         <v>426</v>
@@ -11434,7 +11434,7 @@
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
-        <v>46152.625</v>
+        <v>46154.625</v>
       </c>
       <c r="B234" t="n">
         <v>450</v>
@@ -11481,7 +11481,7 @@
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
-        <v>46152.63541666666</v>
+        <v>46154.63541666666</v>
       </c>
       <c r="B235" t="n">
         <v>322</v>
@@ -11528,7 +11528,7 @@
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
-        <v>46152.64583333334</v>
+        <v>46154.64583333334</v>
       </c>
       <c r="B236" t="n">
         <v>303</v>
@@ -11575,7 +11575,7 @@
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
-        <v>46152.65625</v>
+        <v>46154.65625</v>
       </c>
       <c r="B237" t="n">
         <v>496</v>
@@ -11622,7 +11622,7 @@
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
-        <v>46152.66666666666</v>
+        <v>46154.66666666666</v>
       </c>
       <c r="B238" t="n">
         <v>654</v>
@@ -11669,7 +11669,7 @@
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
-        <v>46152.67708333334</v>
+        <v>46154.67708333334</v>
       </c>
       <c r="B239" t="n">
         <v>781</v>
@@ -11716,7 +11716,7 @@
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
-        <v>46152.6875</v>
+        <v>46154.6875</v>
       </c>
       <c r="B240" t="n">
         <v>795</v>
@@ -11763,7 +11763,7 @@
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
-        <v>46152.69791666666</v>
+        <v>46154.69791666666</v>
       </c>
       <c r="B241" t="n">
         <v>569</v>
@@ -11810,7 +11810,7 @@
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
-        <v>46152.70833333334</v>
+        <v>46154.70833333334</v>
       </c>
       <c r="B242" t="n">
         <v>611</v>
@@ -11857,7 +11857,7 @@
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
-        <v>46152.71875</v>
+        <v>46154.71875</v>
       </c>
       <c r="B243" t="n">
         <v>794</v>
@@ -11904,7 +11904,7 @@
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
-        <v>46152.72916666666</v>
+        <v>46154.72916666666</v>
       </c>
       <c r="B244" t="n">
         <v>635</v>
@@ -11951,7 +11951,7 @@
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
-        <v>46152.73958333334</v>
+        <v>46154.73958333334</v>
       </c>
       <c r="B245" t="n">
         <v>642</v>
@@ -11998,7 +11998,7 @@
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
-        <v>46152.75</v>
+        <v>46154.75</v>
       </c>
       <c r="B246" t="n">
         <v>624</v>
@@ -12045,7 +12045,7 @@
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
-        <v>46152.76041666666</v>
+        <v>46154.76041666666</v>
       </c>
       <c r="B247" t="n">
         <v>608</v>
@@ -12092,7 +12092,7 @@
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
-        <v>46152.77083333334</v>
+        <v>46154.77083333334</v>
       </c>
       <c r="B248" t="n">
         <v>656</v>
@@ -12139,7 +12139,7 @@
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
-        <v>46152.78125</v>
+        <v>46154.78125</v>
       </c>
       <c r="B249" t="n">
         <v>512</v>
@@ -12186,7 +12186,7 @@
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
-        <v>46152.79166666666</v>
+        <v>46154.79166666666</v>
       </c>
       <c r="B250" t="n">
         <v>323</v>
@@ -12233,7 +12233,7 @@
     </row>
     <row r="251">
       <c r="A251" s="1" t="n">
-        <v>46152.80208333334</v>
+        <v>46154.80208333334</v>
       </c>
       <c r="B251" t="n">
         <v>438</v>
@@ -12280,7 +12280,7 @@
     </row>
     <row r="252">
       <c r="A252" s="1" t="n">
-        <v>46152.8125</v>
+        <v>46154.8125</v>
       </c>
       <c r="B252" t="n">
         <v>613</v>
@@ -12327,7 +12327,7 @@
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
-        <v>46152.82291666666</v>
+        <v>46154.82291666666</v>
       </c>
       <c r="B253" t="n">
         <v>547</v>
@@ -12374,7 +12374,7 @@
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
-        <v>46152.83333333334</v>
+        <v>46154.83333333334</v>
       </c>
       <c r="B254" t="n">
         <v>402</v>
@@ -12421,7 +12421,7 @@
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
-        <v>46152.84375</v>
+        <v>46154.84375</v>
       </c>
       <c r="B255" t="n">
         <v>341</v>
@@ -12468,7 +12468,7 @@
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
-        <v>46152.85416666666</v>
+        <v>46154.85416666666</v>
       </c>
       <c r="B256" t="n">
         <v>264</v>
@@ -12515,7 +12515,7 @@
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
-        <v>46152.86458333334</v>
+        <v>46154.86458333334</v>
       </c>
       <c r="B257" t="n">
         <v>116</v>
@@ -12562,7 +12562,7 @@
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
-        <v>46152.875</v>
+        <v>46154.875</v>
       </c>
       <c r="B258" t="n">
         <v>0</v>
@@ -12609,7 +12609,7 @@
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
-        <v>46152.88541666666</v>
+        <v>46154.88541666666</v>
       </c>
       <c r="B259" t="n">
         <v>10</v>
@@ -12656,7 +12656,7 @@
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
-        <v>46152.89583333334</v>
+        <v>46154.89583333334</v>
       </c>
       <c r="B260" t="n">
         <v>39</v>
@@ -12703,7 +12703,7 @@
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
-        <v>46152.90625</v>
+        <v>46154.90625</v>
       </c>
       <c r="B261" t="n">
         <v>109</v>
@@ -12750,7 +12750,7 @@
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
-        <v>46152.91666666666</v>
+        <v>46154.91666666666</v>
       </c>
       <c r="B262" t="n">
         <v>193</v>
@@ -12797,7 +12797,7 @@
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
-        <v>46152.92708333334</v>
+        <v>46154.92708333334</v>
       </c>
       <c r="B263" t="n">
         <v>217</v>
@@ -12844,7 +12844,7 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>46152.9375</v>
+        <v>46154.9375</v>
       </c>
       <c r="B264" t="n">
         <v>185</v>
@@ -12891,7 +12891,7 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>46152.94791666666</v>
+        <v>46154.94791666666</v>
       </c>
       <c r="B265" t="n">
         <v>27</v>
@@ -12938,7 +12938,7 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>46152.95833333334</v>
+        <v>46154.95833333334</v>
       </c>
       <c r="B266" t="n">
         <v>0</v>
@@ -12985,7 +12985,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>46152.96875</v>
+        <v>46154.96875</v>
       </c>
       <c r="B267" t="n">
         <v>0</v>
@@ -13032,7 +13032,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>46152.97916666666</v>
+        <v>46154.97916666666</v>
       </c>
       <c r="B268" t="n">
         <v>0</v>
@@ -13079,7 +13079,7 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>46152.98958333334</v>
+        <v>46154.98958333334</v>
       </c>
       <c r="B269" t="n">
         <v>0</v>
@@ -13126,7 +13126,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>46153</v>
+        <v>46155</v>
       </c>
       <c r="B270" t="n">
         <v>0</v>
@@ -13173,7 +13173,7 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>46153.01041666666</v>
+        <v>46155.01041666666</v>
       </c>
       <c r="B271" t="n">
         <v>10</v>
@@ -13220,7 +13220,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>46153.02083333334</v>
+        <v>46155.02083333334</v>
       </c>
       <c r="B272" t="n">
         <v>35</v>
@@ -13267,7 +13267,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>46153.03125</v>
+        <v>46155.03125</v>
       </c>
       <c r="B273" t="n">
         <v>62</v>
@@ -13314,7 +13314,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>46153.04166666666</v>
+        <v>46155.04166666666</v>
       </c>
       <c r="B274" t="n">
         <v>80</v>
@@ -13361,7 +13361,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>46153.05208333334</v>
+        <v>46155.05208333334</v>
       </c>
       <c r="B275" t="n">
         <v>27</v>
@@ -13408,7 +13408,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>46153.0625</v>
+        <v>46155.0625</v>
       </c>
       <c r="B276" t="n">
         <v>0</v>
@@ -13455,7 +13455,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>46153.07291666666</v>
+        <v>46155.07291666666</v>
       </c>
       <c r="B277" t="n">
         <v>4</v>
@@ -13502,7 +13502,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>46153.08333333334</v>
+        <v>46155.08333333334</v>
       </c>
       <c r="B278" t="n">
         <v>11</v>
@@ -13549,7 +13549,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>46153.09375</v>
+        <v>46155.09375</v>
       </c>
       <c r="B279" t="n">
         <v>20</v>
@@ -13596,7 +13596,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>46153.10416666666</v>
+        <v>46155.10416666666</v>
       </c>
       <c r="B280" t="n">
         <v>33</v>
@@ -13643,7 +13643,7 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>46153.11458333334</v>
+        <v>46155.11458333334</v>
       </c>
       <c r="B281" t="n">
         <v>17</v>
@@ -13690,7 +13690,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>46153.125</v>
+        <v>46155.125</v>
       </c>
       <c r="B282" t="n">
         <v>19</v>
@@ -13737,7 +13737,7 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>46153.13541666666</v>
+        <v>46155.13541666666</v>
       </c>
       <c r="B283" t="n">
         <v>26</v>
@@ -13784,7 +13784,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>46153.14583333334</v>
+        <v>46155.14583333334</v>
       </c>
       <c r="B284" t="n">
         <v>65</v>
@@ -13831,7 +13831,7 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>46153.15625</v>
+        <v>46155.15625</v>
       </c>
       <c r="B285" t="n">
         <v>256</v>
@@ -13878,7 +13878,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>46153.16666666666</v>
+        <v>46155.16666666666</v>
       </c>
       <c r="B286" t="n">
         <v>528</v>
@@ -13925,7 +13925,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>46153.17708333334</v>
+        <v>46155.17708333334</v>
       </c>
       <c r="B287" t="n">
         <v>850</v>
@@ -13972,7 +13972,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>46153.1875</v>
+        <v>46155.1875</v>
       </c>
       <c r="B288" t="n">
         <v>967</v>
@@ -14019,7 +14019,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>46153.19791666666</v>
+        <v>46155.19791666666</v>
       </c>
       <c r="B289" t="n">
         <v>755</v>
@@ -14066,7 +14066,7 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>46153.20833333334</v>
+        <v>46155.20833333334</v>
       </c>
       <c r="B290" t="n">
         <v>800</v>
@@ -14113,7 +14113,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>46153.21875</v>
+        <v>46155.21875</v>
       </c>
       <c r="B291" t="n">
         <v>656</v>
@@ -14160,7 +14160,7 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>46153.22916666666</v>
+        <v>46155.22916666666</v>
       </c>
       <c r="B292" t="n">
         <v>515</v>
@@ -14207,7 +14207,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>46153.23958333334</v>
+        <v>46155.23958333334</v>
       </c>
       <c r="B293" t="n">
         <v>474</v>
@@ -14254,7 +14254,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>46153.25</v>
+        <v>46155.25</v>
       </c>
       <c r="B294" t="n">
         <v>601</v>
@@ -14301,7 +14301,7 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>46153.26041666666</v>
+        <v>46155.26041666666</v>
       </c>
       <c r="B295" t="n">
         <v>632</v>
@@ -14348,7 +14348,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>46153.27083333334</v>
+        <v>46155.27083333334</v>
       </c>
       <c r="B296" t="n">
         <v>592</v>
@@ -14395,7 +14395,7 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>46153.28125</v>
+        <v>46155.28125</v>
       </c>
       <c r="B297" t="n">
         <v>493</v>
@@ -14442,7 +14442,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>46153.29166666666</v>
+        <v>46155.29166666666</v>
       </c>
       <c r="B298" t="n">
         <v>448</v>
@@ -14489,7 +14489,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>46153.30208333334</v>
+        <v>46155.30208333334</v>
       </c>
       <c r="B299" t="n">
         <v>459</v>
@@ -14536,7 +14536,7 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>46153.3125</v>
+        <v>46155.3125</v>
       </c>
       <c r="B300" t="n">
         <v>432</v>
@@ -14583,7 +14583,7 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>46153.32291666666</v>
+        <v>46155.32291666666</v>
       </c>
       <c r="B301" t="n">
         <v>368</v>
@@ -14630,7 +14630,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>46153.33333333334</v>
+        <v>46155.33333333334</v>
       </c>
       <c r="B302" t="n">
         <v>320</v>
@@ -14677,7 +14677,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>46153.34375</v>
+        <v>46155.34375</v>
       </c>
       <c r="B303" t="n">
         <v>237</v>
@@ -14724,7 +14724,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>46153.35416666666</v>
+        <v>46155.35416666666</v>
       </c>
       <c r="B304" t="n">
         <v>262</v>
@@ -14771,7 +14771,7 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>46153.36458333334</v>
+        <v>46155.36458333334</v>
       </c>
       <c r="B305" t="n">
         <v>445</v>
@@ -14818,7 +14818,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>46153.375</v>
+        <v>46155.375</v>
       </c>
       <c r="B306" t="n">
         <v>627</v>
@@ -14865,7 +14865,7 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>46153.38541666666</v>
+        <v>46155.38541666666</v>
       </c>
       <c r="B307" t="n">
         <v>623</v>
@@ -14912,7 +14912,7 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>46153.39583333334</v>
+        <v>46155.39583333334</v>
       </c>
       <c r="B308" t="n">
         <v>576</v>
@@ -14959,7 +14959,7 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>46153.40625</v>
+        <v>46155.40625</v>
       </c>
       <c r="B309" t="n">
         <v>542</v>
@@ -15006,7 +15006,7 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
-        <v>46153.41666666666</v>
+        <v>46155.41666666666</v>
       </c>
       <c r="B310" t="n">
         <v>484</v>
@@ -15053,7 +15053,7 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
-        <v>46153.42708333334</v>
+        <v>46155.42708333334</v>
       </c>
       <c r="B311" t="n">
         <v>377</v>
@@ -15100,7 +15100,7 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>46153.4375</v>
+        <v>46155.4375</v>
       </c>
       <c r="B312" t="n">
         <v>281</v>
@@ -15147,7 +15147,7 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>46153.44791666666</v>
+        <v>46155.44791666666</v>
       </c>
       <c r="B313" t="n">
         <v>386</v>
@@ -15194,7 +15194,7 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>46153.45833333334</v>
+        <v>46155.45833333334</v>
       </c>
       <c r="B314" t="n">
         <v>548</v>
@@ -15241,7 +15241,7 @@
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
-        <v>46153.46875</v>
+        <v>46155.46875</v>
       </c>
       <c r="B315" t="n">
         <v>620</v>
@@ -15288,7 +15288,7 @@
     </row>
     <row r="316">
       <c r="A316" s="1" t="n">
-        <v>46153.47916666666</v>
+        <v>46155.47916666666</v>
       </c>
       <c r="B316" t="n">
         <v>531</v>
@@ -15335,7 +15335,7 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>46153.48958333334</v>
+        <v>46155.48958333334</v>
       </c>
       <c r="B317" t="n">
         <v>491</v>
@@ -15382,7 +15382,7 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>46153.5</v>
+        <v>46155.5</v>
       </c>
       <c r="B318" t="n">
         <v>385</v>
@@ -15429,7 +15429,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>46153.51041666666</v>
+        <v>46155.51041666666</v>
       </c>
       <c r="B319" t="n">
         <v>397</v>
@@ -15476,7 +15476,7 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
-        <v>46153.52083333334</v>
+        <v>46155.52083333334</v>
       </c>
       <c r="B320" t="n">
         <v>490</v>
@@ -15523,7 +15523,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>46153.53125</v>
+        <v>46155.53125</v>
       </c>
       <c r="B321" t="n">
         <v>547</v>
@@ -15570,7 +15570,7 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>46153.54166666666</v>
+        <v>46155.54166666666</v>
       </c>
       <c r="B322" t="n">
         <v>415</v>
@@ -15617,7 +15617,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>46153.55208333334</v>
+        <v>46155.55208333334</v>
       </c>
       <c r="B323" t="n">
         <v>228</v>
@@ -15664,7 +15664,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>46153.5625</v>
+        <v>46155.5625</v>
       </c>
       <c r="B324" t="n">
         <v>309</v>
@@ -15711,7 +15711,7 @@
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>46153.57291666666</v>
+        <v>46155.57291666666</v>
       </c>
       <c r="B325" t="n">
         <v>411</v>
@@ -15758,7 +15758,7 @@
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>46153.58333333334</v>
+        <v>46155.58333333334</v>
       </c>
       <c r="B326" t="n">
         <v>385</v>
@@ -15805,7 +15805,7 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>46153.59375</v>
+        <v>46155.59375</v>
       </c>
       <c r="B327" t="n">
         <v>436</v>
@@ -15852,7 +15852,7 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>46153.60416666666</v>
+        <v>46155.60416666666</v>
       </c>
       <c r="B328" t="n">
         <v>446</v>
@@ -15899,7 +15899,7 @@
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
-        <v>46153.61458333334</v>
+        <v>46155.61458333334</v>
       </c>
       <c r="B329" t="n">
         <v>426</v>
@@ -15946,7 +15946,7 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>46153.625</v>
+        <v>46155.625</v>
       </c>
       <c r="B330" t="n">
         <v>450</v>
@@ -15993,7 +15993,7 @@
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
-        <v>46153.63541666666</v>
+        <v>46155.63541666666</v>
       </c>
       <c r="B331" t="n">
         <v>322</v>
@@ -16040,7 +16040,7 @@
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
-        <v>46153.64583333334</v>
+        <v>46155.64583333334</v>
       </c>
       <c r="B332" t="n">
         <v>303</v>
@@ -16087,7 +16087,7 @@
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
-        <v>46153.65625</v>
+        <v>46155.65625</v>
       </c>
       <c r="B333" t="n">
         <v>496</v>
@@ -16134,7 +16134,7 @@
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
-        <v>46153.66666666666</v>
+        <v>46155.66666666666</v>
       </c>
       <c r="B334" t="n">
         <v>654</v>
@@ -16181,7 +16181,7 @@
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
-        <v>46153.67708333334</v>
+        <v>46155.67708333334</v>
       </c>
       <c r="B335" t="n">
         <v>781</v>
@@ -16228,7 +16228,7 @@
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
-        <v>46153.6875</v>
+        <v>46155.6875</v>
       </c>
       <c r="B336" t="n">
         <v>795</v>
@@ -16275,7 +16275,7 @@
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
-        <v>46153.69791666666</v>
+        <v>46155.69791666666</v>
       </c>
       <c r="B337" t="n">
         <v>569</v>
@@ -16322,7 +16322,7 @@
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
-        <v>46153.70833333334</v>
+        <v>46155.70833333334</v>
       </c>
       <c r="B338" t="n">
         <v>611</v>
@@ -16369,7 +16369,7 @@
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
-        <v>46153.71875</v>
+        <v>46155.71875</v>
       </c>
       <c r="B339" t="n">
         <v>794</v>
@@ -16416,7 +16416,7 @@
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
-        <v>46153.72916666666</v>
+        <v>46155.72916666666</v>
       </c>
       <c r="B340" t="n">
         <v>635</v>
@@ -16463,7 +16463,7 @@
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
-        <v>46153.73958333334</v>
+        <v>46155.73958333334</v>
       </c>
       <c r="B341" t="n">
         <v>642</v>
@@ -16510,7 +16510,7 @@
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
-        <v>46153.75</v>
+        <v>46155.75</v>
       </c>
       <c r="B342" t="n">
         <v>624</v>
@@ -16557,7 +16557,7 @@
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
-        <v>46153.76041666666</v>
+        <v>46155.76041666666</v>
       </c>
       <c r="B343" t="n">
         <v>608</v>
@@ -16604,7 +16604,7 @@
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
-        <v>46153.77083333334</v>
+        <v>46155.77083333334</v>
       </c>
       <c r="B344" t="n">
         <v>656</v>
@@ -16651,7 +16651,7 @@
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
-        <v>46153.78125</v>
+        <v>46155.78125</v>
       </c>
       <c r="B345" t="n">
         <v>512</v>
@@ -16698,7 +16698,7 @@
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
-        <v>46153.79166666666</v>
+        <v>46155.79166666666</v>
       </c>
       <c r="B346" t="n">
         <v>323</v>
@@ -16745,7 +16745,7 @@
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
-        <v>46153.80208333334</v>
+        <v>46155.80208333334</v>
       </c>
       <c r="B347" t="n">
         <v>438</v>
@@ -16792,7 +16792,7 @@
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
-        <v>46153.8125</v>
+        <v>46155.8125</v>
       </c>
       <c r="B348" t="n">
         <v>613</v>
@@ -16839,7 +16839,7 @@
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
-        <v>46153.82291666666</v>
+        <v>46155.82291666666</v>
       </c>
       <c r="B349" t="n">
         <v>547</v>
@@ -16886,7 +16886,7 @@
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
-        <v>46153.83333333334</v>
+        <v>46155.83333333334</v>
       </c>
       <c r="B350" t="n">
         <v>402</v>
@@ -16933,7 +16933,7 @@
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
-        <v>46153.84375</v>
+        <v>46155.84375</v>
       </c>
       <c r="B351" t="n">
         <v>341</v>
@@ -16980,7 +16980,7 @@
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
-        <v>46153.85416666666</v>
+        <v>46155.85416666666</v>
       </c>
       <c r="B352" t="n">
         <v>264</v>
@@ -17027,7 +17027,7 @@
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
-        <v>46153.86458333334</v>
+        <v>46155.86458333334</v>
       </c>
       <c r="B353" t="n">
         <v>116</v>
@@ -17074,7 +17074,7 @@
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
-        <v>46153.875</v>
+        <v>46155.875</v>
       </c>
       <c r="B354" t="n">
         <v>0</v>
@@ -17121,7 +17121,7 @@
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
-        <v>46153.88541666666</v>
+        <v>46155.88541666666</v>
       </c>
       <c r="B355" t="n">
         <v>10</v>
@@ -17168,7 +17168,7 @@
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
-        <v>46153.89583333334</v>
+        <v>46155.89583333334</v>
       </c>
       <c r="B356" t="n">
         <v>39</v>
@@ -17215,7 +17215,7 @@
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
-        <v>46153.90625</v>
+        <v>46155.90625</v>
       </c>
       <c r="B357" t="n">
         <v>109</v>
@@ -17262,7 +17262,7 @@
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
-        <v>46153.91666666666</v>
+        <v>46155.91666666666</v>
       </c>
       <c r="B358" t="n">
         <v>193</v>
@@ -17309,7 +17309,7 @@
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
-        <v>46153.92708333334</v>
+        <v>46155.92708333334</v>
       </c>
       <c r="B359" t="n">
         <v>217</v>
@@ -17356,7 +17356,7 @@
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
-        <v>46153.9375</v>
+        <v>46155.9375</v>
       </c>
       <c r="B360" t="n">
         <v>185</v>
@@ -17403,7 +17403,7 @@
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
-        <v>46153.94791666666</v>
+        <v>46155.94791666666</v>
       </c>
       <c r="B361" t="n">
         <v>27</v>
@@ -17450,7 +17450,7 @@
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
-        <v>46153.95833333334</v>
+        <v>46155.95833333334</v>
       </c>
       <c r="B362" t="n">
         <v>0</v>
@@ -17497,7 +17497,7 @@
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
-        <v>46153.96875</v>
+        <v>46155.96875</v>
       </c>
       <c r="B363" t="n">
         <v>0</v>
@@ -17544,7 +17544,7 @@
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
-        <v>46153.97916666666</v>
+        <v>46155.97916666666</v>
       </c>
       <c r="B364" t="n">
         <v>0</v>
@@ -17591,7 +17591,7 @@
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
-        <v>46153.98958333334</v>
+        <v>46155.98958333334</v>
       </c>
       <c r="B365" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update flight demand data and modify short term passenger data file
</commit_message>
<xml_diff>
--- a/data/short term PAX.xlsx
+++ b/data/short term PAX.xlsx
@@ -530,7 +530,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46152.20833333334</v>
+        <v>46153.20833333334</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
@@ -577,7 +577,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46152.21875</v>
+        <v>46153.21875</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
@@ -624,7 +624,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46152.22916666666</v>
+        <v>46153.22916666666</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -671,7 +671,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46152.23958333334</v>
+        <v>46153.23958333334</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
@@ -718,7 +718,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46152.25</v>
+        <v>46153.25</v>
       </c>
       <c r="B6" t="n">
         <v>27</v>
@@ -765,7 +765,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46152.26041666666</v>
+        <v>46153.26041666666</v>
       </c>
       <c r="B7" t="n">
         <v>82</v>
@@ -812,7 +812,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46152.27083333334</v>
+        <v>46153.27083333334</v>
       </c>
       <c r="B8" t="n">
         <v>180</v>
@@ -859,7 +859,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46152.28125</v>
+        <v>46153.28125</v>
       </c>
       <c r="B9" t="n">
         <v>275</v>
@@ -906,7 +906,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46152.29166666666</v>
+        <v>46153.29166666666</v>
       </c>
       <c r="B10" t="n">
         <v>342</v>
@@ -953,7 +953,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46152.30208333334</v>
+        <v>46153.30208333334</v>
       </c>
       <c r="B11" t="n">
         <v>327</v>
@@ -1000,7 +1000,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46152.3125</v>
+        <v>46153.3125</v>
       </c>
       <c r="B12" t="n">
         <v>386</v>
@@ -1047,7 +1047,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46152.32291666666</v>
+        <v>46153.32291666666</v>
       </c>
       <c r="B13" t="n">
         <v>401</v>
@@ -1094,7 +1094,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46152.33333333334</v>
+        <v>46153.33333333334</v>
       </c>
       <c r="B14" t="n">
         <v>399</v>
@@ -1141,7 +1141,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46152.34375</v>
+        <v>46153.34375</v>
       </c>
       <c r="B15" t="n">
         <v>384</v>
@@ -1188,7 +1188,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46152.35416666666</v>
+        <v>46153.35416666666</v>
       </c>
       <c r="B16" t="n">
         <v>438</v>
@@ -1235,7 +1235,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46152.36458333334</v>
+        <v>46153.36458333334</v>
       </c>
       <c r="B17" t="n">
         <v>433</v>
@@ -1282,7 +1282,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46152.375</v>
+        <v>46153.375</v>
       </c>
       <c r="B18" t="n">
         <v>398</v>
@@ -1329,7 +1329,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46152.38541666666</v>
+        <v>46153.38541666666</v>
       </c>
       <c r="B19" t="n">
         <v>463</v>
@@ -1376,7 +1376,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46152.39583333334</v>
+        <v>46153.39583333334</v>
       </c>
       <c r="B20" t="n">
         <v>422</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46152.40625</v>
+        <v>46153.40625</v>
       </c>
       <c r="B21" t="n">
         <v>448</v>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46152.41666666666</v>
+        <v>46153.41666666666</v>
       </c>
       <c r="B22" t="n">
         <v>603</v>
@@ -1517,7 +1517,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46152.42708333334</v>
+        <v>46153.42708333334</v>
       </c>
       <c r="B23" t="n">
         <v>621</v>
@@ -1564,7 +1564,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46152.4375</v>
+        <v>46153.4375</v>
       </c>
       <c r="B24" t="n">
         <v>521</v>
@@ -1611,7 +1611,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46152.44791666666</v>
+        <v>46153.44791666666</v>
       </c>
       <c r="B25" t="n">
         <v>392</v>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46152.45833333334</v>
+        <v>46153.45833333334</v>
       </c>
       <c r="B26" t="n">
         <v>358</v>
@@ -1705,7 +1705,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46152.46875</v>
+        <v>46153.46875</v>
       </c>
       <c r="B27" t="n">
         <v>487</v>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46152.47916666666</v>
+        <v>46153.47916666666</v>
       </c>
       <c r="B28" t="n">
         <v>557</v>
@@ -1799,7 +1799,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46152.48958333334</v>
+        <v>46153.48958333334</v>
       </c>
       <c r="B29" t="n">
         <v>565</v>
@@ -1846,7 +1846,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46152.5</v>
+        <v>46153.5</v>
       </c>
       <c r="B30" t="n">
         <v>387</v>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46152.51041666666</v>
+        <v>46153.51041666666</v>
       </c>
       <c r="B31" t="n">
         <v>227</v>
@@ -1940,7 +1940,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46152.52083333334</v>
+        <v>46153.52083333334</v>
       </c>
       <c r="B32" t="n">
         <v>382</v>
@@ -1987,7 +1987,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46152.53125</v>
+        <v>46153.53125</v>
       </c>
       <c r="B33" t="n">
         <v>612</v>
@@ -2034,7 +2034,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46152.54166666666</v>
+        <v>46153.54166666666</v>
       </c>
       <c r="B34" t="n">
         <v>699</v>
@@ -2081,7 +2081,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46152.55208333334</v>
+        <v>46153.55208333334</v>
       </c>
       <c r="B35" t="n">
         <v>627</v>
@@ -2128,7 +2128,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46152.5625</v>
+        <v>46153.5625</v>
       </c>
       <c r="B36" t="n">
         <v>538</v>
@@ -2175,7 +2175,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46152.57291666666</v>
+        <v>46153.57291666666</v>
       </c>
       <c r="B37" t="n">
         <v>464</v>
@@ -2222,7 +2222,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46152.58333333334</v>
+        <v>46153.58333333334</v>
       </c>
       <c r="B38" t="n">
         <v>402</v>
@@ -2269,7 +2269,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46152.59375</v>
+        <v>46153.59375</v>
       </c>
       <c r="B39" t="n">
         <v>262</v>
@@ -2316,7 +2316,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46152.60416666666</v>
+        <v>46153.60416666666</v>
       </c>
       <c r="B40" t="n">
         <v>228</v>
@@ -2363,7 +2363,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46152.61458333334</v>
+        <v>46153.61458333334</v>
       </c>
       <c r="B41" t="n">
         <v>350</v>
@@ -2410,7 +2410,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46152.625</v>
+        <v>46153.625</v>
       </c>
       <c r="B42" t="n">
         <v>506</v>
@@ -2457,7 +2457,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46152.63541666666</v>
+        <v>46153.63541666666</v>
       </c>
       <c r="B43" t="n">
         <v>530</v>
@@ -2504,7 +2504,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46152.64583333334</v>
+        <v>46153.64583333334</v>
       </c>
       <c r="B44" t="n">
         <v>459</v>
@@ -2551,7 +2551,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46152.65625</v>
+        <v>46153.65625</v>
       </c>
       <c r="B45" t="n">
         <v>398</v>
@@ -2598,7 +2598,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46152.66666666666</v>
+        <v>46153.66666666666</v>
       </c>
       <c r="B46" t="n">
         <v>488</v>
@@ -2645,7 +2645,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46152.67708333334</v>
+        <v>46153.67708333334</v>
       </c>
       <c r="B47" t="n">
         <v>532</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46152.6875</v>
+        <v>46153.6875</v>
       </c>
       <c r="B48" t="n">
         <v>716</v>
@@ -2739,7 +2739,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46152.69791666666</v>
+        <v>46153.69791666666</v>
       </c>
       <c r="B49" t="n">
         <v>673</v>
@@ -2786,7 +2786,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46152.70833333334</v>
+        <v>46153.70833333334</v>
       </c>
       <c r="B50" t="n">
         <v>504</v>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46152.71875</v>
+        <v>46153.71875</v>
       </c>
       <c r="B51" t="n">
         <v>616</v>
@@ -2880,7 +2880,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46152.72916666666</v>
+        <v>46153.72916666666</v>
       </c>
       <c r="B52" t="n">
         <v>569</v>
@@ -2927,7 +2927,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46152.73958333334</v>
+        <v>46153.73958333334</v>
       </c>
       <c r="B53" t="n">
         <v>619</v>
@@ -2974,7 +2974,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>46152.75</v>
+        <v>46153.75</v>
       </c>
       <c r="B54" t="n">
         <v>597</v>
@@ -3021,7 +3021,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>46152.76041666666</v>
+        <v>46153.76041666666</v>
       </c>
       <c r="B55" t="n">
         <v>373</v>
@@ -3068,7 +3068,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>46152.77083333334</v>
+        <v>46153.77083333334</v>
       </c>
       <c r="B56" t="n">
         <v>298</v>
@@ -3115,7 +3115,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>46152.78125</v>
+        <v>46153.78125</v>
       </c>
       <c r="B57" t="n">
         <v>325</v>
@@ -3162,7 +3162,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46152.79166666666</v>
+        <v>46153.79166666666</v>
       </c>
       <c r="B58" t="n">
         <v>350</v>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>46152.80208333334</v>
+        <v>46153.80208333334</v>
       </c>
       <c r="B59" t="n">
         <v>373</v>
@@ -3256,7 +3256,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46152.8125</v>
+        <v>46153.8125</v>
       </c>
       <c r="B60" t="n">
         <v>344</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46152.82291666666</v>
+        <v>46153.82291666666</v>
       </c>
       <c r="B61" t="n">
         <v>385</v>
@@ -3350,7 +3350,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>46152.83333333334</v>
+        <v>46153.83333333334</v>
       </c>
       <c r="B62" t="n">
         <v>439</v>
@@ -3397,7 +3397,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>46152.84375</v>
+        <v>46153.84375</v>
       </c>
       <c r="B63" t="n">
         <v>408</v>
@@ -3444,7 +3444,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>46152.85416666666</v>
+        <v>46153.85416666666</v>
       </c>
       <c r="B64" t="n">
         <v>319</v>
@@ -3491,7 +3491,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>46152.86458333334</v>
+        <v>46153.86458333334</v>
       </c>
       <c r="B65" t="n">
         <v>166</v>
@@ -3538,7 +3538,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46152.875</v>
+        <v>46153.875</v>
       </c>
       <c r="B66" t="n">
         <v>29</v>
@@ -3585,7 +3585,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>46152.88541666666</v>
+        <v>46153.88541666666</v>
       </c>
       <c r="B67" t="n">
         <v>61</v>
@@ -3632,7 +3632,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>46152.89583333334</v>
+        <v>46153.89583333334</v>
       </c>
       <c r="B68" t="n">
         <v>107</v>
@@ -3679,7 +3679,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>46152.90625</v>
+        <v>46153.90625</v>
       </c>
       <c r="B69" t="n">
         <v>93</v>
@@ -3726,7 +3726,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>46152.91666666666</v>
+        <v>46153.91666666666</v>
       </c>
       <c r="B70" t="n">
         <v>115</v>
@@ -3773,7 +3773,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>46152.92708333334</v>
+        <v>46153.92708333334</v>
       </c>
       <c r="B71" t="n">
         <v>58</v>
@@ -3820,7 +3820,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>46152.9375</v>
+        <v>46153.9375</v>
       </c>
       <c r="B72" t="n">
         <v>0</v>
@@ -3867,7 +3867,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46152.94791666666</v>
+        <v>46153.94791666666</v>
       </c>
       <c r="B73" t="n">
         <v>0</v>
@@ -3914,7 +3914,7 @@
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>46152.95833333334</v>
+        <v>46153.95833333334</v>
       </c>
       <c r="B74" t="n">
         <v>0</v>
@@ -3961,7 +3961,7 @@
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>46152.96875</v>
+        <v>46153.96875</v>
       </c>
       <c r="B75" t="n">
         <v>0</v>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>46152.97916666666</v>
+        <v>46153.97916666666</v>
       </c>
       <c r="B76" t="n">
         <v>0</v>
@@ -4055,7 +4055,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>46152.98958333334</v>
+        <v>46153.98958333334</v>
       </c>
       <c r="B77" t="n">
         <v>0</v>
@@ -4102,7 +4102,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B78" t="n">
         <v>0</v>
@@ -4149,7 +4149,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>46153.01041666666</v>
+        <v>46154.01041666666</v>
       </c>
       <c r="B79" t="n">
         <v>10</v>
@@ -4196,7 +4196,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>46153.02083333334</v>
+        <v>46154.02083333334</v>
       </c>
       <c r="B80" t="n">
         <v>28</v>
@@ -4243,7 +4243,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>46153.03125</v>
+        <v>46154.03125</v>
       </c>
       <c r="B81" t="n">
         <v>48</v>
@@ -4290,7 +4290,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>46153.04166666666</v>
+        <v>46154.04166666666</v>
       </c>
       <c r="B82" t="n">
         <v>58</v>
@@ -4337,7 +4337,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>46153.05208333334</v>
+        <v>46154.05208333334</v>
       </c>
       <c r="B83" t="n">
         <v>9</v>
@@ -4384,7 +4384,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46153.0625</v>
+        <v>46154.0625</v>
       </c>
       <c r="B84" t="n">
         <v>0</v>
@@ -4431,7 +4431,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46153.07291666666</v>
+        <v>46154.07291666666</v>
       </c>
       <c r="B85" t="n">
         <v>4</v>
@@ -4478,7 +4478,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>46153.08333333334</v>
+        <v>46154.08333333334</v>
       </c>
       <c r="B86" t="n">
         <v>11</v>
@@ -4525,7 +4525,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46153.09375</v>
+        <v>46154.09375</v>
       </c>
       <c r="B87" t="n">
         <v>20</v>
@@ -4572,7 +4572,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>46153.10416666666</v>
+        <v>46154.10416666666</v>
       </c>
       <c r="B88" t="n">
         <v>33</v>
@@ -4619,7 +4619,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>46153.11458333334</v>
+        <v>46154.11458333334</v>
       </c>
       <c r="B89" t="n">
         <v>17</v>
@@ -4666,7 +4666,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46153.125</v>
+        <v>46154.125</v>
       </c>
       <c r="B90" t="n">
         <v>27</v>
@@ -4713,7 +4713,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46153.13541666666</v>
+        <v>46154.13541666666</v>
       </c>
       <c r="B91" t="n">
         <v>41</v>
@@ -4760,7 +4760,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46153.14583333334</v>
+        <v>46154.14583333334</v>
       </c>
       <c r="B92" t="n">
         <v>75</v>
@@ -4807,7 +4807,7 @@
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>46153.15625</v>
+        <v>46154.15625</v>
       </c>
       <c r="B93" t="n">
         <v>268</v>
@@ -4854,7 +4854,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>46153.16666666666</v>
+        <v>46154.16666666666</v>
       </c>
       <c r="B94" t="n">
         <v>527</v>
@@ -4901,7 +4901,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>46153.17708333334</v>
+        <v>46154.17708333334</v>
       </c>
       <c r="B95" t="n">
         <v>888</v>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46153.1875</v>
+        <v>46154.1875</v>
       </c>
       <c r="B96" t="n">
         <v>1032</v>
@@ -4995,7 +4995,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>46153.19791666666</v>
+        <v>46154.19791666666</v>
       </c>
       <c r="B97" t="n">
         <v>780</v>
@@ -5042,7 +5042,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46153.20833333334</v>
+        <v>46154.20833333334</v>
       </c>
       <c r="B98" t="n">
         <v>847</v>
@@ -5089,7 +5089,7 @@
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>46153.21875</v>
+        <v>46154.21875</v>
       </c>
       <c r="B99" t="n">
         <v>689</v>
@@ -5136,7 +5136,7 @@
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>46153.22916666666</v>
+        <v>46154.22916666666</v>
       </c>
       <c r="B100" t="n">
         <v>660</v>
@@ -5183,7 +5183,7 @@
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>46153.23958333334</v>
+        <v>46154.23958333334</v>
       </c>
       <c r="B101" t="n">
         <v>671</v>
@@ -5230,7 +5230,7 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>46153.25</v>
+        <v>46154.25</v>
       </c>
       <c r="B102" t="n">
         <v>627</v>
@@ -5277,7 +5277,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>46153.26041666666</v>
+        <v>46154.26041666666</v>
       </c>
       <c r="B103" t="n">
         <v>513</v>
@@ -5324,7 +5324,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>46153.27083333334</v>
+        <v>46154.27083333334</v>
       </c>
       <c r="B104" t="n">
         <v>544</v>
@@ -5371,7 +5371,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>46153.28125</v>
+        <v>46154.28125</v>
       </c>
       <c r="B105" t="n">
         <v>417</v>
@@ -5418,7 +5418,7 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>46153.29166666666</v>
+        <v>46154.29166666666</v>
       </c>
       <c r="B106" t="n">
         <v>285</v>
@@ -5465,7 +5465,7 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>46153.30208333334</v>
+        <v>46154.30208333334</v>
       </c>
       <c r="B107" t="n">
         <v>290</v>
@@ -5512,7 +5512,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>46153.3125</v>
+        <v>46154.3125</v>
       </c>
       <c r="B108" t="n">
         <v>323</v>
@@ -5559,7 +5559,7 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>46153.32291666666</v>
+        <v>46154.32291666666</v>
       </c>
       <c r="B109" t="n">
         <v>271</v>
@@ -5606,7 +5606,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>46153.33333333334</v>
+        <v>46154.33333333334</v>
       </c>
       <c r="B110" t="n">
         <v>246</v>
@@ -5653,7 +5653,7 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>46153.34375</v>
+        <v>46154.34375</v>
       </c>
       <c r="B111" t="n">
         <v>287</v>
@@ -5700,7 +5700,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>46153.35416666666</v>
+        <v>46154.35416666666</v>
       </c>
       <c r="B112" t="n">
         <v>275</v>
@@ -5747,7 +5747,7 @@
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>46153.36458333334</v>
+        <v>46154.36458333334</v>
       </c>
       <c r="B113" t="n">
         <v>447</v>
@@ -5794,7 +5794,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>46153.375</v>
+        <v>46154.375</v>
       </c>
       <c r="B114" t="n">
         <v>566</v>
@@ -5841,7 +5841,7 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>46153.38541666666</v>
+        <v>46154.38541666666</v>
       </c>
       <c r="B115" t="n">
         <v>590</v>
@@ -5888,7 +5888,7 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>46153.39583333334</v>
+        <v>46154.39583333334</v>
       </c>
       <c r="B116" t="n">
         <v>558</v>
@@ -5935,7 +5935,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>46153.40625</v>
+        <v>46154.40625</v>
       </c>
       <c r="B117" t="n">
         <v>354</v>
@@ -5982,7 +5982,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>46153.41666666666</v>
+        <v>46154.41666666666</v>
       </c>
       <c r="B118" t="n">
         <v>483</v>
@@ -6029,7 +6029,7 @@
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>46153.42708333334</v>
+        <v>46154.42708333334</v>
       </c>
       <c r="B119" t="n">
         <v>537</v>
@@ -6076,7 +6076,7 @@
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>46153.4375</v>
+        <v>46154.4375</v>
       </c>
       <c r="B120" t="n">
         <v>558</v>
@@ -6123,7 +6123,7 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46153.44791666666</v>
+        <v>46154.44791666666</v>
       </c>
       <c r="B121" t="n">
         <v>570</v>
@@ -6170,7 +6170,7 @@
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46153.45833333334</v>
+        <v>46154.45833333334</v>
       </c>
       <c r="B122" t="n">
         <v>424</v>
@@ -6217,7 +6217,7 @@
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>46153.46875</v>
+        <v>46154.46875</v>
       </c>
       <c r="B123" t="n">
         <v>377</v>
@@ -6264,7 +6264,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>46153.47916666666</v>
+        <v>46154.47916666666</v>
       </c>
       <c r="B124" t="n">
         <v>372</v>
@@ -6311,7 +6311,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>46153.48958333334</v>
+        <v>46154.48958333334</v>
       </c>
       <c r="B125" t="n">
         <v>374</v>
@@ -6358,7 +6358,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46153.5</v>
+        <v>46154.5</v>
       </c>
       <c r="B126" t="n">
         <v>508</v>
@@ -6405,7 +6405,7 @@
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>46153.51041666666</v>
+        <v>46154.51041666666</v>
       </c>
       <c r="B127" t="n">
         <v>482</v>
@@ -6452,7 +6452,7 @@
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>46153.52083333334</v>
+        <v>46154.52083333334</v>
       </c>
       <c r="B128" t="n">
         <v>416</v>
@@ -6499,7 +6499,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46153.53125</v>
+        <v>46154.53125</v>
       </c>
       <c r="B129" t="n">
         <v>498</v>
@@ -6546,7 +6546,7 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>46153.54166666666</v>
+        <v>46154.54166666666</v>
       </c>
       <c r="B130" t="n">
         <v>378</v>
@@ -6593,7 +6593,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>46153.55208333334</v>
+        <v>46154.55208333334</v>
       </c>
       <c r="B131" t="n">
         <v>245</v>
@@ -6640,7 +6640,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>46153.5625</v>
+        <v>46154.5625</v>
       </c>
       <c r="B132" t="n">
         <v>253</v>
@@ -6687,7 +6687,7 @@
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>46153.57291666666</v>
+        <v>46154.57291666666</v>
       </c>
       <c r="B133" t="n">
         <v>302</v>
@@ -6734,7 +6734,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>46153.58333333334</v>
+        <v>46154.58333333334</v>
       </c>
       <c r="B134" t="n">
         <v>405</v>
@@ -6781,7 +6781,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>46153.59375</v>
+        <v>46154.59375</v>
       </c>
       <c r="B135" t="n">
         <v>472</v>
@@ -6828,7 +6828,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46153.60416666666</v>
+        <v>46154.60416666666</v>
       </c>
       <c r="B136" t="n">
         <v>591</v>
@@ -6875,7 +6875,7 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46153.61458333334</v>
+        <v>46154.61458333334</v>
       </c>
       <c r="B137" t="n">
         <v>607</v>
@@ -6922,7 +6922,7 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46153.625</v>
+        <v>46154.625</v>
       </c>
       <c r="B138" t="n">
         <v>441</v>
@@ -6969,7 +6969,7 @@
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46153.63541666666</v>
+        <v>46154.63541666666</v>
       </c>
       <c r="B139" t="n">
         <v>309</v>
@@ -7016,7 +7016,7 @@
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46153.64583333334</v>
+        <v>46154.64583333334</v>
       </c>
       <c r="B140" t="n">
         <v>406</v>
@@ -7063,7 +7063,7 @@
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46153.65625</v>
+        <v>46154.65625</v>
       </c>
       <c r="B141" t="n">
         <v>545</v>
@@ -7110,7 +7110,7 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46153.66666666666</v>
+        <v>46154.66666666666</v>
       </c>
       <c r="B142" t="n">
         <v>659</v>
@@ -7157,7 +7157,7 @@
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46153.67708333334</v>
+        <v>46154.67708333334</v>
       </c>
       <c r="B143" t="n">
         <v>904</v>
@@ -7204,7 +7204,7 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46153.6875</v>
+        <v>46154.6875</v>
       </c>
       <c r="B144" t="n">
         <v>870</v>
@@ -7251,7 +7251,7 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46153.69791666666</v>
+        <v>46154.69791666666</v>
       </c>
       <c r="B145" t="n">
         <v>773</v>
@@ -7298,7 +7298,7 @@
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>46153.70833333334</v>
+        <v>46154.70833333334</v>
       </c>
       <c r="B146" t="n">
         <v>654</v>
@@ -7345,7 +7345,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>46153.71875</v>
+        <v>46154.71875</v>
       </c>
       <c r="B147" t="n">
         <v>472</v>
@@ -7392,7 +7392,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>46153.72916666666</v>
+        <v>46154.72916666666</v>
       </c>
       <c r="B148" t="n">
         <v>483</v>
@@ -7439,7 +7439,7 @@
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>46153.73958333334</v>
+        <v>46154.73958333334</v>
       </c>
       <c r="B149" t="n">
         <v>597</v>
@@ -7486,7 +7486,7 @@
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46153.75</v>
+        <v>46154.75</v>
       </c>
       <c r="B150" t="n">
         <v>597</v>
@@ -7533,7 +7533,7 @@
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>46153.76041666666</v>
+        <v>46154.76041666666</v>
       </c>
       <c r="B151" t="n">
         <v>569</v>
@@ -7580,7 +7580,7 @@
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>46153.77083333334</v>
+        <v>46154.77083333334</v>
       </c>
       <c r="B152" t="n">
         <v>423</v>
@@ -7627,7 +7627,7 @@
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>46153.78125</v>
+        <v>46154.78125</v>
       </c>
       <c r="B153" t="n">
         <v>269</v>
@@ -7674,7 +7674,7 @@
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>46153.79166666666</v>
+        <v>46154.79166666666</v>
       </c>
       <c r="B154" t="n">
         <v>312</v>
@@ -7721,7 +7721,7 @@
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>46153.80208333334</v>
+        <v>46154.80208333334</v>
       </c>
       <c r="B155" t="n">
         <v>557</v>
@@ -7768,7 +7768,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>46153.8125</v>
+        <v>46154.8125</v>
       </c>
       <c r="B156" t="n">
         <v>690</v>
@@ -7815,7 +7815,7 @@
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>46153.82291666666</v>
+        <v>46154.82291666666</v>
       </c>
       <c r="B157" t="n">
         <v>511</v>
@@ -7862,7 +7862,7 @@
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
-        <v>46153.83333333334</v>
+        <v>46154.83333333334</v>
       </c>
       <c r="B158" t="n">
         <v>188</v>
@@ -7909,7 +7909,7 @@
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
-        <v>46153.84375</v>
+        <v>46154.84375</v>
       </c>
       <c r="B159" t="n">
         <v>204</v>
@@ -7956,7 +7956,7 @@
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
-        <v>46153.85416666666</v>
+        <v>46154.85416666666</v>
       </c>
       <c r="B160" t="n">
         <v>287</v>
@@ -8003,7 +8003,7 @@
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
-        <v>46153.86458333334</v>
+        <v>46154.86458333334</v>
       </c>
       <c r="B161" t="n">
         <v>177</v>
@@ -8050,7 +8050,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>46153.875</v>
+        <v>46154.875</v>
       </c>
       <c r="B162" t="n">
         <v>9</v>
@@ -8097,7 +8097,7 @@
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
-        <v>46153.88541666666</v>
+        <v>46154.88541666666</v>
       </c>
       <c r="B163" t="n">
         <v>0</v>
@@ -8144,7 +8144,7 @@
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
-        <v>46153.89583333334</v>
+        <v>46154.89583333334</v>
       </c>
       <c r="B164" t="n">
         <v>0</v>
@@ -8191,7 +8191,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>46153.90625</v>
+        <v>46154.90625</v>
       </c>
       <c r="B165" t="n">
         <v>15</v>
@@ -8238,7 +8238,7 @@
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
-        <v>46153.91666666666</v>
+        <v>46154.91666666666</v>
       </c>
       <c r="B166" t="n">
         <v>69</v>
@@ -8285,7 +8285,7 @@
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
-        <v>46153.92708333334</v>
+        <v>46154.92708333334</v>
       </c>
       <c r="B167" t="n">
         <v>126</v>
@@ -8332,7 +8332,7 @@
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
-        <v>46153.9375</v>
+        <v>46154.9375</v>
       </c>
       <c r="B168" t="n">
         <v>175</v>
@@ -8379,7 +8379,7 @@
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
-        <v>46153.94791666666</v>
+        <v>46154.94791666666</v>
       </c>
       <c r="B169" t="n">
         <v>82</v>
@@ -8426,7 +8426,7 @@
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
-        <v>46153.95833333334</v>
+        <v>46154.95833333334</v>
       </c>
       <c r="B170" t="n">
         <v>0</v>
@@ -8473,7 +8473,7 @@
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
-        <v>46153.96875</v>
+        <v>46154.96875</v>
       </c>
       <c r="B171" t="n">
         <v>0</v>
@@ -8520,7 +8520,7 @@
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
-        <v>46153.97916666666</v>
+        <v>46154.97916666666</v>
       </c>
       <c r="B172" t="n">
         <v>0</v>
@@ -8567,7 +8567,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>46153.98958333334</v>
+        <v>46154.98958333334</v>
       </c>
       <c r="B173" t="n">
         <v>0</v>
@@ -8614,7 +8614,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B174" t="n">
         <v>0</v>
@@ -8661,7 +8661,7 @@
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
-        <v>46154.01041666666</v>
+        <v>46155.01041666666</v>
       </c>
       <c r="B175" t="n">
         <v>10</v>
@@ -8708,7 +8708,7 @@
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
-        <v>46154.02083333334</v>
+        <v>46155.02083333334</v>
       </c>
       <c r="B176" t="n">
         <v>35</v>
@@ -8755,7 +8755,7 @@
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
-        <v>46154.03125</v>
+        <v>46155.03125</v>
       </c>
       <c r="B177" t="n">
         <v>62</v>
@@ -8802,7 +8802,7 @@
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
-        <v>46154.04166666666</v>
+        <v>46155.04166666666</v>
       </c>
       <c r="B178" t="n">
         <v>80</v>
@@ -8849,7 +8849,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>46154.05208333334</v>
+        <v>46155.05208333334</v>
       </c>
       <c r="B179" t="n">
         <v>27</v>
@@ -8896,7 +8896,7 @@
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
-        <v>46154.0625</v>
+        <v>46155.0625</v>
       </c>
       <c r="B180" t="n">
         <v>0</v>
@@ -8943,7 +8943,7 @@
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
-        <v>46154.07291666666</v>
+        <v>46155.07291666666</v>
       </c>
       <c r="B181" t="n">
         <v>4</v>
@@ -8990,7 +8990,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>46154.08333333334</v>
+        <v>46155.08333333334</v>
       </c>
       <c r="B182" t="n">
         <v>11</v>
@@ -9037,7 +9037,7 @@
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
-        <v>46154.09375</v>
+        <v>46155.09375</v>
       </c>
       <c r="B183" t="n">
         <v>20</v>
@@ -9084,7 +9084,7 @@
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
-        <v>46154.10416666666</v>
+        <v>46155.10416666666</v>
       </c>
       <c r="B184" t="n">
         <v>33</v>
@@ -9131,7 +9131,7 @@
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
-        <v>46154.11458333334</v>
+        <v>46155.11458333334</v>
       </c>
       <c r="B185" t="n">
         <v>17</v>
@@ -9178,7 +9178,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>46154.125</v>
+        <v>46155.125</v>
       </c>
       <c r="B186" t="n">
         <v>19</v>
@@ -9225,7 +9225,7 @@
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
-        <v>46154.13541666666</v>
+        <v>46155.13541666666</v>
       </c>
       <c r="B187" t="n">
         <v>26</v>
@@ -9272,7 +9272,7 @@
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
-        <v>46154.14583333334</v>
+        <v>46155.14583333334</v>
       </c>
       <c r="B188" t="n">
         <v>65</v>
@@ -9319,7 +9319,7 @@
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
-        <v>46154.15625</v>
+        <v>46155.15625</v>
       </c>
       <c r="B189" t="n">
         <v>256</v>
@@ -9366,7 +9366,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>46154.16666666666</v>
+        <v>46155.16666666666</v>
       </c>
       <c r="B190" t="n">
         <v>528</v>
@@ -9413,7 +9413,7 @@
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
-        <v>46154.17708333334</v>
+        <v>46155.17708333334</v>
       </c>
       <c r="B191" t="n">
         <v>850</v>
@@ -9460,7 +9460,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>46154.1875</v>
+        <v>46155.1875</v>
       </c>
       <c r="B192" t="n">
         <v>967</v>
@@ -9507,7 +9507,7 @@
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
-        <v>46154.19791666666</v>
+        <v>46155.19791666666</v>
       </c>
       <c r="B193" t="n">
         <v>755</v>
@@ -9554,7 +9554,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>46154.20833333334</v>
+        <v>46155.20833333334</v>
       </c>
       <c r="B194" t="n">
         <v>800</v>
@@ -9601,7 +9601,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>46154.21875</v>
+        <v>46155.21875</v>
       </c>
       <c r="B195" t="n">
         <v>656</v>
@@ -9648,7 +9648,7 @@
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
-        <v>46154.22916666666</v>
+        <v>46155.22916666666</v>
       </c>
       <c r="B196" t="n">
         <v>515</v>
@@ -9695,7 +9695,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>46154.23958333334</v>
+        <v>46155.23958333334</v>
       </c>
       <c r="B197" t="n">
         <v>474</v>
@@ -9742,7 +9742,7 @@
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
-        <v>46154.25</v>
+        <v>46155.25</v>
       </c>
       <c r="B198" t="n">
         <v>601</v>
@@ -9789,7 +9789,7 @@
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
-        <v>46154.26041666666</v>
+        <v>46155.26041666666</v>
       </c>
       <c r="B199" t="n">
         <v>632</v>
@@ -9836,7 +9836,7 @@
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
-        <v>46154.27083333334</v>
+        <v>46155.27083333334</v>
       </c>
       <c r="B200" t="n">
         <v>592</v>
@@ -9883,7 +9883,7 @@
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
-        <v>46154.28125</v>
+        <v>46155.28125</v>
       </c>
       <c r="B201" t="n">
         <v>493</v>
@@ -9930,7 +9930,7 @@
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
-        <v>46154.29166666666</v>
+        <v>46155.29166666666</v>
       </c>
       <c r="B202" t="n">
         <v>448</v>
@@ -9977,7 +9977,7 @@
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
-        <v>46154.30208333334</v>
+        <v>46155.30208333334</v>
       </c>
       <c r="B203" t="n">
         <v>459</v>
@@ -10024,7 +10024,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>46154.3125</v>
+        <v>46155.3125</v>
       </c>
       <c r="B204" t="n">
         <v>432</v>
@@ -10071,7 +10071,7 @@
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
-        <v>46154.32291666666</v>
+        <v>46155.32291666666</v>
       </c>
       <c r="B205" t="n">
         <v>368</v>
@@ -10118,7 +10118,7 @@
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
-        <v>46154.33333333334</v>
+        <v>46155.33333333334</v>
       </c>
       <c r="B206" t="n">
         <v>320</v>
@@ -10165,7 +10165,7 @@
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
-        <v>46154.34375</v>
+        <v>46155.34375</v>
       </c>
       <c r="B207" t="n">
         <v>237</v>
@@ -10212,7 +10212,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>46154.35416666666</v>
+        <v>46155.35416666666</v>
       </c>
       <c r="B208" t="n">
         <v>262</v>
@@ -10259,7 +10259,7 @@
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">
-        <v>46154.36458333334</v>
+        <v>46155.36458333334</v>
       </c>
       <c r="B209" t="n">
         <v>445</v>
@@ -10306,7 +10306,7 @@
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
-        <v>46154.375</v>
+        <v>46155.375</v>
       </c>
       <c r="B210" t="n">
         <v>627</v>
@@ -10353,7 +10353,7 @@
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
-        <v>46154.38541666666</v>
+        <v>46155.38541666666</v>
       </c>
       <c r="B211" t="n">
         <v>623</v>
@@ -10400,7 +10400,7 @@
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
-        <v>46154.39583333334</v>
+        <v>46155.39583333334</v>
       </c>
       <c r="B212" t="n">
         <v>576</v>
@@ -10447,7 +10447,7 @@
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
-        <v>46154.40625</v>
+        <v>46155.40625</v>
       </c>
       <c r="B213" t="n">
         <v>542</v>
@@ -10494,7 +10494,7 @@
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
-        <v>46154.41666666666</v>
+        <v>46155.41666666666</v>
       </c>
       <c r="B214" t="n">
         <v>484</v>
@@ -10541,7 +10541,7 @@
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
-        <v>46154.42708333334</v>
+        <v>46155.42708333334</v>
       </c>
       <c r="B215" t="n">
         <v>377</v>
@@ -10588,7 +10588,7 @@
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
-        <v>46154.4375</v>
+        <v>46155.4375</v>
       </c>
       <c r="B216" t="n">
         <v>281</v>
@@ -10635,7 +10635,7 @@
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
-        <v>46154.44791666666</v>
+        <v>46155.44791666666</v>
       </c>
       <c r="B217" t="n">
         <v>386</v>
@@ -10682,7 +10682,7 @@
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
-        <v>46154.45833333334</v>
+        <v>46155.45833333334</v>
       </c>
       <c r="B218" t="n">
         <v>548</v>
@@ -10729,7 +10729,7 @@
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
-        <v>46154.46875</v>
+        <v>46155.46875</v>
       </c>
       <c r="B219" t="n">
         <v>620</v>
@@ -10776,7 +10776,7 @@
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
-        <v>46154.47916666666</v>
+        <v>46155.47916666666</v>
       </c>
       <c r="B220" t="n">
         <v>531</v>
@@ -10823,7 +10823,7 @@
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
-        <v>46154.48958333334</v>
+        <v>46155.48958333334</v>
       </c>
       <c r="B221" t="n">
         <v>491</v>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
-        <v>46154.5</v>
+        <v>46155.5</v>
       </c>
       <c r="B222" t="n">
         <v>385</v>
@@ -10917,7 +10917,7 @@
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
-        <v>46154.51041666666</v>
+        <v>46155.51041666666</v>
       </c>
       <c r="B223" t="n">
         <v>397</v>
@@ -10964,7 +10964,7 @@
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
-        <v>46154.52083333334</v>
+        <v>46155.52083333334</v>
       </c>
       <c r="B224" t="n">
         <v>490</v>
@@ -11011,7 +11011,7 @@
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
-        <v>46154.53125</v>
+        <v>46155.53125</v>
       </c>
       <c r="B225" t="n">
         <v>547</v>
@@ -11058,7 +11058,7 @@
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
-        <v>46154.54166666666</v>
+        <v>46155.54166666666</v>
       </c>
       <c r="B226" t="n">
         <v>415</v>
@@ -11105,7 +11105,7 @@
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
-        <v>46154.55208333334</v>
+        <v>46155.55208333334</v>
       </c>
       <c r="B227" t="n">
         <v>228</v>
@@ -11152,7 +11152,7 @@
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
-        <v>46154.5625</v>
+        <v>46155.5625</v>
       </c>
       <c r="B228" t="n">
         <v>309</v>
@@ -11199,7 +11199,7 @@
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
-        <v>46154.57291666666</v>
+        <v>46155.57291666666</v>
       </c>
       <c r="B229" t="n">
         <v>411</v>
@@ -11246,7 +11246,7 @@
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
-        <v>46154.58333333334</v>
+        <v>46155.58333333334</v>
       </c>
       <c r="B230" t="n">
         <v>385</v>
@@ -11293,7 +11293,7 @@
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
-        <v>46154.59375</v>
+        <v>46155.59375</v>
       </c>
       <c r="B231" t="n">
         <v>436</v>
@@ -11340,7 +11340,7 @@
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
-        <v>46154.60416666666</v>
+        <v>46155.60416666666</v>
       </c>
       <c r="B232" t="n">
         <v>446</v>
@@ -11387,7 +11387,7 @@
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
-        <v>46154.61458333334</v>
+        <v>46155.61458333334</v>
       </c>
       <c r="B233" t="n">
         <v>426</v>
@@ -11434,7 +11434,7 @@
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
-        <v>46154.625</v>
+        <v>46155.625</v>
       </c>
       <c r="B234" t="n">
         <v>450</v>
@@ -11481,7 +11481,7 @@
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
-        <v>46154.63541666666</v>
+        <v>46155.63541666666</v>
       </c>
       <c r="B235" t="n">
         <v>322</v>
@@ -11528,7 +11528,7 @@
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
-        <v>46154.64583333334</v>
+        <v>46155.64583333334</v>
       </c>
       <c r="B236" t="n">
         <v>303</v>
@@ -11575,7 +11575,7 @@
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
-        <v>46154.65625</v>
+        <v>46155.65625</v>
       </c>
       <c r="B237" t="n">
         <v>496</v>
@@ -11622,7 +11622,7 @@
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
-        <v>46154.66666666666</v>
+        <v>46155.66666666666</v>
       </c>
       <c r="B238" t="n">
         <v>654</v>
@@ -11669,7 +11669,7 @@
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
-        <v>46154.67708333334</v>
+        <v>46155.67708333334</v>
       </c>
       <c r="B239" t="n">
         <v>781</v>
@@ -11716,7 +11716,7 @@
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
-        <v>46154.6875</v>
+        <v>46155.6875</v>
       </c>
       <c r="B240" t="n">
         <v>795</v>
@@ -11763,7 +11763,7 @@
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
-        <v>46154.69791666666</v>
+        <v>46155.69791666666</v>
       </c>
       <c r="B241" t="n">
         <v>569</v>
@@ -11810,7 +11810,7 @@
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
-        <v>46154.70833333334</v>
+        <v>46155.70833333334</v>
       </c>
       <c r="B242" t="n">
         <v>611</v>
@@ -11857,7 +11857,7 @@
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
-        <v>46154.71875</v>
+        <v>46155.71875</v>
       </c>
       <c r="B243" t="n">
         <v>794</v>
@@ -11904,7 +11904,7 @@
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
-        <v>46154.72916666666</v>
+        <v>46155.72916666666</v>
       </c>
       <c r="B244" t="n">
         <v>635</v>
@@ -11951,7 +11951,7 @@
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
-        <v>46154.73958333334</v>
+        <v>46155.73958333334</v>
       </c>
       <c r="B245" t="n">
         <v>642</v>
@@ -11998,7 +11998,7 @@
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
-        <v>46154.75</v>
+        <v>46155.75</v>
       </c>
       <c r="B246" t="n">
         <v>624</v>
@@ -12045,7 +12045,7 @@
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
-        <v>46154.76041666666</v>
+        <v>46155.76041666666</v>
       </c>
       <c r="B247" t="n">
         <v>608</v>
@@ -12092,7 +12092,7 @@
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
-        <v>46154.77083333334</v>
+        <v>46155.77083333334</v>
       </c>
       <c r="B248" t="n">
         <v>656</v>
@@ -12139,7 +12139,7 @@
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
-        <v>46154.78125</v>
+        <v>46155.78125</v>
       </c>
       <c r="B249" t="n">
         <v>512</v>
@@ -12186,7 +12186,7 @@
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
-        <v>46154.79166666666</v>
+        <v>46155.79166666666</v>
       </c>
       <c r="B250" t="n">
         <v>323</v>
@@ -12233,7 +12233,7 @@
     </row>
     <row r="251">
       <c r="A251" s="1" t="n">
-        <v>46154.80208333334</v>
+        <v>46155.80208333334</v>
       </c>
       <c r="B251" t="n">
         <v>438</v>
@@ -12280,7 +12280,7 @@
     </row>
     <row r="252">
       <c r="A252" s="1" t="n">
-        <v>46154.8125</v>
+        <v>46155.8125</v>
       </c>
       <c r="B252" t="n">
         <v>613</v>
@@ -12327,7 +12327,7 @@
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
-        <v>46154.82291666666</v>
+        <v>46155.82291666666</v>
       </c>
       <c r="B253" t="n">
         <v>547</v>
@@ -12374,7 +12374,7 @@
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
-        <v>46154.83333333334</v>
+        <v>46155.83333333334</v>
       </c>
       <c r="B254" t="n">
         <v>402</v>
@@ -12421,7 +12421,7 @@
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
-        <v>46154.84375</v>
+        <v>46155.84375</v>
       </c>
       <c r="B255" t="n">
         <v>341</v>
@@ -12468,7 +12468,7 @@
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
-        <v>46154.85416666666</v>
+        <v>46155.85416666666</v>
       </c>
       <c r="B256" t="n">
         <v>264</v>
@@ -12515,7 +12515,7 @@
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
-        <v>46154.86458333334</v>
+        <v>46155.86458333334</v>
       </c>
       <c r="B257" t="n">
         <v>116</v>
@@ -12562,7 +12562,7 @@
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
-        <v>46154.875</v>
+        <v>46155.875</v>
       </c>
       <c r="B258" t="n">
         <v>0</v>
@@ -12609,7 +12609,7 @@
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
-        <v>46154.88541666666</v>
+        <v>46155.88541666666</v>
       </c>
       <c r="B259" t="n">
         <v>10</v>
@@ -12656,7 +12656,7 @@
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
-        <v>46154.89583333334</v>
+        <v>46155.89583333334</v>
       </c>
       <c r="B260" t="n">
         <v>39</v>
@@ -12703,7 +12703,7 @@
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
-        <v>46154.90625</v>
+        <v>46155.90625</v>
       </c>
       <c r="B261" t="n">
         <v>109</v>
@@ -12750,7 +12750,7 @@
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
-        <v>46154.91666666666</v>
+        <v>46155.91666666666</v>
       </c>
       <c r="B262" t="n">
         <v>193</v>
@@ -12797,7 +12797,7 @@
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
-        <v>46154.92708333334</v>
+        <v>46155.92708333334</v>
       </c>
       <c r="B263" t="n">
         <v>217</v>
@@ -12844,7 +12844,7 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>46154.9375</v>
+        <v>46155.9375</v>
       </c>
       <c r="B264" t="n">
         <v>185</v>
@@ -12891,7 +12891,7 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>46154.94791666666</v>
+        <v>46155.94791666666</v>
       </c>
       <c r="B265" t="n">
         <v>27</v>
@@ -12938,7 +12938,7 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>46154.95833333334</v>
+        <v>46155.95833333334</v>
       </c>
       <c r="B266" t="n">
         <v>0</v>
@@ -12985,7 +12985,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>46154.96875</v>
+        <v>46155.96875</v>
       </c>
       <c r="B267" t="n">
         <v>0</v>
@@ -13032,7 +13032,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>46154.97916666666</v>
+        <v>46155.97916666666</v>
       </c>
       <c r="B268" t="n">
         <v>0</v>
@@ -13079,7 +13079,7 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>46154.98958333334</v>
+        <v>46155.98958333334</v>
       </c>
       <c r="B269" t="n">
         <v>0</v>
@@ -13126,7 +13126,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B270" t="n">
         <v>0</v>
@@ -13173,7 +13173,7 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>46155.01041666666</v>
+        <v>46156.01041666666</v>
       </c>
       <c r="B271" t="n">
         <v>10</v>
@@ -13220,7 +13220,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>46155.02083333334</v>
+        <v>46156.02083333334</v>
       </c>
       <c r="B272" t="n">
         <v>35</v>
@@ -13267,7 +13267,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>46155.03125</v>
+        <v>46156.03125</v>
       </c>
       <c r="B273" t="n">
         <v>62</v>
@@ -13314,7 +13314,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>46155.04166666666</v>
+        <v>46156.04166666666</v>
       </c>
       <c r="B274" t="n">
         <v>80</v>
@@ -13361,7 +13361,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>46155.05208333334</v>
+        <v>46156.05208333334</v>
       </c>
       <c r="B275" t="n">
         <v>27</v>
@@ -13408,7 +13408,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>46155.0625</v>
+        <v>46156.0625</v>
       </c>
       <c r="B276" t="n">
         <v>0</v>
@@ -13455,7 +13455,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>46155.07291666666</v>
+        <v>46156.07291666666</v>
       </c>
       <c r="B277" t="n">
         <v>4</v>
@@ -13502,7 +13502,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>46155.08333333334</v>
+        <v>46156.08333333334</v>
       </c>
       <c r="B278" t="n">
         <v>11</v>
@@ -13549,7 +13549,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>46155.09375</v>
+        <v>46156.09375</v>
       </c>
       <c r="B279" t="n">
         <v>20</v>
@@ -13596,7 +13596,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>46155.10416666666</v>
+        <v>46156.10416666666</v>
       </c>
       <c r="B280" t="n">
         <v>33</v>
@@ -13643,7 +13643,7 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>46155.11458333334</v>
+        <v>46156.11458333334</v>
       </c>
       <c r="B281" t="n">
         <v>17</v>
@@ -13690,7 +13690,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>46155.125</v>
+        <v>46156.125</v>
       </c>
       <c r="B282" t="n">
         <v>19</v>
@@ -13737,7 +13737,7 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>46155.13541666666</v>
+        <v>46156.13541666666</v>
       </c>
       <c r="B283" t="n">
         <v>26</v>
@@ -13784,7 +13784,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>46155.14583333334</v>
+        <v>46156.14583333334</v>
       </c>
       <c r="B284" t="n">
         <v>65</v>
@@ -13831,7 +13831,7 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>46155.15625</v>
+        <v>46156.15625</v>
       </c>
       <c r="B285" t="n">
         <v>256</v>
@@ -13878,7 +13878,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>46155.16666666666</v>
+        <v>46156.16666666666</v>
       </c>
       <c r="B286" t="n">
         <v>528</v>
@@ -13925,7 +13925,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>46155.17708333334</v>
+        <v>46156.17708333334</v>
       </c>
       <c r="B287" t="n">
         <v>850</v>
@@ -13972,7 +13972,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>46155.1875</v>
+        <v>46156.1875</v>
       </c>
       <c r="B288" t="n">
         <v>967</v>
@@ -14019,7 +14019,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>46155.19791666666</v>
+        <v>46156.19791666666</v>
       </c>
       <c r="B289" t="n">
         <v>755</v>
@@ -14066,7 +14066,7 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>46155.20833333334</v>
+        <v>46156.20833333334</v>
       </c>
       <c r="B290" t="n">
         <v>800</v>
@@ -14113,7 +14113,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>46155.21875</v>
+        <v>46156.21875</v>
       </c>
       <c r="B291" t="n">
         <v>656</v>
@@ -14160,7 +14160,7 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>46155.22916666666</v>
+        <v>46156.22916666666</v>
       </c>
       <c r="B292" t="n">
         <v>515</v>
@@ -14207,7 +14207,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>46155.23958333334</v>
+        <v>46156.23958333334</v>
       </c>
       <c r="B293" t="n">
         <v>474</v>
@@ -14254,7 +14254,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>46155.25</v>
+        <v>46156.25</v>
       </c>
       <c r="B294" t="n">
         <v>601</v>
@@ -14301,7 +14301,7 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>46155.26041666666</v>
+        <v>46156.26041666666</v>
       </c>
       <c r="B295" t="n">
         <v>632</v>
@@ -14348,7 +14348,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>46155.27083333334</v>
+        <v>46156.27083333334</v>
       </c>
       <c r="B296" t="n">
         <v>592</v>
@@ -14395,7 +14395,7 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>46155.28125</v>
+        <v>46156.28125</v>
       </c>
       <c r="B297" t="n">
         <v>493</v>
@@ -14442,7 +14442,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>46155.29166666666</v>
+        <v>46156.29166666666</v>
       </c>
       <c r="B298" t="n">
         <v>448</v>
@@ -14489,7 +14489,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>46155.30208333334</v>
+        <v>46156.30208333334</v>
       </c>
       <c r="B299" t="n">
         <v>459</v>
@@ -14536,7 +14536,7 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>46155.3125</v>
+        <v>46156.3125</v>
       </c>
       <c r="B300" t="n">
         <v>432</v>
@@ -14583,7 +14583,7 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>46155.32291666666</v>
+        <v>46156.32291666666</v>
       </c>
       <c r="B301" t="n">
         <v>368</v>
@@ -14630,7 +14630,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>46155.33333333334</v>
+        <v>46156.33333333334</v>
       </c>
       <c r="B302" t="n">
         <v>320</v>
@@ -14677,7 +14677,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>46155.34375</v>
+        <v>46156.34375</v>
       </c>
       <c r="B303" t="n">
         <v>237</v>
@@ -14724,7 +14724,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>46155.35416666666</v>
+        <v>46156.35416666666</v>
       </c>
       <c r="B304" t="n">
         <v>262</v>
@@ -14771,7 +14771,7 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>46155.36458333334</v>
+        <v>46156.36458333334</v>
       </c>
       <c r="B305" t="n">
         <v>445</v>
@@ -14818,7 +14818,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>46155.375</v>
+        <v>46156.375</v>
       </c>
       <c r="B306" t="n">
         <v>627</v>
@@ -14865,7 +14865,7 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>46155.38541666666</v>
+        <v>46156.38541666666</v>
       </c>
       <c r="B307" t="n">
         <v>623</v>
@@ -14912,7 +14912,7 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>46155.39583333334</v>
+        <v>46156.39583333334</v>
       </c>
       <c r="B308" t="n">
         <v>576</v>
@@ -14959,7 +14959,7 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>46155.40625</v>
+        <v>46156.40625</v>
       </c>
       <c r="B309" t="n">
         <v>542</v>
@@ -15006,7 +15006,7 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
-        <v>46155.41666666666</v>
+        <v>46156.41666666666</v>
       </c>
       <c r="B310" t="n">
         <v>484</v>
@@ -15053,7 +15053,7 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
-        <v>46155.42708333334</v>
+        <v>46156.42708333334</v>
       </c>
       <c r="B311" t="n">
         <v>377</v>
@@ -15100,7 +15100,7 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>46155.4375</v>
+        <v>46156.4375</v>
       </c>
       <c r="B312" t="n">
         <v>281</v>
@@ -15147,7 +15147,7 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>46155.44791666666</v>
+        <v>46156.44791666666</v>
       </c>
       <c r="B313" t="n">
         <v>386</v>
@@ -15194,7 +15194,7 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>46155.45833333334</v>
+        <v>46156.45833333334</v>
       </c>
       <c r="B314" t="n">
         <v>548</v>
@@ -15241,7 +15241,7 @@
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
-        <v>46155.46875</v>
+        <v>46156.46875</v>
       </c>
       <c r="B315" t="n">
         <v>620</v>
@@ -15288,7 +15288,7 @@
     </row>
     <row r="316">
       <c r="A316" s="1" t="n">
-        <v>46155.47916666666</v>
+        <v>46156.47916666666</v>
       </c>
       <c r="B316" t="n">
         <v>531</v>
@@ -15335,7 +15335,7 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>46155.48958333334</v>
+        <v>46156.48958333334</v>
       </c>
       <c r="B317" t="n">
         <v>491</v>
@@ -15382,7 +15382,7 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>46155.5</v>
+        <v>46156.5</v>
       </c>
       <c r="B318" t="n">
         <v>385</v>
@@ -15429,7 +15429,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>46155.51041666666</v>
+        <v>46156.51041666666</v>
       </c>
       <c r="B319" t="n">
         <v>397</v>
@@ -15476,7 +15476,7 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
-        <v>46155.52083333334</v>
+        <v>46156.52083333334</v>
       </c>
       <c r="B320" t="n">
         <v>490</v>
@@ -15523,7 +15523,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>46155.53125</v>
+        <v>46156.53125</v>
       </c>
       <c r="B321" t="n">
         <v>547</v>
@@ -15570,7 +15570,7 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>46155.54166666666</v>
+        <v>46156.54166666666</v>
       </c>
       <c r="B322" t="n">
         <v>415</v>
@@ -15617,7 +15617,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>46155.55208333334</v>
+        <v>46156.55208333334</v>
       </c>
       <c r="B323" t="n">
         <v>228</v>
@@ -15664,7 +15664,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>46155.5625</v>
+        <v>46156.5625</v>
       </c>
       <c r="B324" t="n">
         <v>309</v>
@@ -15711,7 +15711,7 @@
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>46155.57291666666</v>
+        <v>46156.57291666666</v>
       </c>
       <c r="B325" t="n">
         <v>411</v>
@@ -15758,7 +15758,7 @@
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>46155.58333333334</v>
+        <v>46156.58333333334</v>
       </c>
       <c r="B326" t="n">
         <v>385</v>
@@ -15805,7 +15805,7 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>46155.59375</v>
+        <v>46156.59375</v>
       </c>
       <c r="B327" t="n">
         <v>436</v>
@@ -15852,7 +15852,7 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>46155.60416666666</v>
+        <v>46156.60416666666</v>
       </c>
       <c r="B328" t="n">
         <v>446</v>
@@ -15899,7 +15899,7 @@
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
-        <v>46155.61458333334</v>
+        <v>46156.61458333334</v>
       </c>
       <c r="B329" t="n">
         <v>426</v>
@@ -15946,7 +15946,7 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>46155.625</v>
+        <v>46156.625</v>
       </c>
       <c r="B330" t="n">
         <v>450</v>
@@ -15993,7 +15993,7 @@
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
-        <v>46155.63541666666</v>
+        <v>46156.63541666666</v>
       </c>
       <c r="B331" t="n">
         <v>322</v>
@@ -16040,7 +16040,7 @@
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
-        <v>46155.64583333334</v>
+        <v>46156.64583333334</v>
       </c>
       <c r="B332" t="n">
         <v>303</v>
@@ -16087,7 +16087,7 @@
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
-        <v>46155.65625</v>
+        <v>46156.65625</v>
       </c>
       <c r="B333" t="n">
         <v>496</v>
@@ -16134,7 +16134,7 @@
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
-        <v>46155.66666666666</v>
+        <v>46156.66666666666</v>
       </c>
       <c r="B334" t="n">
         <v>654</v>
@@ -16181,7 +16181,7 @@
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
-        <v>46155.67708333334</v>
+        <v>46156.67708333334</v>
       </c>
       <c r="B335" t="n">
         <v>781</v>
@@ -16228,7 +16228,7 @@
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
-        <v>46155.6875</v>
+        <v>46156.6875</v>
       </c>
       <c r="B336" t="n">
         <v>795</v>
@@ -16275,7 +16275,7 @@
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
-        <v>46155.69791666666</v>
+        <v>46156.69791666666</v>
       </c>
       <c r="B337" t="n">
         <v>569</v>
@@ -16322,7 +16322,7 @@
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
-        <v>46155.70833333334</v>
+        <v>46156.70833333334</v>
       </c>
       <c r="B338" t="n">
         <v>611</v>
@@ -16369,7 +16369,7 @@
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
-        <v>46155.71875</v>
+        <v>46156.71875</v>
       </c>
       <c r="B339" t="n">
         <v>794</v>
@@ -16416,7 +16416,7 @@
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
-        <v>46155.72916666666</v>
+        <v>46156.72916666666</v>
       </c>
       <c r="B340" t="n">
         <v>635</v>
@@ -16463,7 +16463,7 @@
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
-        <v>46155.73958333334</v>
+        <v>46156.73958333334</v>
       </c>
       <c r="B341" t="n">
         <v>642</v>
@@ -16510,7 +16510,7 @@
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
-        <v>46155.75</v>
+        <v>46156.75</v>
       </c>
       <c r="B342" t="n">
         <v>624</v>
@@ -16557,7 +16557,7 @@
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
-        <v>46155.76041666666</v>
+        <v>46156.76041666666</v>
       </c>
       <c r="B343" t="n">
         <v>608</v>
@@ -16604,7 +16604,7 @@
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
-        <v>46155.77083333334</v>
+        <v>46156.77083333334</v>
       </c>
       <c r="B344" t="n">
         <v>656</v>
@@ -16651,7 +16651,7 @@
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
-        <v>46155.78125</v>
+        <v>46156.78125</v>
       </c>
       <c r="B345" t="n">
         <v>512</v>
@@ -16698,7 +16698,7 @@
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
-        <v>46155.79166666666</v>
+        <v>46156.79166666666</v>
       </c>
       <c r="B346" t="n">
         <v>323</v>
@@ -16745,7 +16745,7 @@
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
-        <v>46155.80208333334</v>
+        <v>46156.80208333334</v>
       </c>
       <c r="B347" t="n">
         <v>438</v>
@@ -16792,7 +16792,7 @@
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
-        <v>46155.8125</v>
+        <v>46156.8125</v>
       </c>
       <c r="B348" t="n">
         <v>613</v>
@@ -16839,7 +16839,7 @@
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
-        <v>46155.82291666666</v>
+        <v>46156.82291666666</v>
       </c>
       <c r="B349" t="n">
         <v>547</v>
@@ -16886,7 +16886,7 @@
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
-        <v>46155.83333333334</v>
+        <v>46156.83333333334</v>
       </c>
       <c r="B350" t="n">
         <v>402</v>
@@ -16933,7 +16933,7 @@
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
-        <v>46155.84375</v>
+        <v>46156.84375</v>
       </c>
       <c r="B351" t="n">
         <v>341</v>
@@ -16980,7 +16980,7 @@
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
-        <v>46155.85416666666</v>
+        <v>46156.85416666666</v>
       </c>
       <c r="B352" t="n">
         <v>264</v>
@@ -17027,7 +17027,7 @@
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
-        <v>46155.86458333334</v>
+        <v>46156.86458333334</v>
       </c>
       <c r="B353" t="n">
         <v>116</v>
@@ -17074,7 +17074,7 @@
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
-        <v>46155.875</v>
+        <v>46156.875</v>
       </c>
       <c r="B354" t="n">
         <v>0</v>
@@ -17121,7 +17121,7 @@
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
-        <v>46155.88541666666</v>
+        <v>46156.88541666666</v>
       </c>
       <c r="B355" t="n">
         <v>10</v>
@@ -17168,7 +17168,7 @@
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
-        <v>46155.89583333334</v>
+        <v>46156.89583333334</v>
       </c>
       <c r="B356" t="n">
         <v>39</v>
@@ -17215,7 +17215,7 @@
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
-        <v>46155.90625</v>
+        <v>46156.90625</v>
       </c>
       <c r="B357" t="n">
         <v>109</v>
@@ -17262,7 +17262,7 @@
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
-        <v>46155.91666666666</v>
+        <v>46156.91666666666</v>
       </c>
       <c r="B358" t="n">
         <v>193</v>
@@ -17309,7 +17309,7 @@
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
-        <v>46155.92708333334</v>
+        <v>46156.92708333334</v>
       </c>
       <c r="B359" t="n">
         <v>217</v>
@@ -17356,7 +17356,7 @@
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
-        <v>46155.9375</v>
+        <v>46156.9375</v>
       </c>
       <c r="B360" t="n">
         <v>185</v>
@@ -17403,7 +17403,7 @@
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
-        <v>46155.94791666666</v>
+        <v>46156.94791666666</v>
       </c>
       <c r="B361" t="n">
         <v>27</v>
@@ -17450,7 +17450,7 @@
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
-        <v>46155.95833333334</v>
+        <v>46156.95833333334</v>
       </c>
       <c r="B362" t="n">
         <v>0</v>
@@ -17497,7 +17497,7 @@
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
-        <v>46155.96875</v>
+        <v>46156.96875</v>
       </c>
       <c r="B363" t="n">
         <v>0</v>
@@ -17544,7 +17544,7 @@
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
-        <v>46155.97916666666</v>
+        <v>46156.97916666666</v>
       </c>
       <c r="B364" t="n">
         <v>0</v>
@@ -17591,7 +17591,7 @@
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
-        <v>46155.98958333334</v>
+        <v>46156.98958333334</v>
       </c>
       <c r="B365" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Refactor staff schedule data and update forecast and historical passenger data
- Updated staff schedule CSV to include additional dates and employee shifts.
- Rearranged forecast passenger results for 2026 to correct date alignment.
- Adjusted historical passenger data to ensure chronological order and accuracy.
- Modified short term passenger demand script to integrate data from an Excel file.
- Enhanced CSS styles for better visual distinction of data categories.
- Updated JavaScript to display peak week start date correctly in KPI section.
</commit_message>
<xml_diff>
--- a/data/short term PAX.xlsx
+++ b/data/short term PAX.xlsx
@@ -1225,7 +1225,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" s="5">
       <c r="A2" s="3" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>0</v>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="3" ht="16" customHeight="1" s="5">
       <c r="A3" s="3" t="n">
-        <v>46154.01041666666</v>
+        <v>46155.01041666666</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>10</v>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="4" ht="16" customHeight="1" s="5">
       <c r="A4" s="3" t="n">
-        <v>46154.02083333334</v>
+        <v>46155.02083333334</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>28</v>
@@ -1366,7 +1366,7 @@
     </row>
     <row r="5" ht="16" customHeight="1" s="5">
       <c r="A5" s="3" t="n">
-        <v>46154.03125</v>
+        <v>46155.03125</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>48</v>
@@ -1413,7 +1413,7 @@
     </row>
     <row r="6" ht="16" customHeight="1" s="5">
       <c r="A6" s="3" t="n">
-        <v>46154.04166666666</v>
+        <v>46155.04166666666</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>58</v>
@@ -1460,7 +1460,7 @@
     </row>
     <row r="7" ht="16" customHeight="1" s="5">
       <c r="A7" s="3" t="n">
-        <v>46154.05208333334</v>
+        <v>46155.05208333334</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>9</v>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="8" ht="16" customHeight="1" s="5">
       <c r="A8" s="3" t="n">
-        <v>46154.0625</v>
+        <v>46155.0625</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="9" ht="16" customHeight="1" s="5">
       <c r="A9" s="3" t="n">
-        <v>46154.07291666666</v>
+        <v>46155.07291666666</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>4</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="10" ht="16" customHeight="1" s="5">
       <c r="A10" s="3" t="n">
-        <v>46154.08333333334</v>
+        <v>46155.08333333334</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>11</v>
@@ -1648,7 +1648,7 @@
     </row>
     <row r="11" ht="16" customHeight="1" s="5">
       <c r="A11" s="3" t="n">
-        <v>46154.09375</v>
+        <v>46155.09375</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>20</v>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="12" ht="16" customHeight="1" s="5">
       <c r="A12" s="3" t="n">
-        <v>46154.10416666666</v>
+        <v>46155.10416666666</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>33</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="13" ht="16" customHeight="1" s="5">
       <c r="A13" s="3" t="n">
-        <v>46154.11458333334</v>
+        <v>46155.11458333334</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>17</v>
@@ -1789,7 +1789,7 @@
     </row>
     <row r="14" ht="16" customHeight="1" s="5">
       <c r="A14" s="3" t="n">
-        <v>46154.125</v>
+        <v>46155.125</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>27</v>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="15" ht="16" customHeight="1" s="5">
       <c r="A15" s="3" t="n">
-        <v>46154.13541666666</v>
+        <v>46155.13541666666</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>41</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="16" ht="16" customHeight="1" s="5">
       <c r="A16" s="3" t="n">
-        <v>46154.14583333334</v>
+        <v>46155.14583333334</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>75</v>
@@ -1930,7 +1930,7 @@
     </row>
     <row r="17" ht="16" customHeight="1" s="5">
       <c r="A17" s="3" t="n">
-        <v>46154.15625</v>
+        <v>46155.15625</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>268</v>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="18" ht="16" customHeight="1" s="5">
       <c r="A18" s="3" t="n">
-        <v>46154.16666666666</v>
+        <v>46155.16666666666</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>527</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="19" ht="16" customHeight="1" s="5">
       <c r="A19" s="3" t="n">
-        <v>46154.17708333334</v>
+        <v>46155.17708333334</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>888</v>
@@ -2071,7 +2071,7 @@
     </row>
     <row r="20" ht="16" customHeight="1" s="5">
       <c r="A20" s="3" t="n">
-        <v>46154.1875</v>
+        <v>46155.1875</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>1032</v>
@@ -2118,7 +2118,7 @@
     </row>
     <row r="21" ht="16" customHeight="1" s="5">
       <c r="A21" s="3" t="n">
-        <v>46154.19791666666</v>
+        <v>46155.19791666666</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>780</v>
@@ -2165,7 +2165,7 @@
     </row>
     <row r="22" ht="16" customHeight="1" s="5">
       <c r="A22" s="3" t="n">
-        <v>46154.20833333334</v>
+        <v>46155.20833333334</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>0</v>
@@ -2212,7 +2212,7 @@
     </row>
     <row r="23" ht="16" customHeight="1" s="5">
       <c r="A23" s="3" t="n">
-        <v>46154.21875</v>
+        <v>46155.21875</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>0</v>
@@ -2259,7 +2259,7 @@
     </row>
     <row r="24" ht="16" customHeight="1" s="5">
       <c r="A24" s="3" t="n">
-        <v>46154.22916666666</v>
+        <v>46155.22916666666</v>
       </c>
       <c r="B24" s="4" t="n">
         <v>0</v>
@@ -2306,7 +2306,7 @@
     </row>
     <row r="25" ht="16" customHeight="1" s="5">
       <c r="A25" s="3" t="n">
-        <v>46154.23958333334</v>
+        <v>46155.23958333334</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>1</v>
@@ -2353,7 +2353,7 @@
     </row>
     <row r="26" ht="16" customHeight="1" s="5">
       <c r="A26" s="3" t="n">
-        <v>46154.25</v>
+        <v>46155.25</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>27</v>
@@ -2400,7 +2400,7 @@
     </row>
     <row r="27" ht="16" customHeight="1" s="5">
       <c r="A27" s="3" t="n">
-        <v>46154.26041666666</v>
+        <v>46155.26041666666</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>82</v>
@@ -2447,7 +2447,7 @@
     </row>
     <row r="28" ht="16" customHeight="1" s="5">
       <c r="A28" s="3" t="n">
-        <v>46154.27083333334</v>
+        <v>46155.27083333334</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>180</v>
@@ -2494,7 +2494,7 @@
     </row>
     <row r="29" ht="16" customHeight="1" s="5">
       <c r="A29" s="3" t="n">
-        <v>46154.28125</v>
+        <v>46155.28125</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>275</v>
@@ -2541,7 +2541,7 @@
     </row>
     <row r="30" ht="16" customHeight="1" s="5">
       <c r="A30" s="3" t="n">
-        <v>46154.29166666666</v>
+        <v>46155.29166666666</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>342</v>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="31" ht="16" customHeight="1" s="5">
       <c r="A31" s="3" t="n">
-        <v>46154.30208333334</v>
+        <v>46155.30208333334</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>327</v>
@@ -2635,7 +2635,7 @@
     </row>
     <row r="32" ht="16" customHeight="1" s="5">
       <c r="A32" s="3" t="n">
-        <v>46154.3125</v>
+        <v>46155.3125</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>386</v>
@@ -2682,7 +2682,7 @@
     </row>
     <row r="33" ht="16" customHeight="1" s="5">
       <c r="A33" s="3" t="n">
-        <v>46154.32291666666</v>
+        <v>46155.32291666666</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>401</v>
@@ -2729,7 +2729,7 @@
     </row>
     <row r="34" ht="16" customHeight="1" s="5">
       <c r="A34" s="3" t="n">
-        <v>46154.33333333334</v>
+        <v>46155.33333333334</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>399</v>
@@ -2776,7 +2776,7 @@
     </row>
     <row r="35" ht="16" customHeight="1" s="5">
       <c r="A35" s="3" t="n">
-        <v>46154.34375</v>
+        <v>46155.34375</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>384</v>
@@ -2823,7 +2823,7 @@
     </row>
     <row r="36" ht="16" customHeight="1" s="5">
       <c r="A36" s="3" t="n">
-        <v>46154.35416666666</v>
+        <v>46155.35416666666</v>
       </c>
       <c r="B36" s="4" t="n">
         <v>438</v>
@@ -2870,7 +2870,7 @@
     </row>
     <row r="37" ht="16" customHeight="1" s="5">
       <c r="A37" s="3" t="n">
-        <v>46154.36458333334</v>
+        <v>46155.36458333334</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>433</v>
@@ -2917,7 +2917,7 @@
     </row>
     <row r="38" ht="16" customHeight="1" s="5">
       <c r="A38" s="3" t="n">
-        <v>46154.375</v>
+        <v>46155.375</v>
       </c>
       <c r="B38" s="4" t="n">
         <v>398</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="39" ht="16" customHeight="1" s="5">
       <c r="A39" s="3" t="n">
-        <v>46154.38541666666</v>
+        <v>46155.38541666666</v>
       </c>
       <c r="B39" s="4" t="n">
         <v>463</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="40" ht="16" customHeight="1" s="5">
       <c r="A40" s="3" t="n">
-        <v>46154.39583333334</v>
+        <v>46155.39583333334</v>
       </c>
       <c r="B40" s="4" t="n">
         <v>422</v>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="41" ht="16" customHeight="1" s="5">
       <c r="A41" s="3" t="n">
-        <v>46154.40625</v>
+        <v>46155.40625</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>448</v>
@@ -3105,7 +3105,7 @@
     </row>
     <row r="42" ht="16" customHeight="1" s="5">
       <c r="A42" s="3" t="n">
-        <v>46154.41666666666</v>
+        <v>46155.41666666666</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>603</v>
@@ -3152,7 +3152,7 @@
     </row>
     <row r="43" ht="16" customHeight="1" s="5">
       <c r="A43" s="3" t="n">
-        <v>46154.42708333334</v>
+        <v>46155.42708333334</v>
       </c>
       <c r="B43" s="4" t="n">
         <v>621</v>
@@ -3199,7 +3199,7 @@
     </row>
     <row r="44" ht="16" customHeight="1" s="5">
       <c r="A44" s="3" t="n">
-        <v>46154.4375</v>
+        <v>46155.4375</v>
       </c>
       <c r="B44" s="4" t="n">
         <v>521</v>
@@ -3246,7 +3246,7 @@
     </row>
     <row r="45" ht="16" customHeight="1" s="5">
       <c r="A45" s="3" t="n">
-        <v>46154.44791666666</v>
+        <v>46155.44791666666</v>
       </c>
       <c r="B45" s="4" t="n">
         <v>392</v>
@@ -3293,7 +3293,7 @@
     </row>
     <row r="46" ht="16" customHeight="1" s="5">
       <c r="A46" s="3" t="n">
-        <v>46154.45833333334</v>
+        <v>46155.45833333334</v>
       </c>
       <c r="B46" s="4" t="n">
         <v>358</v>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="47" ht="16" customHeight="1" s="5">
       <c r="A47" s="3" t="n">
-        <v>46154.46875</v>
+        <v>46155.46875</v>
       </c>
       <c r="B47" s="4" t="n">
         <v>487</v>
@@ -3387,7 +3387,7 @@
     </row>
     <row r="48" ht="16" customHeight="1" s="5">
       <c r="A48" s="3" t="n">
-        <v>46154.47916666666</v>
+        <v>46155.47916666666</v>
       </c>
       <c r="B48" s="4" t="n">
         <v>557</v>
@@ -3434,7 +3434,7 @@
     </row>
     <row r="49" ht="16" customHeight="1" s="5">
       <c r="A49" s="3" t="n">
-        <v>46154.48958333334</v>
+        <v>46155.48958333334</v>
       </c>
       <c r="B49" s="4" t="n">
         <v>565</v>
@@ -3481,7 +3481,7 @@
     </row>
     <row r="50" ht="16" customHeight="1" s="5">
       <c r="A50" s="3" t="n">
-        <v>46154.5</v>
+        <v>46155.5</v>
       </c>
       <c r="B50" s="4" t="n">
         <v>387</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="51" ht="16" customHeight="1" s="5">
       <c r="A51" s="3" t="n">
-        <v>46154.51041666666</v>
+        <v>46155.51041666666</v>
       </c>
       <c r="B51" s="4" t="n">
         <v>227</v>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="52" ht="16" customHeight="1" s="5">
       <c r="A52" s="3" t="n">
-        <v>46154.52083333334</v>
+        <v>46155.52083333334</v>
       </c>
       <c r="B52" s="4" t="n">
         <v>382</v>
@@ -3622,7 +3622,7 @@
     </row>
     <row r="53" ht="16" customHeight="1" s="5">
       <c r="A53" s="3" t="n">
-        <v>46154.53125</v>
+        <v>46155.53125</v>
       </c>
       <c r="B53" s="4" t="n">
         <v>612</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="54" ht="16" customHeight="1" s="5">
       <c r="A54" s="3" t="n">
-        <v>46154.54166666666</v>
+        <v>46155.54166666666</v>
       </c>
       <c r="B54" s="4" t="n">
         <v>699</v>
@@ -3716,7 +3716,7 @@
     </row>
     <row r="55" ht="16" customHeight="1" s="5">
       <c r="A55" s="3" t="n">
-        <v>46154.55208333334</v>
+        <v>46155.55208333334</v>
       </c>
       <c r="B55" s="4" t="n">
         <v>627</v>
@@ -3763,7 +3763,7 @@
     </row>
     <row r="56" ht="16" customHeight="1" s="5">
       <c r="A56" s="3" t="n">
-        <v>46154.5625</v>
+        <v>46155.5625</v>
       </c>
       <c r="B56" s="4" t="n">
         <v>538</v>
@@ -3810,7 +3810,7 @@
     </row>
     <row r="57" ht="16" customHeight="1" s="5">
       <c r="A57" s="3" t="n">
-        <v>46154.57291666666</v>
+        <v>46155.57291666666</v>
       </c>
       <c r="B57" s="4" t="n">
         <v>464</v>
@@ -3857,7 +3857,7 @@
     </row>
     <row r="58" ht="16" customHeight="1" s="5">
       <c r="A58" s="3" t="n">
-        <v>46154.58333333334</v>
+        <v>46155.58333333334</v>
       </c>
       <c r="B58" s="4" t="n">
         <v>402</v>
@@ -3904,7 +3904,7 @@
     </row>
     <row r="59" ht="16" customHeight="1" s="5">
       <c r="A59" s="3" t="n">
-        <v>46154.59375</v>
+        <v>46155.59375</v>
       </c>
       <c r="B59" s="4" t="n">
         <v>262</v>
@@ -3951,7 +3951,7 @@
     </row>
     <row r="60" ht="16" customHeight="1" s="5">
       <c r="A60" s="3" t="n">
-        <v>46154.60416666666</v>
+        <v>46155.60416666666</v>
       </c>
       <c r="B60" s="4" t="n">
         <v>228</v>
@@ -3998,7 +3998,7 @@
     </row>
     <row r="61" ht="16" customHeight="1" s="5">
       <c r="A61" s="3" t="n">
-        <v>46154.61458333334</v>
+        <v>46155.61458333334</v>
       </c>
       <c r="B61" s="4" t="n">
         <v>350</v>
@@ -4045,7 +4045,7 @@
     </row>
     <row r="62" ht="16" customHeight="1" s="5">
       <c r="A62" s="3" t="n">
-        <v>46154.625</v>
+        <v>46155.625</v>
       </c>
       <c r="B62" s="4" t="n">
         <v>506</v>
@@ -4092,7 +4092,7 @@
     </row>
     <row r="63" ht="16" customHeight="1" s="5">
       <c r="A63" s="3" t="n">
-        <v>46154.63541666666</v>
+        <v>46155.63541666666</v>
       </c>
       <c r="B63" s="4" t="n">
         <v>530</v>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="64" ht="16" customHeight="1" s="5">
       <c r="A64" s="3" t="n">
-        <v>46154.64583333334</v>
+        <v>46155.64583333334</v>
       </c>
       <c r="B64" s="4" t="n">
         <v>459</v>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="65" ht="16" customHeight="1" s="5">
       <c r="A65" s="3" t="n">
-        <v>46154.65625</v>
+        <v>46155.65625</v>
       </c>
       <c r="B65" s="4" t="n">
         <v>398</v>
@@ -4233,7 +4233,7 @@
     </row>
     <row r="66" ht="16" customHeight="1" s="5">
       <c r="A66" s="3" t="n">
-        <v>46154.66666666666</v>
+        <v>46155.66666666666</v>
       </c>
       <c r="B66" s="4" t="n">
         <v>488</v>
@@ -4280,7 +4280,7 @@
     </row>
     <row r="67" ht="16" customHeight="1" s="5">
       <c r="A67" s="3" t="n">
-        <v>46154.67708333334</v>
+        <v>46155.67708333334</v>
       </c>
       <c r="B67" s="4" t="n">
         <v>532</v>
@@ -4327,7 +4327,7 @@
     </row>
     <row r="68" ht="16" customHeight="1" s="5">
       <c r="A68" s="3" t="n">
-        <v>46154.6875</v>
+        <v>46155.6875</v>
       </c>
       <c r="B68" s="4" t="n">
         <v>716</v>
@@ -4374,7 +4374,7 @@
     </row>
     <row r="69" ht="16" customHeight="1" s="5">
       <c r="A69" s="3" t="n">
-        <v>46154.69791666666</v>
+        <v>46155.69791666666</v>
       </c>
       <c r="B69" s="4" t="n">
         <v>673</v>
@@ -4421,7 +4421,7 @@
     </row>
     <row r="70" ht="16" customHeight="1" s="5">
       <c r="A70" s="3" t="n">
-        <v>46154.70833333334</v>
+        <v>46155.70833333334</v>
       </c>
       <c r="B70" s="4" t="n">
         <v>504</v>
@@ -4468,7 +4468,7 @@
     </row>
     <row r="71" ht="16" customHeight="1" s="5">
       <c r="A71" s="3" t="n">
-        <v>46154.71875</v>
+        <v>46155.71875</v>
       </c>
       <c r="B71" s="4" t="n">
         <v>616</v>
@@ -4515,7 +4515,7 @@
     </row>
     <row r="72" ht="16" customHeight="1" s="5">
       <c r="A72" s="3" t="n">
-        <v>46154.72916666666</v>
+        <v>46155.72916666666</v>
       </c>
       <c r="B72" s="4" t="n">
         <v>569</v>
@@ -4562,7 +4562,7 @@
     </row>
     <row r="73" ht="16" customHeight="1" s="5">
       <c r="A73" s="3" t="n">
-        <v>46154.73958333334</v>
+        <v>46155.73958333334</v>
       </c>
       <c r="B73" s="4" t="n">
         <v>619</v>
@@ -4609,7 +4609,7 @@
     </row>
     <row r="74" ht="16" customHeight="1" s="5">
       <c r="A74" s="3" t="n">
-        <v>46154.75</v>
+        <v>46155.75</v>
       </c>
       <c r="B74" s="4" t="n">
         <v>597</v>
@@ -4656,7 +4656,7 @@
     </row>
     <row r="75" ht="16" customHeight="1" s="5">
       <c r="A75" s="3" t="n">
-        <v>46154.76041666666</v>
+        <v>46155.76041666666</v>
       </c>
       <c r="B75" s="4" t="n">
         <v>373</v>
@@ -4703,7 +4703,7 @@
     </row>
     <row r="76" ht="16" customHeight="1" s="5">
       <c r="A76" s="3" t="n">
-        <v>46154.77083333334</v>
+        <v>46155.77083333334</v>
       </c>
       <c r="B76" s="4" t="n">
         <v>298</v>
@@ -4750,7 +4750,7 @@
     </row>
     <row r="77" ht="16" customHeight="1" s="5">
       <c r="A77" s="3" t="n">
-        <v>46154.78125</v>
+        <v>46155.78125</v>
       </c>
       <c r="B77" s="4" t="n">
         <v>325</v>
@@ -4797,7 +4797,7 @@
     </row>
     <row r="78" ht="16" customHeight="1" s="5">
       <c r="A78" s="3" t="n">
-        <v>46154.79166666666</v>
+        <v>46155.79166666666</v>
       </c>
       <c r="B78" s="4" t="n">
         <v>350</v>
@@ -4844,7 +4844,7 @@
     </row>
     <row r="79" ht="16" customHeight="1" s="5">
       <c r="A79" s="3" t="n">
-        <v>46154.80208333334</v>
+        <v>46155.80208333334</v>
       </c>
       <c r="B79" s="4" t="n">
         <v>373</v>
@@ -4891,7 +4891,7 @@
     </row>
     <row r="80" ht="16" customHeight="1" s="5">
       <c r="A80" s="3" t="n">
-        <v>46154.8125</v>
+        <v>46155.8125</v>
       </c>
       <c r="B80" s="4" t="n">
         <v>344</v>
@@ -4938,7 +4938,7 @@
     </row>
     <row r="81" ht="16" customHeight="1" s="5">
       <c r="A81" s="3" t="n">
-        <v>46154.82291666666</v>
+        <v>46155.82291666666</v>
       </c>
       <c r="B81" s="4" t="n">
         <v>385</v>
@@ -4985,7 +4985,7 @@
     </row>
     <row r="82" ht="16" customHeight="1" s="5">
       <c r="A82" s="3" t="n">
-        <v>46154.83333333334</v>
+        <v>46155.83333333334</v>
       </c>
       <c r="B82" s="4" t="n">
         <v>439</v>
@@ -5032,7 +5032,7 @@
     </row>
     <row r="83" ht="16" customHeight="1" s="5">
       <c r="A83" s="3" t="n">
-        <v>46154.84375</v>
+        <v>46155.84375</v>
       </c>
       <c r="B83" s="4" t="n">
         <v>408</v>
@@ -5079,7 +5079,7 @@
     </row>
     <row r="84" ht="16" customHeight="1" s="5">
       <c r="A84" s="3" t="n">
-        <v>46154.85416666666</v>
+        <v>46155.85416666666</v>
       </c>
       <c r="B84" s="4" t="n">
         <v>319</v>
@@ -5126,7 +5126,7 @@
     </row>
     <row r="85" ht="16" customHeight="1" s="5">
       <c r="A85" s="3" t="n">
-        <v>46154.86458333334</v>
+        <v>46155.86458333334</v>
       </c>
       <c r="B85" s="4" t="n">
         <v>166</v>
@@ -5173,7 +5173,7 @@
     </row>
     <row r="86" ht="16" customHeight="1" s="5">
       <c r="A86" s="3" t="n">
-        <v>46154.875</v>
+        <v>46155.875</v>
       </c>
       <c r="B86" s="4" t="n">
         <v>29</v>
@@ -5220,7 +5220,7 @@
     </row>
     <row r="87" ht="16" customHeight="1" s="5">
       <c r="A87" s="3" t="n">
-        <v>46154.88541666666</v>
+        <v>46155.88541666666</v>
       </c>
       <c r="B87" s="4" t="n">
         <v>61</v>
@@ -5267,7 +5267,7 @@
     </row>
     <row r="88" ht="16" customHeight="1" s="5">
       <c r="A88" s="3" t="n">
-        <v>46154.89583333334</v>
+        <v>46155.89583333334</v>
       </c>
       <c r="B88" s="4" t="n">
         <v>107</v>
@@ -5314,7 +5314,7 @@
     </row>
     <row r="89" ht="16" customHeight="1" s="5">
       <c r="A89" s="3" t="n">
-        <v>46154.90625</v>
+        <v>46155.90625</v>
       </c>
       <c r="B89" s="4" t="n">
         <v>93</v>
@@ -5361,7 +5361,7 @@
     </row>
     <row r="90" ht="16" customHeight="1" s="5">
       <c r="A90" s="3" t="n">
-        <v>46154.91666666666</v>
+        <v>46155.91666666666</v>
       </c>
       <c r="B90" s="4" t="n">
         <v>115</v>
@@ -5408,7 +5408,7 @@
     </row>
     <row r="91" ht="16" customHeight="1" s="5">
       <c r="A91" s="3" t="n">
-        <v>46154.92708333334</v>
+        <v>46155.92708333334</v>
       </c>
       <c r="B91" s="4" t="n">
         <v>58</v>
@@ -5455,7 +5455,7 @@
     </row>
     <row r="92" ht="16" customHeight="1" s="5">
       <c r="A92" s="3" t="n">
-        <v>46154.9375</v>
+        <v>46155.9375</v>
       </c>
       <c r="B92" s="4" t="n">
         <v>0</v>
@@ -5502,7 +5502,7 @@
     </row>
     <row r="93" ht="16" customHeight="1" s="5">
       <c r="A93" s="3" t="n">
-        <v>46154.94791666666</v>
+        <v>46155.94791666666</v>
       </c>
       <c r="B93" s="4" t="n">
         <v>0</v>
@@ -5549,7 +5549,7 @@
     </row>
     <row r="94" ht="16" customHeight="1" s="5">
       <c r="A94" s="3" t="n">
-        <v>46154.95833333334</v>
+        <v>46155.95833333334</v>
       </c>
       <c r="B94" s="4" t="n">
         <v>0</v>
@@ -5596,7 +5596,7 @@
     </row>
     <row r="95" ht="16" customHeight="1" s="5">
       <c r="A95" s="3" t="n">
-        <v>46154.96875</v>
+        <v>46155.96875</v>
       </c>
       <c r="B95" s="4" t="n">
         <v>0</v>
@@ -5643,7 +5643,7 @@
     </row>
     <row r="96" ht="16" customHeight="1" s="5">
       <c r="A96" s="3" t="n">
-        <v>46154.97916666666</v>
+        <v>46155.97916666666</v>
       </c>
       <c r="B96" s="4" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
     </row>
     <row r="97" ht="16" customHeight="1" s="5">
       <c r="A97" s="3" t="n">
-        <v>46154.98958333334</v>
+        <v>46155.98958333334</v>
       </c>
       <c r="B97" s="4" t="n">
         <v>0</v>
@@ -5737,7 +5737,7 @@
     </row>
     <row r="98" ht="16" customHeight="1" s="5">
       <c r="A98" s="3" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B98" s="4" t="n">
         <v>0</v>
@@ -5784,7 +5784,7 @@
     </row>
     <row r="99" ht="16" customHeight="1" s="5">
       <c r="A99" s="3" t="n">
-        <v>46155.01041666666</v>
+        <v>46156.01041666666</v>
       </c>
       <c r="B99" s="4" t="n">
         <v>10</v>
@@ -5831,7 +5831,7 @@
     </row>
     <row r="100" ht="16" customHeight="1" s="5">
       <c r="A100" s="3" t="n">
-        <v>46155.02083333334</v>
+        <v>46156.02083333334</v>
       </c>
       <c r="B100" s="4" t="n">
         <v>28</v>
@@ -5878,7 +5878,7 @@
     </row>
     <row r="101" ht="16" customHeight="1" s="5">
       <c r="A101" s="3" t="n">
-        <v>46155.03125</v>
+        <v>46156.03125</v>
       </c>
       <c r="B101" s="4" t="n">
         <v>48</v>
@@ -5925,7 +5925,7 @@
     </row>
     <row r="102" ht="16" customHeight="1" s="5">
       <c r="A102" s="3" t="n">
-        <v>46155.04166666666</v>
+        <v>46156.04166666666</v>
       </c>
       <c r="B102" s="4" t="n">
         <v>58</v>
@@ -5972,7 +5972,7 @@
     </row>
     <row r="103" ht="16" customHeight="1" s="5">
       <c r="A103" s="3" t="n">
-        <v>46155.05208333334</v>
+        <v>46156.05208333334</v>
       </c>
       <c r="B103" s="4" t="n">
         <v>9</v>
@@ -6019,7 +6019,7 @@
     </row>
     <row r="104" ht="16" customHeight="1" s="5">
       <c r="A104" s="3" t="n">
-        <v>46155.0625</v>
+        <v>46156.0625</v>
       </c>
       <c r="B104" s="4" t="n">
         <v>0</v>
@@ -6066,7 +6066,7 @@
     </row>
     <row r="105" ht="16" customHeight="1" s="5">
       <c r="A105" s="3" t="n">
-        <v>46155.07291666666</v>
+        <v>46156.07291666666</v>
       </c>
       <c r="B105" s="4" t="n">
         <v>4</v>
@@ -6113,7 +6113,7 @@
     </row>
     <row r="106" ht="16" customHeight="1" s="5">
       <c r="A106" s="3" t="n">
-        <v>46155.08333333334</v>
+        <v>46156.08333333334</v>
       </c>
       <c r="B106" s="4" t="n">
         <v>11</v>
@@ -6160,7 +6160,7 @@
     </row>
     <row r="107" ht="16" customHeight="1" s="5">
       <c r="A107" s="3" t="n">
-        <v>46155.09375</v>
+        <v>46156.09375</v>
       </c>
       <c r="B107" s="4" t="n">
         <v>20</v>
@@ -6207,7 +6207,7 @@
     </row>
     <row r="108" ht="16" customHeight="1" s="5">
       <c r="A108" s="3" t="n">
-        <v>46155.10416666666</v>
+        <v>46156.10416666666</v>
       </c>
       <c r="B108" s="4" t="n">
         <v>33</v>
@@ -6254,7 +6254,7 @@
     </row>
     <row r="109" ht="16" customHeight="1" s="5">
       <c r="A109" s="3" t="n">
-        <v>46155.11458333334</v>
+        <v>46156.11458333334</v>
       </c>
       <c r="B109" s="4" t="n">
         <v>17</v>
@@ -6301,7 +6301,7 @@
     </row>
     <row r="110" ht="16" customHeight="1" s="5">
       <c r="A110" s="3" t="n">
-        <v>46155.125</v>
+        <v>46156.125</v>
       </c>
       <c r="B110" s="4" t="n">
         <v>27</v>
@@ -6348,7 +6348,7 @@
     </row>
     <row r="111" ht="16" customHeight="1" s="5">
       <c r="A111" s="3" t="n">
-        <v>46155.13541666666</v>
+        <v>46156.13541666666</v>
       </c>
       <c r="B111" s="4" t="n">
         <v>41</v>
@@ -6395,7 +6395,7 @@
     </row>
     <row r="112" ht="16" customHeight="1" s="5">
       <c r="A112" s="3" t="n">
-        <v>46155.14583333334</v>
+        <v>46156.14583333334</v>
       </c>
       <c r="B112" s="4" t="n">
         <v>75</v>
@@ -6442,7 +6442,7 @@
     </row>
     <row r="113" ht="16" customHeight="1" s="5">
       <c r="A113" s="3" t="n">
-        <v>46155.15625</v>
+        <v>46156.15625</v>
       </c>
       <c r="B113" s="4" t="n">
         <v>268</v>
@@ -6489,7 +6489,7 @@
     </row>
     <row r="114" ht="16" customHeight="1" s="5">
       <c r="A114" s="3" t="n">
-        <v>46155.16666666666</v>
+        <v>46156.16666666666</v>
       </c>
       <c r="B114" s="4" t="n">
         <v>527</v>
@@ -6536,7 +6536,7 @@
     </row>
     <row r="115" ht="16" customHeight="1" s="5">
       <c r="A115" s="3" t="n">
-        <v>46155.17708333334</v>
+        <v>46156.17708333334</v>
       </c>
       <c r="B115" s="4" t="n">
         <v>888</v>
@@ -6583,7 +6583,7 @@
     </row>
     <row r="116" ht="16" customHeight="1" s="5">
       <c r="A116" s="3" t="n">
-        <v>46155.1875</v>
+        <v>46156.1875</v>
       </c>
       <c r="B116" s="4" t="n">
         <v>1032</v>
@@ -6630,7 +6630,7 @@
     </row>
     <row r="117" ht="16" customHeight="1" s="5">
       <c r="A117" s="3" t="n">
-        <v>46155.19791666666</v>
+        <v>46156.19791666666</v>
       </c>
       <c r="B117" s="4" t="n">
         <v>780</v>
@@ -6677,7 +6677,7 @@
     </row>
     <row r="118" ht="16" customHeight="1" s="5">
       <c r="A118" s="3" t="n">
-        <v>46155.20833333334</v>
+        <v>46156.20833333334</v>
       </c>
       <c r="B118" s="4" t="n">
         <v>847</v>
@@ -6724,7 +6724,7 @@
     </row>
     <row r="119" ht="16" customHeight="1" s="5">
       <c r="A119" s="3" t="n">
-        <v>46155.21875</v>
+        <v>46156.21875</v>
       </c>
       <c r="B119" s="4" t="n">
         <v>689</v>
@@ -6771,7 +6771,7 @@
     </row>
     <row r="120" ht="16" customHeight="1" s="5">
       <c r="A120" s="3" t="n">
-        <v>46155.22916666666</v>
+        <v>46156.22916666666</v>
       </c>
       <c r="B120" s="4" t="n">
         <v>660</v>
@@ -6818,7 +6818,7 @@
     </row>
     <row r="121" ht="16" customHeight="1" s="5">
       <c r="A121" s="3" t="n">
-        <v>46155.23958333334</v>
+        <v>46156.23958333334</v>
       </c>
       <c r="B121" s="4" t="n">
         <v>671</v>
@@ -6865,7 +6865,7 @@
     </row>
     <row r="122" ht="16" customHeight="1" s="5">
       <c r="A122" s="3" t="n">
-        <v>46155.25</v>
+        <v>46156.25</v>
       </c>
       <c r="B122" s="4" t="n">
         <v>627</v>
@@ -6912,7 +6912,7 @@
     </row>
     <row r="123" ht="16" customHeight="1" s="5">
       <c r="A123" s="3" t="n">
-        <v>46155.26041666666</v>
+        <v>46156.26041666666</v>
       </c>
       <c r="B123" s="4" t="n">
         <v>513</v>
@@ -6959,7 +6959,7 @@
     </row>
     <row r="124" ht="16" customHeight="1" s="5">
       <c r="A124" s="3" t="n">
-        <v>46155.27083333334</v>
+        <v>46156.27083333334</v>
       </c>
       <c r="B124" s="4" t="n">
         <v>544</v>
@@ -7006,7 +7006,7 @@
     </row>
     <row r="125" ht="16" customHeight="1" s="5">
       <c r="A125" s="3" t="n">
-        <v>46155.28125</v>
+        <v>46156.28125</v>
       </c>
       <c r="B125" s="4" t="n">
         <v>417</v>
@@ -7053,7 +7053,7 @@
     </row>
     <row r="126" ht="16" customHeight="1" s="5">
       <c r="A126" s="3" t="n">
-        <v>46155.29166666666</v>
+        <v>46156.29166666666</v>
       </c>
       <c r="B126" s="4" t="n">
         <v>285</v>
@@ -7100,7 +7100,7 @@
     </row>
     <row r="127" ht="16" customHeight="1" s="5">
       <c r="A127" s="3" t="n">
-        <v>46155.30208333334</v>
+        <v>46156.30208333334</v>
       </c>
       <c r="B127" s="4" t="n">
         <v>290</v>
@@ -7147,7 +7147,7 @@
     </row>
     <row r="128" ht="16" customHeight="1" s="5">
       <c r="A128" s="3" t="n">
-        <v>46155.3125</v>
+        <v>46156.3125</v>
       </c>
       <c r="B128" s="4" t="n">
         <v>323</v>
@@ -7194,7 +7194,7 @@
     </row>
     <row r="129" ht="16" customHeight="1" s="5">
       <c r="A129" s="3" t="n">
-        <v>46155.32291666666</v>
+        <v>46156.32291666666</v>
       </c>
       <c r="B129" s="4" t="n">
         <v>271</v>
@@ -7241,7 +7241,7 @@
     </row>
     <row r="130" ht="16" customHeight="1" s="5">
       <c r="A130" s="3" t="n">
-        <v>46155.33333333334</v>
+        <v>46156.33333333334</v>
       </c>
       <c r="B130" s="4" t="n">
         <v>246</v>
@@ -7288,7 +7288,7 @@
     </row>
     <row r="131" ht="16" customHeight="1" s="5">
       <c r="A131" s="3" t="n">
-        <v>46155.34375</v>
+        <v>46156.34375</v>
       </c>
       <c r="B131" s="4" t="n">
         <v>287</v>
@@ -7335,7 +7335,7 @@
     </row>
     <row r="132" ht="16" customHeight="1" s="5">
       <c r="A132" s="3" t="n">
-        <v>46155.35416666666</v>
+        <v>46156.35416666666</v>
       </c>
       <c r="B132" s="4" t="n">
         <v>275</v>
@@ -7382,7 +7382,7 @@
     </row>
     <row r="133" ht="16" customHeight="1" s="5">
       <c r="A133" s="3" t="n">
-        <v>46155.36458333334</v>
+        <v>46156.36458333334</v>
       </c>
       <c r="B133" s="4" t="n">
         <v>447</v>
@@ -7429,7 +7429,7 @@
     </row>
     <row r="134" ht="16" customHeight="1" s="5">
       <c r="A134" s="3" t="n">
-        <v>46155.375</v>
+        <v>46156.375</v>
       </c>
       <c r="B134" s="4" t="n">
         <v>566</v>
@@ -7476,7 +7476,7 @@
     </row>
     <row r="135" ht="16" customHeight="1" s="5">
       <c r="A135" s="3" t="n">
-        <v>46155.38541666666</v>
+        <v>46156.38541666666</v>
       </c>
       <c r="B135" s="4" t="n">
         <v>590</v>
@@ -7523,7 +7523,7 @@
     </row>
     <row r="136" ht="16" customHeight="1" s="5">
       <c r="A136" s="3" t="n">
-        <v>46155.39583333334</v>
+        <v>46156.39583333334</v>
       </c>
       <c r="B136" s="4" t="n">
         <v>558</v>
@@ -7570,7 +7570,7 @@
     </row>
     <row r="137" ht="16" customHeight="1" s="5">
       <c r="A137" s="3" t="n">
-        <v>46155.40625</v>
+        <v>46156.40625</v>
       </c>
       <c r="B137" s="4" t="n">
         <v>354</v>
@@ -7617,7 +7617,7 @@
     </row>
     <row r="138" ht="16" customHeight="1" s="5">
       <c r="A138" s="3" t="n">
-        <v>46155.41666666666</v>
+        <v>46156.41666666666</v>
       </c>
       <c r="B138" s="4" t="n">
         <v>483</v>
@@ -7664,7 +7664,7 @@
     </row>
     <row r="139" ht="16" customHeight="1" s="5">
       <c r="A139" s="3" t="n">
-        <v>46155.42708333334</v>
+        <v>46156.42708333334</v>
       </c>
       <c r="B139" s="4" t="n">
         <v>537</v>
@@ -7711,7 +7711,7 @@
     </row>
     <row r="140" ht="16" customHeight="1" s="5">
       <c r="A140" s="3" t="n">
-        <v>46155.4375</v>
+        <v>46156.4375</v>
       </c>
       <c r="B140" s="4" t="n">
         <v>558</v>
@@ -7758,7 +7758,7 @@
     </row>
     <row r="141" ht="16" customHeight="1" s="5">
       <c r="A141" s="3" t="n">
-        <v>46155.44791666666</v>
+        <v>46156.44791666666</v>
       </c>
       <c r="B141" s="4" t="n">
         <v>570</v>
@@ -7805,7 +7805,7 @@
     </row>
     <row r="142" ht="16" customHeight="1" s="5">
       <c r="A142" s="3" t="n">
-        <v>46155.45833333334</v>
+        <v>46156.45833333334</v>
       </c>
       <c r="B142" s="4" t="n">
         <v>424</v>
@@ -7852,7 +7852,7 @@
     </row>
     <row r="143" ht="16" customHeight="1" s="5">
       <c r="A143" s="3" t="n">
-        <v>46155.46875</v>
+        <v>46156.46875</v>
       </c>
       <c r="B143" s="4" t="n">
         <v>377</v>
@@ -7899,7 +7899,7 @@
     </row>
     <row r="144" ht="16" customHeight="1" s="5">
       <c r="A144" s="3" t="n">
-        <v>46155.47916666666</v>
+        <v>46156.47916666666</v>
       </c>
       <c r="B144" s="4" t="n">
         <v>372</v>
@@ -7946,7 +7946,7 @@
     </row>
     <row r="145" ht="16" customHeight="1" s="5">
       <c r="A145" s="3" t="n">
-        <v>46155.48958333334</v>
+        <v>46156.48958333334</v>
       </c>
       <c r="B145" s="4" t="n">
         <v>374</v>
@@ -7993,7 +7993,7 @@
     </row>
     <row r="146" ht="16" customHeight="1" s="5">
       <c r="A146" s="3" t="n">
-        <v>46155.5</v>
+        <v>46156.5</v>
       </c>
       <c r="B146" s="4" t="n">
         <v>508</v>
@@ -8040,7 +8040,7 @@
     </row>
     <row r="147" ht="16" customHeight="1" s="5">
       <c r="A147" s="3" t="n">
-        <v>46155.51041666666</v>
+        <v>46156.51041666666</v>
       </c>
       <c r="B147" s="4" t="n">
         <v>482</v>
@@ -8087,7 +8087,7 @@
     </row>
     <row r="148" ht="16" customHeight="1" s="5">
       <c r="A148" s="3" t="n">
-        <v>46155.52083333334</v>
+        <v>46156.52083333334</v>
       </c>
       <c r="B148" s="4" t="n">
         <v>416</v>
@@ -8134,7 +8134,7 @@
     </row>
     <row r="149" ht="16" customHeight="1" s="5">
       <c r="A149" s="3" t="n">
-        <v>46155.53125</v>
+        <v>46156.53125</v>
       </c>
       <c r="B149" s="4" t="n">
         <v>498</v>
@@ -8181,7 +8181,7 @@
     </row>
     <row r="150" ht="16" customHeight="1" s="5">
       <c r="A150" s="3" t="n">
-        <v>46155.54166666666</v>
+        <v>46156.54166666666</v>
       </c>
       <c r="B150" s="4" t="n">
         <v>378</v>
@@ -8228,7 +8228,7 @@
     </row>
     <row r="151" ht="16" customHeight="1" s="5">
       <c r="A151" s="3" t="n">
-        <v>46155.55208333334</v>
+        <v>46156.55208333334</v>
       </c>
       <c r="B151" s="4" t="n">
         <v>245</v>
@@ -8275,7 +8275,7 @@
     </row>
     <row r="152" ht="16" customHeight="1" s="5">
       <c r="A152" s="3" t="n">
-        <v>46155.5625</v>
+        <v>46156.5625</v>
       </c>
       <c r="B152" s="4" t="n">
         <v>253</v>
@@ -8322,7 +8322,7 @@
     </row>
     <row r="153" ht="16" customHeight="1" s="5">
       <c r="A153" s="3" t="n">
-        <v>46155.57291666666</v>
+        <v>46156.57291666666</v>
       </c>
       <c r="B153" s="4" t="n">
         <v>302</v>
@@ -8369,7 +8369,7 @@
     </row>
     <row r="154" ht="16" customHeight="1" s="5">
       <c r="A154" s="3" t="n">
-        <v>46155.58333333334</v>
+        <v>46156.58333333334</v>
       </c>
       <c r="B154" s="4" t="n">
         <v>405</v>
@@ -8416,7 +8416,7 @@
     </row>
     <row r="155" ht="16" customHeight="1" s="5">
       <c r="A155" s="3" t="n">
-        <v>46155.59375</v>
+        <v>46156.59375</v>
       </c>
       <c r="B155" s="4" t="n">
         <v>472</v>
@@ -8463,7 +8463,7 @@
     </row>
     <row r="156" ht="16" customHeight="1" s="5">
       <c r="A156" s="3" t="n">
-        <v>46155.60416666666</v>
+        <v>46156.60416666666</v>
       </c>
       <c r="B156" s="4" t="n">
         <v>591</v>
@@ -8510,7 +8510,7 @@
     </row>
     <row r="157" ht="16" customHeight="1" s="5">
       <c r="A157" s="3" t="n">
-        <v>46155.61458333334</v>
+        <v>46156.61458333334</v>
       </c>
       <c r="B157" s="4" t="n">
         <v>607</v>
@@ -8557,7 +8557,7 @@
     </row>
     <row r="158" ht="16" customHeight="1" s="5">
       <c r="A158" s="3" t="n">
-        <v>46155.625</v>
+        <v>46156.625</v>
       </c>
       <c r="B158" s="4" t="n">
         <v>441</v>
@@ -8604,7 +8604,7 @@
     </row>
     <row r="159" ht="16" customHeight="1" s="5">
       <c r="A159" s="3" t="n">
-        <v>46155.63541666666</v>
+        <v>46156.63541666666</v>
       </c>
       <c r="B159" s="4" t="n">
         <v>309</v>
@@ -8651,7 +8651,7 @@
     </row>
     <row r="160" ht="16" customHeight="1" s="5">
       <c r="A160" s="3" t="n">
-        <v>46155.64583333334</v>
+        <v>46156.64583333334</v>
       </c>
       <c r="B160" s="4" t="n">
         <v>406</v>
@@ -8698,7 +8698,7 @@
     </row>
     <row r="161" ht="16" customHeight="1" s="5">
       <c r="A161" s="3" t="n">
-        <v>46155.65625</v>
+        <v>46156.65625</v>
       </c>
       <c r="B161" s="4" t="n">
         <v>545</v>
@@ -8745,7 +8745,7 @@
     </row>
     <row r="162" ht="16" customHeight="1" s="5">
       <c r="A162" s="3" t="n">
-        <v>46155.66666666666</v>
+        <v>46156.66666666666</v>
       </c>
       <c r="B162" s="4" t="n">
         <v>659</v>
@@ -8792,7 +8792,7 @@
     </row>
     <row r="163" ht="16" customHeight="1" s="5">
       <c r="A163" s="3" t="n">
-        <v>46155.67708333334</v>
+        <v>46156.67708333334</v>
       </c>
       <c r="B163" s="4" t="n">
         <v>904</v>
@@ -8839,7 +8839,7 @@
     </row>
     <row r="164" ht="16" customHeight="1" s="5">
       <c r="A164" s="3" t="n">
-        <v>46155.6875</v>
+        <v>46156.6875</v>
       </c>
       <c r="B164" s="4" t="n">
         <v>870</v>
@@ -8886,7 +8886,7 @@
     </row>
     <row r="165" ht="16" customHeight="1" s="5">
       <c r="A165" s="3" t="n">
-        <v>46155.69791666666</v>
+        <v>46156.69791666666</v>
       </c>
       <c r="B165" s="4" t="n">
         <v>773</v>
@@ -8933,7 +8933,7 @@
     </row>
     <row r="166" ht="16" customHeight="1" s="5">
       <c r="A166" s="3" t="n">
-        <v>46155.70833333334</v>
+        <v>46156.70833333334</v>
       </c>
       <c r="B166" s="4" t="n">
         <v>654</v>
@@ -8980,7 +8980,7 @@
     </row>
     <row r="167" ht="16" customHeight="1" s="5">
       <c r="A167" s="3" t="n">
-        <v>46155.71875</v>
+        <v>46156.71875</v>
       </c>
       <c r="B167" s="4" t="n">
         <v>472</v>
@@ -9027,7 +9027,7 @@
     </row>
     <row r="168" ht="16" customHeight="1" s="5">
       <c r="A168" s="3" t="n">
-        <v>46155.72916666666</v>
+        <v>46156.72916666666</v>
       </c>
       <c r="B168" s="4" t="n">
         <v>483</v>
@@ -9074,7 +9074,7 @@
     </row>
     <row r="169" ht="16" customHeight="1" s="5">
       <c r="A169" s="3" t="n">
-        <v>46155.73958333334</v>
+        <v>46156.73958333334</v>
       </c>
       <c r="B169" s="4" t="n">
         <v>597</v>
@@ -9121,7 +9121,7 @@
     </row>
     <row r="170" ht="16" customHeight="1" s="5">
       <c r="A170" s="3" t="n">
-        <v>46155.75</v>
+        <v>46156.75</v>
       </c>
       <c r="B170" s="4" t="n">
         <v>597</v>
@@ -9168,7 +9168,7 @@
     </row>
     <row r="171" ht="16" customHeight="1" s="5">
       <c r="A171" s="3" t="n">
-        <v>46155.76041666666</v>
+        <v>46156.76041666666</v>
       </c>
       <c r="B171" s="4" t="n">
         <v>569</v>
@@ -9215,7 +9215,7 @@
     </row>
     <row r="172" ht="16" customHeight="1" s="5">
       <c r="A172" s="3" t="n">
-        <v>46155.77083333334</v>
+        <v>46156.77083333334</v>
       </c>
       <c r="B172" s="4" t="n">
         <v>423</v>
@@ -9262,7 +9262,7 @@
     </row>
     <row r="173" ht="16" customHeight="1" s="5">
       <c r="A173" s="3" t="n">
-        <v>46155.78125</v>
+        <v>46156.78125</v>
       </c>
       <c r="B173" s="4" t="n">
         <v>269</v>
@@ -9309,7 +9309,7 @@
     </row>
     <row r="174" ht="16" customHeight="1" s="5">
       <c r="A174" s="3" t="n">
-        <v>46155.79166666666</v>
+        <v>46156.79166666666</v>
       </c>
       <c r="B174" s="4" t="n">
         <v>312</v>
@@ -9356,7 +9356,7 @@
     </row>
     <row r="175" ht="16" customHeight="1" s="5">
       <c r="A175" s="3" t="n">
-        <v>46155.80208333334</v>
+        <v>46156.80208333334</v>
       </c>
       <c r="B175" s="4" t="n">
         <v>557</v>
@@ -9403,7 +9403,7 @@
     </row>
     <row r="176" ht="16" customHeight="1" s="5">
       <c r="A176" s="3" t="n">
-        <v>46155.8125</v>
+        <v>46156.8125</v>
       </c>
       <c r="B176" s="4" t="n">
         <v>690</v>
@@ -9450,7 +9450,7 @@
     </row>
     <row r="177" ht="16" customHeight="1" s="5">
       <c r="A177" s="3" t="n">
-        <v>46155.82291666666</v>
+        <v>46156.82291666666</v>
       </c>
       <c r="B177" s="4" t="n">
         <v>511</v>
@@ -9497,7 +9497,7 @@
     </row>
     <row r="178" ht="16" customHeight="1" s="5">
       <c r="A178" s="3" t="n">
-        <v>46155.83333333334</v>
+        <v>46156.83333333334</v>
       </c>
       <c r="B178" s="4" t="n">
         <v>188</v>
@@ -9544,7 +9544,7 @@
     </row>
     <row r="179" ht="16" customHeight="1" s="5">
       <c r="A179" s="3" t="n">
-        <v>46155.84375</v>
+        <v>46156.84375</v>
       </c>
       <c r="B179" s="4" t="n">
         <v>204</v>
@@ -9591,7 +9591,7 @@
     </row>
     <row r="180" ht="16" customHeight="1" s="5">
       <c r="A180" s="3" t="n">
-        <v>46155.85416666666</v>
+        <v>46156.85416666666</v>
       </c>
       <c r="B180" s="4" t="n">
         <v>287</v>
@@ -9638,7 +9638,7 @@
     </row>
     <row r="181" ht="16" customHeight="1" s="5">
       <c r="A181" s="3" t="n">
-        <v>46155.86458333334</v>
+        <v>46156.86458333334</v>
       </c>
       <c r="B181" s="4" t="n">
         <v>177</v>
@@ -9685,7 +9685,7 @@
     </row>
     <row r="182" ht="16" customHeight="1" s="5">
       <c r="A182" s="3" t="n">
-        <v>46155.875</v>
+        <v>46156.875</v>
       </c>
       <c r="B182" s="4" t="n">
         <v>9</v>
@@ -9732,7 +9732,7 @@
     </row>
     <row r="183" ht="16" customHeight="1" s="5">
       <c r="A183" s="3" t="n">
-        <v>46155.88541666666</v>
+        <v>46156.88541666666</v>
       </c>
       <c r="B183" s="4" t="n">
         <v>0</v>
@@ -9779,7 +9779,7 @@
     </row>
     <row r="184" ht="16" customHeight="1" s="5">
       <c r="A184" s="3" t="n">
-        <v>46155.89583333334</v>
+        <v>46156.89583333334</v>
       </c>
       <c r="B184" s="4" t="n">
         <v>0</v>
@@ -9826,7 +9826,7 @@
     </row>
     <row r="185" ht="16" customHeight="1" s="5">
       <c r="A185" s="3" t="n">
-        <v>46155.90625</v>
+        <v>46156.90625</v>
       </c>
       <c r="B185" s="4" t="n">
         <v>15</v>
@@ -9873,7 +9873,7 @@
     </row>
     <row r="186" ht="16" customHeight="1" s="5">
       <c r="A186" s="3" t="n">
-        <v>46155.91666666666</v>
+        <v>46156.91666666666</v>
       </c>
       <c r="B186" s="4" t="n">
         <v>69</v>
@@ -9920,7 +9920,7 @@
     </row>
     <row r="187" ht="16" customHeight="1" s="5">
       <c r="A187" s="3" t="n">
-        <v>46155.92708333334</v>
+        <v>46156.92708333334</v>
       </c>
       <c r="B187" s="4" t="n">
         <v>126</v>
@@ -9967,7 +9967,7 @@
     </row>
     <row r="188" ht="16" customHeight="1" s="5">
       <c r="A188" s="3" t="n">
-        <v>46155.9375</v>
+        <v>46156.9375</v>
       </c>
       <c r="B188" s="4" t="n">
         <v>175</v>
@@ -10014,7 +10014,7 @@
     </row>
     <row r="189" ht="16" customHeight="1" s="5">
       <c r="A189" s="3" t="n">
-        <v>46155.94791666666</v>
+        <v>46156.94791666666</v>
       </c>
       <c r="B189" s="4" t="n">
         <v>82</v>
@@ -10061,7 +10061,7 @@
     </row>
     <row r="190" ht="16" customHeight="1" s="5">
       <c r="A190" s="3" t="n">
-        <v>46155.95833333334</v>
+        <v>46156.95833333334</v>
       </c>
       <c r="B190" s="4" t="n">
         <v>0</v>
@@ -10108,7 +10108,7 @@
     </row>
     <row r="191" ht="16" customHeight="1" s="5">
       <c r="A191" s="3" t="n">
-        <v>46155.96875</v>
+        <v>46156.96875</v>
       </c>
       <c r="B191" s="4" t="n">
         <v>0</v>
@@ -10155,7 +10155,7 @@
     </row>
     <row r="192" ht="16" customHeight="1" s="5">
       <c r="A192" s="3" t="n">
-        <v>46155.97916666666</v>
+        <v>46156.97916666666</v>
       </c>
       <c r="B192" s="4" t="n">
         <v>0</v>
@@ -10202,7 +10202,7 @@
     </row>
     <row r="193" ht="16" customHeight="1" s="5">
       <c r="A193" s="3" t="n">
-        <v>46155.98958333334</v>
+        <v>46156.98958333334</v>
       </c>
       <c r="B193" s="4" t="n">
         <v>0</v>
@@ -10249,7 +10249,7 @@
     </row>
     <row r="194" ht="16" customHeight="1" s="5">
       <c r="A194" s="3" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B194" s="4" t="n">
         <v>0</v>
@@ -10296,7 +10296,7 @@
     </row>
     <row r="195" ht="16" customHeight="1" s="5">
       <c r="A195" s="3" t="n">
-        <v>46156.01041666666</v>
+        <v>46157.01041666666</v>
       </c>
       <c r="B195" s="4" t="n">
         <v>10</v>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="196" ht="16" customHeight="1" s="5">
       <c r="A196" s="3" t="n">
-        <v>46156.02083333334</v>
+        <v>46157.02083333334</v>
       </c>
       <c r="B196" s="4" t="n">
         <v>35</v>
@@ -10390,7 +10390,7 @@
     </row>
     <row r="197" ht="16" customHeight="1" s="5">
       <c r="A197" s="3" t="n">
-        <v>46156.03125</v>
+        <v>46157.03125</v>
       </c>
       <c r="B197" s="4" t="n">
         <v>62</v>
@@ -10437,7 +10437,7 @@
     </row>
     <row r="198" ht="16" customHeight="1" s="5">
       <c r="A198" s="3" t="n">
-        <v>46156.04166666666</v>
+        <v>46157.04166666666</v>
       </c>
       <c r="B198" s="4" t="n">
         <v>80</v>
@@ -10484,7 +10484,7 @@
     </row>
     <row r="199" ht="16" customHeight="1" s="5">
       <c r="A199" s="3" t="n">
-        <v>46156.05208333334</v>
+        <v>46157.05208333334</v>
       </c>
       <c r="B199" s="4" t="n">
         <v>27</v>
@@ -10531,7 +10531,7 @@
     </row>
     <row r="200" ht="16" customHeight="1" s="5">
       <c r="A200" s="3" t="n">
-        <v>46156.0625</v>
+        <v>46157.0625</v>
       </c>
       <c r="B200" s="4" t="n">
         <v>0</v>
@@ -10578,7 +10578,7 @@
     </row>
     <row r="201" ht="16" customHeight="1" s="5">
       <c r="A201" s="3" t="n">
-        <v>46156.07291666666</v>
+        <v>46157.07291666666</v>
       </c>
       <c r="B201" s="4" t="n">
         <v>4</v>
@@ -10625,7 +10625,7 @@
     </row>
     <row r="202" ht="16" customHeight="1" s="5">
       <c r="A202" s="3" t="n">
-        <v>46156.08333333334</v>
+        <v>46157.08333333334</v>
       </c>
       <c r="B202" s="4" t="n">
         <v>11</v>
@@ -10672,7 +10672,7 @@
     </row>
     <row r="203" ht="16" customHeight="1" s="5">
       <c r="A203" s="3" t="n">
-        <v>46156.09375</v>
+        <v>46157.09375</v>
       </c>
       <c r="B203" s="4" t="n">
         <v>20</v>
@@ -10719,7 +10719,7 @@
     </row>
     <row r="204" ht="16" customHeight="1" s="5">
       <c r="A204" s="3" t="n">
-        <v>46156.10416666666</v>
+        <v>46157.10416666666</v>
       </c>
       <c r="B204" s="4" t="n">
         <v>33</v>
@@ -10766,7 +10766,7 @@
     </row>
     <row r="205" ht="16" customHeight="1" s="5">
       <c r="A205" s="3" t="n">
-        <v>46156.11458333334</v>
+        <v>46157.11458333334</v>
       </c>
       <c r="B205" s="4" t="n">
         <v>17</v>
@@ -10813,7 +10813,7 @@
     </row>
     <row r="206" ht="16" customHeight="1" s="5">
       <c r="A206" s="3" t="n">
-        <v>46156.125</v>
+        <v>46157.125</v>
       </c>
       <c r="B206" s="4" t="n">
         <v>19</v>
@@ -10860,7 +10860,7 @@
     </row>
     <row r="207" ht="16" customHeight="1" s="5">
       <c r="A207" s="3" t="n">
-        <v>46156.13541666666</v>
+        <v>46157.13541666666</v>
       </c>
       <c r="B207" s="4" t="n">
         <v>26</v>
@@ -10907,7 +10907,7 @@
     </row>
     <row r="208" ht="16" customHeight="1" s="5">
       <c r="A208" s="3" t="n">
-        <v>46156.14583333334</v>
+        <v>46157.14583333334</v>
       </c>
       <c r="B208" s="4" t="n">
         <v>65</v>
@@ -10954,7 +10954,7 @@
     </row>
     <row r="209" ht="16" customHeight="1" s="5">
       <c r="A209" s="3" t="n">
-        <v>46156.15625</v>
+        <v>46157.15625</v>
       </c>
       <c r="B209" s="4" t="n">
         <v>256</v>
@@ -11001,7 +11001,7 @@
     </row>
     <row r="210" ht="16" customHeight="1" s="5">
       <c r="A210" s="3" t="n">
-        <v>46156.16666666666</v>
+        <v>46157.16666666666</v>
       </c>
       <c r="B210" s="4" t="n">
         <v>528</v>
@@ -11048,7 +11048,7 @@
     </row>
     <row r="211" ht="16" customHeight="1" s="5">
       <c r="A211" s="3" t="n">
-        <v>46156.17708333334</v>
+        <v>46157.17708333334</v>
       </c>
       <c r="B211" s="4" t="n">
         <v>850</v>
@@ -11095,7 +11095,7 @@
     </row>
     <row r="212" ht="16" customHeight="1" s="5">
       <c r="A212" s="3" t="n">
-        <v>46156.1875</v>
+        <v>46157.1875</v>
       </c>
       <c r="B212" s="4" t="n">
         <v>967</v>
@@ -11142,7 +11142,7 @@
     </row>
     <row r="213" ht="16" customHeight="1" s="5">
       <c r="A213" s="3" t="n">
-        <v>46156.19791666666</v>
+        <v>46157.19791666666</v>
       </c>
       <c r="B213" s="4" t="n">
         <v>755</v>
@@ -11189,7 +11189,7 @@
     </row>
     <row r="214" ht="16" customHeight="1" s="5">
       <c r="A214" s="3" t="n">
-        <v>46156.20833333334</v>
+        <v>46157.20833333334</v>
       </c>
       <c r="B214" s="4" t="n">
         <v>800</v>
@@ -11236,7 +11236,7 @@
     </row>
     <row r="215" ht="16" customHeight="1" s="5">
       <c r="A215" s="3" t="n">
-        <v>46156.21875</v>
+        <v>46157.21875</v>
       </c>
       <c r="B215" s="4" t="n">
         <v>656</v>
@@ -11283,7 +11283,7 @@
     </row>
     <row r="216" ht="16" customHeight="1" s="5">
       <c r="A216" s="3" t="n">
-        <v>46156.22916666666</v>
+        <v>46157.22916666666</v>
       </c>
       <c r="B216" s="4" t="n">
         <v>515</v>
@@ -11330,7 +11330,7 @@
     </row>
     <row r="217" ht="16" customHeight="1" s="5">
       <c r="A217" s="3" t="n">
-        <v>46156.23958333334</v>
+        <v>46157.23958333334</v>
       </c>
       <c r="B217" s="4" t="n">
         <v>474</v>
@@ -11377,7 +11377,7 @@
     </row>
     <row r="218" ht="16" customHeight="1" s="5">
       <c r="A218" s="3" t="n">
-        <v>46156.25</v>
+        <v>46157.25</v>
       </c>
       <c r="B218" s="4" t="n">
         <v>601</v>
@@ -11424,7 +11424,7 @@
     </row>
     <row r="219" ht="16" customHeight="1" s="5">
       <c r="A219" s="3" t="n">
-        <v>46156.26041666666</v>
+        <v>46157.26041666666</v>
       </c>
       <c r="B219" s="4" t="n">
         <v>632</v>
@@ -11471,7 +11471,7 @@
     </row>
     <row r="220" ht="16" customHeight="1" s="5">
       <c r="A220" s="3" t="n">
-        <v>46156.27083333334</v>
+        <v>46157.27083333334</v>
       </c>
       <c r="B220" s="4" t="n">
         <v>592</v>
@@ -11518,7 +11518,7 @@
     </row>
     <row r="221" ht="16" customHeight="1" s="5">
       <c r="A221" s="3" t="n">
-        <v>46156.28125</v>
+        <v>46157.28125</v>
       </c>
       <c r="B221" s="4" t="n">
         <v>493</v>
@@ -11565,7 +11565,7 @@
     </row>
     <row r="222" ht="16" customHeight="1" s="5">
       <c r="A222" s="3" t="n">
-        <v>46156.29166666666</v>
+        <v>46157.29166666666</v>
       </c>
       <c r="B222" s="4" t="n">
         <v>448</v>
@@ -11612,7 +11612,7 @@
     </row>
     <row r="223" ht="16" customHeight="1" s="5">
       <c r="A223" s="3" t="n">
-        <v>46156.30208333334</v>
+        <v>46157.30208333334</v>
       </c>
       <c r="B223" s="4" t="n">
         <v>459</v>
@@ -11659,7 +11659,7 @@
     </row>
     <row r="224" ht="16" customHeight="1" s="5">
       <c r="A224" s="3" t="n">
-        <v>46156.3125</v>
+        <v>46157.3125</v>
       </c>
       <c r="B224" s="4" t="n">
         <v>432</v>
@@ -11706,7 +11706,7 @@
     </row>
     <row r="225" ht="16" customHeight="1" s="5">
       <c r="A225" s="3" t="n">
-        <v>46156.32291666666</v>
+        <v>46157.32291666666</v>
       </c>
       <c r="B225" s="4" t="n">
         <v>368</v>
@@ -11753,7 +11753,7 @@
     </row>
     <row r="226" ht="16" customHeight="1" s="5">
       <c r="A226" s="3" t="n">
-        <v>46156.33333333334</v>
+        <v>46157.33333333334</v>
       </c>
       <c r="B226" s="4" t="n">
         <v>320</v>
@@ -11800,7 +11800,7 @@
     </row>
     <row r="227" ht="16" customHeight="1" s="5">
       <c r="A227" s="3" t="n">
-        <v>46156.34375</v>
+        <v>46157.34375</v>
       </c>
       <c r="B227" s="4" t="n">
         <v>237</v>
@@ -11847,7 +11847,7 @@
     </row>
     <row r="228" ht="16" customHeight="1" s="5">
       <c r="A228" s="3" t="n">
-        <v>46156.35416666666</v>
+        <v>46157.35416666666</v>
       </c>
       <c r="B228" s="4" t="n">
         <v>262</v>
@@ -11894,7 +11894,7 @@
     </row>
     <row r="229" ht="16" customHeight="1" s="5">
       <c r="A229" s="3" t="n">
-        <v>46156.36458333334</v>
+        <v>46157.36458333334</v>
       </c>
       <c r="B229" s="4" t="n">
         <v>445</v>
@@ -11941,7 +11941,7 @@
     </row>
     <row r="230" ht="16" customHeight="1" s="5">
       <c r="A230" s="3" t="n">
-        <v>46156.375</v>
+        <v>46157.375</v>
       </c>
       <c r="B230" s="4" t="n">
         <v>627</v>
@@ -11988,7 +11988,7 @@
     </row>
     <row r="231" ht="16" customHeight="1" s="5">
       <c r="A231" s="3" t="n">
-        <v>46156.38541666666</v>
+        <v>46157.38541666666</v>
       </c>
       <c r="B231" s="4" t="n">
         <v>623</v>
@@ -12035,7 +12035,7 @@
     </row>
     <row r="232" ht="16" customHeight="1" s="5">
       <c r="A232" s="3" t="n">
-        <v>46156.39583333334</v>
+        <v>46157.39583333334</v>
       </c>
       <c r="B232" s="4" t="n">
         <v>576</v>
@@ -12082,7 +12082,7 @@
     </row>
     <row r="233" ht="16" customHeight="1" s="5">
       <c r="A233" s="3" t="n">
-        <v>46156.40625</v>
+        <v>46157.40625</v>
       </c>
       <c r="B233" s="4" t="n">
         <v>542</v>
@@ -12129,7 +12129,7 @@
     </row>
     <row r="234" ht="16" customHeight="1" s="5">
       <c r="A234" s="3" t="n">
-        <v>46156.41666666666</v>
+        <v>46157.41666666666</v>
       </c>
       <c r="B234" s="4" t="n">
         <v>484</v>
@@ -12176,7 +12176,7 @@
     </row>
     <row r="235" ht="16" customHeight="1" s="5">
       <c r="A235" s="3" t="n">
-        <v>46156.42708333334</v>
+        <v>46157.42708333334</v>
       </c>
       <c r="B235" s="4" t="n">
         <v>377</v>
@@ -12223,7 +12223,7 @@
     </row>
     <row r="236" ht="16" customHeight="1" s="5">
       <c r="A236" s="3" t="n">
-        <v>46156.4375</v>
+        <v>46157.4375</v>
       </c>
       <c r="B236" s="4" t="n">
         <v>281</v>
@@ -12270,7 +12270,7 @@
     </row>
     <row r="237" ht="16" customHeight="1" s="5">
       <c r="A237" s="3" t="n">
-        <v>46156.44791666666</v>
+        <v>46157.44791666666</v>
       </c>
       <c r="B237" s="4" t="n">
         <v>386</v>
@@ -12317,7 +12317,7 @@
     </row>
     <row r="238" ht="16" customHeight="1" s="5">
       <c r="A238" s="3" t="n">
-        <v>46156.45833333334</v>
+        <v>46157.45833333334</v>
       </c>
       <c r="B238" s="4" t="n">
         <v>548</v>
@@ -12364,7 +12364,7 @@
     </row>
     <row r="239" ht="16" customHeight="1" s="5">
       <c r="A239" s="3" t="n">
-        <v>46156.46875</v>
+        <v>46157.46875</v>
       </c>
       <c r="B239" s="4" t="n">
         <v>620</v>
@@ -12411,7 +12411,7 @@
     </row>
     <row r="240" ht="16" customHeight="1" s="5">
       <c r="A240" s="3" t="n">
-        <v>46156.47916666666</v>
+        <v>46157.47916666666</v>
       </c>
       <c r="B240" s="4" t="n">
         <v>531</v>
@@ -12458,7 +12458,7 @@
     </row>
     <row r="241" ht="16" customHeight="1" s="5">
       <c r="A241" s="3" t="n">
-        <v>46156.48958333334</v>
+        <v>46157.48958333334</v>
       </c>
       <c r="B241" s="4" t="n">
         <v>491</v>
@@ -12505,7 +12505,7 @@
     </row>
     <row r="242" ht="16" customHeight="1" s="5">
       <c r="A242" s="3" t="n">
-        <v>46156.5</v>
+        <v>46157.5</v>
       </c>
       <c r="B242" s="4" t="n">
         <v>385</v>
@@ -12552,7 +12552,7 @@
     </row>
     <row r="243" ht="16" customHeight="1" s="5">
       <c r="A243" s="3" t="n">
-        <v>46156.51041666666</v>
+        <v>46157.51041666666</v>
       </c>
       <c r="B243" s="4" t="n">
         <v>397</v>
@@ -12599,7 +12599,7 @@
     </row>
     <row r="244" ht="16" customHeight="1" s="5">
       <c r="A244" s="3" t="n">
-        <v>46156.52083333334</v>
+        <v>46157.52083333334</v>
       </c>
       <c r="B244" s="4" t="n">
         <v>490</v>
@@ -12646,7 +12646,7 @@
     </row>
     <row r="245" ht="16" customHeight="1" s="5">
       <c r="A245" s="3" t="n">
-        <v>46156.53125</v>
+        <v>46157.53125</v>
       </c>
       <c r="B245" s="4" t="n">
         <v>547</v>
@@ -12693,7 +12693,7 @@
     </row>
     <row r="246" ht="16" customHeight="1" s="5">
       <c r="A246" s="3" t="n">
-        <v>46156.54166666666</v>
+        <v>46157.54166666666</v>
       </c>
       <c r="B246" s="4" t="n">
         <v>415</v>
@@ -12740,7 +12740,7 @@
     </row>
     <row r="247" ht="16" customHeight="1" s="5">
       <c r="A247" s="3" t="n">
-        <v>46156.55208333334</v>
+        <v>46157.55208333334</v>
       </c>
       <c r="B247" s="4" t="n">
         <v>228</v>
@@ -12787,7 +12787,7 @@
     </row>
     <row r="248" ht="16" customHeight="1" s="5">
       <c r="A248" s="3" t="n">
-        <v>46156.5625</v>
+        <v>46157.5625</v>
       </c>
       <c r="B248" s="4" t="n">
         <v>309</v>
@@ -12834,7 +12834,7 @@
     </row>
     <row r="249" ht="16" customHeight="1" s="5">
       <c r="A249" s="3" t="n">
-        <v>46156.57291666666</v>
+        <v>46157.57291666666</v>
       </c>
       <c r="B249" s="4" t="n">
         <v>411</v>
@@ -12881,7 +12881,7 @@
     </row>
     <row r="250" ht="16" customHeight="1" s="5">
       <c r="A250" s="3" t="n">
-        <v>46156.58333333334</v>
+        <v>46157.58333333334</v>
       </c>
       <c r="B250" s="4" t="n">
         <v>385</v>
@@ -12928,7 +12928,7 @@
     </row>
     <row r="251" ht="16" customHeight="1" s="5">
       <c r="A251" s="3" t="n">
-        <v>46156.59375</v>
+        <v>46157.59375</v>
       </c>
       <c r="B251" s="4" t="n">
         <v>436</v>
@@ -12975,7 +12975,7 @@
     </row>
     <row r="252" ht="16" customHeight="1" s="5">
       <c r="A252" s="3" t="n">
-        <v>46156.60416666666</v>
+        <v>46157.60416666666</v>
       </c>
       <c r="B252" s="4" t="n">
         <v>446</v>
@@ -13022,7 +13022,7 @@
     </row>
     <row r="253" ht="16" customHeight="1" s="5">
       <c r="A253" s="3" t="n">
-        <v>46156.61458333334</v>
+        <v>46157.61458333334</v>
       </c>
       <c r="B253" s="4" t="n">
         <v>426</v>
@@ -13069,7 +13069,7 @@
     </row>
     <row r="254" ht="16" customHeight="1" s="5">
       <c r="A254" s="3" t="n">
-        <v>46156.625</v>
+        <v>46157.625</v>
       </c>
       <c r="B254" s="4" t="n">
         <v>450</v>
@@ -13116,7 +13116,7 @@
     </row>
     <row r="255" ht="16" customHeight="1" s="5">
       <c r="A255" s="3" t="n">
-        <v>46156.63541666666</v>
+        <v>46157.63541666666</v>
       </c>
       <c r="B255" s="4" t="n">
         <v>322</v>
@@ -13163,7 +13163,7 @@
     </row>
     <row r="256" ht="16" customHeight="1" s="5">
       <c r="A256" s="3" t="n">
-        <v>46156.64583333334</v>
+        <v>46157.64583333334</v>
       </c>
       <c r="B256" s="4" t="n">
         <v>303</v>
@@ -13210,7 +13210,7 @@
     </row>
     <row r="257" ht="16" customHeight="1" s="5">
       <c r="A257" s="3" t="n">
-        <v>46156.65625</v>
+        <v>46157.65625</v>
       </c>
       <c r="B257" s="4" t="n">
         <v>496</v>
@@ -13257,7 +13257,7 @@
     </row>
     <row r="258" ht="16" customHeight="1" s="5">
       <c r="A258" s="3" t="n">
-        <v>46156.66666666666</v>
+        <v>46157.66666666666</v>
       </c>
       <c r="B258" s="4" t="n">
         <v>654</v>
@@ -13304,7 +13304,7 @@
     </row>
     <row r="259" ht="16" customHeight="1" s="5">
       <c r="A259" s="3" t="n">
-        <v>46156.67708333334</v>
+        <v>46157.67708333334</v>
       </c>
       <c r="B259" s="4" t="n">
         <v>781</v>
@@ -13351,7 +13351,7 @@
     </row>
     <row r="260" ht="16" customHeight="1" s="5">
       <c r="A260" s="3" t="n">
-        <v>46156.6875</v>
+        <v>46157.6875</v>
       </c>
       <c r="B260" s="4" t="n">
         <v>795</v>
@@ -13398,7 +13398,7 @@
     </row>
     <row r="261" ht="16" customHeight="1" s="5">
       <c r="A261" s="3" t="n">
-        <v>46156.69791666666</v>
+        <v>46157.69791666666</v>
       </c>
       <c r="B261" s="4" t="n">
         <v>569</v>
@@ -13445,7 +13445,7 @@
     </row>
     <row r="262" ht="16" customHeight="1" s="5">
       <c r="A262" s="3" t="n">
-        <v>46156.70833333334</v>
+        <v>46157.70833333334</v>
       </c>
       <c r="B262" s="4" t="n">
         <v>611</v>
@@ -13492,7 +13492,7 @@
     </row>
     <row r="263" ht="16" customHeight="1" s="5">
       <c r="A263" s="3" t="n">
-        <v>46156.71875</v>
+        <v>46157.71875</v>
       </c>
       <c r="B263" s="4" t="n">
         <v>794</v>
@@ -13539,7 +13539,7 @@
     </row>
     <row r="264" ht="16" customHeight="1" s="5">
       <c r="A264" s="3" t="n">
-        <v>46156.72916666666</v>
+        <v>46157.72916666666</v>
       </c>
       <c r="B264" s="4" t="n">
         <v>635</v>
@@ -13586,7 +13586,7 @@
     </row>
     <row r="265" ht="16" customHeight="1" s="5">
       <c r="A265" s="3" t="n">
-        <v>46156.73958333334</v>
+        <v>46157.73958333334</v>
       </c>
       <c r="B265" s="4" t="n">
         <v>642</v>
@@ -13633,7 +13633,7 @@
     </row>
     <row r="266" ht="16" customHeight="1" s="5">
       <c r="A266" s="3" t="n">
-        <v>46156.75</v>
+        <v>46157.75</v>
       </c>
       <c r="B266" s="4" t="n">
         <v>624</v>
@@ -13680,7 +13680,7 @@
     </row>
     <row r="267" ht="16" customHeight="1" s="5">
       <c r="A267" s="3" t="n">
-        <v>46156.76041666666</v>
+        <v>46157.76041666666</v>
       </c>
       <c r="B267" s="4" t="n">
         <v>608</v>
@@ -13727,7 +13727,7 @@
     </row>
     <row r="268" ht="16" customHeight="1" s="5">
       <c r="A268" s="3" t="n">
-        <v>46156.77083333334</v>
+        <v>46157.77083333334</v>
       </c>
       <c r="B268" s="4" t="n">
         <v>656</v>
@@ -13774,7 +13774,7 @@
     </row>
     <row r="269" ht="16" customHeight="1" s="5">
       <c r="A269" s="3" t="n">
-        <v>46156.78125</v>
+        <v>46157.78125</v>
       </c>
       <c r="B269" s="4" t="n">
         <v>512</v>
@@ -13821,7 +13821,7 @@
     </row>
     <row r="270" ht="16" customHeight="1" s="5">
       <c r="A270" s="3" t="n">
-        <v>46156.79166666666</v>
+        <v>46157.79166666666</v>
       </c>
       <c r="B270" s="4" t="n">
         <v>323</v>
@@ -13868,7 +13868,7 @@
     </row>
     <row r="271" ht="16" customHeight="1" s="5">
       <c r="A271" s="3" t="n">
-        <v>46156.80208333334</v>
+        <v>46157.80208333334</v>
       </c>
       <c r="B271" s="4" t="n">
         <v>438</v>
@@ -13915,7 +13915,7 @@
     </row>
     <row r="272" ht="16" customHeight="1" s="5">
       <c r="A272" s="3" t="n">
-        <v>46156.8125</v>
+        <v>46157.8125</v>
       </c>
       <c r="B272" s="4" t="n">
         <v>613</v>
@@ -13962,7 +13962,7 @@
     </row>
     <row r="273" ht="16" customHeight="1" s="5">
       <c r="A273" s="3" t="n">
-        <v>46156.82291666666</v>
+        <v>46157.82291666666</v>
       </c>
       <c r="B273" s="4" t="n">
         <v>547</v>
@@ -14009,7 +14009,7 @@
     </row>
     <row r="274" ht="16" customHeight="1" s="5">
       <c r="A274" s="3" t="n">
-        <v>46156.83333333334</v>
+        <v>46157.83333333334</v>
       </c>
       <c r="B274" s="4" t="n">
         <v>402</v>
@@ -14056,7 +14056,7 @@
     </row>
     <row r="275" ht="16" customHeight="1" s="5">
       <c r="A275" s="3" t="n">
-        <v>46156.84375</v>
+        <v>46157.84375</v>
       </c>
       <c r="B275" s="4" t="n">
         <v>341</v>
@@ -14103,7 +14103,7 @@
     </row>
     <row r="276" ht="16" customHeight="1" s="5">
       <c r="A276" s="3" t="n">
-        <v>46156.85416666666</v>
+        <v>46157.85416666666</v>
       </c>
       <c r="B276" s="4" t="n">
         <v>264</v>
@@ -14150,7 +14150,7 @@
     </row>
     <row r="277" ht="16" customHeight="1" s="5">
       <c r="A277" s="3" t="n">
-        <v>46156.86458333334</v>
+        <v>46157.86458333334</v>
       </c>
       <c r="B277" s="4" t="n">
         <v>116</v>
@@ -14197,7 +14197,7 @@
     </row>
     <row r="278" ht="16" customHeight="1" s="5">
       <c r="A278" s="3" t="n">
-        <v>46156.875</v>
+        <v>46157.875</v>
       </c>
       <c r="B278" s="4" t="n">
         <v>0</v>
@@ -14244,7 +14244,7 @@
     </row>
     <row r="279" ht="16" customHeight="1" s="5">
       <c r="A279" s="3" t="n">
-        <v>46156.88541666666</v>
+        <v>46157.88541666666</v>
       </c>
       <c r="B279" s="4" t="n">
         <v>10</v>
@@ -14291,7 +14291,7 @@
     </row>
     <row r="280" ht="16" customHeight="1" s="5">
       <c r="A280" s="3" t="n">
-        <v>46156.89583333334</v>
+        <v>46157.89583333334</v>
       </c>
       <c r="B280" s="4" t="n">
         <v>39</v>
@@ -14338,7 +14338,7 @@
     </row>
     <row r="281" ht="16" customHeight="1" s="5">
       <c r="A281" s="3" t="n">
-        <v>46156.90625</v>
+        <v>46157.90625</v>
       </c>
       <c r="B281" s="4" t="n">
         <v>109</v>
@@ -14385,7 +14385,7 @@
     </row>
     <row r="282" ht="16" customHeight="1" s="5">
       <c r="A282" s="3" t="n">
-        <v>46156.91666666666</v>
+        <v>46157.91666666666</v>
       </c>
       <c r="B282" s="4" t="n">
         <v>193</v>
@@ -14432,7 +14432,7 @@
     </row>
     <row r="283" ht="16" customHeight="1" s="5">
       <c r="A283" s="3" t="n">
-        <v>46156.92708333334</v>
+        <v>46157.92708333334</v>
       </c>
       <c r="B283" s="4" t="n">
         <v>217</v>
@@ -14479,7 +14479,7 @@
     </row>
     <row r="284" ht="16" customHeight="1" s="5">
       <c r="A284" s="3" t="n">
-        <v>46156.9375</v>
+        <v>46157.9375</v>
       </c>
       <c r="B284" s="4" t="n">
         <v>185</v>
@@ -14526,7 +14526,7 @@
     </row>
     <row r="285" ht="16" customHeight="1" s="5">
       <c r="A285" s="3" t="n">
-        <v>46156.94791666666</v>
+        <v>46157.94791666666</v>
       </c>
       <c r="B285" s="4" t="n">
         <v>27</v>
@@ -14573,7 +14573,7 @@
     </row>
     <row r="286" ht="16" customHeight="1" s="5">
       <c r="A286" s="3" t="n">
-        <v>46156.95833333334</v>
+        <v>46157.95833333334</v>
       </c>
       <c r="B286" s="4" t="n">
         <v>0</v>
@@ -14620,7 +14620,7 @@
     </row>
     <row r="287" ht="16" customHeight="1" s="5">
       <c r="A287" s="3" t="n">
-        <v>46156.96875</v>
+        <v>46157.96875</v>
       </c>
       <c r="B287" s="4" t="n">
         <v>0</v>
@@ -14667,7 +14667,7 @@
     </row>
     <row r="288" ht="16" customHeight="1" s="5">
       <c r="A288" s="3" t="n">
-        <v>46156.97916666666</v>
+        <v>46157.97916666666</v>
       </c>
       <c r="B288" s="4" t="n">
         <v>0</v>
@@ -14714,7 +14714,7 @@
     </row>
     <row r="289" ht="16" customHeight="1" s="5">
       <c r="A289" s="3" t="n">
-        <v>46156.98958333334</v>
+        <v>46157.98958333334</v>
       </c>
       <c r="B289" s="4" t="n">
         <v>0</v>
@@ -14761,7 +14761,7 @@
     </row>
     <row r="290" ht="16" customHeight="1" s="5">
       <c r="A290" s="3" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B290" s="4" t="n">
         <v>0</v>
@@ -14808,7 +14808,7 @@
     </row>
     <row r="291" ht="16" customHeight="1" s="5">
       <c r="A291" s="3" t="n">
-        <v>46157.01041666666</v>
+        <v>46158.01041666666</v>
       </c>
       <c r="B291" s="4" t="n">
         <v>10</v>
@@ -14855,7 +14855,7 @@
     </row>
     <row r="292" ht="16" customHeight="1" s="5">
       <c r="A292" s="3" t="n">
-        <v>46157.02083333334</v>
+        <v>46158.02083333334</v>
       </c>
       <c r="B292" s="4" t="n">
         <v>35</v>
@@ -14902,7 +14902,7 @@
     </row>
     <row r="293" ht="16" customHeight="1" s="5">
       <c r="A293" s="3" t="n">
-        <v>46157.03125</v>
+        <v>46158.03125</v>
       </c>
       <c r="B293" s="4" t="n">
         <v>62</v>
@@ -14949,7 +14949,7 @@
     </row>
     <row r="294" ht="16" customHeight="1" s="5">
       <c r="A294" s="3" t="n">
-        <v>46157.04166666666</v>
+        <v>46158.04166666666</v>
       </c>
       <c r="B294" s="4" t="n">
         <v>80</v>
@@ -14996,7 +14996,7 @@
     </row>
     <row r="295" ht="16" customHeight="1" s="5">
       <c r="A295" s="3" t="n">
-        <v>46157.05208333334</v>
+        <v>46158.05208333334</v>
       </c>
       <c r="B295" s="4" t="n">
         <v>27</v>
@@ -15043,7 +15043,7 @@
     </row>
     <row r="296" ht="16" customHeight="1" s="5">
       <c r="A296" s="3" t="n">
-        <v>46157.0625</v>
+        <v>46158.0625</v>
       </c>
       <c r="B296" s="4" t="n">
         <v>0</v>
@@ -15090,7 +15090,7 @@
     </row>
     <row r="297" ht="16" customHeight="1" s="5">
       <c r="A297" s="3" t="n">
-        <v>46157.07291666666</v>
+        <v>46158.07291666666</v>
       </c>
       <c r="B297" s="4" t="n">
         <v>4</v>
@@ -15137,7 +15137,7 @@
     </row>
     <row r="298" ht="16" customHeight="1" s="5">
       <c r="A298" s="3" t="n">
-        <v>46157.08333333334</v>
+        <v>46158.08333333334</v>
       </c>
       <c r="B298" s="4" t="n">
         <v>11</v>
@@ -15184,7 +15184,7 @@
     </row>
     <row r="299" ht="16" customHeight="1" s="5">
       <c r="A299" s="3" t="n">
-        <v>46157.09375</v>
+        <v>46158.09375</v>
       </c>
       <c r="B299" s="4" t="n">
         <v>20</v>
@@ -15231,7 +15231,7 @@
     </row>
     <row r="300" ht="16" customHeight="1" s="5">
       <c r="A300" s="3" t="n">
-        <v>46157.10416666666</v>
+        <v>46158.10416666666</v>
       </c>
       <c r="B300" s="4" t="n">
         <v>33</v>
@@ -15278,7 +15278,7 @@
     </row>
     <row r="301" ht="16" customHeight="1" s="5">
       <c r="A301" s="3" t="n">
-        <v>46157.11458333334</v>
+        <v>46158.11458333334</v>
       </c>
       <c r="B301" s="4" t="n">
         <v>17</v>
@@ -15325,7 +15325,7 @@
     </row>
     <row r="302" ht="16" customHeight="1" s="5">
       <c r="A302" s="3" t="n">
-        <v>46157.125</v>
+        <v>46158.125</v>
       </c>
       <c r="B302" s="4" t="n">
         <v>19</v>
@@ -15372,7 +15372,7 @@
     </row>
     <row r="303" ht="16" customHeight="1" s="5">
       <c r="A303" s="3" t="n">
-        <v>46157.13541666666</v>
+        <v>46158.13541666666</v>
       </c>
       <c r="B303" s="4" t="n">
         <v>26</v>
@@ -15419,7 +15419,7 @@
     </row>
     <row r="304" ht="16" customHeight="1" s="5">
       <c r="A304" s="3" t="n">
-        <v>46157.14583333334</v>
+        <v>46158.14583333334</v>
       </c>
       <c r="B304" s="4" t="n">
         <v>65</v>
@@ -15466,7 +15466,7 @@
     </row>
     <row r="305" ht="16" customHeight="1" s="5">
       <c r="A305" s="3" t="n">
-        <v>46157.15625</v>
+        <v>46158.15625</v>
       </c>
       <c r="B305" s="4" t="n">
         <v>256</v>
@@ -15513,7 +15513,7 @@
     </row>
     <row r="306" ht="16" customHeight="1" s="5">
       <c r="A306" s="3" t="n">
-        <v>46157.16666666666</v>
+        <v>46158.16666666666</v>
       </c>
       <c r="B306" s="4" t="n">
         <v>528</v>
@@ -15560,7 +15560,7 @@
     </row>
     <row r="307" ht="16" customHeight="1" s="5">
       <c r="A307" s="3" t="n">
-        <v>46157.17708333334</v>
+        <v>46158.17708333334</v>
       </c>
       <c r="B307" s="4" t="n">
         <v>850</v>
@@ -15607,7 +15607,7 @@
     </row>
     <row r="308" ht="16" customHeight="1" s="5">
       <c r="A308" s="3" t="n">
-        <v>46157.1875</v>
+        <v>46158.1875</v>
       </c>
       <c r="B308" s="4" t="n">
         <v>967</v>
@@ -15654,7 +15654,7 @@
     </row>
     <row r="309" ht="16" customHeight="1" s="5">
       <c r="A309" s="3" t="n">
-        <v>46157.19791666666</v>
+        <v>46158.19791666666</v>
       </c>
       <c r="B309" s="4" t="n">
         <v>755</v>
@@ -15701,7 +15701,7 @@
     </row>
     <row r="310" ht="16" customHeight="1" s="5">
       <c r="A310" s="3" t="n">
-        <v>46157.20833333334</v>
+        <v>46158.20833333334</v>
       </c>
       <c r="B310" s="4" t="n">
         <v>800</v>
@@ -15748,7 +15748,7 @@
     </row>
     <row r="311" ht="16" customHeight="1" s="5">
       <c r="A311" s="3" t="n">
-        <v>46157.21875</v>
+        <v>46158.21875</v>
       </c>
       <c r="B311" s="4" t="n">
         <v>656</v>
@@ -15795,7 +15795,7 @@
     </row>
     <row r="312" ht="16" customHeight="1" s="5">
       <c r="A312" s="3" t="n">
-        <v>46157.22916666666</v>
+        <v>46158.22916666666</v>
       </c>
       <c r="B312" s="4" t="n">
         <v>515</v>
@@ -15842,7 +15842,7 @@
     </row>
     <row r="313" ht="16" customHeight="1" s="5">
       <c r="A313" s="3" t="n">
-        <v>46157.23958333334</v>
+        <v>46158.23958333334</v>
       </c>
       <c r="B313" s="4" t="n">
         <v>474</v>
@@ -15889,7 +15889,7 @@
     </row>
     <row r="314" ht="16" customHeight="1" s="5">
       <c r="A314" s="3" t="n">
-        <v>46157.25</v>
+        <v>46158.25</v>
       </c>
       <c r="B314" s="4" t="n">
         <v>601</v>
@@ -15936,7 +15936,7 @@
     </row>
     <row r="315" ht="16" customHeight="1" s="5">
       <c r="A315" s="3" t="n">
-        <v>46157.26041666666</v>
+        <v>46158.26041666666</v>
       </c>
       <c r="B315" s="4" t="n">
         <v>632</v>
@@ -15983,7 +15983,7 @@
     </row>
     <row r="316" ht="16" customHeight="1" s="5">
       <c r="A316" s="3" t="n">
-        <v>46157.27083333334</v>
+        <v>46158.27083333334</v>
       </c>
       <c r="B316" s="4" t="n">
         <v>592</v>
@@ -16030,7 +16030,7 @@
     </row>
     <row r="317" ht="16" customHeight="1" s="5">
       <c r="A317" s="3" t="n">
-        <v>46157.28125</v>
+        <v>46158.28125</v>
       </c>
       <c r="B317" s="4" t="n">
         <v>493</v>
@@ -16077,7 +16077,7 @@
     </row>
     <row r="318" ht="16" customHeight="1" s="5">
       <c r="A318" s="3" t="n">
-        <v>46157.29166666666</v>
+        <v>46158.29166666666</v>
       </c>
       <c r="B318" s="4" t="n">
         <v>448</v>
@@ -16124,7 +16124,7 @@
     </row>
     <row r="319" ht="16" customHeight="1" s="5">
       <c r="A319" s="3" t="n">
-        <v>46157.30208333334</v>
+        <v>46158.30208333334</v>
       </c>
       <c r="B319" s="4" t="n">
         <v>459</v>
@@ -16171,7 +16171,7 @@
     </row>
     <row r="320" ht="16" customHeight="1" s="5">
       <c r="A320" s="3" t="n">
-        <v>46157.3125</v>
+        <v>46158.3125</v>
       </c>
       <c r="B320" s="4" t="n">
         <v>432</v>
@@ -16218,7 +16218,7 @@
     </row>
     <row r="321" ht="16" customHeight="1" s="5">
       <c r="A321" s="3" t="n">
-        <v>46157.32291666666</v>
+        <v>46158.32291666666</v>
       </c>
       <c r="B321" s="4" t="n">
         <v>368</v>
@@ -16265,7 +16265,7 @@
     </row>
     <row r="322" ht="16" customHeight="1" s="5">
       <c r="A322" s="3" t="n">
-        <v>46157.33333333334</v>
+        <v>46158.33333333334</v>
       </c>
       <c r="B322" s="4" t="n">
         <v>320</v>
@@ -16312,7 +16312,7 @@
     </row>
     <row r="323" ht="16" customHeight="1" s="5">
       <c r="A323" s="3" t="n">
-        <v>46157.34375</v>
+        <v>46158.34375</v>
       </c>
       <c r="B323" s="4" t="n">
         <v>237</v>
@@ -16359,7 +16359,7 @@
     </row>
     <row r="324" ht="16" customHeight="1" s="5">
       <c r="A324" s="3" t="n">
-        <v>46157.35416666666</v>
+        <v>46158.35416666666</v>
       </c>
       <c r="B324" s="4" t="n">
         <v>262</v>
@@ -16406,7 +16406,7 @@
     </row>
     <row r="325" ht="16" customHeight="1" s="5">
       <c r="A325" s="3" t="n">
-        <v>46157.36458333334</v>
+        <v>46158.36458333334</v>
       </c>
       <c r="B325" s="4" t="n">
         <v>445</v>
@@ -16453,7 +16453,7 @@
     </row>
     <row r="326" ht="16" customHeight="1" s="5">
       <c r="A326" s="3" t="n">
-        <v>46157.375</v>
+        <v>46158.375</v>
       </c>
       <c r="B326" s="4" t="n">
         <v>627</v>
@@ -16500,7 +16500,7 @@
     </row>
     <row r="327" ht="16" customHeight="1" s="5">
       <c r="A327" s="3" t="n">
-        <v>46157.38541666666</v>
+        <v>46158.38541666666</v>
       </c>
       <c r="B327" s="4" t="n">
         <v>623</v>
@@ -16547,7 +16547,7 @@
     </row>
     <row r="328" ht="16" customHeight="1" s="5">
       <c r="A328" s="3" t="n">
-        <v>46157.39583333334</v>
+        <v>46158.39583333334</v>
       </c>
       <c r="B328" s="4" t="n">
         <v>576</v>
@@ -16594,7 +16594,7 @@
     </row>
     <row r="329" ht="16" customHeight="1" s="5">
       <c r="A329" s="3" t="n">
-        <v>46157.40625</v>
+        <v>46158.40625</v>
       </c>
       <c r="B329" s="4" t="n">
         <v>542</v>
@@ -16641,7 +16641,7 @@
     </row>
     <row r="330" ht="16" customHeight="1" s="5">
       <c r="A330" s="3" t="n">
-        <v>46157.41666666666</v>
+        <v>46158.41666666666</v>
       </c>
       <c r="B330" s="4" t="n">
         <v>484</v>
@@ -16688,7 +16688,7 @@
     </row>
     <row r="331" ht="16" customHeight="1" s="5">
       <c r="A331" s="3" t="n">
-        <v>46157.42708333334</v>
+        <v>46158.42708333334</v>
       </c>
       <c r="B331" s="4" t="n">
         <v>377</v>
@@ -16735,7 +16735,7 @@
     </row>
     <row r="332" ht="16" customHeight="1" s="5">
       <c r="A332" s="3" t="n">
-        <v>46157.4375</v>
+        <v>46158.4375</v>
       </c>
       <c r="B332" s="4" t="n">
         <v>281</v>
@@ -16782,7 +16782,7 @@
     </row>
     <row r="333" ht="16" customHeight="1" s="5">
       <c r="A333" s="3" t="n">
-        <v>46157.44791666666</v>
+        <v>46158.44791666666</v>
       </c>
       <c r="B333" s="4" t="n">
         <v>386</v>
@@ -16829,7 +16829,7 @@
     </row>
     <row r="334" ht="16" customHeight="1" s="5">
       <c r="A334" s="3" t="n">
-        <v>46157.45833333334</v>
+        <v>46158.45833333334</v>
       </c>
       <c r="B334" s="4" t="n">
         <v>548</v>
@@ -16876,7 +16876,7 @@
     </row>
     <row r="335" ht="16" customHeight="1" s="5">
       <c r="A335" s="3" t="n">
-        <v>46157.46875</v>
+        <v>46158.46875</v>
       </c>
       <c r="B335" s="4" t="n">
         <v>620</v>
@@ -16923,7 +16923,7 @@
     </row>
     <row r="336" ht="16" customHeight="1" s="5">
       <c r="A336" s="3" t="n">
-        <v>46157.47916666666</v>
+        <v>46158.47916666666</v>
       </c>
       <c r="B336" s="4" t="n">
         <v>531</v>
@@ -16970,7 +16970,7 @@
     </row>
     <row r="337" ht="16" customHeight="1" s="5">
       <c r="A337" s="3" t="n">
-        <v>46157.48958333334</v>
+        <v>46158.48958333334</v>
       </c>
       <c r="B337" s="4" t="n">
         <v>491</v>
@@ -17017,7 +17017,7 @@
     </row>
     <row r="338" ht="16" customHeight="1" s="5">
       <c r="A338" s="3" t="n">
-        <v>46157.5</v>
+        <v>46158.5</v>
       </c>
       <c r="B338" s="4" t="n">
         <v>385</v>
@@ -17064,7 +17064,7 @@
     </row>
     <row r="339" ht="16" customHeight="1" s="5">
       <c r="A339" s="3" t="n">
-        <v>46157.51041666666</v>
+        <v>46158.51041666666</v>
       </c>
       <c r="B339" s="4" t="n">
         <v>397</v>
@@ -17111,7 +17111,7 @@
     </row>
     <row r="340" ht="16" customHeight="1" s="5">
       <c r="A340" s="3" t="n">
-        <v>46157.52083333334</v>
+        <v>46158.52083333334</v>
       </c>
       <c r="B340" s="4" t="n">
         <v>490</v>
@@ -17158,7 +17158,7 @@
     </row>
     <row r="341" ht="16" customHeight="1" s="5">
       <c r="A341" s="3" t="n">
-        <v>46157.53125</v>
+        <v>46158.53125</v>
       </c>
       <c r="B341" s="4" t="n">
         <v>547</v>
@@ -17205,7 +17205,7 @@
     </row>
     <row r="342" ht="16" customHeight="1" s="5">
       <c r="A342" s="3" t="n">
-        <v>46157.54166666666</v>
+        <v>46158.54166666666</v>
       </c>
       <c r="B342" s="4" t="n">
         <v>415</v>
@@ -17252,7 +17252,7 @@
     </row>
     <row r="343" ht="16" customHeight="1" s="5">
       <c r="A343" s="3" t="n">
-        <v>46157.55208333334</v>
+        <v>46158.55208333334</v>
       </c>
       <c r="B343" s="4" t="n">
         <v>228</v>
@@ -17299,7 +17299,7 @@
     </row>
     <row r="344" ht="16" customHeight="1" s="5">
       <c r="A344" s="3" t="n">
-        <v>46157.5625</v>
+        <v>46158.5625</v>
       </c>
       <c r="B344" s="4" t="n">
         <v>309</v>
@@ -17346,7 +17346,7 @@
     </row>
     <row r="345" ht="16" customHeight="1" s="5">
       <c r="A345" s="3" t="n">
-        <v>46157.57291666666</v>
+        <v>46158.57291666666</v>
       </c>
       <c r="B345" s="4" t="n">
         <v>411</v>
@@ -17393,7 +17393,7 @@
     </row>
     <row r="346" ht="16" customHeight="1" s="5">
       <c r="A346" s="3" t="n">
-        <v>46157.58333333334</v>
+        <v>46158.58333333334</v>
       </c>
       <c r="B346" s="4" t="n">
         <v>385</v>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="347" ht="16" customHeight="1" s="5">
       <c r="A347" s="3" t="n">
-        <v>46157.59375</v>
+        <v>46158.59375</v>
       </c>
       <c r="B347" s="4" t="n">
         <v>436</v>
@@ -17487,7 +17487,7 @@
     </row>
     <row r="348" ht="16" customHeight="1" s="5">
       <c r="A348" s="3" t="n">
-        <v>46157.60416666666</v>
+        <v>46158.60416666666</v>
       </c>
       <c r="B348" s="4" t="n">
         <v>446</v>
@@ -17534,7 +17534,7 @@
     </row>
     <row r="349" ht="16" customHeight="1" s="5">
       <c r="A349" s="3" t="n">
-        <v>46157.61458333334</v>
+        <v>46158.61458333334</v>
       </c>
       <c r="B349" s="4" t="n">
         <v>426</v>
@@ -17581,7 +17581,7 @@
     </row>
     <row r="350" ht="16" customHeight="1" s="5">
       <c r="A350" s="3" t="n">
-        <v>46157.625</v>
+        <v>46158.625</v>
       </c>
       <c r="B350" s="4" t="n">
         <v>450</v>
@@ -17628,7 +17628,7 @@
     </row>
     <row r="351" ht="16" customHeight="1" s="5">
       <c r="A351" s="3" t="n">
-        <v>46157.63541666666</v>
+        <v>46158.63541666666</v>
       </c>
       <c r="B351" s="4" t="n">
         <v>322</v>
@@ -17675,7 +17675,7 @@
     </row>
     <row r="352" ht="16" customHeight="1" s="5">
       <c r="A352" s="3" t="n">
-        <v>46157.64583333334</v>
+        <v>46158.64583333334</v>
       </c>
       <c r="B352" s="4" t="n">
         <v>303</v>
@@ -17722,7 +17722,7 @@
     </row>
     <row r="353" ht="16" customHeight="1" s="5">
       <c r="A353" s="3" t="n">
-        <v>46157.65625</v>
+        <v>46158.65625</v>
       </c>
       <c r="B353" s="4" t="n">
         <v>496</v>
@@ -17769,7 +17769,7 @@
     </row>
     <row r="354" ht="16" customHeight="1" s="5">
       <c r="A354" s="3" t="n">
-        <v>46157.66666666666</v>
+        <v>46158.66666666666</v>
       </c>
       <c r="B354" s="4" t="n">
         <v>654</v>
@@ -17816,7 +17816,7 @@
     </row>
     <row r="355" ht="16" customHeight="1" s="5">
       <c r="A355" s="3" t="n">
-        <v>46157.67708333334</v>
+        <v>46158.67708333334</v>
       </c>
       <c r="B355" s="4" t="n">
         <v>781</v>
@@ -17863,7 +17863,7 @@
     </row>
     <row r="356" ht="16" customHeight="1" s="5">
       <c r="A356" s="3" t="n">
-        <v>46157.6875</v>
+        <v>46158.6875</v>
       </c>
       <c r="B356" s="4" t="n">
         <v>795</v>
@@ -17910,7 +17910,7 @@
     </row>
     <row r="357" ht="16" customHeight="1" s="5">
       <c r="A357" s="3" t="n">
-        <v>46157.69791666666</v>
+        <v>46158.69791666666</v>
       </c>
       <c r="B357" s="4" t="n">
         <v>569</v>
@@ -17957,7 +17957,7 @@
     </row>
     <row r="358" ht="16" customHeight="1" s="5">
       <c r="A358" s="3" t="n">
-        <v>46157.70833333334</v>
+        <v>46158.70833333334</v>
       </c>
       <c r="B358" s="4" t="n">
         <v>611</v>
@@ -18004,7 +18004,7 @@
     </row>
     <row r="359" ht="16" customHeight="1" s="5">
       <c r="A359" s="3" t="n">
-        <v>46157.71875</v>
+        <v>46158.71875</v>
       </c>
       <c r="B359" s="4" t="n">
         <v>794</v>
@@ -18051,7 +18051,7 @@
     </row>
     <row r="360" ht="16" customHeight="1" s="5">
       <c r="A360" s="3" t="n">
-        <v>46157.72916666666</v>
+        <v>46158.72916666666</v>
       </c>
       <c r="B360" s="4" t="n">
         <v>635</v>
@@ -18098,7 +18098,7 @@
     </row>
     <row r="361" ht="16" customHeight="1" s="5">
       <c r="A361" s="3" t="n">
-        <v>46157.73958333334</v>
+        <v>46158.73958333334</v>
       </c>
       <c r="B361" s="4" t="n">
         <v>642</v>
@@ -18145,7 +18145,7 @@
     </row>
     <row r="362" ht="16" customHeight="1" s="5">
       <c r="A362" s="3" t="n">
-        <v>46157.75</v>
+        <v>46158.75</v>
       </c>
       <c r="B362" s="4" t="n">
         <v>624</v>
@@ -18192,7 +18192,7 @@
     </row>
     <row r="363" ht="16" customHeight="1" s="5">
       <c r="A363" s="3" t="n">
-        <v>46157.76041666666</v>
+        <v>46158.76041666666</v>
       </c>
       <c r="B363" s="4" t="n">
         <v>608</v>
@@ -18239,7 +18239,7 @@
     </row>
     <row r="364" ht="16" customHeight="1" s="5">
       <c r="A364" s="3" t="n">
-        <v>46157.77083333334</v>
+        <v>46158.77083333334</v>
       </c>
       <c r="B364" s="4" t="n">
         <v>656</v>
@@ -18286,7 +18286,7 @@
     </row>
     <row r="365" ht="16" customHeight="1" s="5">
       <c r="A365" s="3" t="n">
-        <v>46157.78125</v>
+        <v>46158.78125</v>
       </c>
       <c r="B365" s="4" t="n">
         <v>512</v>
@@ -18333,7 +18333,7 @@
     </row>
     <row r="366" ht="16" customHeight="1" s="5">
       <c r="A366" s="3" t="n">
-        <v>46157.79166666666</v>
+        <v>46158.79166666666</v>
       </c>
       <c r="B366" s="4" t="n">
         <v>323</v>
@@ -18380,7 +18380,7 @@
     </row>
     <row r="367" ht="16" customHeight="1" s="5">
       <c r="A367" s="3" t="n">
-        <v>46157.80208333334</v>
+        <v>46158.80208333334</v>
       </c>
       <c r="B367" s="4" t="n">
         <v>438</v>
@@ -18427,7 +18427,7 @@
     </row>
     <row r="368" ht="16" customHeight="1" s="5">
       <c r="A368" s="3" t="n">
-        <v>46157.8125</v>
+        <v>46158.8125</v>
       </c>
       <c r="B368" s="4" t="n">
         <v>613</v>
@@ -18474,7 +18474,7 @@
     </row>
     <row r="369" ht="16" customHeight="1" s="5">
       <c r="A369" s="3" t="n">
-        <v>46157.82291666666</v>
+        <v>46158.82291666666</v>
       </c>
       <c r="B369" s="4" t="n">
         <v>547</v>
@@ -18521,7 +18521,7 @@
     </row>
     <row r="370" ht="16" customHeight="1" s="5">
       <c r="A370" s="3" t="n">
-        <v>46157.83333333334</v>
+        <v>46158.83333333334</v>
       </c>
       <c r="B370" s="4" t="n">
         <v>402</v>
@@ -18568,7 +18568,7 @@
     </row>
     <row r="371" ht="16" customHeight="1" s="5">
       <c r="A371" s="3" t="n">
-        <v>46157.84375</v>
+        <v>46158.84375</v>
       </c>
       <c r="B371" s="4" t="n">
         <v>341</v>
@@ -18615,7 +18615,7 @@
     </row>
     <row r="372" ht="16" customHeight="1" s="5">
       <c r="A372" s="3" t="n">
-        <v>46157.85416666666</v>
+        <v>46158.85416666666</v>
       </c>
       <c r="B372" s="4" t="n">
         <v>264</v>
@@ -18662,7 +18662,7 @@
     </row>
     <row r="373" ht="16" customHeight="1" s="5">
       <c r="A373" s="3" t="n">
-        <v>46157.86458333334</v>
+        <v>46158.86458333334</v>
       </c>
       <c r="B373" s="4" t="n">
         <v>116</v>
@@ -18709,7 +18709,7 @@
     </row>
     <row r="374" ht="16" customHeight="1" s="5">
       <c r="A374" s="3" t="n">
-        <v>46157.875</v>
+        <v>46158.875</v>
       </c>
       <c r="B374" s="4" t="n">
         <v>0</v>
@@ -18756,7 +18756,7 @@
     </row>
     <row r="375" ht="16" customHeight="1" s="5">
       <c r="A375" s="3" t="n">
-        <v>46157.88541666666</v>
+        <v>46158.88541666666</v>
       </c>
       <c r="B375" s="4" t="n">
         <v>10</v>
@@ -18803,7 +18803,7 @@
     </row>
     <row r="376" ht="16" customHeight="1" s="5">
       <c r="A376" s="3" t="n">
-        <v>46157.89583333334</v>
+        <v>46158.89583333334</v>
       </c>
       <c r="B376" s="4" t="n">
         <v>39</v>
@@ -18850,7 +18850,7 @@
     </row>
     <row r="377" ht="16" customHeight="1" s="5">
       <c r="A377" s="3" t="n">
-        <v>46157.90625</v>
+        <v>46158.90625</v>
       </c>
       <c r="B377" s="4" t="n">
         <v>109</v>
@@ -18897,7 +18897,7 @@
     </row>
     <row r="378" ht="16" customHeight="1" s="5">
       <c r="A378" s="3" t="n">
-        <v>46157.91666666666</v>
+        <v>46158.91666666666</v>
       </c>
       <c r="B378" s="4" t="n">
         <v>193</v>
@@ -18944,7 +18944,7 @@
     </row>
     <row r="379" ht="16" customHeight="1" s="5">
       <c r="A379" s="3" t="n">
-        <v>46157.92708333334</v>
+        <v>46158.92708333334</v>
       </c>
       <c r="B379" s="4" t="n">
         <v>217</v>
@@ -18991,7 +18991,7 @@
     </row>
     <row r="380" ht="16" customHeight="1" s="5">
       <c r="A380" s="3" t="n">
-        <v>46157.9375</v>
+        <v>46158.9375</v>
       </c>
       <c r="B380" s="4" t="n">
         <v>185</v>
@@ -19038,7 +19038,7 @@
     </row>
     <row r="381" ht="16" customHeight="1" s="5">
       <c r="A381" s="3" t="n">
-        <v>46157.94791666666</v>
+        <v>46158.94791666666</v>
       </c>
       <c r="B381" s="4" t="n">
         <v>27</v>
@@ -19085,7 +19085,7 @@
     </row>
     <row r="382" ht="16" customHeight="1" s="5">
       <c r="A382" s="3" t="n">
-        <v>46157.95833333334</v>
+        <v>46158.95833333334</v>
       </c>
       <c r="B382" s="4" t="n">
         <v>0</v>
@@ -19132,7 +19132,7 @@
     </row>
     <row r="383" ht="16" customHeight="1" s="5">
       <c r="A383" s="3" t="n">
-        <v>46157.96875</v>
+        <v>46158.96875</v>
       </c>
       <c r="B383" s="4" t="n">
         <v>0</v>
@@ -19179,7 +19179,7 @@
     </row>
     <row r="384" ht="16" customHeight="1" s="5">
       <c r="A384" s="3" t="n">
-        <v>46157.97916666666</v>
+        <v>46158.97916666666</v>
       </c>
       <c r="B384" s="4" t="n">
         <v>0</v>
@@ -19226,7 +19226,7 @@
     </row>
     <row r="385" ht="16" customHeight="1" s="5">
       <c r="A385" s="3" t="n">
-        <v>46157.98958333334</v>
+        <v>46158.98958333334</v>
       </c>
       <c r="B385" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat: Add passenger flow skill timeline card and update styles
- Introduced a new component for displaying passenger flow by skill with interactive buttons for selection.
- Updated styles for the new component to enhance visual presentation.
- Modified the intraday optimization script to integrate the new passenger skill timeline card.
- Adjusted the default delay input value in the scenario form from 30 to 60 minutes.
- Added a new Excel file for flight delay effects data.
</commit_message>
<xml_diff>
--- a/data/short term PAX.xlsx
+++ b/data/short term PAX.xlsx
@@ -1225,7 +1225,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" s="5">
       <c r="A2" s="3" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>0</v>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="3" ht="16" customHeight="1" s="5">
       <c r="A3" s="3" t="n">
-        <v>46155.01041666666</v>
+        <v>46156.01041666666</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>10</v>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="4" ht="16" customHeight="1" s="5">
       <c r="A4" s="3" t="n">
-        <v>46155.02083333334</v>
+        <v>46156.02083333334</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>28</v>
@@ -1366,7 +1366,7 @@
     </row>
     <row r="5" ht="16" customHeight="1" s="5">
       <c r="A5" s="3" t="n">
-        <v>46155.03125</v>
+        <v>46156.03125</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>48</v>
@@ -1413,7 +1413,7 @@
     </row>
     <row r="6" ht="16" customHeight="1" s="5">
       <c r="A6" s="3" t="n">
-        <v>46155.04166666666</v>
+        <v>46156.04166666666</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>58</v>
@@ -1460,7 +1460,7 @@
     </row>
     <row r="7" ht="16" customHeight="1" s="5">
       <c r="A7" s="3" t="n">
-        <v>46155.05208333334</v>
+        <v>46156.05208333334</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>9</v>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="8" ht="16" customHeight="1" s="5">
       <c r="A8" s="3" t="n">
-        <v>46155.0625</v>
+        <v>46156.0625</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="9" ht="16" customHeight="1" s="5">
       <c r="A9" s="3" t="n">
-        <v>46155.07291666666</v>
+        <v>46156.07291666666</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>4</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="10" ht="16" customHeight="1" s="5">
       <c r="A10" s="3" t="n">
-        <v>46155.08333333334</v>
+        <v>46156.08333333334</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>11</v>
@@ -1648,7 +1648,7 @@
     </row>
     <row r="11" ht="16" customHeight="1" s="5">
       <c r="A11" s="3" t="n">
-        <v>46155.09375</v>
+        <v>46156.09375</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>20</v>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="12" ht="16" customHeight="1" s="5">
       <c r="A12" s="3" t="n">
-        <v>46155.10416666666</v>
+        <v>46156.10416666666</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>33</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="13" ht="16" customHeight="1" s="5">
       <c r="A13" s="3" t="n">
-        <v>46155.11458333334</v>
+        <v>46156.11458333334</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>17</v>
@@ -1789,7 +1789,7 @@
     </row>
     <row r="14" ht="16" customHeight="1" s="5">
       <c r="A14" s="3" t="n">
-        <v>46155.125</v>
+        <v>46156.125</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>27</v>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="15" ht="16" customHeight="1" s="5">
       <c r="A15" s="3" t="n">
-        <v>46155.13541666666</v>
+        <v>46156.13541666666</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>41</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="16" ht="16" customHeight="1" s="5">
       <c r="A16" s="3" t="n">
-        <v>46155.14583333334</v>
+        <v>46156.14583333334</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>75</v>
@@ -1930,7 +1930,7 @@
     </row>
     <row r="17" ht="16" customHeight="1" s="5">
       <c r="A17" s="3" t="n">
-        <v>46155.15625</v>
+        <v>46156.15625</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>268</v>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="18" ht="16" customHeight="1" s="5">
       <c r="A18" s="3" t="n">
-        <v>46155.16666666666</v>
+        <v>46156.16666666666</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>527</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="19" ht="16" customHeight="1" s="5">
       <c r="A19" s="3" t="n">
-        <v>46155.17708333334</v>
+        <v>46156.17708333334</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>888</v>
@@ -2071,7 +2071,7 @@
     </row>
     <row r="20" ht="16" customHeight="1" s="5">
       <c r="A20" s="3" t="n">
-        <v>46155.1875</v>
+        <v>46156.1875</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>1032</v>
@@ -2118,7 +2118,7 @@
     </row>
     <row r="21" ht="16" customHeight="1" s="5">
       <c r="A21" s="3" t="n">
-        <v>46155.19791666666</v>
+        <v>46156.19791666666</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>780</v>
@@ -2165,7 +2165,7 @@
     </row>
     <row r="22" ht="16" customHeight="1" s="5">
       <c r="A22" s="3" t="n">
-        <v>46155.20833333334</v>
+        <v>46156.20833333334</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>0</v>
@@ -2212,7 +2212,7 @@
     </row>
     <row r="23" ht="16" customHeight="1" s="5">
       <c r="A23" s="3" t="n">
-        <v>46155.21875</v>
+        <v>46156.21875</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>0</v>
@@ -2259,7 +2259,7 @@
     </row>
     <row r="24" ht="16" customHeight="1" s="5">
       <c r="A24" s="3" t="n">
-        <v>46155.22916666666</v>
+        <v>46156.22916666666</v>
       </c>
       <c r="B24" s="4" t="n">
         <v>0</v>
@@ -2306,7 +2306,7 @@
     </row>
     <row r="25" ht="16" customHeight="1" s="5">
       <c r="A25" s="3" t="n">
-        <v>46155.23958333334</v>
+        <v>46156.23958333334</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>1</v>
@@ -2353,7 +2353,7 @@
     </row>
     <row r="26" ht="16" customHeight="1" s="5">
       <c r="A26" s="3" t="n">
-        <v>46155.25</v>
+        <v>46156.25</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>27</v>
@@ -2400,7 +2400,7 @@
     </row>
     <row r="27" ht="16" customHeight="1" s="5">
       <c r="A27" s="3" t="n">
-        <v>46155.26041666666</v>
+        <v>46156.26041666666</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>82</v>
@@ -2447,7 +2447,7 @@
     </row>
     <row r="28" ht="16" customHeight="1" s="5">
       <c r="A28" s="3" t="n">
-        <v>46155.27083333334</v>
+        <v>46156.27083333334</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>180</v>
@@ -2494,7 +2494,7 @@
     </row>
     <row r="29" ht="16" customHeight="1" s="5">
       <c r="A29" s="3" t="n">
-        <v>46155.28125</v>
+        <v>46156.28125</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>275</v>
@@ -2541,7 +2541,7 @@
     </row>
     <row r="30" ht="16" customHeight="1" s="5">
       <c r="A30" s="3" t="n">
-        <v>46155.29166666666</v>
+        <v>46156.29166666666</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>342</v>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="31" ht="16" customHeight="1" s="5">
       <c r="A31" s="3" t="n">
-        <v>46155.30208333334</v>
+        <v>46156.30208333334</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>327</v>
@@ -2635,7 +2635,7 @@
     </row>
     <row r="32" ht="16" customHeight="1" s="5">
       <c r="A32" s="3" t="n">
-        <v>46155.3125</v>
+        <v>46156.3125</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>386</v>
@@ -2682,7 +2682,7 @@
     </row>
     <row r="33" ht="16" customHeight="1" s="5">
       <c r="A33" s="3" t="n">
-        <v>46155.32291666666</v>
+        <v>46156.32291666666</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>401</v>
@@ -2729,7 +2729,7 @@
     </row>
     <row r="34" ht="16" customHeight="1" s="5">
       <c r="A34" s="3" t="n">
-        <v>46155.33333333334</v>
+        <v>46156.33333333334</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>399</v>
@@ -2776,7 +2776,7 @@
     </row>
     <row r="35" ht="16" customHeight="1" s="5">
       <c r="A35" s="3" t="n">
-        <v>46155.34375</v>
+        <v>46156.34375</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>384</v>
@@ -2823,7 +2823,7 @@
     </row>
     <row r="36" ht="16" customHeight="1" s="5">
       <c r="A36" s="3" t="n">
-        <v>46155.35416666666</v>
+        <v>46156.35416666666</v>
       </c>
       <c r="B36" s="4" t="n">
         <v>438</v>
@@ -2870,7 +2870,7 @@
     </row>
     <row r="37" ht="16" customHeight="1" s="5">
       <c r="A37" s="3" t="n">
-        <v>46155.36458333334</v>
+        <v>46156.36458333334</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>433</v>
@@ -2917,7 +2917,7 @@
     </row>
     <row r="38" ht="16" customHeight="1" s="5">
       <c r="A38" s="3" t="n">
-        <v>46155.375</v>
+        <v>46156.375</v>
       </c>
       <c r="B38" s="4" t="n">
         <v>398</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="39" ht="16" customHeight="1" s="5">
       <c r="A39" s="3" t="n">
-        <v>46155.38541666666</v>
+        <v>46156.38541666666</v>
       </c>
       <c r="B39" s="4" t="n">
         <v>463</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="40" ht="16" customHeight="1" s="5">
       <c r="A40" s="3" t="n">
-        <v>46155.39583333334</v>
+        <v>46156.39583333334</v>
       </c>
       <c r="B40" s="4" t="n">
         <v>422</v>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="41" ht="16" customHeight="1" s="5">
       <c r="A41" s="3" t="n">
-        <v>46155.40625</v>
+        <v>46156.40625</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>448</v>
@@ -3105,7 +3105,7 @@
     </row>
     <row r="42" ht="16" customHeight="1" s="5">
       <c r="A42" s="3" t="n">
-        <v>46155.41666666666</v>
+        <v>46156.41666666666</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>603</v>
@@ -3152,7 +3152,7 @@
     </row>
     <row r="43" ht="16" customHeight="1" s="5">
       <c r="A43" s="3" t="n">
-        <v>46155.42708333334</v>
+        <v>46156.42708333334</v>
       </c>
       <c r="B43" s="4" t="n">
         <v>621</v>
@@ -3199,7 +3199,7 @@
     </row>
     <row r="44" ht="16" customHeight="1" s="5">
       <c r="A44" s="3" t="n">
-        <v>46155.4375</v>
+        <v>46156.4375</v>
       </c>
       <c r="B44" s="4" t="n">
         <v>521</v>
@@ -3246,7 +3246,7 @@
     </row>
     <row r="45" ht="16" customHeight="1" s="5">
       <c r="A45" s="3" t="n">
-        <v>46155.44791666666</v>
+        <v>46156.44791666666</v>
       </c>
       <c r="B45" s="4" t="n">
         <v>392</v>
@@ -3293,7 +3293,7 @@
     </row>
     <row r="46" ht="16" customHeight="1" s="5">
       <c r="A46" s="3" t="n">
-        <v>46155.45833333334</v>
+        <v>46156.45833333334</v>
       </c>
       <c r="B46" s="4" t="n">
         <v>358</v>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="47" ht="16" customHeight="1" s="5">
       <c r="A47" s="3" t="n">
-        <v>46155.46875</v>
+        <v>46156.46875</v>
       </c>
       <c r="B47" s="4" t="n">
         <v>487</v>
@@ -3387,7 +3387,7 @@
     </row>
     <row r="48" ht="16" customHeight="1" s="5">
       <c r="A48" s="3" t="n">
-        <v>46155.47916666666</v>
+        <v>46156.47916666666</v>
       </c>
       <c r="B48" s="4" t="n">
         <v>557</v>
@@ -3434,7 +3434,7 @@
     </row>
     <row r="49" ht="16" customHeight="1" s="5">
       <c r="A49" s="3" t="n">
-        <v>46155.48958333334</v>
+        <v>46156.48958333334</v>
       </c>
       <c r="B49" s="4" t="n">
         <v>565</v>
@@ -3481,7 +3481,7 @@
     </row>
     <row r="50" ht="16" customHeight="1" s="5">
       <c r="A50" s="3" t="n">
-        <v>46155.5</v>
+        <v>46156.5</v>
       </c>
       <c r="B50" s="4" t="n">
         <v>387</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="51" ht="16" customHeight="1" s="5">
       <c r="A51" s="3" t="n">
-        <v>46155.51041666666</v>
+        <v>46156.51041666666</v>
       </c>
       <c r="B51" s="4" t="n">
         <v>227</v>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="52" ht="16" customHeight="1" s="5">
       <c r="A52" s="3" t="n">
-        <v>46155.52083333334</v>
+        <v>46156.52083333334</v>
       </c>
       <c r="B52" s="4" t="n">
         <v>382</v>
@@ -3622,7 +3622,7 @@
     </row>
     <row r="53" ht="16" customHeight="1" s="5">
       <c r="A53" s="3" t="n">
-        <v>46155.53125</v>
+        <v>46156.53125</v>
       </c>
       <c r="B53" s="4" t="n">
         <v>612</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="54" ht="16" customHeight="1" s="5">
       <c r="A54" s="3" t="n">
-        <v>46155.54166666666</v>
+        <v>46156.54166666666</v>
       </c>
       <c r="B54" s="4" t="n">
         <v>699</v>
@@ -3716,7 +3716,7 @@
     </row>
     <row r="55" ht="16" customHeight="1" s="5">
       <c r="A55" s="3" t="n">
-        <v>46155.55208333334</v>
+        <v>46156.55208333334</v>
       </c>
       <c r="B55" s="4" t="n">
         <v>627</v>
@@ -3763,7 +3763,7 @@
     </row>
     <row r="56" ht="16" customHeight="1" s="5">
       <c r="A56" s="3" t="n">
-        <v>46155.5625</v>
+        <v>46156.5625</v>
       </c>
       <c r="B56" s="4" t="n">
         <v>538</v>
@@ -3810,7 +3810,7 @@
     </row>
     <row r="57" ht="16" customHeight="1" s="5">
       <c r="A57" s="3" t="n">
-        <v>46155.57291666666</v>
+        <v>46156.57291666666</v>
       </c>
       <c r="B57" s="4" t="n">
         <v>464</v>
@@ -3857,7 +3857,7 @@
     </row>
     <row r="58" ht="16" customHeight="1" s="5">
       <c r="A58" s="3" t="n">
-        <v>46155.58333333334</v>
+        <v>46156.58333333334</v>
       </c>
       <c r="B58" s="4" t="n">
         <v>402</v>
@@ -3904,7 +3904,7 @@
     </row>
     <row r="59" ht="16" customHeight="1" s="5">
       <c r="A59" s="3" t="n">
-        <v>46155.59375</v>
+        <v>46156.59375</v>
       </c>
       <c r="B59" s="4" t="n">
         <v>262</v>
@@ -3951,7 +3951,7 @@
     </row>
     <row r="60" ht="16" customHeight="1" s="5">
       <c r="A60" s="3" t="n">
-        <v>46155.60416666666</v>
+        <v>46156.60416666666</v>
       </c>
       <c r="B60" s="4" t="n">
         <v>228</v>
@@ -3998,7 +3998,7 @@
     </row>
     <row r="61" ht="16" customHeight="1" s="5">
       <c r="A61" s="3" t="n">
-        <v>46155.61458333334</v>
+        <v>46156.61458333334</v>
       </c>
       <c r="B61" s="4" t="n">
         <v>350</v>
@@ -4045,7 +4045,7 @@
     </row>
     <row r="62" ht="16" customHeight="1" s="5">
       <c r="A62" s="3" t="n">
-        <v>46155.625</v>
+        <v>46156.625</v>
       </c>
       <c r="B62" s="4" t="n">
         <v>506</v>
@@ -4092,7 +4092,7 @@
     </row>
     <row r="63" ht="16" customHeight="1" s="5">
       <c r="A63" s="3" t="n">
-        <v>46155.63541666666</v>
+        <v>46156.63541666666</v>
       </c>
       <c r="B63" s="4" t="n">
         <v>530</v>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="64" ht="16" customHeight="1" s="5">
       <c r="A64" s="3" t="n">
-        <v>46155.64583333334</v>
+        <v>46156.64583333334</v>
       </c>
       <c r="B64" s="4" t="n">
         <v>459</v>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="65" ht="16" customHeight="1" s="5">
       <c r="A65" s="3" t="n">
-        <v>46155.65625</v>
+        <v>46156.65625</v>
       </c>
       <c r="B65" s="4" t="n">
         <v>398</v>
@@ -4233,7 +4233,7 @@
     </row>
     <row r="66" ht="16" customHeight="1" s="5">
       <c r="A66" s="3" t="n">
-        <v>46155.66666666666</v>
+        <v>46156.66666666666</v>
       </c>
       <c r="B66" s="4" t="n">
         <v>488</v>
@@ -4280,7 +4280,7 @@
     </row>
     <row r="67" ht="16" customHeight="1" s="5">
       <c r="A67" s="3" t="n">
-        <v>46155.67708333334</v>
+        <v>46156.67708333334</v>
       </c>
       <c r="B67" s="4" t="n">
         <v>532</v>
@@ -4327,7 +4327,7 @@
     </row>
     <row r="68" ht="16" customHeight="1" s="5">
       <c r="A68" s="3" t="n">
-        <v>46155.6875</v>
+        <v>46156.6875</v>
       </c>
       <c r="B68" s="4" t="n">
         <v>716</v>
@@ -4374,7 +4374,7 @@
     </row>
     <row r="69" ht="16" customHeight="1" s="5">
       <c r="A69" s="3" t="n">
-        <v>46155.69791666666</v>
+        <v>46156.69791666666</v>
       </c>
       <c r="B69" s="4" t="n">
         <v>673</v>
@@ -4421,7 +4421,7 @@
     </row>
     <row r="70" ht="16" customHeight="1" s="5">
       <c r="A70" s="3" t="n">
-        <v>46155.70833333334</v>
+        <v>46156.70833333334</v>
       </c>
       <c r="B70" s="4" t="n">
         <v>504</v>
@@ -4468,7 +4468,7 @@
     </row>
     <row r="71" ht="16" customHeight="1" s="5">
       <c r="A71" s="3" t="n">
-        <v>46155.71875</v>
+        <v>46156.71875</v>
       </c>
       <c r="B71" s="4" t="n">
         <v>616</v>
@@ -4515,7 +4515,7 @@
     </row>
     <row r="72" ht="16" customHeight="1" s="5">
       <c r="A72" s="3" t="n">
-        <v>46155.72916666666</v>
+        <v>46156.72916666666</v>
       </c>
       <c r="B72" s="4" t="n">
         <v>569</v>
@@ -4562,7 +4562,7 @@
     </row>
     <row r="73" ht="16" customHeight="1" s="5">
       <c r="A73" s="3" t="n">
-        <v>46155.73958333334</v>
+        <v>46156.73958333334</v>
       </c>
       <c r="B73" s="4" t="n">
         <v>619</v>
@@ -4609,7 +4609,7 @@
     </row>
     <row r="74" ht="16" customHeight="1" s="5">
       <c r="A74" s="3" t="n">
-        <v>46155.75</v>
+        <v>46156.75</v>
       </c>
       <c r="B74" s="4" t="n">
         <v>597</v>
@@ -4656,7 +4656,7 @@
     </row>
     <row r="75" ht="16" customHeight="1" s="5">
       <c r="A75" s="3" t="n">
-        <v>46155.76041666666</v>
+        <v>46156.76041666666</v>
       </c>
       <c r="B75" s="4" t="n">
         <v>373</v>
@@ -4703,7 +4703,7 @@
     </row>
     <row r="76" ht="16" customHeight="1" s="5">
       <c r="A76" s="3" t="n">
-        <v>46155.77083333334</v>
+        <v>46156.77083333334</v>
       </c>
       <c r="B76" s="4" t="n">
         <v>298</v>
@@ -4750,7 +4750,7 @@
     </row>
     <row r="77" ht="16" customHeight="1" s="5">
       <c r="A77" s="3" t="n">
-        <v>46155.78125</v>
+        <v>46156.78125</v>
       </c>
       <c r="B77" s="4" t="n">
         <v>325</v>
@@ -4797,7 +4797,7 @@
     </row>
     <row r="78" ht="16" customHeight="1" s="5">
       <c r="A78" s="3" t="n">
-        <v>46155.79166666666</v>
+        <v>46156.79166666666</v>
       </c>
       <c r="B78" s="4" t="n">
         <v>350</v>
@@ -4844,7 +4844,7 @@
     </row>
     <row r="79" ht="16" customHeight="1" s="5">
       <c r="A79" s="3" t="n">
-        <v>46155.80208333334</v>
+        <v>46156.80208333334</v>
       </c>
       <c r="B79" s="4" t="n">
         <v>373</v>
@@ -4891,7 +4891,7 @@
     </row>
     <row r="80" ht="16" customHeight="1" s="5">
       <c r="A80" s="3" t="n">
-        <v>46155.8125</v>
+        <v>46156.8125</v>
       </c>
       <c r="B80" s="4" t="n">
         <v>344</v>
@@ -4938,7 +4938,7 @@
     </row>
     <row r="81" ht="16" customHeight="1" s="5">
       <c r="A81" s="3" t="n">
-        <v>46155.82291666666</v>
+        <v>46156.82291666666</v>
       </c>
       <c r="B81" s="4" t="n">
         <v>385</v>
@@ -4985,7 +4985,7 @@
     </row>
     <row r="82" ht="16" customHeight="1" s="5">
       <c r="A82" s="3" t="n">
-        <v>46155.83333333334</v>
+        <v>46156.83333333334</v>
       </c>
       <c r="B82" s="4" t="n">
         <v>439</v>
@@ -5032,7 +5032,7 @@
     </row>
     <row r="83" ht="16" customHeight="1" s="5">
       <c r="A83" s="3" t="n">
-        <v>46155.84375</v>
+        <v>46156.84375</v>
       </c>
       <c r="B83" s="4" t="n">
         <v>408</v>
@@ -5079,7 +5079,7 @@
     </row>
     <row r="84" ht="16" customHeight="1" s="5">
       <c r="A84" s="3" t="n">
-        <v>46155.85416666666</v>
+        <v>46156.85416666666</v>
       </c>
       <c r="B84" s="4" t="n">
         <v>319</v>
@@ -5126,7 +5126,7 @@
     </row>
     <row r="85" ht="16" customHeight="1" s="5">
       <c r="A85" s="3" t="n">
-        <v>46155.86458333334</v>
+        <v>46156.86458333334</v>
       </c>
       <c r="B85" s="4" t="n">
         <v>166</v>
@@ -5173,7 +5173,7 @@
     </row>
     <row r="86" ht="16" customHeight="1" s="5">
       <c r="A86" s="3" t="n">
-        <v>46155.875</v>
+        <v>46156.875</v>
       </c>
       <c r="B86" s="4" t="n">
         <v>29</v>
@@ -5220,7 +5220,7 @@
     </row>
     <row r="87" ht="16" customHeight="1" s="5">
       <c r="A87" s="3" t="n">
-        <v>46155.88541666666</v>
+        <v>46156.88541666666</v>
       </c>
       <c r="B87" s="4" t="n">
         <v>61</v>
@@ -5267,7 +5267,7 @@
     </row>
     <row r="88" ht="16" customHeight="1" s="5">
       <c r="A88" s="3" t="n">
-        <v>46155.89583333334</v>
+        <v>46156.89583333334</v>
       </c>
       <c r="B88" s="4" t="n">
         <v>107</v>
@@ -5314,7 +5314,7 @@
     </row>
     <row r="89" ht="16" customHeight="1" s="5">
       <c r="A89" s="3" t="n">
-        <v>46155.90625</v>
+        <v>46156.90625</v>
       </c>
       <c r="B89" s="4" t="n">
         <v>93</v>
@@ -5361,7 +5361,7 @@
     </row>
     <row r="90" ht="16" customHeight="1" s="5">
       <c r="A90" s="3" t="n">
-        <v>46155.91666666666</v>
+        <v>46156.91666666666</v>
       </c>
       <c r="B90" s="4" t="n">
         <v>115</v>
@@ -5408,7 +5408,7 @@
     </row>
     <row r="91" ht="16" customHeight="1" s="5">
       <c r="A91" s="3" t="n">
-        <v>46155.92708333334</v>
+        <v>46156.92708333334</v>
       </c>
       <c r="B91" s="4" t="n">
         <v>58</v>
@@ -5455,7 +5455,7 @@
     </row>
     <row r="92" ht="16" customHeight="1" s="5">
       <c r="A92" s="3" t="n">
-        <v>46155.9375</v>
+        <v>46156.9375</v>
       </c>
       <c r="B92" s="4" t="n">
         <v>0</v>
@@ -5502,7 +5502,7 @@
     </row>
     <row r="93" ht="16" customHeight="1" s="5">
       <c r="A93" s="3" t="n">
-        <v>46155.94791666666</v>
+        <v>46156.94791666666</v>
       </c>
       <c r="B93" s="4" t="n">
         <v>0</v>
@@ -5549,7 +5549,7 @@
     </row>
     <row r="94" ht="16" customHeight="1" s="5">
       <c r="A94" s="3" t="n">
-        <v>46155.95833333334</v>
+        <v>46156.95833333334</v>
       </c>
       <c r="B94" s="4" t="n">
         <v>0</v>
@@ -5596,7 +5596,7 @@
     </row>
     <row r="95" ht="16" customHeight="1" s="5">
       <c r="A95" s="3" t="n">
-        <v>46155.96875</v>
+        <v>46156.96875</v>
       </c>
       <c r="B95" s="4" t="n">
         <v>0</v>
@@ -5643,7 +5643,7 @@
     </row>
     <row r="96" ht="16" customHeight="1" s="5">
       <c r="A96" s="3" t="n">
-        <v>46155.97916666666</v>
+        <v>46156.97916666666</v>
       </c>
       <c r="B96" s="4" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
     </row>
     <row r="97" ht="16" customHeight="1" s="5">
       <c r="A97" s="3" t="n">
-        <v>46155.98958333334</v>
+        <v>46156.98958333334</v>
       </c>
       <c r="B97" s="4" t="n">
         <v>0</v>
@@ -5737,7 +5737,7 @@
     </row>
     <row r="98" ht="16" customHeight="1" s="5">
       <c r="A98" s="3" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B98" s="4" t="n">
         <v>0</v>
@@ -5784,7 +5784,7 @@
     </row>
     <row r="99" ht="16" customHeight="1" s="5">
       <c r="A99" s="3" t="n">
-        <v>46156.01041666666</v>
+        <v>46157.01041666666</v>
       </c>
       <c r="B99" s="4" t="n">
         <v>10</v>
@@ -5831,7 +5831,7 @@
     </row>
     <row r="100" ht="16" customHeight="1" s="5">
       <c r="A100" s="3" t="n">
-        <v>46156.02083333334</v>
+        <v>46157.02083333334</v>
       </c>
       <c r="B100" s="4" t="n">
         <v>28</v>
@@ -5878,7 +5878,7 @@
     </row>
     <row r="101" ht="16" customHeight="1" s="5">
       <c r="A101" s="3" t="n">
-        <v>46156.03125</v>
+        <v>46157.03125</v>
       </c>
       <c r="B101" s="4" t="n">
         <v>48</v>
@@ -5925,7 +5925,7 @@
     </row>
     <row r="102" ht="16" customHeight="1" s="5">
       <c r="A102" s="3" t="n">
-        <v>46156.04166666666</v>
+        <v>46157.04166666666</v>
       </c>
       <c r="B102" s="4" t="n">
         <v>58</v>
@@ -5972,7 +5972,7 @@
     </row>
     <row r="103" ht="16" customHeight="1" s="5">
       <c r="A103" s="3" t="n">
-        <v>46156.05208333334</v>
+        <v>46157.05208333334</v>
       </c>
       <c r="B103" s="4" t="n">
         <v>9</v>
@@ -6019,7 +6019,7 @@
     </row>
     <row r="104" ht="16" customHeight="1" s="5">
       <c r="A104" s="3" t="n">
-        <v>46156.0625</v>
+        <v>46157.0625</v>
       </c>
       <c r="B104" s="4" t="n">
         <v>0</v>
@@ -6066,7 +6066,7 @@
     </row>
     <row r="105" ht="16" customHeight="1" s="5">
       <c r="A105" s="3" t="n">
-        <v>46156.07291666666</v>
+        <v>46157.07291666666</v>
       </c>
       <c r="B105" s="4" t="n">
         <v>4</v>
@@ -6113,7 +6113,7 @@
     </row>
     <row r="106" ht="16" customHeight="1" s="5">
       <c r="A106" s="3" t="n">
-        <v>46156.08333333334</v>
+        <v>46157.08333333334</v>
       </c>
       <c r="B106" s="4" t="n">
         <v>11</v>
@@ -6160,7 +6160,7 @@
     </row>
     <row r="107" ht="16" customHeight="1" s="5">
       <c r="A107" s="3" t="n">
-        <v>46156.09375</v>
+        <v>46157.09375</v>
       </c>
       <c r="B107" s="4" t="n">
         <v>20</v>
@@ -6207,7 +6207,7 @@
     </row>
     <row r="108" ht="16" customHeight="1" s="5">
       <c r="A108" s="3" t="n">
-        <v>46156.10416666666</v>
+        <v>46157.10416666666</v>
       </c>
       <c r="B108" s="4" t="n">
         <v>33</v>
@@ -6254,7 +6254,7 @@
     </row>
     <row r="109" ht="16" customHeight="1" s="5">
       <c r="A109" s="3" t="n">
-        <v>46156.11458333334</v>
+        <v>46157.11458333334</v>
       </c>
       <c r="B109" s="4" t="n">
         <v>17</v>
@@ -6301,7 +6301,7 @@
     </row>
     <row r="110" ht="16" customHeight="1" s="5">
       <c r="A110" s="3" t="n">
-        <v>46156.125</v>
+        <v>46157.125</v>
       </c>
       <c r="B110" s="4" t="n">
         <v>27</v>
@@ -6348,7 +6348,7 @@
     </row>
     <row r="111" ht="16" customHeight="1" s="5">
       <c r="A111" s="3" t="n">
-        <v>46156.13541666666</v>
+        <v>46157.13541666666</v>
       </c>
       <c r="B111" s="4" t="n">
         <v>41</v>
@@ -6395,7 +6395,7 @@
     </row>
     <row r="112" ht="16" customHeight="1" s="5">
       <c r="A112" s="3" t="n">
-        <v>46156.14583333334</v>
+        <v>46157.14583333334</v>
       </c>
       <c r="B112" s="4" t="n">
         <v>75</v>
@@ -6442,7 +6442,7 @@
     </row>
     <row r="113" ht="16" customHeight="1" s="5">
       <c r="A113" s="3" t="n">
-        <v>46156.15625</v>
+        <v>46157.15625</v>
       </c>
       <c r="B113" s="4" t="n">
         <v>268</v>
@@ -6489,7 +6489,7 @@
     </row>
     <row r="114" ht="16" customHeight="1" s="5">
       <c r="A114" s="3" t="n">
-        <v>46156.16666666666</v>
+        <v>46157.16666666666</v>
       </c>
       <c r="B114" s="4" t="n">
         <v>527</v>
@@ -6536,7 +6536,7 @@
     </row>
     <row r="115" ht="16" customHeight="1" s="5">
       <c r="A115" s="3" t="n">
-        <v>46156.17708333334</v>
+        <v>46157.17708333334</v>
       </c>
       <c r="B115" s="4" t="n">
         <v>888</v>
@@ -6583,7 +6583,7 @@
     </row>
     <row r="116" ht="16" customHeight="1" s="5">
       <c r="A116" s="3" t="n">
-        <v>46156.1875</v>
+        <v>46157.1875</v>
       </c>
       <c r="B116" s="4" t="n">
         <v>1032</v>
@@ -6630,7 +6630,7 @@
     </row>
     <row r="117" ht="16" customHeight="1" s="5">
       <c r="A117" s="3" t="n">
-        <v>46156.19791666666</v>
+        <v>46157.19791666666</v>
       </c>
       <c r="B117" s="4" t="n">
         <v>780</v>
@@ -6677,7 +6677,7 @@
     </row>
     <row r="118" ht="16" customHeight="1" s="5">
       <c r="A118" s="3" t="n">
-        <v>46156.20833333334</v>
+        <v>46157.20833333334</v>
       </c>
       <c r="B118" s="4" t="n">
         <v>847</v>
@@ -6724,7 +6724,7 @@
     </row>
     <row r="119" ht="16" customHeight="1" s="5">
       <c r="A119" s="3" t="n">
-        <v>46156.21875</v>
+        <v>46157.21875</v>
       </c>
       <c r="B119" s="4" t="n">
         <v>689</v>
@@ -6771,7 +6771,7 @@
     </row>
     <row r="120" ht="16" customHeight="1" s="5">
       <c r="A120" s="3" t="n">
-        <v>46156.22916666666</v>
+        <v>46157.22916666666</v>
       </c>
       <c r="B120" s="4" t="n">
         <v>660</v>
@@ -6818,7 +6818,7 @@
     </row>
     <row r="121" ht="16" customHeight="1" s="5">
       <c r="A121" s="3" t="n">
-        <v>46156.23958333334</v>
+        <v>46157.23958333334</v>
       </c>
       <c r="B121" s="4" t="n">
         <v>671</v>
@@ -6865,7 +6865,7 @@
     </row>
     <row r="122" ht="16" customHeight="1" s="5">
       <c r="A122" s="3" t="n">
-        <v>46156.25</v>
+        <v>46157.25</v>
       </c>
       <c r="B122" s="4" t="n">
         <v>627</v>
@@ -6912,7 +6912,7 @@
     </row>
     <row r="123" ht="16" customHeight="1" s="5">
       <c r="A123" s="3" t="n">
-        <v>46156.26041666666</v>
+        <v>46157.26041666666</v>
       </c>
       <c r="B123" s="4" t="n">
         <v>513</v>
@@ -6959,7 +6959,7 @@
     </row>
     <row r="124" ht="16" customHeight="1" s="5">
       <c r="A124" s="3" t="n">
-        <v>46156.27083333334</v>
+        <v>46157.27083333334</v>
       </c>
       <c r="B124" s="4" t="n">
         <v>544</v>
@@ -7006,7 +7006,7 @@
     </row>
     <row r="125" ht="16" customHeight="1" s="5">
       <c r="A125" s="3" t="n">
-        <v>46156.28125</v>
+        <v>46157.28125</v>
       </c>
       <c r="B125" s="4" t="n">
         <v>417</v>
@@ -7053,7 +7053,7 @@
     </row>
     <row r="126" ht="16" customHeight="1" s="5">
       <c r="A126" s="3" t="n">
-        <v>46156.29166666666</v>
+        <v>46157.29166666666</v>
       </c>
       <c r="B126" s="4" t="n">
         <v>285</v>
@@ -7100,7 +7100,7 @@
     </row>
     <row r="127" ht="16" customHeight="1" s="5">
       <c r="A127" s="3" t="n">
-        <v>46156.30208333334</v>
+        <v>46157.30208333334</v>
       </c>
       <c r="B127" s="4" t="n">
         <v>290</v>
@@ -7147,7 +7147,7 @@
     </row>
     <row r="128" ht="16" customHeight="1" s="5">
       <c r="A128" s="3" t="n">
-        <v>46156.3125</v>
+        <v>46157.3125</v>
       </c>
       <c r="B128" s="4" t="n">
         <v>323</v>
@@ -7194,7 +7194,7 @@
     </row>
     <row r="129" ht="16" customHeight="1" s="5">
       <c r="A129" s="3" t="n">
-        <v>46156.32291666666</v>
+        <v>46157.32291666666</v>
       </c>
       <c r="B129" s="4" t="n">
         <v>271</v>
@@ -7241,7 +7241,7 @@
     </row>
     <row r="130" ht="16" customHeight="1" s="5">
       <c r="A130" s="3" t="n">
-        <v>46156.33333333334</v>
+        <v>46157.33333333334</v>
       </c>
       <c r="B130" s="4" t="n">
         <v>246</v>
@@ -7288,7 +7288,7 @@
     </row>
     <row r="131" ht="16" customHeight="1" s="5">
       <c r="A131" s="3" t="n">
-        <v>46156.34375</v>
+        <v>46157.34375</v>
       </c>
       <c r="B131" s="4" t="n">
         <v>287</v>
@@ -7335,7 +7335,7 @@
     </row>
     <row r="132" ht="16" customHeight="1" s="5">
       <c r="A132" s="3" t="n">
-        <v>46156.35416666666</v>
+        <v>46157.35416666666</v>
       </c>
       <c r="B132" s="4" t="n">
         <v>275</v>
@@ -7382,7 +7382,7 @@
     </row>
     <row r="133" ht="16" customHeight="1" s="5">
       <c r="A133" s="3" t="n">
-        <v>46156.36458333334</v>
+        <v>46157.36458333334</v>
       </c>
       <c r="B133" s="4" t="n">
         <v>447</v>
@@ -7429,7 +7429,7 @@
     </row>
     <row r="134" ht="16" customHeight="1" s="5">
       <c r="A134" s="3" t="n">
-        <v>46156.375</v>
+        <v>46157.375</v>
       </c>
       <c r="B134" s="4" t="n">
         <v>566</v>
@@ -7476,7 +7476,7 @@
     </row>
     <row r="135" ht="16" customHeight="1" s="5">
       <c r="A135" s="3" t="n">
-        <v>46156.38541666666</v>
+        <v>46157.38541666666</v>
       </c>
       <c r="B135" s="4" t="n">
         <v>590</v>
@@ -7523,7 +7523,7 @@
     </row>
     <row r="136" ht="16" customHeight="1" s="5">
       <c r="A136" s="3" t="n">
-        <v>46156.39583333334</v>
+        <v>46157.39583333334</v>
       </c>
       <c r="B136" s="4" t="n">
         <v>558</v>
@@ -7570,7 +7570,7 @@
     </row>
     <row r="137" ht="16" customHeight="1" s="5">
       <c r="A137" s="3" t="n">
-        <v>46156.40625</v>
+        <v>46157.40625</v>
       </c>
       <c r="B137" s="4" t="n">
         <v>354</v>
@@ -7617,7 +7617,7 @@
     </row>
     <row r="138" ht="16" customHeight="1" s="5">
       <c r="A138" s="3" t="n">
-        <v>46156.41666666666</v>
+        <v>46157.41666666666</v>
       </c>
       <c r="B138" s="4" t="n">
         <v>483</v>
@@ -7664,7 +7664,7 @@
     </row>
     <row r="139" ht="16" customHeight="1" s="5">
       <c r="A139" s="3" t="n">
-        <v>46156.42708333334</v>
+        <v>46157.42708333334</v>
       </c>
       <c r="B139" s="4" t="n">
         <v>537</v>
@@ -7711,7 +7711,7 @@
     </row>
     <row r="140" ht="16" customHeight="1" s="5">
       <c r="A140" s="3" t="n">
-        <v>46156.4375</v>
+        <v>46157.4375</v>
       </c>
       <c r="B140" s="4" t="n">
         <v>558</v>
@@ -7758,7 +7758,7 @@
     </row>
     <row r="141" ht="16" customHeight="1" s="5">
       <c r="A141" s="3" t="n">
-        <v>46156.44791666666</v>
+        <v>46157.44791666666</v>
       </c>
       <c r="B141" s="4" t="n">
         <v>570</v>
@@ -7805,7 +7805,7 @@
     </row>
     <row r="142" ht="16" customHeight="1" s="5">
       <c r="A142" s="3" t="n">
-        <v>46156.45833333334</v>
+        <v>46157.45833333334</v>
       </c>
       <c r="B142" s="4" t="n">
         <v>424</v>
@@ -7852,7 +7852,7 @@
     </row>
     <row r="143" ht="16" customHeight="1" s="5">
       <c r="A143" s="3" t="n">
-        <v>46156.46875</v>
+        <v>46157.46875</v>
       </c>
       <c r="B143" s="4" t="n">
         <v>377</v>
@@ -7899,7 +7899,7 @@
     </row>
     <row r="144" ht="16" customHeight="1" s="5">
       <c r="A144" s="3" t="n">
-        <v>46156.47916666666</v>
+        <v>46157.47916666666</v>
       </c>
       <c r="B144" s="4" t="n">
         <v>372</v>
@@ -7946,7 +7946,7 @@
     </row>
     <row r="145" ht="16" customHeight="1" s="5">
       <c r="A145" s="3" t="n">
-        <v>46156.48958333334</v>
+        <v>46157.48958333334</v>
       </c>
       <c r="B145" s="4" t="n">
         <v>374</v>
@@ -7993,7 +7993,7 @@
     </row>
     <row r="146" ht="16" customHeight="1" s="5">
       <c r="A146" s="3" t="n">
-        <v>46156.5</v>
+        <v>46157.5</v>
       </c>
       <c r="B146" s="4" t="n">
         <v>508</v>
@@ -8040,7 +8040,7 @@
     </row>
     <row r="147" ht="16" customHeight="1" s="5">
       <c r="A147" s="3" t="n">
-        <v>46156.51041666666</v>
+        <v>46157.51041666666</v>
       </c>
       <c r="B147" s="4" t="n">
         <v>482</v>
@@ -8087,7 +8087,7 @@
     </row>
     <row r="148" ht="16" customHeight="1" s="5">
       <c r="A148" s="3" t="n">
-        <v>46156.52083333334</v>
+        <v>46157.52083333334</v>
       </c>
       <c r="B148" s="4" t="n">
         <v>416</v>
@@ -8134,7 +8134,7 @@
     </row>
     <row r="149" ht="16" customHeight="1" s="5">
       <c r="A149" s="3" t="n">
-        <v>46156.53125</v>
+        <v>46157.53125</v>
       </c>
       <c r="B149" s="4" t="n">
         <v>498</v>
@@ -8181,7 +8181,7 @@
     </row>
     <row r="150" ht="16" customHeight="1" s="5">
       <c r="A150" s="3" t="n">
-        <v>46156.54166666666</v>
+        <v>46157.54166666666</v>
       </c>
       <c r="B150" s="4" t="n">
         <v>378</v>
@@ -8228,7 +8228,7 @@
     </row>
     <row r="151" ht="16" customHeight="1" s="5">
       <c r="A151" s="3" t="n">
-        <v>46156.55208333334</v>
+        <v>46157.55208333334</v>
       </c>
       <c r="B151" s="4" t="n">
         <v>245</v>
@@ -8275,7 +8275,7 @@
     </row>
     <row r="152" ht="16" customHeight="1" s="5">
       <c r="A152" s="3" t="n">
-        <v>46156.5625</v>
+        <v>46157.5625</v>
       </c>
       <c r="B152" s="4" t="n">
         <v>253</v>
@@ -8322,7 +8322,7 @@
     </row>
     <row r="153" ht="16" customHeight="1" s="5">
       <c r="A153" s="3" t="n">
-        <v>46156.57291666666</v>
+        <v>46157.57291666666</v>
       </c>
       <c r="B153" s="4" t="n">
         <v>302</v>
@@ -8369,7 +8369,7 @@
     </row>
     <row r="154" ht="16" customHeight="1" s="5">
       <c r="A154" s="3" t="n">
-        <v>46156.58333333334</v>
+        <v>46157.58333333334</v>
       </c>
       <c r="B154" s="4" t="n">
         <v>405</v>
@@ -8416,7 +8416,7 @@
     </row>
     <row r="155" ht="16" customHeight="1" s="5">
       <c r="A155" s="3" t="n">
-        <v>46156.59375</v>
+        <v>46157.59375</v>
       </c>
       <c r="B155" s="4" t="n">
         <v>472</v>
@@ -8463,7 +8463,7 @@
     </row>
     <row r="156" ht="16" customHeight="1" s="5">
       <c r="A156" s="3" t="n">
-        <v>46156.60416666666</v>
+        <v>46157.60416666666</v>
       </c>
       <c r="B156" s="4" t="n">
         <v>591</v>
@@ -8510,7 +8510,7 @@
     </row>
     <row r="157" ht="16" customHeight="1" s="5">
       <c r="A157" s="3" t="n">
-        <v>46156.61458333334</v>
+        <v>46157.61458333334</v>
       </c>
       <c r="B157" s="4" t="n">
         <v>607</v>
@@ -8557,7 +8557,7 @@
     </row>
     <row r="158" ht="16" customHeight="1" s="5">
       <c r="A158" s="3" t="n">
-        <v>46156.625</v>
+        <v>46157.625</v>
       </c>
       <c r="B158" s="4" t="n">
         <v>441</v>
@@ -8604,7 +8604,7 @@
     </row>
     <row r="159" ht="16" customHeight="1" s="5">
       <c r="A159" s="3" t="n">
-        <v>46156.63541666666</v>
+        <v>46157.63541666666</v>
       </c>
       <c r="B159" s="4" t="n">
         <v>309</v>
@@ -8651,7 +8651,7 @@
     </row>
     <row r="160" ht="16" customHeight="1" s="5">
       <c r="A160" s="3" t="n">
-        <v>46156.64583333334</v>
+        <v>46157.64583333334</v>
       </c>
       <c r="B160" s="4" t="n">
         <v>406</v>
@@ -8698,7 +8698,7 @@
     </row>
     <row r="161" ht="16" customHeight="1" s="5">
       <c r="A161" s="3" t="n">
-        <v>46156.65625</v>
+        <v>46157.65625</v>
       </c>
       <c r="B161" s="4" t="n">
         <v>545</v>
@@ -8745,7 +8745,7 @@
     </row>
     <row r="162" ht="16" customHeight="1" s="5">
       <c r="A162" s="3" t="n">
-        <v>46156.66666666666</v>
+        <v>46157.66666666666</v>
       </c>
       <c r="B162" s="4" t="n">
         <v>659</v>
@@ -8792,7 +8792,7 @@
     </row>
     <row r="163" ht="16" customHeight="1" s="5">
       <c r="A163" s="3" t="n">
-        <v>46156.67708333334</v>
+        <v>46157.67708333334</v>
       </c>
       <c r="B163" s="4" t="n">
         <v>904</v>
@@ -8839,7 +8839,7 @@
     </row>
     <row r="164" ht="16" customHeight="1" s="5">
       <c r="A164" s="3" t="n">
-        <v>46156.6875</v>
+        <v>46157.6875</v>
       </c>
       <c r="B164" s="4" t="n">
         <v>870</v>
@@ -8886,7 +8886,7 @@
     </row>
     <row r="165" ht="16" customHeight="1" s="5">
       <c r="A165" s="3" t="n">
-        <v>46156.69791666666</v>
+        <v>46157.69791666666</v>
       </c>
       <c r="B165" s="4" t="n">
         <v>773</v>
@@ -8933,7 +8933,7 @@
     </row>
     <row r="166" ht="16" customHeight="1" s="5">
       <c r="A166" s="3" t="n">
-        <v>46156.70833333334</v>
+        <v>46157.70833333334</v>
       </c>
       <c r="B166" s="4" t="n">
         <v>654</v>
@@ -8980,7 +8980,7 @@
     </row>
     <row r="167" ht="16" customHeight="1" s="5">
       <c r="A167" s="3" t="n">
-        <v>46156.71875</v>
+        <v>46157.71875</v>
       </c>
       <c r="B167" s="4" t="n">
         <v>472</v>
@@ -9027,7 +9027,7 @@
     </row>
     <row r="168" ht="16" customHeight="1" s="5">
       <c r="A168" s="3" t="n">
-        <v>46156.72916666666</v>
+        <v>46157.72916666666</v>
       </c>
       <c r="B168" s="4" t="n">
         <v>483</v>
@@ -9074,7 +9074,7 @@
     </row>
     <row r="169" ht="16" customHeight="1" s="5">
       <c r="A169" s="3" t="n">
-        <v>46156.73958333334</v>
+        <v>46157.73958333334</v>
       </c>
       <c r="B169" s="4" t="n">
         <v>597</v>
@@ -9121,7 +9121,7 @@
     </row>
     <row r="170" ht="16" customHeight="1" s="5">
       <c r="A170" s="3" t="n">
-        <v>46156.75</v>
+        <v>46157.75</v>
       </c>
       <c r="B170" s="4" t="n">
         <v>597</v>
@@ -9168,7 +9168,7 @@
     </row>
     <row r="171" ht="16" customHeight="1" s="5">
       <c r="A171" s="3" t="n">
-        <v>46156.76041666666</v>
+        <v>46157.76041666666</v>
       </c>
       <c r="B171" s="4" t="n">
         <v>569</v>
@@ -9215,7 +9215,7 @@
     </row>
     <row r="172" ht="16" customHeight="1" s="5">
       <c r="A172" s="3" t="n">
-        <v>46156.77083333334</v>
+        <v>46157.77083333334</v>
       </c>
       <c r="B172" s="4" t="n">
         <v>423</v>
@@ -9262,7 +9262,7 @@
     </row>
     <row r="173" ht="16" customHeight="1" s="5">
       <c r="A173" s="3" t="n">
-        <v>46156.78125</v>
+        <v>46157.78125</v>
       </c>
       <c r="B173" s="4" t="n">
         <v>269</v>
@@ -9309,7 +9309,7 @@
     </row>
     <row r="174" ht="16" customHeight="1" s="5">
       <c r="A174" s="3" t="n">
-        <v>46156.79166666666</v>
+        <v>46157.79166666666</v>
       </c>
       <c r="B174" s="4" t="n">
         <v>312</v>
@@ -9356,7 +9356,7 @@
     </row>
     <row r="175" ht="16" customHeight="1" s="5">
       <c r="A175" s="3" t="n">
-        <v>46156.80208333334</v>
+        <v>46157.80208333334</v>
       </c>
       <c r="B175" s="4" t="n">
         <v>557</v>
@@ -9403,7 +9403,7 @@
     </row>
     <row r="176" ht="16" customHeight="1" s="5">
       <c r="A176" s="3" t="n">
-        <v>46156.8125</v>
+        <v>46157.8125</v>
       </c>
       <c r="B176" s="4" t="n">
         <v>690</v>
@@ -9450,7 +9450,7 @@
     </row>
     <row r="177" ht="16" customHeight="1" s="5">
       <c r="A177" s="3" t="n">
-        <v>46156.82291666666</v>
+        <v>46157.82291666666</v>
       </c>
       <c r="B177" s="4" t="n">
         <v>511</v>
@@ -9497,7 +9497,7 @@
     </row>
     <row r="178" ht="16" customHeight="1" s="5">
       <c r="A178" s="3" t="n">
-        <v>46156.83333333334</v>
+        <v>46157.83333333334</v>
       </c>
       <c r="B178" s="4" t="n">
         <v>188</v>
@@ -9544,7 +9544,7 @@
     </row>
     <row r="179" ht="16" customHeight="1" s="5">
       <c r="A179" s="3" t="n">
-        <v>46156.84375</v>
+        <v>46157.84375</v>
       </c>
       <c r="B179" s="4" t="n">
         <v>204</v>
@@ -9591,7 +9591,7 @@
     </row>
     <row r="180" ht="16" customHeight="1" s="5">
       <c r="A180" s="3" t="n">
-        <v>46156.85416666666</v>
+        <v>46157.85416666666</v>
       </c>
       <c r="B180" s="4" t="n">
         <v>287</v>
@@ -9638,7 +9638,7 @@
     </row>
     <row r="181" ht="16" customHeight="1" s="5">
       <c r="A181" s="3" t="n">
-        <v>46156.86458333334</v>
+        <v>46157.86458333334</v>
       </c>
       <c r="B181" s="4" t="n">
         <v>177</v>
@@ -9685,7 +9685,7 @@
     </row>
     <row r="182" ht="16" customHeight="1" s="5">
       <c r="A182" s="3" t="n">
-        <v>46156.875</v>
+        <v>46157.875</v>
       </c>
       <c r="B182" s="4" t="n">
         <v>9</v>
@@ -9732,7 +9732,7 @@
     </row>
     <row r="183" ht="16" customHeight="1" s="5">
       <c r="A183" s="3" t="n">
-        <v>46156.88541666666</v>
+        <v>46157.88541666666</v>
       </c>
       <c r="B183" s="4" t="n">
         <v>0</v>
@@ -9779,7 +9779,7 @@
     </row>
     <row r="184" ht="16" customHeight="1" s="5">
       <c r="A184" s="3" t="n">
-        <v>46156.89583333334</v>
+        <v>46157.89583333334</v>
       </c>
       <c r="B184" s="4" t="n">
         <v>0</v>
@@ -9826,7 +9826,7 @@
     </row>
     <row r="185" ht="16" customHeight="1" s="5">
       <c r="A185" s="3" t="n">
-        <v>46156.90625</v>
+        <v>46157.90625</v>
       </c>
       <c r="B185" s="4" t="n">
         <v>15</v>
@@ -9873,7 +9873,7 @@
     </row>
     <row r="186" ht="16" customHeight="1" s="5">
       <c r="A186" s="3" t="n">
-        <v>46156.91666666666</v>
+        <v>46157.91666666666</v>
       </c>
       <c r="B186" s="4" t="n">
         <v>69</v>
@@ -9920,7 +9920,7 @@
     </row>
     <row r="187" ht="16" customHeight="1" s="5">
       <c r="A187" s="3" t="n">
-        <v>46156.92708333334</v>
+        <v>46157.92708333334</v>
       </c>
       <c r="B187" s="4" t="n">
         <v>126</v>
@@ -9967,7 +9967,7 @@
     </row>
     <row r="188" ht="16" customHeight="1" s="5">
       <c r="A188" s="3" t="n">
-        <v>46156.9375</v>
+        <v>46157.9375</v>
       </c>
       <c r="B188" s="4" t="n">
         <v>175</v>
@@ -10014,7 +10014,7 @@
     </row>
     <row r="189" ht="16" customHeight="1" s="5">
       <c r="A189" s="3" t="n">
-        <v>46156.94791666666</v>
+        <v>46157.94791666666</v>
       </c>
       <c r="B189" s="4" t="n">
         <v>82</v>
@@ -10061,7 +10061,7 @@
     </row>
     <row r="190" ht="16" customHeight="1" s="5">
       <c r="A190" s="3" t="n">
-        <v>46156.95833333334</v>
+        <v>46157.95833333334</v>
       </c>
       <c r="B190" s="4" t="n">
         <v>0</v>
@@ -10108,7 +10108,7 @@
     </row>
     <row r="191" ht="16" customHeight="1" s="5">
       <c r="A191" s="3" t="n">
-        <v>46156.96875</v>
+        <v>46157.96875</v>
       </c>
       <c r="B191" s="4" t="n">
         <v>0</v>
@@ -10155,7 +10155,7 @@
     </row>
     <row r="192" ht="16" customHeight="1" s="5">
       <c r="A192" s="3" t="n">
-        <v>46156.97916666666</v>
+        <v>46157.97916666666</v>
       </c>
       <c r="B192" s="4" t="n">
         <v>0</v>
@@ -10202,7 +10202,7 @@
     </row>
     <row r="193" ht="16" customHeight="1" s="5">
       <c r="A193" s="3" t="n">
-        <v>46156.98958333334</v>
+        <v>46157.98958333334</v>
       </c>
       <c r="B193" s="4" t="n">
         <v>0</v>
@@ -10249,7 +10249,7 @@
     </row>
     <row r="194" ht="16" customHeight="1" s="5">
       <c r="A194" s="3" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B194" s="4" t="n">
         <v>0</v>
@@ -10296,7 +10296,7 @@
     </row>
     <row r="195" ht="16" customHeight="1" s="5">
       <c r="A195" s="3" t="n">
-        <v>46157.01041666666</v>
+        <v>46158.01041666666</v>
       </c>
       <c r="B195" s="4" t="n">
         <v>10</v>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="196" ht="16" customHeight="1" s="5">
       <c r="A196" s="3" t="n">
-        <v>46157.02083333334</v>
+        <v>46158.02083333334</v>
       </c>
       <c r="B196" s="4" t="n">
         <v>35</v>
@@ -10390,7 +10390,7 @@
     </row>
     <row r="197" ht="16" customHeight="1" s="5">
       <c r="A197" s="3" t="n">
-        <v>46157.03125</v>
+        <v>46158.03125</v>
       </c>
       <c r="B197" s="4" t="n">
         <v>62</v>
@@ -10437,7 +10437,7 @@
     </row>
     <row r="198" ht="16" customHeight="1" s="5">
       <c r="A198" s="3" t="n">
-        <v>46157.04166666666</v>
+        <v>46158.04166666666</v>
       </c>
       <c r="B198" s="4" t="n">
         <v>80</v>
@@ -10484,7 +10484,7 @@
     </row>
     <row r="199" ht="16" customHeight="1" s="5">
       <c r="A199" s="3" t="n">
-        <v>46157.05208333334</v>
+        <v>46158.05208333334</v>
       </c>
       <c r="B199" s="4" t="n">
         <v>27</v>
@@ -10531,7 +10531,7 @@
     </row>
     <row r="200" ht="16" customHeight="1" s="5">
       <c r="A200" s="3" t="n">
-        <v>46157.0625</v>
+        <v>46158.0625</v>
       </c>
       <c r="B200" s="4" t="n">
         <v>0</v>
@@ -10578,7 +10578,7 @@
     </row>
     <row r="201" ht="16" customHeight="1" s="5">
       <c r="A201" s="3" t="n">
-        <v>46157.07291666666</v>
+        <v>46158.07291666666</v>
       </c>
       <c r="B201" s="4" t="n">
         <v>4</v>
@@ -10625,7 +10625,7 @@
     </row>
     <row r="202" ht="16" customHeight="1" s="5">
       <c r="A202" s="3" t="n">
-        <v>46157.08333333334</v>
+        <v>46158.08333333334</v>
       </c>
       <c r="B202" s="4" t="n">
         <v>11</v>
@@ -10672,7 +10672,7 @@
     </row>
     <row r="203" ht="16" customHeight="1" s="5">
       <c r="A203" s="3" t="n">
-        <v>46157.09375</v>
+        <v>46158.09375</v>
       </c>
       <c r="B203" s="4" t="n">
         <v>20</v>
@@ -10719,7 +10719,7 @@
     </row>
     <row r="204" ht="16" customHeight="1" s="5">
       <c r="A204" s="3" t="n">
-        <v>46157.10416666666</v>
+        <v>46158.10416666666</v>
       </c>
       <c r="B204" s="4" t="n">
         <v>33</v>
@@ -10766,7 +10766,7 @@
     </row>
     <row r="205" ht="16" customHeight="1" s="5">
       <c r="A205" s="3" t="n">
-        <v>46157.11458333334</v>
+        <v>46158.11458333334</v>
       </c>
       <c r="B205" s="4" t="n">
         <v>17</v>
@@ -10813,7 +10813,7 @@
     </row>
     <row r="206" ht="16" customHeight="1" s="5">
       <c r="A206" s="3" t="n">
-        <v>46157.125</v>
+        <v>46158.125</v>
       </c>
       <c r="B206" s="4" t="n">
         <v>19</v>
@@ -10860,7 +10860,7 @@
     </row>
     <row r="207" ht="16" customHeight="1" s="5">
       <c r="A207" s="3" t="n">
-        <v>46157.13541666666</v>
+        <v>46158.13541666666</v>
       </c>
       <c r="B207" s="4" t="n">
         <v>26</v>
@@ -10907,7 +10907,7 @@
     </row>
     <row r="208" ht="16" customHeight="1" s="5">
       <c r="A208" s="3" t="n">
-        <v>46157.14583333334</v>
+        <v>46158.14583333334</v>
       </c>
       <c r="B208" s="4" t="n">
         <v>65</v>
@@ -10954,7 +10954,7 @@
     </row>
     <row r="209" ht="16" customHeight="1" s="5">
       <c r="A209" s="3" t="n">
-        <v>46157.15625</v>
+        <v>46158.15625</v>
       </c>
       <c r="B209" s="4" t="n">
         <v>256</v>
@@ -11001,7 +11001,7 @@
     </row>
     <row r="210" ht="16" customHeight="1" s="5">
       <c r="A210" s="3" t="n">
-        <v>46157.16666666666</v>
+        <v>46158.16666666666</v>
       </c>
       <c r="B210" s="4" t="n">
         <v>528</v>
@@ -11048,7 +11048,7 @@
     </row>
     <row r="211" ht="16" customHeight="1" s="5">
       <c r="A211" s="3" t="n">
-        <v>46157.17708333334</v>
+        <v>46158.17708333334</v>
       </c>
       <c r="B211" s="4" t="n">
         <v>850</v>
@@ -11095,7 +11095,7 @@
     </row>
     <row r="212" ht="16" customHeight="1" s="5">
       <c r="A212" s="3" t="n">
-        <v>46157.1875</v>
+        <v>46158.1875</v>
       </c>
       <c r="B212" s="4" t="n">
         <v>967</v>
@@ -11142,7 +11142,7 @@
     </row>
     <row r="213" ht="16" customHeight="1" s="5">
       <c r="A213" s="3" t="n">
-        <v>46157.19791666666</v>
+        <v>46158.19791666666</v>
       </c>
       <c r="B213" s="4" t="n">
         <v>755</v>
@@ -11189,7 +11189,7 @@
     </row>
     <row r="214" ht="16" customHeight="1" s="5">
       <c r="A214" s="3" t="n">
-        <v>46157.20833333334</v>
+        <v>46158.20833333334</v>
       </c>
       <c r="B214" s="4" t="n">
         <v>800</v>
@@ -11236,7 +11236,7 @@
     </row>
     <row r="215" ht="16" customHeight="1" s="5">
       <c r="A215" s="3" t="n">
-        <v>46157.21875</v>
+        <v>46158.21875</v>
       </c>
       <c r="B215" s="4" t="n">
         <v>656</v>
@@ -11283,7 +11283,7 @@
     </row>
     <row r="216" ht="16" customHeight="1" s="5">
       <c r="A216" s="3" t="n">
-        <v>46157.22916666666</v>
+        <v>46158.22916666666</v>
       </c>
       <c r="B216" s="4" t="n">
         <v>515</v>
@@ -11330,7 +11330,7 @@
     </row>
     <row r="217" ht="16" customHeight="1" s="5">
       <c r="A217" s="3" t="n">
-        <v>46157.23958333334</v>
+        <v>46158.23958333334</v>
       </c>
       <c r="B217" s="4" t="n">
         <v>474</v>
@@ -11377,7 +11377,7 @@
     </row>
     <row r="218" ht="16" customHeight="1" s="5">
       <c r="A218" s="3" t="n">
-        <v>46157.25</v>
+        <v>46158.25</v>
       </c>
       <c r="B218" s="4" t="n">
         <v>601</v>
@@ -11424,7 +11424,7 @@
     </row>
     <row r="219" ht="16" customHeight="1" s="5">
       <c r="A219" s="3" t="n">
-        <v>46157.26041666666</v>
+        <v>46158.26041666666</v>
       </c>
       <c r="B219" s="4" t="n">
         <v>632</v>
@@ -11471,7 +11471,7 @@
     </row>
     <row r="220" ht="16" customHeight="1" s="5">
       <c r="A220" s="3" t="n">
-        <v>46157.27083333334</v>
+        <v>46158.27083333334</v>
       </c>
       <c r="B220" s="4" t="n">
         <v>592</v>
@@ -11518,7 +11518,7 @@
     </row>
     <row r="221" ht="16" customHeight="1" s="5">
       <c r="A221" s="3" t="n">
-        <v>46157.28125</v>
+        <v>46158.28125</v>
       </c>
       <c r="B221" s="4" t="n">
         <v>493</v>
@@ -11565,7 +11565,7 @@
     </row>
     <row r="222" ht="16" customHeight="1" s="5">
       <c r="A222" s="3" t="n">
-        <v>46157.29166666666</v>
+        <v>46158.29166666666</v>
       </c>
       <c r="B222" s="4" t="n">
         <v>448</v>
@@ -11612,7 +11612,7 @@
     </row>
     <row r="223" ht="16" customHeight="1" s="5">
       <c r="A223" s="3" t="n">
-        <v>46157.30208333334</v>
+        <v>46158.30208333334</v>
       </c>
       <c r="B223" s="4" t="n">
         <v>459</v>
@@ -11659,7 +11659,7 @@
     </row>
     <row r="224" ht="16" customHeight="1" s="5">
       <c r="A224" s="3" t="n">
-        <v>46157.3125</v>
+        <v>46158.3125</v>
       </c>
       <c r="B224" s="4" t="n">
         <v>432</v>
@@ -11706,7 +11706,7 @@
     </row>
     <row r="225" ht="16" customHeight="1" s="5">
       <c r="A225" s="3" t="n">
-        <v>46157.32291666666</v>
+        <v>46158.32291666666</v>
       </c>
       <c r="B225" s="4" t="n">
         <v>368</v>
@@ -11753,7 +11753,7 @@
     </row>
     <row r="226" ht="16" customHeight="1" s="5">
       <c r="A226" s="3" t="n">
-        <v>46157.33333333334</v>
+        <v>46158.33333333334</v>
       </c>
       <c r="B226" s="4" t="n">
         <v>320</v>
@@ -11800,7 +11800,7 @@
     </row>
     <row r="227" ht="16" customHeight="1" s="5">
       <c r="A227" s="3" t="n">
-        <v>46157.34375</v>
+        <v>46158.34375</v>
       </c>
       <c r="B227" s="4" t="n">
         <v>237</v>
@@ -11847,7 +11847,7 @@
     </row>
     <row r="228" ht="16" customHeight="1" s="5">
       <c r="A228" s="3" t="n">
-        <v>46157.35416666666</v>
+        <v>46158.35416666666</v>
       </c>
       <c r="B228" s="4" t="n">
         <v>262</v>
@@ -11894,7 +11894,7 @@
     </row>
     <row r="229" ht="16" customHeight="1" s="5">
       <c r="A229" s="3" t="n">
-        <v>46157.36458333334</v>
+        <v>46158.36458333334</v>
       </c>
       <c r="B229" s="4" t="n">
         <v>445</v>
@@ -11941,7 +11941,7 @@
     </row>
     <row r="230" ht="16" customHeight="1" s="5">
       <c r="A230" s="3" t="n">
-        <v>46157.375</v>
+        <v>46158.375</v>
       </c>
       <c r="B230" s="4" t="n">
         <v>627</v>
@@ -11988,7 +11988,7 @@
     </row>
     <row r="231" ht="16" customHeight="1" s="5">
       <c r="A231" s="3" t="n">
-        <v>46157.38541666666</v>
+        <v>46158.38541666666</v>
       </c>
       <c r="B231" s="4" t="n">
         <v>623</v>
@@ -12035,7 +12035,7 @@
     </row>
     <row r="232" ht="16" customHeight="1" s="5">
       <c r="A232" s="3" t="n">
-        <v>46157.39583333334</v>
+        <v>46158.39583333334</v>
       </c>
       <c r="B232" s="4" t="n">
         <v>576</v>
@@ -12082,7 +12082,7 @@
     </row>
     <row r="233" ht="16" customHeight="1" s="5">
       <c r="A233" s="3" t="n">
-        <v>46157.40625</v>
+        <v>46158.40625</v>
       </c>
       <c r="B233" s="4" t="n">
         <v>542</v>
@@ -12129,7 +12129,7 @@
     </row>
     <row r="234" ht="16" customHeight="1" s="5">
       <c r="A234" s="3" t="n">
-        <v>46157.41666666666</v>
+        <v>46158.41666666666</v>
       </c>
       <c r="B234" s="4" t="n">
         <v>484</v>
@@ -12176,7 +12176,7 @@
     </row>
     <row r="235" ht="16" customHeight="1" s="5">
       <c r="A235" s="3" t="n">
-        <v>46157.42708333334</v>
+        <v>46158.42708333334</v>
       </c>
       <c r="B235" s="4" t="n">
         <v>377</v>
@@ -12223,7 +12223,7 @@
     </row>
     <row r="236" ht="16" customHeight="1" s="5">
       <c r="A236" s="3" t="n">
-        <v>46157.4375</v>
+        <v>46158.4375</v>
       </c>
       <c r="B236" s="4" t="n">
         <v>281</v>
@@ -12270,7 +12270,7 @@
     </row>
     <row r="237" ht="16" customHeight="1" s="5">
       <c r="A237" s="3" t="n">
-        <v>46157.44791666666</v>
+        <v>46158.44791666666</v>
       </c>
       <c r="B237" s="4" t="n">
         <v>386</v>
@@ -12317,7 +12317,7 @@
     </row>
     <row r="238" ht="16" customHeight="1" s="5">
       <c r="A238" s="3" t="n">
-        <v>46157.45833333334</v>
+        <v>46158.45833333334</v>
       </c>
       <c r="B238" s="4" t="n">
         <v>548</v>
@@ -12364,7 +12364,7 @@
     </row>
     <row r="239" ht="16" customHeight="1" s="5">
       <c r="A239" s="3" t="n">
-        <v>46157.46875</v>
+        <v>46158.46875</v>
       </c>
       <c r="B239" s="4" t="n">
         <v>620</v>
@@ -12411,7 +12411,7 @@
     </row>
     <row r="240" ht="16" customHeight="1" s="5">
       <c r="A240" s="3" t="n">
-        <v>46157.47916666666</v>
+        <v>46158.47916666666</v>
       </c>
       <c r="B240" s="4" t="n">
         <v>531</v>
@@ -12458,7 +12458,7 @@
     </row>
     <row r="241" ht="16" customHeight="1" s="5">
       <c r="A241" s="3" t="n">
-        <v>46157.48958333334</v>
+        <v>46158.48958333334</v>
       </c>
       <c r="B241" s="4" t="n">
         <v>491</v>
@@ -12505,7 +12505,7 @@
     </row>
     <row r="242" ht="16" customHeight="1" s="5">
       <c r="A242" s="3" t="n">
-        <v>46157.5</v>
+        <v>46158.5</v>
       </c>
       <c r="B242" s="4" t="n">
         <v>385</v>
@@ -12552,7 +12552,7 @@
     </row>
     <row r="243" ht="16" customHeight="1" s="5">
       <c r="A243" s="3" t="n">
-        <v>46157.51041666666</v>
+        <v>46158.51041666666</v>
       </c>
       <c r="B243" s="4" t="n">
         <v>397</v>
@@ -12599,7 +12599,7 @@
     </row>
     <row r="244" ht="16" customHeight="1" s="5">
       <c r="A244" s="3" t="n">
-        <v>46157.52083333334</v>
+        <v>46158.52083333334</v>
       </c>
       <c r="B244" s="4" t="n">
         <v>490</v>
@@ -12646,7 +12646,7 @@
     </row>
     <row r="245" ht="16" customHeight="1" s="5">
       <c r="A245" s="3" t="n">
-        <v>46157.53125</v>
+        <v>46158.53125</v>
       </c>
       <c r="B245" s="4" t="n">
         <v>547</v>
@@ -12693,7 +12693,7 @@
     </row>
     <row r="246" ht="16" customHeight="1" s="5">
       <c r="A246" s="3" t="n">
-        <v>46157.54166666666</v>
+        <v>46158.54166666666</v>
       </c>
       <c r="B246" s="4" t="n">
         <v>415</v>
@@ -12740,7 +12740,7 @@
     </row>
     <row r="247" ht="16" customHeight="1" s="5">
       <c r="A247" s="3" t="n">
-        <v>46157.55208333334</v>
+        <v>46158.55208333334</v>
       </c>
       <c r="B247" s="4" t="n">
         <v>228</v>
@@ -12787,7 +12787,7 @@
     </row>
     <row r="248" ht="16" customHeight="1" s="5">
       <c r="A248" s="3" t="n">
-        <v>46157.5625</v>
+        <v>46158.5625</v>
       </c>
       <c r="B248" s="4" t="n">
         <v>309</v>
@@ -12834,7 +12834,7 @@
     </row>
     <row r="249" ht="16" customHeight="1" s="5">
       <c r="A249" s="3" t="n">
-        <v>46157.57291666666</v>
+        <v>46158.57291666666</v>
       </c>
       <c r="B249" s="4" t="n">
         <v>411</v>
@@ -12881,7 +12881,7 @@
     </row>
     <row r="250" ht="16" customHeight="1" s="5">
       <c r="A250" s="3" t="n">
-        <v>46157.58333333334</v>
+        <v>46158.58333333334</v>
       </c>
       <c r="B250" s="4" t="n">
         <v>385</v>
@@ -12928,7 +12928,7 @@
     </row>
     <row r="251" ht="16" customHeight="1" s="5">
       <c r="A251" s="3" t="n">
-        <v>46157.59375</v>
+        <v>46158.59375</v>
       </c>
       <c r="B251" s="4" t="n">
         <v>436</v>
@@ -12975,7 +12975,7 @@
     </row>
     <row r="252" ht="16" customHeight="1" s="5">
       <c r="A252" s="3" t="n">
-        <v>46157.60416666666</v>
+        <v>46158.60416666666</v>
       </c>
       <c r="B252" s="4" t="n">
         <v>446</v>
@@ -13022,7 +13022,7 @@
     </row>
     <row r="253" ht="16" customHeight="1" s="5">
       <c r="A253" s="3" t="n">
-        <v>46157.61458333334</v>
+        <v>46158.61458333334</v>
       </c>
       <c r="B253" s="4" t="n">
         <v>426</v>
@@ -13069,7 +13069,7 @@
     </row>
     <row r="254" ht="16" customHeight="1" s="5">
       <c r="A254" s="3" t="n">
-        <v>46157.625</v>
+        <v>46158.625</v>
       </c>
       <c r="B254" s="4" t="n">
         <v>450</v>
@@ -13116,7 +13116,7 @@
     </row>
     <row r="255" ht="16" customHeight="1" s="5">
       <c r="A255" s="3" t="n">
-        <v>46157.63541666666</v>
+        <v>46158.63541666666</v>
       </c>
       <c r="B255" s="4" t="n">
         <v>322</v>
@@ -13163,7 +13163,7 @@
     </row>
     <row r="256" ht="16" customHeight="1" s="5">
       <c r="A256" s="3" t="n">
-        <v>46157.64583333334</v>
+        <v>46158.64583333334</v>
       </c>
       <c r="B256" s="4" t="n">
         <v>303</v>
@@ -13210,7 +13210,7 @@
     </row>
     <row r="257" ht="16" customHeight="1" s="5">
       <c r="A257" s="3" t="n">
-        <v>46157.65625</v>
+        <v>46158.65625</v>
       </c>
       <c r="B257" s="4" t="n">
         <v>496</v>
@@ -13257,7 +13257,7 @@
     </row>
     <row r="258" ht="16" customHeight="1" s="5">
       <c r="A258" s="3" t="n">
-        <v>46157.66666666666</v>
+        <v>46158.66666666666</v>
       </c>
       <c r="B258" s="4" t="n">
         <v>654</v>
@@ -13304,7 +13304,7 @@
     </row>
     <row r="259" ht="16" customHeight="1" s="5">
       <c r="A259" s="3" t="n">
-        <v>46157.67708333334</v>
+        <v>46158.67708333334</v>
       </c>
       <c r="B259" s="4" t="n">
         <v>781</v>
@@ -13351,7 +13351,7 @@
     </row>
     <row r="260" ht="16" customHeight="1" s="5">
       <c r="A260" s="3" t="n">
-        <v>46157.6875</v>
+        <v>46158.6875</v>
       </c>
       <c r="B260" s="4" t="n">
         <v>795</v>
@@ -13398,7 +13398,7 @@
     </row>
     <row r="261" ht="16" customHeight="1" s="5">
       <c r="A261" s="3" t="n">
-        <v>46157.69791666666</v>
+        <v>46158.69791666666</v>
       </c>
       <c r="B261" s="4" t="n">
         <v>569</v>
@@ -13445,7 +13445,7 @@
     </row>
     <row r="262" ht="16" customHeight="1" s="5">
       <c r="A262" s="3" t="n">
-        <v>46157.70833333334</v>
+        <v>46158.70833333334</v>
       </c>
       <c r="B262" s="4" t="n">
         <v>611</v>
@@ -13492,7 +13492,7 @@
     </row>
     <row r="263" ht="16" customHeight="1" s="5">
       <c r="A263" s="3" t="n">
-        <v>46157.71875</v>
+        <v>46158.71875</v>
       </c>
       <c r="B263" s="4" t="n">
         <v>794</v>
@@ -13539,7 +13539,7 @@
     </row>
     <row r="264" ht="16" customHeight="1" s="5">
       <c r="A264" s="3" t="n">
-        <v>46157.72916666666</v>
+        <v>46158.72916666666</v>
       </c>
       <c r="B264" s="4" t="n">
         <v>635</v>
@@ -13586,7 +13586,7 @@
     </row>
     <row r="265" ht="16" customHeight="1" s="5">
       <c r="A265" s="3" t="n">
-        <v>46157.73958333334</v>
+        <v>46158.73958333334</v>
       </c>
       <c r="B265" s="4" t="n">
         <v>642</v>
@@ -13633,7 +13633,7 @@
     </row>
     <row r="266" ht="16" customHeight="1" s="5">
       <c r="A266" s="3" t="n">
-        <v>46157.75</v>
+        <v>46158.75</v>
       </c>
       <c r="B266" s="4" t="n">
         <v>624</v>
@@ -13680,7 +13680,7 @@
     </row>
     <row r="267" ht="16" customHeight="1" s="5">
       <c r="A267" s="3" t="n">
-        <v>46157.76041666666</v>
+        <v>46158.76041666666</v>
       </c>
       <c r="B267" s="4" t="n">
         <v>608</v>
@@ -13727,7 +13727,7 @@
     </row>
     <row r="268" ht="16" customHeight="1" s="5">
       <c r="A268" s="3" t="n">
-        <v>46157.77083333334</v>
+        <v>46158.77083333334</v>
       </c>
       <c r="B268" s="4" t="n">
         <v>656</v>
@@ -13774,7 +13774,7 @@
     </row>
     <row r="269" ht="16" customHeight="1" s="5">
       <c r="A269" s="3" t="n">
-        <v>46157.78125</v>
+        <v>46158.78125</v>
       </c>
       <c r="B269" s="4" t="n">
         <v>512</v>
@@ -13821,7 +13821,7 @@
     </row>
     <row r="270" ht="16" customHeight="1" s="5">
       <c r="A270" s="3" t="n">
-        <v>46157.79166666666</v>
+        <v>46158.79166666666</v>
       </c>
       <c r="B270" s="4" t="n">
         <v>323</v>
@@ -13868,7 +13868,7 @@
     </row>
     <row r="271" ht="16" customHeight="1" s="5">
       <c r="A271" s="3" t="n">
-        <v>46157.80208333334</v>
+        <v>46158.80208333334</v>
       </c>
       <c r="B271" s="4" t="n">
         <v>438</v>
@@ -13915,7 +13915,7 @@
     </row>
     <row r="272" ht="16" customHeight="1" s="5">
       <c r="A272" s="3" t="n">
-        <v>46157.8125</v>
+        <v>46158.8125</v>
       </c>
       <c r="B272" s="4" t="n">
         <v>613</v>
@@ -13962,7 +13962,7 @@
     </row>
     <row r="273" ht="16" customHeight="1" s="5">
       <c r="A273" s="3" t="n">
-        <v>46157.82291666666</v>
+        <v>46158.82291666666</v>
       </c>
       <c r="B273" s="4" t="n">
         <v>547</v>
@@ -14009,7 +14009,7 @@
     </row>
     <row r="274" ht="16" customHeight="1" s="5">
       <c r="A274" s="3" t="n">
-        <v>46157.83333333334</v>
+        <v>46158.83333333334</v>
       </c>
       <c r="B274" s="4" t="n">
         <v>402</v>
@@ -14056,7 +14056,7 @@
     </row>
     <row r="275" ht="16" customHeight="1" s="5">
       <c r="A275" s="3" t="n">
-        <v>46157.84375</v>
+        <v>46158.84375</v>
       </c>
       <c r="B275" s="4" t="n">
         <v>341</v>
@@ -14103,7 +14103,7 @@
     </row>
     <row r="276" ht="16" customHeight="1" s="5">
       <c r="A276" s="3" t="n">
-        <v>46157.85416666666</v>
+        <v>46158.85416666666</v>
       </c>
       <c r="B276" s="4" t="n">
         <v>264</v>
@@ -14150,7 +14150,7 @@
     </row>
     <row r="277" ht="16" customHeight="1" s="5">
       <c r="A277" s="3" t="n">
-        <v>46157.86458333334</v>
+        <v>46158.86458333334</v>
       </c>
       <c r="B277" s="4" t="n">
         <v>116</v>
@@ -14197,7 +14197,7 @@
     </row>
     <row r="278" ht="16" customHeight="1" s="5">
       <c r="A278" s="3" t="n">
-        <v>46157.875</v>
+        <v>46158.875</v>
       </c>
       <c r="B278" s="4" t="n">
         <v>0</v>
@@ -14244,7 +14244,7 @@
     </row>
     <row r="279" ht="16" customHeight="1" s="5">
       <c r="A279" s="3" t="n">
-        <v>46157.88541666666</v>
+        <v>46158.88541666666</v>
       </c>
       <c r="B279" s="4" t="n">
         <v>10</v>
@@ -14291,7 +14291,7 @@
     </row>
     <row r="280" ht="16" customHeight="1" s="5">
       <c r="A280" s="3" t="n">
-        <v>46157.89583333334</v>
+        <v>46158.89583333334</v>
       </c>
       <c r="B280" s="4" t="n">
         <v>39</v>
@@ -14338,7 +14338,7 @@
     </row>
     <row r="281" ht="16" customHeight="1" s="5">
       <c r="A281" s="3" t="n">
-        <v>46157.90625</v>
+        <v>46158.90625</v>
       </c>
       <c r="B281" s="4" t="n">
         <v>109</v>
@@ -14385,7 +14385,7 @@
     </row>
     <row r="282" ht="16" customHeight="1" s="5">
       <c r="A282" s="3" t="n">
-        <v>46157.91666666666</v>
+        <v>46158.91666666666</v>
       </c>
       <c r="B282" s="4" t="n">
         <v>193</v>
@@ -14432,7 +14432,7 @@
     </row>
     <row r="283" ht="16" customHeight="1" s="5">
       <c r="A283" s="3" t="n">
-        <v>46157.92708333334</v>
+        <v>46158.92708333334</v>
       </c>
       <c r="B283" s="4" t="n">
         <v>217</v>
@@ -14479,7 +14479,7 @@
     </row>
     <row r="284" ht="16" customHeight="1" s="5">
       <c r="A284" s="3" t="n">
-        <v>46157.9375</v>
+        <v>46158.9375</v>
       </c>
       <c r="B284" s="4" t="n">
         <v>185</v>
@@ -14526,7 +14526,7 @@
     </row>
     <row r="285" ht="16" customHeight="1" s="5">
       <c r="A285" s="3" t="n">
-        <v>46157.94791666666</v>
+        <v>46158.94791666666</v>
       </c>
       <c r="B285" s="4" t="n">
         <v>27</v>
@@ -14573,7 +14573,7 @@
     </row>
     <row r="286" ht="16" customHeight="1" s="5">
       <c r="A286" s="3" t="n">
-        <v>46157.95833333334</v>
+        <v>46158.95833333334</v>
       </c>
       <c r="B286" s="4" t="n">
         <v>0</v>
@@ -14620,7 +14620,7 @@
     </row>
     <row r="287" ht="16" customHeight="1" s="5">
       <c r="A287" s="3" t="n">
-        <v>46157.96875</v>
+        <v>46158.96875</v>
       </c>
       <c r="B287" s="4" t="n">
         <v>0</v>
@@ -14667,7 +14667,7 @@
     </row>
     <row r="288" ht="16" customHeight="1" s="5">
       <c r="A288" s="3" t="n">
-        <v>46157.97916666666</v>
+        <v>46158.97916666666</v>
       </c>
       <c r="B288" s="4" t="n">
         <v>0</v>
@@ -14714,7 +14714,7 @@
     </row>
     <row r="289" ht="16" customHeight="1" s="5">
       <c r="A289" s="3" t="n">
-        <v>46157.98958333334</v>
+        <v>46158.98958333334</v>
       </c>
       <c r="B289" s="4" t="n">
         <v>0</v>
@@ -14761,7 +14761,7 @@
     </row>
     <row r="290" ht="16" customHeight="1" s="5">
       <c r="A290" s="3" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
       <c r="B290" s="4" t="n">
         <v>0</v>
@@ -14808,7 +14808,7 @@
     </row>
     <row r="291" ht="16" customHeight="1" s="5">
       <c r="A291" s="3" t="n">
-        <v>46158.01041666666</v>
+        <v>46159.01041666666</v>
       </c>
       <c r="B291" s="4" t="n">
         <v>10</v>
@@ -14855,7 +14855,7 @@
     </row>
     <row r="292" ht="16" customHeight="1" s="5">
       <c r="A292" s="3" t="n">
-        <v>46158.02083333334</v>
+        <v>46159.02083333334</v>
       </c>
       <c r="B292" s="4" t="n">
         <v>35</v>
@@ -14902,7 +14902,7 @@
     </row>
     <row r="293" ht="16" customHeight="1" s="5">
       <c r="A293" s="3" t="n">
-        <v>46158.03125</v>
+        <v>46159.03125</v>
       </c>
       <c r="B293" s="4" t="n">
         <v>62</v>
@@ -14949,7 +14949,7 @@
     </row>
     <row r="294" ht="16" customHeight="1" s="5">
       <c r="A294" s="3" t="n">
-        <v>46158.04166666666</v>
+        <v>46159.04166666666</v>
       </c>
       <c r="B294" s="4" t="n">
         <v>80</v>
@@ -14996,7 +14996,7 @@
     </row>
     <row r="295" ht="16" customHeight="1" s="5">
       <c r="A295" s="3" t="n">
-        <v>46158.05208333334</v>
+        <v>46159.05208333334</v>
       </c>
       <c r="B295" s="4" t="n">
         <v>27</v>
@@ -15043,7 +15043,7 @@
     </row>
     <row r="296" ht="16" customHeight="1" s="5">
       <c r="A296" s="3" t="n">
-        <v>46158.0625</v>
+        <v>46159.0625</v>
       </c>
       <c r="B296" s="4" t="n">
         <v>0</v>
@@ -15090,7 +15090,7 @@
     </row>
     <row r="297" ht="16" customHeight="1" s="5">
       <c r="A297" s="3" t="n">
-        <v>46158.07291666666</v>
+        <v>46159.07291666666</v>
       </c>
       <c r="B297" s="4" t="n">
         <v>4</v>
@@ -15137,7 +15137,7 @@
     </row>
     <row r="298" ht="16" customHeight="1" s="5">
       <c r="A298" s="3" t="n">
-        <v>46158.08333333334</v>
+        <v>46159.08333333334</v>
       </c>
       <c r="B298" s="4" t="n">
         <v>11</v>
@@ -15184,7 +15184,7 @@
     </row>
     <row r="299" ht="16" customHeight="1" s="5">
       <c r="A299" s="3" t="n">
-        <v>46158.09375</v>
+        <v>46159.09375</v>
       </c>
       <c r="B299" s="4" t="n">
         <v>20</v>
@@ -15231,7 +15231,7 @@
     </row>
     <row r="300" ht="16" customHeight="1" s="5">
       <c r="A300" s="3" t="n">
-        <v>46158.10416666666</v>
+        <v>46159.10416666666</v>
       </c>
       <c r="B300" s="4" t="n">
         <v>33</v>
@@ -15278,7 +15278,7 @@
     </row>
     <row r="301" ht="16" customHeight="1" s="5">
       <c r="A301" s="3" t="n">
-        <v>46158.11458333334</v>
+        <v>46159.11458333334</v>
       </c>
       <c r="B301" s="4" t="n">
         <v>17</v>
@@ -15325,7 +15325,7 @@
     </row>
     <row r="302" ht="16" customHeight="1" s="5">
       <c r="A302" s="3" t="n">
-        <v>46158.125</v>
+        <v>46159.125</v>
       </c>
       <c r="B302" s="4" t="n">
         <v>19</v>
@@ -15372,7 +15372,7 @@
     </row>
     <row r="303" ht="16" customHeight="1" s="5">
       <c r="A303" s="3" t="n">
-        <v>46158.13541666666</v>
+        <v>46159.13541666666</v>
       </c>
       <c r="B303" s="4" t="n">
         <v>26</v>
@@ -15419,7 +15419,7 @@
     </row>
     <row r="304" ht="16" customHeight="1" s="5">
       <c r="A304" s="3" t="n">
-        <v>46158.14583333334</v>
+        <v>46159.14583333334</v>
       </c>
       <c r="B304" s="4" t="n">
         <v>65</v>
@@ -15466,7 +15466,7 @@
     </row>
     <row r="305" ht="16" customHeight="1" s="5">
       <c r="A305" s="3" t="n">
-        <v>46158.15625</v>
+        <v>46159.15625</v>
       </c>
       <c r="B305" s="4" t="n">
         <v>256</v>
@@ -15513,7 +15513,7 @@
     </row>
     <row r="306" ht="16" customHeight="1" s="5">
       <c r="A306" s="3" t="n">
-        <v>46158.16666666666</v>
+        <v>46159.16666666666</v>
       </c>
       <c r="B306" s="4" t="n">
         <v>528</v>
@@ -15560,7 +15560,7 @@
     </row>
     <row r="307" ht="16" customHeight="1" s="5">
       <c r="A307" s="3" t="n">
-        <v>46158.17708333334</v>
+        <v>46159.17708333334</v>
       </c>
       <c r="B307" s="4" t="n">
         <v>850</v>
@@ -15607,7 +15607,7 @@
     </row>
     <row r="308" ht="16" customHeight="1" s="5">
       <c r="A308" s="3" t="n">
-        <v>46158.1875</v>
+        <v>46159.1875</v>
       </c>
       <c r="B308" s="4" t="n">
         <v>967</v>
@@ -15654,7 +15654,7 @@
     </row>
     <row r="309" ht="16" customHeight="1" s="5">
       <c r="A309" s="3" t="n">
-        <v>46158.19791666666</v>
+        <v>46159.19791666666</v>
       </c>
       <c r="B309" s="4" t="n">
         <v>755</v>
@@ -15701,7 +15701,7 @@
     </row>
     <row r="310" ht="16" customHeight="1" s="5">
       <c r="A310" s="3" t="n">
-        <v>46158.20833333334</v>
+        <v>46159.20833333334</v>
       </c>
       <c r="B310" s="4" t="n">
         <v>800</v>
@@ -15748,7 +15748,7 @@
     </row>
     <row r="311" ht="16" customHeight="1" s="5">
       <c r="A311" s="3" t="n">
-        <v>46158.21875</v>
+        <v>46159.21875</v>
       </c>
       <c r="B311" s="4" t="n">
         <v>656</v>
@@ -15795,7 +15795,7 @@
     </row>
     <row r="312" ht="16" customHeight="1" s="5">
       <c r="A312" s="3" t="n">
-        <v>46158.22916666666</v>
+        <v>46159.22916666666</v>
       </c>
       <c r="B312" s="4" t="n">
         <v>515</v>
@@ -15842,7 +15842,7 @@
     </row>
     <row r="313" ht="16" customHeight="1" s="5">
       <c r="A313" s="3" t="n">
-        <v>46158.23958333334</v>
+        <v>46159.23958333334</v>
       </c>
       <c r="B313" s="4" t="n">
         <v>474</v>
@@ -15889,7 +15889,7 @@
     </row>
     <row r="314" ht="16" customHeight="1" s="5">
       <c r="A314" s="3" t="n">
-        <v>46158.25</v>
+        <v>46159.25</v>
       </c>
       <c r="B314" s="4" t="n">
         <v>601</v>
@@ -15936,7 +15936,7 @@
     </row>
     <row r="315" ht="16" customHeight="1" s="5">
       <c r="A315" s="3" t="n">
-        <v>46158.26041666666</v>
+        <v>46159.26041666666</v>
       </c>
       <c r="B315" s="4" t="n">
         <v>632</v>
@@ -15983,7 +15983,7 @@
     </row>
     <row r="316" ht="16" customHeight="1" s="5">
       <c r="A316" s="3" t="n">
-        <v>46158.27083333334</v>
+        <v>46159.27083333334</v>
       </c>
       <c r="B316" s="4" t="n">
         <v>592</v>
@@ -16030,7 +16030,7 @@
     </row>
     <row r="317" ht="16" customHeight="1" s="5">
       <c r="A317" s="3" t="n">
-        <v>46158.28125</v>
+        <v>46159.28125</v>
       </c>
       <c r="B317" s="4" t="n">
         <v>493</v>
@@ -16077,7 +16077,7 @@
     </row>
     <row r="318" ht="16" customHeight="1" s="5">
       <c r="A318" s="3" t="n">
-        <v>46158.29166666666</v>
+        <v>46159.29166666666</v>
       </c>
       <c r="B318" s="4" t="n">
         <v>448</v>
@@ -16124,7 +16124,7 @@
     </row>
     <row r="319" ht="16" customHeight="1" s="5">
       <c r="A319" s="3" t="n">
-        <v>46158.30208333334</v>
+        <v>46159.30208333334</v>
       </c>
       <c r="B319" s="4" t="n">
         <v>459</v>
@@ -16171,7 +16171,7 @@
     </row>
     <row r="320" ht="16" customHeight="1" s="5">
       <c r="A320" s="3" t="n">
-        <v>46158.3125</v>
+        <v>46159.3125</v>
       </c>
       <c r="B320" s="4" t="n">
         <v>432</v>
@@ -16218,7 +16218,7 @@
     </row>
     <row r="321" ht="16" customHeight="1" s="5">
       <c r="A321" s="3" t="n">
-        <v>46158.32291666666</v>
+        <v>46159.32291666666</v>
       </c>
       <c r="B321" s="4" t="n">
         <v>368</v>
@@ -16265,7 +16265,7 @@
     </row>
     <row r="322" ht="16" customHeight="1" s="5">
       <c r="A322" s="3" t="n">
-        <v>46158.33333333334</v>
+        <v>46159.33333333334</v>
       </c>
       <c r="B322" s="4" t="n">
         <v>320</v>
@@ -16312,7 +16312,7 @@
     </row>
     <row r="323" ht="16" customHeight="1" s="5">
       <c r="A323" s="3" t="n">
-        <v>46158.34375</v>
+        <v>46159.34375</v>
       </c>
       <c r="B323" s="4" t="n">
         <v>237</v>
@@ -16359,7 +16359,7 @@
     </row>
     <row r="324" ht="16" customHeight="1" s="5">
       <c r="A324" s="3" t="n">
-        <v>46158.35416666666</v>
+        <v>46159.35416666666</v>
       </c>
       <c r="B324" s="4" t="n">
         <v>262</v>
@@ -16406,7 +16406,7 @@
     </row>
     <row r="325" ht="16" customHeight="1" s="5">
       <c r="A325" s="3" t="n">
-        <v>46158.36458333334</v>
+        <v>46159.36458333334</v>
       </c>
       <c r="B325" s="4" t="n">
         <v>445</v>
@@ -16453,7 +16453,7 @@
     </row>
     <row r="326" ht="16" customHeight="1" s="5">
       <c r="A326" s="3" t="n">
-        <v>46158.375</v>
+        <v>46159.375</v>
       </c>
       <c r="B326" s="4" t="n">
         <v>627</v>
@@ -16500,7 +16500,7 @@
     </row>
     <row r="327" ht="16" customHeight="1" s="5">
       <c r="A327" s="3" t="n">
-        <v>46158.38541666666</v>
+        <v>46159.38541666666</v>
       </c>
       <c r="B327" s="4" t="n">
         <v>623</v>
@@ -16547,7 +16547,7 @@
     </row>
     <row r="328" ht="16" customHeight="1" s="5">
       <c r="A328" s="3" t="n">
-        <v>46158.39583333334</v>
+        <v>46159.39583333334</v>
       </c>
       <c r="B328" s="4" t="n">
         <v>576</v>
@@ -16594,7 +16594,7 @@
     </row>
     <row r="329" ht="16" customHeight="1" s="5">
       <c r="A329" s="3" t="n">
-        <v>46158.40625</v>
+        <v>46159.40625</v>
       </c>
       <c r="B329" s="4" t="n">
         <v>542</v>
@@ -16641,7 +16641,7 @@
     </row>
     <row r="330" ht="16" customHeight="1" s="5">
       <c r="A330" s="3" t="n">
-        <v>46158.41666666666</v>
+        <v>46159.41666666666</v>
       </c>
       <c r="B330" s="4" t="n">
         <v>484</v>
@@ -16688,7 +16688,7 @@
     </row>
     <row r="331" ht="16" customHeight="1" s="5">
       <c r="A331" s="3" t="n">
-        <v>46158.42708333334</v>
+        <v>46159.42708333334</v>
       </c>
       <c r="B331" s="4" t="n">
         <v>377</v>
@@ -16735,7 +16735,7 @@
     </row>
     <row r="332" ht="16" customHeight="1" s="5">
       <c r="A332" s="3" t="n">
-        <v>46158.4375</v>
+        <v>46159.4375</v>
       </c>
       <c r="B332" s="4" t="n">
         <v>281</v>
@@ -16782,7 +16782,7 @@
     </row>
     <row r="333" ht="16" customHeight="1" s="5">
       <c r="A333" s="3" t="n">
-        <v>46158.44791666666</v>
+        <v>46159.44791666666</v>
       </c>
       <c r="B333" s="4" t="n">
         <v>386</v>
@@ -16829,7 +16829,7 @@
     </row>
     <row r="334" ht="16" customHeight="1" s="5">
       <c r="A334" s="3" t="n">
-        <v>46158.45833333334</v>
+        <v>46159.45833333334</v>
       </c>
       <c r="B334" s="4" t="n">
         <v>548</v>
@@ -16876,7 +16876,7 @@
     </row>
     <row r="335" ht="16" customHeight="1" s="5">
       <c r="A335" s="3" t="n">
-        <v>46158.46875</v>
+        <v>46159.46875</v>
       </c>
       <c r="B335" s="4" t="n">
         <v>620</v>
@@ -16923,7 +16923,7 @@
     </row>
     <row r="336" ht="16" customHeight="1" s="5">
       <c r="A336" s="3" t="n">
-        <v>46158.47916666666</v>
+        <v>46159.47916666666</v>
       </c>
       <c r="B336" s="4" t="n">
         <v>531</v>
@@ -16970,7 +16970,7 @@
     </row>
     <row r="337" ht="16" customHeight="1" s="5">
       <c r="A337" s="3" t="n">
-        <v>46158.48958333334</v>
+        <v>46159.48958333334</v>
       </c>
       <c r="B337" s="4" t="n">
         <v>491</v>
@@ -17017,7 +17017,7 @@
     </row>
     <row r="338" ht="16" customHeight="1" s="5">
       <c r="A338" s="3" t="n">
-        <v>46158.5</v>
+        <v>46159.5</v>
       </c>
       <c r="B338" s="4" t="n">
         <v>385</v>
@@ -17064,7 +17064,7 @@
     </row>
     <row r="339" ht="16" customHeight="1" s="5">
       <c r="A339" s="3" t="n">
-        <v>46158.51041666666</v>
+        <v>46159.51041666666</v>
       </c>
       <c r="B339" s="4" t="n">
         <v>397</v>
@@ -17111,7 +17111,7 @@
     </row>
     <row r="340" ht="16" customHeight="1" s="5">
       <c r="A340" s="3" t="n">
-        <v>46158.52083333334</v>
+        <v>46159.52083333334</v>
       </c>
       <c r="B340" s="4" t="n">
         <v>490</v>
@@ -17158,7 +17158,7 @@
     </row>
     <row r="341" ht="16" customHeight="1" s="5">
       <c r="A341" s="3" t="n">
-        <v>46158.53125</v>
+        <v>46159.53125</v>
       </c>
       <c r="B341" s="4" t="n">
         <v>547</v>
@@ -17205,7 +17205,7 @@
     </row>
     <row r="342" ht="16" customHeight="1" s="5">
       <c r="A342" s="3" t="n">
-        <v>46158.54166666666</v>
+        <v>46159.54166666666</v>
       </c>
       <c r="B342" s="4" t="n">
         <v>415</v>
@@ -17252,7 +17252,7 @@
     </row>
     <row r="343" ht="16" customHeight="1" s="5">
       <c r="A343" s="3" t="n">
-        <v>46158.55208333334</v>
+        <v>46159.55208333334</v>
       </c>
       <c r="B343" s="4" t="n">
         <v>228</v>
@@ -17299,7 +17299,7 @@
     </row>
     <row r="344" ht="16" customHeight="1" s="5">
       <c r="A344" s="3" t="n">
-        <v>46158.5625</v>
+        <v>46159.5625</v>
       </c>
       <c r="B344" s="4" t="n">
         <v>309</v>
@@ -17346,7 +17346,7 @@
     </row>
     <row r="345" ht="16" customHeight="1" s="5">
       <c r="A345" s="3" t="n">
-        <v>46158.57291666666</v>
+        <v>46159.57291666666</v>
       </c>
       <c r="B345" s="4" t="n">
         <v>411</v>
@@ -17393,7 +17393,7 @@
     </row>
     <row r="346" ht="16" customHeight="1" s="5">
       <c r="A346" s="3" t="n">
-        <v>46158.58333333334</v>
+        <v>46159.58333333334</v>
       </c>
       <c r="B346" s="4" t="n">
         <v>385</v>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="347" ht="16" customHeight="1" s="5">
       <c r="A347" s="3" t="n">
-        <v>46158.59375</v>
+        <v>46159.59375</v>
       </c>
       <c r="B347" s="4" t="n">
         <v>436</v>
@@ -17487,7 +17487,7 @@
     </row>
     <row r="348" ht="16" customHeight="1" s="5">
       <c r="A348" s="3" t="n">
-        <v>46158.60416666666</v>
+        <v>46159.60416666666</v>
       </c>
       <c r="B348" s="4" t="n">
         <v>446</v>
@@ -17534,7 +17534,7 @@
     </row>
     <row r="349" ht="16" customHeight="1" s="5">
       <c r="A349" s="3" t="n">
-        <v>46158.61458333334</v>
+        <v>46159.61458333334</v>
       </c>
       <c r="B349" s="4" t="n">
         <v>426</v>
@@ -17581,7 +17581,7 @@
     </row>
     <row r="350" ht="16" customHeight="1" s="5">
       <c r="A350" s="3" t="n">
-        <v>46158.625</v>
+        <v>46159.625</v>
       </c>
       <c r="B350" s="4" t="n">
         <v>450</v>
@@ -17628,7 +17628,7 @@
     </row>
     <row r="351" ht="16" customHeight="1" s="5">
       <c r="A351" s="3" t="n">
-        <v>46158.63541666666</v>
+        <v>46159.63541666666</v>
       </c>
       <c r="B351" s="4" t="n">
         <v>322</v>
@@ -17675,7 +17675,7 @@
     </row>
     <row r="352" ht="16" customHeight="1" s="5">
       <c r="A352" s="3" t="n">
-        <v>46158.64583333334</v>
+        <v>46159.64583333334</v>
       </c>
       <c r="B352" s="4" t="n">
         <v>303</v>
@@ -17722,7 +17722,7 @@
     </row>
     <row r="353" ht="16" customHeight="1" s="5">
       <c r="A353" s="3" t="n">
-        <v>46158.65625</v>
+        <v>46159.65625</v>
       </c>
       <c r="B353" s="4" t="n">
         <v>496</v>
@@ -17769,7 +17769,7 @@
     </row>
     <row r="354" ht="16" customHeight="1" s="5">
       <c r="A354" s="3" t="n">
-        <v>46158.66666666666</v>
+        <v>46159.66666666666</v>
       </c>
       <c r="B354" s="4" t="n">
         <v>654</v>
@@ -17816,7 +17816,7 @@
     </row>
     <row r="355" ht="16" customHeight="1" s="5">
       <c r="A355" s="3" t="n">
-        <v>46158.67708333334</v>
+        <v>46159.67708333334</v>
       </c>
       <c r="B355" s="4" t="n">
         <v>781</v>
@@ -17863,7 +17863,7 @@
     </row>
     <row r="356" ht="16" customHeight="1" s="5">
       <c r="A356" s="3" t="n">
-        <v>46158.6875</v>
+        <v>46159.6875</v>
       </c>
       <c r="B356" s="4" t="n">
         <v>795</v>
@@ -17910,7 +17910,7 @@
     </row>
     <row r="357" ht="16" customHeight="1" s="5">
       <c r="A357" s="3" t="n">
-        <v>46158.69791666666</v>
+        <v>46159.69791666666</v>
       </c>
       <c r="B357" s="4" t="n">
         <v>569</v>
@@ -17957,7 +17957,7 @@
     </row>
     <row r="358" ht="16" customHeight="1" s="5">
       <c r="A358" s="3" t="n">
-        <v>46158.70833333334</v>
+        <v>46159.70833333334</v>
       </c>
       <c r="B358" s="4" t="n">
         <v>611</v>
@@ -18004,7 +18004,7 @@
     </row>
     <row r="359" ht="16" customHeight="1" s="5">
       <c r="A359" s="3" t="n">
-        <v>46158.71875</v>
+        <v>46159.71875</v>
       </c>
       <c r="B359" s="4" t="n">
         <v>794</v>
@@ -18051,7 +18051,7 @@
     </row>
     <row r="360" ht="16" customHeight="1" s="5">
       <c r="A360" s="3" t="n">
-        <v>46158.72916666666</v>
+        <v>46159.72916666666</v>
       </c>
       <c r="B360" s="4" t="n">
         <v>635</v>
@@ -18098,7 +18098,7 @@
     </row>
     <row r="361" ht="16" customHeight="1" s="5">
       <c r="A361" s="3" t="n">
-        <v>46158.73958333334</v>
+        <v>46159.73958333334</v>
       </c>
       <c r="B361" s="4" t="n">
         <v>642</v>
@@ -18145,7 +18145,7 @@
     </row>
     <row r="362" ht="16" customHeight="1" s="5">
       <c r="A362" s="3" t="n">
-        <v>46158.75</v>
+        <v>46159.75</v>
       </c>
       <c r="B362" s="4" t="n">
         <v>624</v>
@@ -18192,7 +18192,7 @@
     </row>
     <row r="363" ht="16" customHeight="1" s="5">
       <c r="A363" s="3" t="n">
-        <v>46158.76041666666</v>
+        <v>46159.76041666666</v>
       </c>
       <c r="B363" s="4" t="n">
         <v>608</v>
@@ -18239,7 +18239,7 @@
     </row>
     <row r="364" ht="16" customHeight="1" s="5">
       <c r="A364" s="3" t="n">
-        <v>46158.77083333334</v>
+        <v>46159.77083333334</v>
       </c>
       <c r="B364" s="4" t="n">
         <v>656</v>
@@ -18286,7 +18286,7 @@
     </row>
     <row r="365" ht="16" customHeight="1" s="5">
       <c r="A365" s="3" t="n">
-        <v>46158.78125</v>
+        <v>46159.78125</v>
       </c>
       <c r="B365" s="4" t="n">
         <v>512</v>
@@ -18333,7 +18333,7 @@
     </row>
     <row r="366" ht="16" customHeight="1" s="5">
       <c r="A366" s="3" t="n">
-        <v>46158.79166666666</v>
+        <v>46159.79166666666</v>
       </c>
       <c r="B366" s="4" t="n">
         <v>323</v>
@@ -18380,7 +18380,7 @@
     </row>
     <row r="367" ht="16" customHeight="1" s="5">
       <c r="A367" s="3" t="n">
-        <v>46158.80208333334</v>
+        <v>46159.80208333334</v>
       </c>
       <c r="B367" s="4" t="n">
         <v>438</v>
@@ -18427,7 +18427,7 @@
     </row>
     <row r="368" ht="16" customHeight="1" s="5">
       <c r="A368" s="3" t="n">
-        <v>46158.8125</v>
+        <v>46159.8125</v>
       </c>
       <c r="B368" s="4" t="n">
         <v>613</v>
@@ -18474,7 +18474,7 @@
     </row>
     <row r="369" ht="16" customHeight="1" s="5">
       <c r="A369" s="3" t="n">
-        <v>46158.82291666666</v>
+        <v>46159.82291666666</v>
       </c>
       <c r="B369" s="4" t="n">
         <v>547</v>
@@ -18521,7 +18521,7 @@
     </row>
     <row r="370" ht="16" customHeight="1" s="5">
       <c r="A370" s="3" t="n">
-        <v>46158.83333333334</v>
+        <v>46159.83333333334</v>
       </c>
       <c r="B370" s="4" t="n">
         <v>402</v>
@@ -18568,7 +18568,7 @@
     </row>
     <row r="371" ht="16" customHeight="1" s="5">
       <c r="A371" s="3" t="n">
-        <v>46158.84375</v>
+        <v>46159.84375</v>
       </c>
       <c r="B371" s="4" t="n">
         <v>341</v>
@@ -18615,7 +18615,7 @@
     </row>
     <row r="372" ht="16" customHeight="1" s="5">
       <c r="A372" s="3" t="n">
-        <v>46158.85416666666</v>
+        <v>46159.85416666666</v>
       </c>
       <c r="B372" s="4" t="n">
         <v>264</v>
@@ -18662,7 +18662,7 @@
     </row>
     <row r="373" ht="16" customHeight="1" s="5">
       <c r="A373" s="3" t="n">
-        <v>46158.86458333334</v>
+        <v>46159.86458333334</v>
       </c>
       <c r="B373" s="4" t="n">
         <v>116</v>
@@ -18709,7 +18709,7 @@
     </row>
     <row r="374" ht="16" customHeight="1" s="5">
       <c r="A374" s="3" t="n">
-        <v>46158.875</v>
+        <v>46159.875</v>
       </c>
       <c r="B374" s="4" t="n">
         <v>0</v>
@@ -18756,7 +18756,7 @@
     </row>
     <row r="375" ht="16" customHeight="1" s="5">
       <c r="A375" s="3" t="n">
-        <v>46158.88541666666</v>
+        <v>46159.88541666666</v>
       </c>
       <c r="B375" s="4" t="n">
         <v>10</v>
@@ -18803,7 +18803,7 @@
     </row>
     <row r="376" ht="16" customHeight="1" s="5">
       <c r="A376" s="3" t="n">
-        <v>46158.89583333334</v>
+        <v>46159.89583333334</v>
       </c>
       <c r="B376" s="4" t="n">
         <v>39</v>
@@ -18850,7 +18850,7 @@
     </row>
     <row r="377" ht="16" customHeight="1" s="5">
       <c r="A377" s="3" t="n">
-        <v>46158.90625</v>
+        <v>46159.90625</v>
       </c>
       <c r="B377" s="4" t="n">
         <v>109</v>
@@ -18897,7 +18897,7 @@
     </row>
     <row r="378" ht="16" customHeight="1" s="5">
       <c r="A378" s="3" t="n">
-        <v>46158.91666666666</v>
+        <v>46159.91666666666</v>
       </c>
       <c r="B378" s="4" t="n">
         <v>193</v>
@@ -18944,7 +18944,7 @@
     </row>
     <row r="379" ht="16" customHeight="1" s="5">
       <c r="A379" s="3" t="n">
-        <v>46158.92708333334</v>
+        <v>46159.92708333334</v>
       </c>
       <c r="B379" s="4" t="n">
         <v>217</v>
@@ -18991,7 +18991,7 @@
     </row>
     <row r="380" ht="16" customHeight="1" s="5">
       <c r="A380" s="3" t="n">
-        <v>46158.9375</v>
+        <v>46159.9375</v>
       </c>
       <c r="B380" s="4" t="n">
         <v>185</v>
@@ -19038,7 +19038,7 @@
     </row>
     <row r="381" ht="16" customHeight="1" s="5">
       <c r="A381" s="3" t="n">
-        <v>46158.94791666666</v>
+        <v>46159.94791666666</v>
       </c>
       <c r="B381" s="4" t="n">
         <v>27</v>
@@ -19085,7 +19085,7 @@
     </row>
     <row r="382" ht="16" customHeight="1" s="5">
       <c r="A382" s="3" t="n">
-        <v>46158.95833333334</v>
+        <v>46159.95833333334</v>
       </c>
       <c r="B382" s="4" t="n">
         <v>0</v>
@@ -19132,7 +19132,7 @@
     </row>
     <row r="383" ht="16" customHeight="1" s="5">
       <c r="A383" s="3" t="n">
-        <v>46158.96875</v>
+        <v>46159.96875</v>
       </c>
       <c r="B383" s="4" t="n">
         <v>0</v>
@@ -19179,7 +19179,7 @@
     </row>
     <row r="384" ht="16" customHeight="1" s="5">
       <c r="A384" s="3" t="n">
-        <v>46158.97916666666</v>
+        <v>46159.97916666666</v>
       </c>
       <c r="B384" s="4" t="n">
         <v>0</v>
@@ -19226,7 +19226,7 @@
     </row>
     <row r="385" ht="16" customHeight="1" s="5">
       <c r="A385" s="3" t="n">
-        <v>46158.98958333334</v>
+        <v>46159.98958333334</v>
       </c>
       <c r="B385" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Long term UI changes done
</commit_message>
<xml_diff>
--- a/data/short term PAX.xlsx
+++ b/data/short term PAX.xlsx
@@ -1225,7 +1225,7 @@
     </row>
     <row r="2" ht="16" customHeight="1" s="5">
       <c r="A2" s="3" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>0</v>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="3" ht="16" customHeight="1" s="5">
       <c r="A3" s="3" t="n">
-        <v>46156.01041666666</v>
+        <v>46157.01041666666</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>10</v>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="4" ht="16" customHeight="1" s="5">
       <c r="A4" s="3" t="n">
-        <v>46156.02083333334</v>
+        <v>46157.02083333334</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>28</v>
@@ -1366,7 +1366,7 @@
     </row>
     <row r="5" ht="16" customHeight="1" s="5">
       <c r="A5" s="3" t="n">
-        <v>46156.03125</v>
+        <v>46157.03125</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>48</v>
@@ -1413,7 +1413,7 @@
     </row>
     <row r="6" ht="16" customHeight="1" s="5">
       <c r="A6" s="3" t="n">
-        <v>46156.04166666666</v>
+        <v>46157.04166666666</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>58</v>
@@ -1460,7 +1460,7 @@
     </row>
     <row r="7" ht="16" customHeight="1" s="5">
       <c r="A7" s="3" t="n">
-        <v>46156.05208333334</v>
+        <v>46157.05208333334</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>9</v>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="8" ht="16" customHeight="1" s="5">
       <c r="A8" s="3" t="n">
-        <v>46156.0625</v>
+        <v>46157.0625</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>0</v>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="9" ht="16" customHeight="1" s="5">
       <c r="A9" s="3" t="n">
-        <v>46156.07291666666</v>
+        <v>46157.07291666666</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>4</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="10" ht="16" customHeight="1" s="5">
       <c r="A10" s="3" t="n">
-        <v>46156.08333333334</v>
+        <v>46157.08333333334</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>11</v>
@@ -1648,7 +1648,7 @@
     </row>
     <row r="11" ht="16" customHeight="1" s="5">
       <c r="A11" s="3" t="n">
-        <v>46156.09375</v>
+        <v>46157.09375</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>20</v>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="12" ht="16" customHeight="1" s="5">
       <c r="A12" s="3" t="n">
-        <v>46156.10416666666</v>
+        <v>46157.10416666666</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>33</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="13" ht="16" customHeight="1" s="5">
       <c r="A13" s="3" t="n">
-        <v>46156.11458333334</v>
+        <v>46157.11458333334</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>17</v>
@@ -1789,7 +1789,7 @@
     </row>
     <row r="14" ht="16" customHeight="1" s="5">
       <c r="A14" s="3" t="n">
-        <v>46156.125</v>
+        <v>46157.125</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>27</v>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="15" ht="16" customHeight="1" s="5">
       <c r="A15" s="3" t="n">
-        <v>46156.13541666666</v>
+        <v>46157.13541666666</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>41</v>
@@ -1883,7 +1883,7 @@
     </row>
     <row r="16" ht="16" customHeight="1" s="5">
       <c r="A16" s="3" t="n">
-        <v>46156.14583333334</v>
+        <v>46157.14583333334</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>75</v>
@@ -1930,7 +1930,7 @@
     </row>
     <row r="17" ht="16" customHeight="1" s="5">
       <c r="A17" s="3" t="n">
-        <v>46156.15625</v>
+        <v>46157.15625</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>268</v>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="18" ht="16" customHeight="1" s="5">
       <c r="A18" s="3" t="n">
-        <v>46156.16666666666</v>
+        <v>46157.16666666666</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>527</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="19" ht="16" customHeight="1" s="5">
       <c r="A19" s="3" t="n">
-        <v>46156.17708333334</v>
+        <v>46157.17708333334</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>888</v>
@@ -2071,7 +2071,7 @@
     </row>
     <row r="20" ht="16" customHeight="1" s="5">
       <c r="A20" s="3" t="n">
-        <v>46156.1875</v>
+        <v>46157.1875</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>1032</v>
@@ -2118,7 +2118,7 @@
     </row>
     <row r="21" ht="16" customHeight="1" s="5">
       <c r="A21" s="3" t="n">
-        <v>46156.19791666666</v>
+        <v>46157.19791666666</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>780</v>
@@ -2165,7 +2165,7 @@
     </row>
     <row r="22" ht="16" customHeight="1" s="5">
       <c r="A22" s="3" t="n">
-        <v>46156.20833333334</v>
+        <v>46157.20833333334</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>0</v>
@@ -2212,7 +2212,7 @@
     </row>
     <row r="23" ht="16" customHeight="1" s="5">
       <c r="A23" s="3" t="n">
-        <v>46156.21875</v>
+        <v>46157.21875</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>0</v>
@@ -2259,7 +2259,7 @@
     </row>
     <row r="24" ht="16" customHeight="1" s="5">
       <c r="A24" s="3" t="n">
-        <v>46156.22916666666</v>
+        <v>46157.22916666666</v>
       </c>
       <c r="B24" s="4" t="n">
         <v>0</v>
@@ -2306,7 +2306,7 @@
     </row>
     <row r="25" ht="16" customHeight="1" s="5">
       <c r="A25" s="3" t="n">
-        <v>46156.23958333334</v>
+        <v>46157.23958333334</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>1</v>
@@ -2353,7 +2353,7 @@
     </row>
     <row r="26" ht="16" customHeight="1" s="5">
       <c r="A26" s="3" t="n">
-        <v>46156.25</v>
+        <v>46157.25</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>27</v>
@@ -2400,7 +2400,7 @@
     </row>
     <row r="27" ht="16" customHeight="1" s="5">
       <c r="A27" s="3" t="n">
-        <v>46156.26041666666</v>
+        <v>46157.26041666666</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>82</v>
@@ -2447,7 +2447,7 @@
     </row>
     <row r="28" ht="16" customHeight="1" s="5">
       <c r="A28" s="3" t="n">
-        <v>46156.27083333334</v>
+        <v>46157.27083333334</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>180</v>
@@ -2494,7 +2494,7 @@
     </row>
     <row r="29" ht="16" customHeight="1" s="5">
       <c r="A29" s="3" t="n">
-        <v>46156.28125</v>
+        <v>46157.28125</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>275</v>
@@ -2541,7 +2541,7 @@
     </row>
     <row r="30" ht="16" customHeight="1" s="5">
       <c r="A30" s="3" t="n">
-        <v>46156.29166666666</v>
+        <v>46157.29166666666</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>342</v>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="31" ht="16" customHeight="1" s="5">
       <c r="A31" s="3" t="n">
-        <v>46156.30208333334</v>
+        <v>46157.30208333334</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>327</v>
@@ -2635,7 +2635,7 @@
     </row>
     <row r="32" ht="16" customHeight="1" s="5">
       <c r="A32" s="3" t="n">
-        <v>46156.3125</v>
+        <v>46157.3125</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>386</v>
@@ -2682,7 +2682,7 @@
     </row>
     <row r="33" ht="16" customHeight="1" s="5">
       <c r="A33" s="3" t="n">
-        <v>46156.32291666666</v>
+        <v>46157.32291666666</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>401</v>
@@ -2729,7 +2729,7 @@
     </row>
     <row r="34" ht="16" customHeight="1" s="5">
       <c r="A34" s="3" t="n">
-        <v>46156.33333333334</v>
+        <v>46157.33333333334</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>399</v>
@@ -2776,7 +2776,7 @@
     </row>
     <row r="35" ht="16" customHeight="1" s="5">
       <c r="A35" s="3" t="n">
-        <v>46156.34375</v>
+        <v>46157.34375</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>384</v>
@@ -2823,7 +2823,7 @@
     </row>
     <row r="36" ht="16" customHeight="1" s="5">
       <c r="A36" s="3" t="n">
-        <v>46156.35416666666</v>
+        <v>46157.35416666666</v>
       </c>
       <c r="B36" s="4" t="n">
         <v>438</v>
@@ -2870,7 +2870,7 @@
     </row>
     <row r="37" ht="16" customHeight="1" s="5">
       <c r="A37" s="3" t="n">
-        <v>46156.36458333334</v>
+        <v>46157.36458333334</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>433</v>
@@ -2917,7 +2917,7 @@
     </row>
     <row r="38" ht="16" customHeight="1" s="5">
       <c r="A38" s="3" t="n">
-        <v>46156.375</v>
+        <v>46157.375</v>
       </c>
       <c r="B38" s="4" t="n">
         <v>398</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="39" ht="16" customHeight="1" s="5">
       <c r="A39" s="3" t="n">
-        <v>46156.38541666666</v>
+        <v>46157.38541666666</v>
       </c>
       <c r="B39" s="4" t="n">
         <v>463</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="40" ht="16" customHeight="1" s="5">
       <c r="A40" s="3" t="n">
-        <v>46156.39583333334</v>
+        <v>46157.39583333334</v>
       </c>
       <c r="B40" s="4" t="n">
         <v>422</v>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="41" ht="16" customHeight="1" s="5">
       <c r="A41" s="3" t="n">
-        <v>46156.40625</v>
+        <v>46157.40625</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>448</v>
@@ -3105,7 +3105,7 @@
     </row>
     <row r="42" ht="16" customHeight="1" s="5">
       <c r="A42" s="3" t="n">
-        <v>46156.41666666666</v>
+        <v>46157.41666666666</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>603</v>
@@ -3152,7 +3152,7 @@
     </row>
     <row r="43" ht="16" customHeight="1" s="5">
       <c r="A43" s="3" t="n">
-        <v>46156.42708333334</v>
+        <v>46157.42708333334</v>
       </c>
       <c r="B43" s="4" t="n">
         <v>621</v>
@@ -3199,7 +3199,7 @@
     </row>
     <row r="44" ht="16" customHeight="1" s="5">
       <c r="A44" s="3" t="n">
-        <v>46156.4375</v>
+        <v>46157.4375</v>
       </c>
       <c r="B44" s="4" t="n">
         <v>521</v>
@@ -3246,7 +3246,7 @@
     </row>
     <row r="45" ht="16" customHeight="1" s="5">
       <c r="A45" s="3" t="n">
-        <v>46156.44791666666</v>
+        <v>46157.44791666666</v>
       </c>
       <c r="B45" s="4" t="n">
         <v>392</v>
@@ -3293,7 +3293,7 @@
     </row>
     <row r="46" ht="16" customHeight="1" s="5">
       <c r="A46" s="3" t="n">
-        <v>46156.45833333334</v>
+        <v>46157.45833333334</v>
       </c>
       <c r="B46" s="4" t="n">
         <v>358</v>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="47" ht="16" customHeight="1" s="5">
       <c r="A47" s="3" t="n">
-        <v>46156.46875</v>
+        <v>46157.46875</v>
       </c>
       <c r="B47" s="4" t="n">
         <v>487</v>
@@ -3387,7 +3387,7 @@
     </row>
     <row r="48" ht="16" customHeight="1" s="5">
       <c r="A48" s="3" t="n">
-        <v>46156.47916666666</v>
+        <v>46157.47916666666</v>
       </c>
       <c r="B48" s="4" t="n">
         <v>557</v>
@@ -3434,7 +3434,7 @@
     </row>
     <row r="49" ht="16" customHeight="1" s="5">
       <c r="A49" s="3" t="n">
-        <v>46156.48958333334</v>
+        <v>46157.48958333334</v>
       </c>
       <c r="B49" s="4" t="n">
         <v>565</v>
@@ -3481,7 +3481,7 @@
     </row>
     <row r="50" ht="16" customHeight="1" s="5">
       <c r="A50" s="3" t="n">
-        <v>46156.5</v>
+        <v>46157.5</v>
       </c>
       <c r="B50" s="4" t="n">
         <v>387</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="51" ht="16" customHeight="1" s="5">
       <c r="A51" s="3" t="n">
-        <v>46156.51041666666</v>
+        <v>46157.51041666666</v>
       </c>
       <c r="B51" s="4" t="n">
         <v>227</v>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="52" ht="16" customHeight="1" s="5">
       <c r="A52" s="3" t="n">
-        <v>46156.52083333334</v>
+        <v>46157.52083333334</v>
       </c>
       <c r="B52" s="4" t="n">
         <v>382</v>
@@ -3622,7 +3622,7 @@
     </row>
     <row r="53" ht="16" customHeight="1" s="5">
       <c r="A53" s="3" t="n">
-        <v>46156.53125</v>
+        <v>46157.53125</v>
       </c>
       <c r="B53" s="4" t="n">
         <v>612</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="54" ht="16" customHeight="1" s="5">
       <c r="A54" s="3" t="n">
-        <v>46156.54166666666</v>
+        <v>46157.54166666666</v>
       </c>
       <c r="B54" s="4" t="n">
         <v>699</v>
@@ -3716,7 +3716,7 @@
     </row>
     <row r="55" ht="16" customHeight="1" s="5">
       <c r="A55" s="3" t="n">
-        <v>46156.55208333334</v>
+        <v>46157.55208333334</v>
       </c>
       <c r="B55" s="4" t="n">
         <v>627</v>
@@ -3763,7 +3763,7 @@
     </row>
     <row r="56" ht="16" customHeight="1" s="5">
       <c r="A56" s="3" t="n">
-        <v>46156.5625</v>
+        <v>46157.5625</v>
       </c>
       <c r="B56" s="4" t="n">
         <v>538</v>
@@ -3810,7 +3810,7 @@
     </row>
     <row r="57" ht="16" customHeight="1" s="5">
       <c r="A57" s="3" t="n">
-        <v>46156.57291666666</v>
+        <v>46157.57291666666</v>
       </c>
       <c r="B57" s="4" t="n">
         <v>464</v>
@@ -3857,7 +3857,7 @@
     </row>
     <row r="58" ht="16" customHeight="1" s="5">
       <c r="A58" s="3" t="n">
-        <v>46156.58333333334</v>
+        <v>46157.58333333334</v>
       </c>
       <c r="B58" s="4" t="n">
         <v>402</v>
@@ -3904,7 +3904,7 @@
     </row>
     <row r="59" ht="16" customHeight="1" s="5">
       <c r="A59" s="3" t="n">
-        <v>46156.59375</v>
+        <v>46157.59375</v>
       </c>
       <c r="B59" s="4" t="n">
         <v>262</v>
@@ -3951,7 +3951,7 @@
     </row>
     <row r="60" ht="16" customHeight="1" s="5">
       <c r="A60" s="3" t="n">
-        <v>46156.60416666666</v>
+        <v>46157.60416666666</v>
       </c>
       <c r="B60" s="4" t="n">
         <v>228</v>
@@ -3998,7 +3998,7 @@
     </row>
     <row r="61" ht="16" customHeight="1" s="5">
       <c r="A61" s="3" t="n">
-        <v>46156.61458333334</v>
+        <v>46157.61458333334</v>
       </c>
       <c r="B61" s="4" t="n">
         <v>350</v>
@@ -4045,7 +4045,7 @@
     </row>
     <row r="62" ht="16" customHeight="1" s="5">
       <c r="A62" s="3" t="n">
-        <v>46156.625</v>
+        <v>46157.625</v>
       </c>
       <c r="B62" s="4" t="n">
         <v>506</v>
@@ -4092,7 +4092,7 @@
     </row>
     <row r="63" ht="16" customHeight="1" s="5">
       <c r="A63" s="3" t="n">
-        <v>46156.63541666666</v>
+        <v>46157.63541666666</v>
       </c>
       <c r="B63" s="4" t="n">
         <v>530</v>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="64" ht="16" customHeight="1" s="5">
       <c r="A64" s="3" t="n">
-        <v>46156.64583333334</v>
+        <v>46157.64583333334</v>
       </c>
       <c r="B64" s="4" t="n">
         <v>459</v>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="65" ht="16" customHeight="1" s="5">
       <c r="A65" s="3" t="n">
-        <v>46156.65625</v>
+        <v>46157.65625</v>
       </c>
       <c r="B65" s="4" t="n">
         <v>398</v>
@@ -4233,7 +4233,7 @@
     </row>
     <row r="66" ht="16" customHeight="1" s="5">
       <c r="A66" s="3" t="n">
-        <v>46156.66666666666</v>
+        <v>46157.66666666666</v>
       </c>
       <c r="B66" s="4" t="n">
         <v>488</v>
@@ -4280,7 +4280,7 @@
     </row>
     <row r="67" ht="16" customHeight="1" s="5">
       <c r="A67" s="3" t="n">
-        <v>46156.67708333334</v>
+        <v>46157.67708333334</v>
       </c>
       <c r="B67" s="4" t="n">
         <v>532</v>
@@ -4327,7 +4327,7 @@
     </row>
     <row r="68" ht="16" customHeight="1" s="5">
       <c r="A68" s="3" t="n">
-        <v>46156.6875</v>
+        <v>46157.6875</v>
       </c>
       <c r="B68" s="4" t="n">
         <v>716</v>
@@ -4374,7 +4374,7 @@
     </row>
     <row r="69" ht="16" customHeight="1" s="5">
       <c r="A69" s="3" t="n">
-        <v>46156.69791666666</v>
+        <v>46157.69791666666</v>
       </c>
       <c r="B69" s="4" t="n">
         <v>673</v>
@@ -4421,7 +4421,7 @@
     </row>
     <row r="70" ht="16" customHeight="1" s="5">
       <c r="A70" s="3" t="n">
-        <v>46156.70833333334</v>
+        <v>46157.70833333334</v>
       </c>
       <c r="B70" s="4" t="n">
         <v>504</v>
@@ -4468,7 +4468,7 @@
     </row>
     <row r="71" ht="16" customHeight="1" s="5">
       <c r="A71" s="3" t="n">
-        <v>46156.71875</v>
+        <v>46157.71875</v>
       </c>
       <c r="B71" s="4" t="n">
         <v>616</v>
@@ -4515,7 +4515,7 @@
     </row>
     <row r="72" ht="16" customHeight="1" s="5">
       <c r="A72" s="3" t="n">
-        <v>46156.72916666666</v>
+        <v>46157.72916666666</v>
       </c>
       <c r="B72" s="4" t="n">
         <v>569</v>
@@ -4562,7 +4562,7 @@
     </row>
     <row r="73" ht="16" customHeight="1" s="5">
       <c r="A73" s="3" t="n">
-        <v>46156.73958333334</v>
+        <v>46157.73958333334</v>
       </c>
       <c r="B73" s="4" t="n">
         <v>619</v>
@@ -4609,7 +4609,7 @@
     </row>
     <row r="74" ht="16" customHeight="1" s="5">
       <c r="A74" s="3" t="n">
-        <v>46156.75</v>
+        <v>46157.75</v>
       </c>
       <c r="B74" s="4" t="n">
         <v>597</v>
@@ -4656,7 +4656,7 @@
     </row>
     <row r="75" ht="16" customHeight="1" s="5">
       <c r="A75" s="3" t="n">
-        <v>46156.76041666666</v>
+        <v>46157.76041666666</v>
       </c>
       <c r="B75" s="4" t="n">
         <v>373</v>
@@ -4703,7 +4703,7 @@
     </row>
     <row r="76" ht="16" customHeight="1" s="5">
       <c r="A76" s="3" t="n">
-        <v>46156.77083333334</v>
+        <v>46157.77083333334</v>
       </c>
       <c r="B76" s="4" t="n">
         <v>298</v>
@@ -4750,7 +4750,7 @@
     </row>
     <row r="77" ht="16" customHeight="1" s="5">
       <c r="A77" s="3" t="n">
-        <v>46156.78125</v>
+        <v>46157.78125</v>
       </c>
       <c r="B77" s="4" t="n">
         <v>325</v>
@@ -4797,7 +4797,7 @@
     </row>
     <row r="78" ht="16" customHeight="1" s="5">
       <c r="A78" s="3" t="n">
-        <v>46156.79166666666</v>
+        <v>46157.79166666666</v>
       </c>
       <c r="B78" s="4" t="n">
         <v>350</v>
@@ -4844,7 +4844,7 @@
     </row>
     <row r="79" ht="16" customHeight="1" s="5">
       <c r="A79" s="3" t="n">
-        <v>46156.80208333334</v>
+        <v>46157.80208333334</v>
       </c>
       <c r="B79" s="4" t="n">
         <v>373</v>
@@ -4891,7 +4891,7 @@
     </row>
     <row r="80" ht="16" customHeight="1" s="5">
       <c r="A80" s="3" t="n">
-        <v>46156.8125</v>
+        <v>46157.8125</v>
       </c>
       <c r="B80" s="4" t="n">
         <v>344</v>
@@ -4938,7 +4938,7 @@
     </row>
     <row r="81" ht="16" customHeight="1" s="5">
       <c r="A81" s="3" t="n">
-        <v>46156.82291666666</v>
+        <v>46157.82291666666</v>
       </c>
       <c r="B81" s="4" t="n">
         <v>385</v>
@@ -4985,7 +4985,7 @@
     </row>
     <row r="82" ht="16" customHeight="1" s="5">
       <c r="A82" s="3" t="n">
-        <v>46156.83333333334</v>
+        <v>46157.83333333334</v>
       </c>
       <c r="B82" s="4" t="n">
         <v>439</v>
@@ -5032,7 +5032,7 @@
     </row>
     <row r="83" ht="16" customHeight="1" s="5">
       <c r="A83" s="3" t="n">
-        <v>46156.84375</v>
+        <v>46157.84375</v>
       </c>
       <c r="B83" s="4" t="n">
         <v>408</v>
@@ -5079,7 +5079,7 @@
     </row>
     <row r="84" ht="16" customHeight="1" s="5">
       <c r="A84" s="3" t="n">
-        <v>46156.85416666666</v>
+        <v>46157.85416666666</v>
       </c>
       <c r="B84" s="4" t="n">
         <v>319</v>
@@ -5126,7 +5126,7 @@
     </row>
     <row r="85" ht="16" customHeight="1" s="5">
       <c r="A85" s="3" t="n">
-        <v>46156.86458333334</v>
+        <v>46157.86458333334</v>
       </c>
       <c r="B85" s="4" t="n">
         <v>166</v>
@@ -5173,7 +5173,7 @@
     </row>
     <row r="86" ht="16" customHeight="1" s="5">
       <c r="A86" s="3" t="n">
-        <v>46156.875</v>
+        <v>46157.875</v>
       </c>
       <c r="B86" s="4" t="n">
         <v>29</v>
@@ -5220,7 +5220,7 @@
     </row>
     <row r="87" ht="16" customHeight="1" s="5">
       <c r="A87" s="3" t="n">
-        <v>46156.88541666666</v>
+        <v>46157.88541666666</v>
       </c>
       <c r="B87" s="4" t="n">
         <v>61</v>
@@ -5267,7 +5267,7 @@
     </row>
     <row r="88" ht="16" customHeight="1" s="5">
       <c r="A88" s="3" t="n">
-        <v>46156.89583333334</v>
+        <v>46157.89583333334</v>
       </c>
       <c r="B88" s="4" t="n">
         <v>107</v>
@@ -5314,7 +5314,7 @@
     </row>
     <row r="89" ht="16" customHeight="1" s="5">
       <c r="A89" s="3" t="n">
-        <v>46156.90625</v>
+        <v>46157.90625</v>
       </c>
       <c r="B89" s="4" t="n">
         <v>93</v>
@@ -5361,7 +5361,7 @@
     </row>
     <row r="90" ht="16" customHeight="1" s="5">
       <c r="A90" s="3" t="n">
-        <v>46156.91666666666</v>
+        <v>46157.91666666666</v>
       </c>
       <c r="B90" s="4" t="n">
         <v>115</v>
@@ -5408,7 +5408,7 @@
     </row>
     <row r="91" ht="16" customHeight="1" s="5">
       <c r="A91" s="3" t="n">
-        <v>46156.92708333334</v>
+        <v>46157.92708333334</v>
       </c>
       <c r="B91" s="4" t="n">
         <v>58</v>
@@ -5455,7 +5455,7 @@
     </row>
     <row r="92" ht="16" customHeight="1" s="5">
       <c r="A92" s="3" t="n">
-        <v>46156.9375</v>
+        <v>46157.9375</v>
       </c>
       <c r="B92" s="4" t="n">
         <v>0</v>
@@ -5502,7 +5502,7 @@
     </row>
     <row r="93" ht="16" customHeight="1" s="5">
       <c r="A93" s="3" t="n">
-        <v>46156.94791666666</v>
+        <v>46157.94791666666</v>
       </c>
       <c r="B93" s="4" t="n">
         <v>0</v>
@@ -5549,7 +5549,7 @@
     </row>
     <row r="94" ht="16" customHeight="1" s="5">
       <c r="A94" s="3" t="n">
-        <v>46156.95833333334</v>
+        <v>46157.95833333334</v>
       </c>
       <c r="B94" s="4" t="n">
         <v>0</v>
@@ -5596,7 +5596,7 @@
     </row>
     <row r="95" ht="16" customHeight="1" s="5">
       <c r="A95" s="3" t="n">
-        <v>46156.96875</v>
+        <v>46157.96875</v>
       </c>
       <c r="B95" s="4" t="n">
         <v>0</v>
@@ -5643,7 +5643,7 @@
     </row>
     <row r="96" ht="16" customHeight="1" s="5">
       <c r="A96" s="3" t="n">
-        <v>46156.97916666666</v>
+        <v>46157.97916666666</v>
       </c>
       <c r="B96" s="4" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
     </row>
     <row r="97" ht="16" customHeight="1" s="5">
       <c r="A97" s="3" t="n">
-        <v>46156.98958333334</v>
+        <v>46157.98958333334</v>
       </c>
       <c r="B97" s="4" t="n">
         <v>0</v>
@@ -5737,7 +5737,7 @@
     </row>
     <row r="98" ht="16" customHeight="1" s="5">
       <c r="A98" s="3" t="n">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B98" s="4" t="n">
         <v>0</v>
@@ -5784,7 +5784,7 @@
     </row>
     <row r="99" ht="16" customHeight="1" s="5">
       <c r="A99" s="3" t="n">
-        <v>46157.01041666666</v>
+        <v>46158.01041666666</v>
       </c>
       <c r="B99" s="4" t="n">
         <v>10</v>
@@ -5831,7 +5831,7 @@
     </row>
     <row r="100" ht="16" customHeight="1" s="5">
       <c r="A100" s="3" t="n">
-        <v>46157.02083333334</v>
+        <v>46158.02083333334</v>
       </c>
       <c r="B100" s="4" t="n">
         <v>28</v>
@@ -5878,7 +5878,7 @@
     </row>
     <row r="101" ht="16" customHeight="1" s="5">
       <c r="A101" s="3" t="n">
-        <v>46157.03125</v>
+        <v>46158.03125</v>
       </c>
       <c r="B101" s="4" t="n">
         <v>48</v>
@@ -5925,7 +5925,7 @@
     </row>
     <row r="102" ht="16" customHeight="1" s="5">
       <c r="A102" s="3" t="n">
-        <v>46157.04166666666</v>
+        <v>46158.04166666666</v>
       </c>
       <c r="B102" s="4" t="n">
         <v>58</v>
@@ -5972,7 +5972,7 @@
     </row>
     <row r="103" ht="16" customHeight="1" s="5">
       <c r="A103" s="3" t="n">
-        <v>46157.05208333334</v>
+        <v>46158.05208333334</v>
       </c>
       <c r="B103" s="4" t="n">
         <v>9</v>
@@ -6019,7 +6019,7 @@
     </row>
     <row r="104" ht="16" customHeight="1" s="5">
       <c r="A104" s="3" t="n">
-        <v>46157.0625</v>
+        <v>46158.0625</v>
       </c>
       <c r="B104" s="4" t="n">
         <v>0</v>
@@ -6066,7 +6066,7 @@
     </row>
     <row r="105" ht="16" customHeight="1" s="5">
       <c r="A105" s="3" t="n">
-        <v>46157.07291666666</v>
+        <v>46158.07291666666</v>
       </c>
       <c r="B105" s="4" t="n">
         <v>4</v>
@@ -6113,7 +6113,7 @@
     </row>
     <row r="106" ht="16" customHeight="1" s="5">
       <c r="A106" s="3" t="n">
-        <v>46157.08333333334</v>
+        <v>46158.08333333334</v>
       </c>
       <c r="B106" s="4" t="n">
         <v>11</v>
@@ -6160,7 +6160,7 @@
     </row>
     <row r="107" ht="16" customHeight="1" s="5">
       <c r="A107" s="3" t="n">
-        <v>46157.09375</v>
+        <v>46158.09375</v>
       </c>
       <c r="B107" s="4" t="n">
         <v>20</v>
@@ -6207,7 +6207,7 @@
     </row>
     <row r="108" ht="16" customHeight="1" s="5">
       <c r="A108" s="3" t="n">
-        <v>46157.10416666666</v>
+        <v>46158.10416666666</v>
       </c>
       <c r="B108" s="4" t="n">
         <v>33</v>
@@ -6254,7 +6254,7 @@
     </row>
     <row r="109" ht="16" customHeight="1" s="5">
       <c r="A109" s="3" t="n">
-        <v>46157.11458333334</v>
+        <v>46158.11458333334</v>
       </c>
       <c r="B109" s="4" t="n">
         <v>17</v>
@@ -6301,7 +6301,7 @@
     </row>
     <row r="110" ht="16" customHeight="1" s="5">
       <c r="A110" s="3" t="n">
-        <v>46157.125</v>
+        <v>46158.125</v>
       </c>
       <c r="B110" s="4" t="n">
         <v>27</v>
@@ -6348,7 +6348,7 @@
     </row>
     <row r="111" ht="16" customHeight="1" s="5">
       <c r="A111" s="3" t="n">
-        <v>46157.13541666666</v>
+        <v>46158.13541666666</v>
       </c>
       <c r="B111" s="4" t="n">
         <v>41</v>
@@ -6395,7 +6395,7 @@
     </row>
     <row r="112" ht="16" customHeight="1" s="5">
       <c r="A112" s="3" t="n">
-        <v>46157.14583333334</v>
+        <v>46158.14583333334</v>
       </c>
       <c r="B112" s="4" t="n">
         <v>75</v>
@@ -6442,7 +6442,7 @@
     </row>
     <row r="113" ht="16" customHeight="1" s="5">
       <c r="A113" s="3" t="n">
-        <v>46157.15625</v>
+        <v>46158.15625</v>
       </c>
       <c r="B113" s="4" t="n">
         <v>268</v>
@@ -6489,7 +6489,7 @@
     </row>
     <row r="114" ht="16" customHeight="1" s="5">
       <c r="A114" s="3" t="n">
-        <v>46157.16666666666</v>
+        <v>46158.16666666666</v>
       </c>
       <c r="B114" s="4" t="n">
         <v>527</v>
@@ -6536,7 +6536,7 @@
     </row>
     <row r="115" ht="16" customHeight="1" s="5">
       <c r="A115" s="3" t="n">
-        <v>46157.17708333334</v>
+        <v>46158.17708333334</v>
       </c>
       <c r="B115" s="4" t="n">
         <v>888</v>
@@ -6583,7 +6583,7 @@
     </row>
     <row r="116" ht="16" customHeight="1" s="5">
       <c r="A116" s="3" t="n">
-        <v>46157.1875</v>
+        <v>46158.1875</v>
       </c>
       <c r="B116" s="4" t="n">
         <v>1032</v>
@@ -6630,7 +6630,7 @@
     </row>
     <row r="117" ht="16" customHeight="1" s="5">
       <c r="A117" s="3" t="n">
-        <v>46157.19791666666</v>
+        <v>46158.19791666666</v>
       </c>
       <c r="B117" s="4" t="n">
         <v>780</v>
@@ -6677,7 +6677,7 @@
     </row>
     <row r="118" ht="16" customHeight="1" s="5">
       <c r="A118" s="3" t="n">
-        <v>46157.20833333334</v>
+        <v>46158.20833333334</v>
       </c>
       <c r="B118" s="4" t="n">
         <v>847</v>
@@ -6724,7 +6724,7 @@
     </row>
     <row r="119" ht="16" customHeight="1" s="5">
       <c r="A119" s="3" t="n">
-        <v>46157.21875</v>
+        <v>46158.21875</v>
       </c>
       <c r="B119" s="4" t="n">
         <v>689</v>
@@ -6771,7 +6771,7 @@
     </row>
     <row r="120" ht="16" customHeight="1" s="5">
       <c r="A120" s="3" t="n">
-        <v>46157.22916666666</v>
+        <v>46158.22916666666</v>
       </c>
       <c r="B120" s="4" t="n">
         <v>660</v>
@@ -6818,7 +6818,7 @@
     </row>
     <row r="121" ht="16" customHeight="1" s="5">
       <c r="A121" s="3" t="n">
-        <v>46157.23958333334</v>
+        <v>46158.23958333334</v>
       </c>
       <c r="B121" s="4" t="n">
         <v>671</v>
@@ -6865,7 +6865,7 @@
     </row>
     <row r="122" ht="16" customHeight="1" s="5">
       <c r="A122" s="3" t="n">
-        <v>46157.25</v>
+        <v>46158.25</v>
       </c>
       <c r="B122" s="4" t="n">
         <v>627</v>
@@ -6912,7 +6912,7 @@
     </row>
     <row r="123" ht="16" customHeight="1" s="5">
       <c r="A123" s="3" t="n">
-        <v>46157.26041666666</v>
+        <v>46158.26041666666</v>
       </c>
       <c r="B123" s="4" t="n">
         <v>513</v>
@@ -6959,7 +6959,7 @@
     </row>
     <row r="124" ht="16" customHeight="1" s="5">
       <c r="A124" s="3" t="n">
-        <v>46157.27083333334</v>
+        <v>46158.27083333334</v>
       </c>
       <c r="B124" s="4" t="n">
         <v>544</v>
@@ -7006,7 +7006,7 @@
     </row>
     <row r="125" ht="16" customHeight="1" s="5">
       <c r="A125" s="3" t="n">
-        <v>46157.28125</v>
+        <v>46158.28125</v>
       </c>
       <c r="B125" s="4" t="n">
         <v>417</v>
@@ -7053,7 +7053,7 @@
     </row>
     <row r="126" ht="16" customHeight="1" s="5">
       <c r="A126" s="3" t="n">
-        <v>46157.29166666666</v>
+        <v>46158.29166666666</v>
       </c>
       <c r="B126" s="4" t="n">
         <v>285</v>
@@ -7100,7 +7100,7 @@
     </row>
     <row r="127" ht="16" customHeight="1" s="5">
       <c r="A127" s="3" t="n">
-        <v>46157.30208333334</v>
+        <v>46158.30208333334</v>
       </c>
       <c r="B127" s="4" t="n">
         <v>290</v>
@@ -7147,7 +7147,7 @@
     </row>
     <row r="128" ht="16" customHeight="1" s="5">
       <c r="A128" s="3" t="n">
-        <v>46157.3125</v>
+        <v>46158.3125</v>
       </c>
       <c r="B128" s="4" t="n">
         <v>323</v>
@@ -7194,7 +7194,7 @@
     </row>
     <row r="129" ht="16" customHeight="1" s="5">
       <c r="A129" s="3" t="n">
-        <v>46157.32291666666</v>
+        <v>46158.32291666666</v>
       </c>
       <c r="B129" s="4" t="n">
         <v>271</v>
@@ -7241,7 +7241,7 @@
     </row>
     <row r="130" ht="16" customHeight="1" s="5">
       <c r="A130" s="3" t="n">
-        <v>46157.33333333334</v>
+        <v>46158.33333333334</v>
       </c>
       <c r="B130" s="4" t="n">
         <v>246</v>
@@ -7288,7 +7288,7 @@
     </row>
     <row r="131" ht="16" customHeight="1" s="5">
       <c r="A131" s="3" t="n">
-        <v>46157.34375</v>
+        <v>46158.34375</v>
       </c>
       <c r="B131" s="4" t="n">
         <v>287</v>
@@ -7335,7 +7335,7 @@
     </row>
     <row r="132" ht="16" customHeight="1" s="5">
       <c r="A132" s="3" t="n">
-        <v>46157.35416666666</v>
+        <v>46158.35416666666</v>
       </c>
       <c r="B132" s="4" t="n">
         <v>275</v>
@@ -7382,7 +7382,7 @@
     </row>
     <row r="133" ht="16" customHeight="1" s="5">
       <c r="A133" s="3" t="n">
-        <v>46157.36458333334</v>
+        <v>46158.36458333334</v>
       </c>
       <c r="B133" s="4" t="n">
         <v>447</v>
@@ -7429,7 +7429,7 @@
     </row>
     <row r="134" ht="16" customHeight="1" s="5">
       <c r="A134" s="3" t="n">
-        <v>46157.375</v>
+        <v>46158.375</v>
       </c>
       <c r="B134" s="4" t="n">
         <v>566</v>
@@ -7476,7 +7476,7 @@
     </row>
     <row r="135" ht="16" customHeight="1" s="5">
       <c r="A135" s="3" t="n">
-        <v>46157.38541666666</v>
+        <v>46158.38541666666</v>
       </c>
       <c r="B135" s="4" t="n">
         <v>590</v>
@@ -7523,7 +7523,7 @@
     </row>
     <row r="136" ht="16" customHeight="1" s="5">
       <c r="A136" s="3" t="n">
-        <v>46157.39583333334</v>
+        <v>46158.39583333334</v>
       </c>
       <c r="B136" s="4" t="n">
         <v>558</v>
@@ -7570,7 +7570,7 @@
     </row>
     <row r="137" ht="16" customHeight="1" s="5">
       <c r="A137" s="3" t="n">
-        <v>46157.40625</v>
+        <v>46158.40625</v>
       </c>
       <c r="B137" s="4" t="n">
         <v>354</v>
@@ -7617,7 +7617,7 @@
     </row>
     <row r="138" ht="16" customHeight="1" s="5">
       <c r="A138" s="3" t="n">
-        <v>46157.41666666666</v>
+        <v>46158.41666666666</v>
       </c>
       <c r="B138" s="4" t="n">
         <v>483</v>
@@ -7664,7 +7664,7 @@
     </row>
     <row r="139" ht="16" customHeight="1" s="5">
       <c r="A139" s="3" t="n">
-        <v>46157.42708333334</v>
+        <v>46158.42708333334</v>
       </c>
       <c r="B139" s="4" t="n">
         <v>537</v>
@@ -7711,7 +7711,7 @@
     </row>
     <row r="140" ht="16" customHeight="1" s="5">
       <c r="A140" s="3" t="n">
-        <v>46157.4375</v>
+        <v>46158.4375</v>
       </c>
       <c r="B140" s="4" t="n">
         <v>558</v>
@@ -7758,7 +7758,7 @@
     </row>
     <row r="141" ht="16" customHeight="1" s="5">
       <c r="A141" s="3" t="n">
-        <v>46157.44791666666</v>
+        <v>46158.44791666666</v>
       </c>
       <c r="B141" s="4" t="n">
         <v>570</v>
@@ -7805,7 +7805,7 @@
     </row>
     <row r="142" ht="16" customHeight="1" s="5">
       <c r="A142" s="3" t="n">
-        <v>46157.45833333334</v>
+        <v>46158.45833333334</v>
       </c>
       <c r="B142" s="4" t="n">
         <v>424</v>
@@ -7852,7 +7852,7 @@
     </row>
     <row r="143" ht="16" customHeight="1" s="5">
       <c r="A143" s="3" t="n">
-        <v>46157.46875</v>
+        <v>46158.46875</v>
       </c>
       <c r="B143" s="4" t="n">
         <v>377</v>
@@ -7899,7 +7899,7 @@
     </row>
     <row r="144" ht="16" customHeight="1" s="5">
       <c r="A144" s="3" t="n">
-        <v>46157.47916666666</v>
+        <v>46158.47916666666</v>
       </c>
       <c r="B144" s="4" t="n">
         <v>372</v>
@@ -7946,7 +7946,7 @@
     </row>
     <row r="145" ht="16" customHeight="1" s="5">
       <c r="A145" s="3" t="n">
-        <v>46157.48958333334</v>
+        <v>46158.48958333334</v>
       </c>
       <c r="B145" s="4" t="n">
         <v>374</v>
@@ -7993,7 +7993,7 @@
     </row>
     <row r="146" ht="16" customHeight="1" s="5">
       <c r="A146" s="3" t="n">
-        <v>46157.5</v>
+        <v>46158.5</v>
       </c>
       <c r="B146" s="4" t="n">
         <v>508</v>
@@ -8040,7 +8040,7 @@
     </row>
     <row r="147" ht="16" customHeight="1" s="5">
       <c r="A147" s="3" t="n">
-        <v>46157.51041666666</v>
+        <v>46158.51041666666</v>
       </c>
       <c r="B147" s="4" t="n">
         <v>482</v>
@@ -8087,7 +8087,7 @@
     </row>
     <row r="148" ht="16" customHeight="1" s="5">
       <c r="A148" s="3" t="n">
-        <v>46157.52083333334</v>
+        <v>46158.52083333334</v>
       </c>
       <c r="B148" s="4" t="n">
         <v>416</v>
@@ -8134,7 +8134,7 @@
     </row>
     <row r="149" ht="16" customHeight="1" s="5">
       <c r="A149" s="3" t="n">
-        <v>46157.53125</v>
+        <v>46158.53125</v>
       </c>
       <c r="B149" s="4" t="n">
         <v>498</v>
@@ -8181,7 +8181,7 @@
     </row>
     <row r="150" ht="16" customHeight="1" s="5">
       <c r="A150" s="3" t="n">
-        <v>46157.54166666666</v>
+        <v>46158.54166666666</v>
       </c>
       <c r="B150" s="4" t="n">
         <v>378</v>
@@ -8228,7 +8228,7 @@
     </row>
     <row r="151" ht="16" customHeight="1" s="5">
       <c r="A151" s="3" t="n">
-        <v>46157.55208333334</v>
+        <v>46158.55208333334</v>
       </c>
       <c r="B151" s="4" t="n">
         <v>245</v>
@@ -8275,7 +8275,7 @@
     </row>
     <row r="152" ht="16" customHeight="1" s="5">
       <c r="A152" s="3" t="n">
-        <v>46157.5625</v>
+        <v>46158.5625</v>
       </c>
       <c r="B152" s="4" t="n">
         <v>253</v>
@@ -8322,7 +8322,7 @@
     </row>
     <row r="153" ht="16" customHeight="1" s="5">
       <c r="A153" s="3" t="n">
-        <v>46157.57291666666</v>
+        <v>46158.57291666666</v>
       </c>
       <c r="B153" s="4" t="n">
         <v>302</v>
@@ -8369,7 +8369,7 @@
     </row>
     <row r="154" ht="16" customHeight="1" s="5">
       <c r="A154" s="3" t="n">
-        <v>46157.58333333334</v>
+        <v>46158.58333333334</v>
       </c>
       <c r="B154" s="4" t="n">
         <v>405</v>
@@ -8416,7 +8416,7 @@
     </row>
     <row r="155" ht="16" customHeight="1" s="5">
       <c r="A155" s="3" t="n">
-        <v>46157.59375</v>
+        <v>46158.59375</v>
       </c>
       <c r="B155" s="4" t="n">
         <v>472</v>
@@ -8463,7 +8463,7 @@
     </row>
     <row r="156" ht="16" customHeight="1" s="5">
       <c r="A156" s="3" t="n">
-        <v>46157.60416666666</v>
+        <v>46158.60416666666</v>
       </c>
       <c r="B156" s="4" t="n">
         <v>591</v>
@@ -8510,7 +8510,7 @@
     </row>
     <row r="157" ht="16" customHeight="1" s="5">
       <c r="A157" s="3" t="n">
-        <v>46157.61458333334</v>
+        <v>46158.61458333334</v>
       </c>
       <c r="B157" s="4" t="n">
         <v>607</v>
@@ -8557,7 +8557,7 @@
     </row>
     <row r="158" ht="16" customHeight="1" s="5">
       <c r="A158" s="3" t="n">
-        <v>46157.625</v>
+        <v>46158.625</v>
       </c>
       <c r="B158" s="4" t="n">
         <v>441</v>
@@ -8604,7 +8604,7 @@
     </row>
     <row r="159" ht="16" customHeight="1" s="5">
       <c r="A159" s="3" t="n">
-        <v>46157.63541666666</v>
+        <v>46158.63541666666</v>
       </c>
       <c r="B159" s="4" t="n">
         <v>309</v>
@@ -8651,7 +8651,7 @@
     </row>
     <row r="160" ht="16" customHeight="1" s="5">
       <c r="A160" s="3" t="n">
-        <v>46157.64583333334</v>
+        <v>46158.64583333334</v>
       </c>
       <c r="B160" s="4" t="n">
         <v>406</v>
@@ -8698,7 +8698,7 @@
     </row>
     <row r="161" ht="16" customHeight="1" s="5">
       <c r="A161" s="3" t="n">
-        <v>46157.65625</v>
+        <v>46158.65625</v>
       </c>
       <c r="B161" s="4" t="n">
         <v>545</v>
@@ -8745,7 +8745,7 @@
     </row>
     <row r="162" ht="16" customHeight="1" s="5">
       <c r="A162" s="3" t="n">
-        <v>46157.66666666666</v>
+        <v>46158.66666666666</v>
       </c>
       <c r="B162" s="4" t="n">
         <v>659</v>
@@ -8792,7 +8792,7 @@
     </row>
     <row r="163" ht="16" customHeight="1" s="5">
       <c r="A163" s="3" t="n">
-        <v>46157.67708333334</v>
+        <v>46158.67708333334</v>
       </c>
       <c r="B163" s="4" t="n">
         <v>904</v>
@@ -8839,7 +8839,7 @@
     </row>
     <row r="164" ht="16" customHeight="1" s="5">
       <c r="A164" s="3" t="n">
-        <v>46157.6875</v>
+        <v>46158.6875</v>
       </c>
       <c r="B164" s="4" t="n">
         <v>870</v>
@@ -8886,7 +8886,7 @@
     </row>
     <row r="165" ht="16" customHeight="1" s="5">
       <c r="A165" s="3" t="n">
-        <v>46157.69791666666</v>
+        <v>46158.69791666666</v>
       </c>
       <c r="B165" s="4" t="n">
         <v>773</v>
@@ -8933,7 +8933,7 @@
     </row>
     <row r="166" ht="16" customHeight="1" s="5">
       <c r="A166" s="3" t="n">
-        <v>46157.70833333334</v>
+        <v>46158.70833333334</v>
       </c>
       <c r="B166" s="4" t="n">
         <v>654</v>
@@ -8980,7 +8980,7 @@
     </row>
     <row r="167" ht="16" customHeight="1" s="5">
       <c r="A167" s="3" t="n">
-        <v>46157.71875</v>
+        <v>46158.71875</v>
       </c>
       <c r="B167" s="4" t="n">
         <v>472</v>
@@ -9027,7 +9027,7 @@
     </row>
     <row r="168" ht="16" customHeight="1" s="5">
       <c r="A168" s="3" t="n">
-        <v>46157.72916666666</v>
+        <v>46158.72916666666</v>
       </c>
       <c r="B168" s="4" t="n">
         <v>483</v>
@@ -9074,7 +9074,7 @@
     </row>
     <row r="169" ht="16" customHeight="1" s="5">
       <c r="A169" s="3" t="n">
-        <v>46157.73958333334</v>
+        <v>46158.73958333334</v>
       </c>
       <c r="B169" s="4" t="n">
         <v>597</v>
@@ -9121,7 +9121,7 @@
     </row>
     <row r="170" ht="16" customHeight="1" s="5">
       <c r="A170" s="3" t="n">
-        <v>46157.75</v>
+        <v>46158.75</v>
       </c>
       <c r="B170" s="4" t="n">
         <v>597</v>
@@ -9168,7 +9168,7 @@
     </row>
     <row r="171" ht="16" customHeight="1" s="5">
       <c r="A171" s="3" t="n">
-        <v>46157.76041666666</v>
+        <v>46158.76041666666</v>
       </c>
       <c r="B171" s="4" t="n">
         <v>569</v>
@@ -9215,7 +9215,7 @@
     </row>
     <row r="172" ht="16" customHeight="1" s="5">
       <c r="A172" s="3" t="n">
-        <v>46157.77083333334</v>
+        <v>46158.77083333334</v>
       </c>
       <c r="B172" s="4" t="n">
         <v>423</v>
@@ -9262,7 +9262,7 @@
     </row>
     <row r="173" ht="16" customHeight="1" s="5">
       <c r="A173" s="3" t="n">
-        <v>46157.78125</v>
+        <v>46158.78125</v>
       </c>
       <c r="B173" s="4" t="n">
         <v>269</v>
@@ -9309,7 +9309,7 @@
     </row>
     <row r="174" ht="16" customHeight="1" s="5">
       <c r="A174" s="3" t="n">
-        <v>46157.79166666666</v>
+        <v>46158.79166666666</v>
       </c>
       <c r="B174" s="4" t="n">
         <v>312</v>
@@ -9356,7 +9356,7 @@
     </row>
     <row r="175" ht="16" customHeight="1" s="5">
       <c r="A175" s="3" t="n">
-        <v>46157.80208333334</v>
+        <v>46158.80208333334</v>
       </c>
       <c r="B175" s="4" t="n">
         <v>557</v>
@@ -9403,7 +9403,7 @@
     </row>
     <row r="176" ht="16" customHeight="1" s="5">
       <c r="A176" s="3" t="n">
-        <v>46157.8125</v>
+        <v>46158.8125</v>
       </c>
       <c r="B176" s="4" t="n">
         <v>690</v>
@@ -9450,7 +9450,7 @@
     </row>
     <row r="177" ht="16" customHeight="1" s="5">
       <c r="A177" s="3" t="n">
-        <v>46157.82291666666</v>
+        <v>46158.82291666666</v>
       </c>
       <c r="B177" s="4" t="n">
         <v>511</v>
@@ -9497,7 +9497,7 @@
     </row>
     <row r="178" ht="16" customHeight="1" s="5">
       <c r="A178" s="3" t="n">
-        <v>46157.83333333334</v>
+        <v>46158.83333333334</v>
       </c>
       <c r="B178" s="4" t="n">
         <v>188</v>
@@ -9544,7 +9544,7 @@
     </row>
     <row r="179" ht="16" customHeight="1" s="5">
       <c r="A179" s="3" t="n">
-        <v>46157.84375</v>
+        <v>46158.84375</v>
       </c>
       <c r="B179" s="4" t="n">
         <v>204</v>
@@ -9591,7 +9591,7 @@
     </row>
     <row r="180" ht="16" customHeight="1" s="5">
       <c r="A180" s="3" t="n">
-        <v>46157.85416666666</v>
+        <v>46158.85416666666</v>
       </c>
       <c r="B180" s="4" t="n">
         <v>287</v>
@@ -9638,7 +9638,7 @@
     </row>
     <row r="181" ht="16" customHeight="1" s="5">
       <c r="A181" s="3" t="n">
-        <v>46157.86458333334</v>
+        <v>46158.86458333334</v>
       </c>
       <c r="B181" s="4" t="n">
         <v>177</v>
@@ -9685,7 +9685,7 @@
     </row>
     <row r="182" ht="16" customHeight="1" s="5">
       <c r="A182" s="3" t="n">
-        <v>46157.875</v>
+        <v>46158.875</v>
       </c>
       <c r="B182" s="4" t="n">
         <v>9</v>
@@ -9732,7 +9732,7 @@
     </row>
     <row r="183" ht="16" customHeight="1" s="5">
       <c r="A183" s="3" t="n">
-        <v>46157.88541666666</v>
+        <v>46158.88541666666</v>
       </c>
       <c r="B183" s="4" t="n">
         <v>0</v>
@@ -9779,7 +9779,7 @@
     </row>
     <row r="184" ht="16" customHeight="1" s="5">
       <c r="A184" s="3" t="n">
-        <v>46157.89583333334</v>
+        <v>46158.89583333334</v>
       </c>
       <c r="B184" s="4" t="n">
         <v>0</v>
@@ -9826,7 +9826,7 @@
     </row>
     <row r="185" ht="16" customHeight="1" s="5">
       <c r="A185" s="3" t="n">
-        <v>46157.90625</v>
+        <v>46158.90625</v>
       </c>
       <c r="B185" s="4" t="n">
         <v>15</v>
@@ -9873,7 +9873,7 @@
     </row>
     <row r="186" ht="16" customHeight="1" s="5">
       <c r="A186" s="3" t="n">
-        <v>46157.91666666666</v>
+        <v>46158.91666666666</v>
       </c>
       <c r="B186" s="4" t="n">
         <v>69</v>
@@ -9920,7 +9920,7 @@
     </row>
     <row r="187" ht="16" customHeight="1" s="5">
       <c r="A187" s="3" t="n">
-        <v>46157.92708333334</v>
+        <v>46158.92708333334</v>
       </c>
       <c r="B187" s="4" t="n">
         <v>126</v>
@@ -9967,7 +9967,7 @@
     </row>
     <row r="188" ht="16" customHeight="1" s="5">
       <c r="A188" s="3" t="n">
-        <v>46157.9375</v>
+        <v>46158.9375</v>
       </c>
       <c r="B188" s="4" t="n">
         <v>175</v>
@@ -10014,7 +10014,7 @@
     </row>
     <row r="189" ht="16" customHeight="1" s="5">
       <c r="A189" s="3" t="n">
-        <v>46157.94791666666</v>
+        <v>46158.94791666666</v>
       </c>
       <c r="B189" s="4" t="n">
         <v>82</v>
@@ -10061,7 +10061,7 @@
     </row>
     <row r="190" ht="16" customHeight="1" s="5">
       <c r="A190" s="3" t="n">
-        <v>46157.95833333334</v>
+        <v>46158.95833333334</v>
       </c>
       <c r="B190" s="4" t="n">
         <v>0</v>
@@ -10108,7 +10108,7 @@
     </row>
     <row r="191" ht="16" customHeight="1" s="5">
       <c r="A191" s="3" t="n">
-        <v>46157.96875</v>
+        <v>46158.96875</v>
       </c>
       <c r="B191" s="4" t="n">
         <v>0</v>
@@ -10155,7 +10155,7 @@
     </row>
     <row r="192" ht="16" customHeight="1" s="5">
       <c r="A192" s="3" t="n">
-        <v>46157.97916666666</v>
+        <v>46158.97916666666</v>
       </c>
       <c r="B192" s="4" t="n">
         <v>0</v>
@@ -10202,7 +10202,7 @@
     </row>
     <row r="193" ht="16" customHeight="1" s="5">
       <c r="A193" s="3" t="n">
-        <v>46157.98958333334</v>
+        <v>46158.98958333334</v>
       </c>
       <c r="B193" s="4" t="n">
         <v>0</v>
@@ -10249,7 +10249,7 @@
     </row>
     <row r="194" ht="16" customHeight="1" s="5">
       <c r="A194" s="3" t="n">
-        <v>46158</v>
+        <v>46159</v>
       </c>
       <c r="B194" s="4" t="n">
         <v>0</v>
@@ -10296,7 +10296,7 @@
     </row>
     <row r="195" ht="16" customHeight="1" s="5">
       <c r="A195" s="3" t="n">
-        <v>46158.01041666666</v>
+        <v>46159.01041666666</v>
       </c>
       <c r="B195" s="4" t="n">
         <v>10</v>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="196" ht="16" customHeight="1" s="5">
       <c r="A196" s="3" t="n">
-        <v>46158.02083333334</v>
+        <v>46159.02083333334</v>
       </c>
       <c r="B196" s="4" t="n">
         <v>35</v>
@@ -10390,7 +10390,7 @@
     </row>
     <row r="197" ht="16" customHeight="1" s="5">
       <c r="A197" s="3" t="n">
-        <v>46158.03125</v>
+        <v>46159.03125</v>
       </c>
       <c r="B197" s="4" t="n">
         <v>62</v>
@@ -10437,7 +10437,7 @@
     </row>
     <row r="198" ht="16" customHeight="1" s="5">
       <c r="A198" s="3" t="n">
-        <v>46158.04166666666</v>
+        <v>46159.04166666666</v>
       </c>
       <c r="B198" s="4" t="n">
         <v>80</v>
@@ -10484,7 +10484,7 @@
     </row>
     <row r="199" ht="16" customHeight="1" s="5">
       <c r="A199" s="3" t="n">
-        <v>46158.05208333334</v>
+        <v>46159.05208333334</v>
       </c>
       <c r="B199" s="4" t="n">
         <v>27</v>
@@ -10531,7 +10531,7 @@
     </row>
     <row r="200" ht="16" customHeight="1" s="5">
       <c r="A200" s="3" t="n">
-        <v>46158.0625</v>
+        <v>46159.0625</v>
       </c>
       <c r="B200" s="4" t="n">
         <v>0</v>
@@ -10578,7 +10578,7 @@
     </row>
     <row r="201" ht="16" customHeight="1" s="5">
       <c r="A201" s="3" t="n">
-        <v>46158.07291666666</v>
+        <v>46159.07291666666</v>
       </c>
       <c r="B201" s="4" t="n">
         <v>4</v>
@@ -10625,7 +10625,7 @@
     </row>
     <row r="202" ht="16" customHeight="1" s="5">
       <c r="A202" s="3" t="n">
-        <v>46158.08333333334</v>
+        <v>46159.08333333334</v>
       </c>
       <c r="B202" s="4" t="n">
         <v>11</v>
@@ -10672,7 +10672,7 @@
     </row>
     <row r="203" ht="16" customHeight="1" s="5">
       <c r="A203" s="3" t="n">
-        <v>46158.09375</v>
+        <v>46159.09375</v>
       </c>
       <c r="B203" s="4" t="n">
         <v>20</v>
@@ -10719,7 +10719,7 @@
     </row>
     <row r="204" ht="16" customHeight="1" s="5">
       <c r="A204" s="3" t="n">
-        <v>46158.10416666666</v>
+        <v>46159.10416666666</v>
       </c>
       <c r="B204" s="4" t="n">
         <v>33</v>
@@ -10766,7 +10766,7 @@
     </row>
     <row r="205" ht="16" customHeight="1" s="5">
       <c r="A205" s="3" t="n">
-        <v>46158.11458333334</v>
+        <v>46159.11458333334</v>
       </c>
       <c r="B205" s="4" t="n">
         <v>17</v>
@@ -10813,7 +10813,7 @@
     </row>
     <row r="206" ht="16" customHeight="1" s="5">
       <c r="A206" s="3" t="n">
-        <v>46158.125</v>
+        <v>46159.125</v>
       </c>
       <c r="B206" s="4" t="n">
         <v>19</v>
@@ -10860,7 +10860,7 @@
     </row>
     <row r="207" ht="16" customHeight="1" s="5">
       <c r="A207" s="3" t="n">
-        <v>46158.13541666666</v>
+        <v>46159.13541666666</v>
       </c>
       <c r="B207" s="4" t="n">
         <v>26</v>
@@ -10907,7 +10907,7 @@
     </row>
     <row r="208" ht="16" customHeight="1" s="5">
       <c r="A208" s="3" t="n">
-        <v>46158.14583333334</v>
+        <v>46159.14583333334</v>
       </c>
       <c r="B208" s="4" t="n">
         <v>65</v>
@@ -10954,7 +10954,7 @@
     </row>
     <row r="209" ht="16" customHeight="1" s="5">
       <c r="A209" s="3" t="n">
-        <v>46158.15625</v>
+        <v>46159.15625</v>
       </c>
       <c r="B209" s="4" t="n">
         <v>256</v>
@@ -11001,7 +11001,7 @@
     </row>
     <row r="210" ht="16" customHeight="1" s="5">
       <c r="A210" s="3" t="n">
-        <v>46158.16666666666</v>
+        <v>46159.16666666666</v>
       </c>
       <c r="B210" s="4" t="n">
         <v>528</v>
@@ -11048,7 +11048,7 @@
     </row>
     <row r="211" ht="16" customHeight="1" s="5">
       <c r="A211" s="3" t="n">
-        <v>46158.17708333334</v>
+        <v>46159.17708333334</v>
       </c>
       <c r="B211" s="4" t="n">
         <v>850</v>
@@ -11095,7 +11095,7 @@
     </row>
     <row r="212" ht="16" customHeight="1" s="5">
       <c r="A212" s="3" t="n">
-        <v>46158.1875</v>
+        <v>46159.1875</v>
       </c>
       <c r="B212" s="4" t="n">
         <v>967</v>
@@ -11142,7 +11142,7 @@
     </row>
     <row r="213" ht="16" customHeight="1" s="5">
       <c r="A213" s="3" t="n">
-        <v>46158.19791666666</v>
+        <v>46159.19791666666</v>
       </c>
       <c r="B213" s="4" t="n">
         <v>755</v>
@@ -11189,7 +11189,7 @@
     </row>
     <row r="214" ht="16" customHeight="1" s="5">
       <c r="A214" s="3" t="n">
-        <v>46158.20833333334</v>
+        <v>46159.20833333334</v>
       </c>
       <c r="B214" s="4" t="n">
         <v>800</v>
@@ -11236,7 +11236,7 @@
     </row>
     <row r="215" ht="16" customHeight="1" s="5">
       <c r="A215" s="3" t="n">
-        <v>46158.21875</v>
+        <v>46159.21875</v>
       </c>
       <c r="B215" s="4" t="n">
         <v>656</v>
@@ -11283,7 +11283,7 @@
     </row>
     <row r="216" ht="16" customHeight="1" s="5">
       <c r="A216" s="3" t="n">
-        <v>46158.22916666666</v>
+        <v>46159.22916666666</v>
       </c>
       <c r="B216" s="4" t="n">
         <v>515</v>
@@ -11330,7 +11330,7 @@
     </row>
     <row r="217" ht="16" customHeight="1" s="5">
       <c r="A217" s="3" t="n">
-        <v>46158.23958333334</v>
+        <v>46159.23958333334</v>
       </c>
       <c r="B217" s="4" t="n">
         <v>474</v>
@@ -11377,7 +11377,7 @@
     </row>
     <row r="218" ht="16" customHeight="1" s="5">
       <c r="A218" s="3" t="n">
-        <v>46158.25</v>
+        <v>46159.25</v>
       </c>
       <c r="B218" s="4" t="n">
         <v>601</v>
@@ -11424,7 +11424,7 @@
     </row>
     <row r="219" ht="16" customHeight="1" s="5">
       <c r="A219" s="3" t="n">
-        <v>46158.26041666666</v>
+        <v>46159.26041666666</v>
       </c>
       <c r="B219" s="4" t="n">
         <v>632</v>
@@ -11471,7 +11471,7 @@
     </row>
     <row r="220" ht="16" customHeight="1" s="5">
       <c r="A220" s="3" t="n">
-        <v>46158.27083333334</v>
+        <v>46159.27083333334</v>
       </c>
       <c r="B220" s="4" t="n">
         <v>592</v>
@@ -11518,7 +11518,7 @@
     </row>
     <row r="221" ht="16" customHeight="1" s="5">
       <c r="A221" s="3" t="n">
-        <v>46158.28125</v>
+        <v>46159.28125</v>
       </c>
       <c r="B221" s="4" t="n">
         <v>493</v>
@@ -11565,7 +11565,7 @@
     </row>
     <row r="222" ht="16" customHeight="1" s="5">
       <c r="A222" s="3" t="n">
-        <v>46158.29166666666</v>
+        <v>46159.29166666666</v>
       </c>
       <c r="B222" s="4" t="n">
         <v>448</v>
@@ -11612,7 +11612,7 @@
     </row>
     <row r="223" ht="16" customHeight="1" s="5">
       <c r="A223" s="3" t="n">
-        <v>46158.30208333334</v>
+        <v>46159.30208333334</v>
       </c>
       <c r="B223" s="4" t="n">
         <v>459</v>
@@ -11659,7 +11659,7 @@
     </row>
     <row r="224" ht="16" customHeight="1" s="5">
       <c r="A224" s="3" t="n">
-        <v>46158.3125</v>
+        <v>46159.3125</v>
       </c>
       <c r="B224" s="4" t="n">
         <v>432</v>
@@ -11706,7 +11706,7 @@
     </row>
     <row r="225" ht="16" customHeight="1" s="5">
       <c r="A225" s="3" t="n">
-        <v>46158.32291666666</v>
+        <v>46159.32291666666</v>
       </c>
       <c r="B225" s="4" t="n">
         <v>368</v>
@@ -11753,7 +11753,7 @@
     </row>
     <row r="226" ht="16" customHeight="1" s="5">
       <c r="A226" s="3" t="n">
-        <v>46158.33333333334</v>
+        <v>46159.33333333334</v>
       </c>
       <c r="B226" s="4" t="n">
         <v>320</v>
@@ -11800,7 +11800,7 @@
     </row>
     <row r="227" ht="16" customHeight="1" s="5">
       <c r="A227" s="3" t="n">
-        <v>46158.34375</v>
+        <v>46159.34375</v>
       </c>
       <c r="B227" s="4" t="n">
         <v>237</v>
@@ -11847,7 +11847,7 @@
     </row>
     <row r="228" ht="16" customHeight="1" s="5">
       <c r="A228" s="3" t="n">
-        <v>46158.35416666666</v>
+        <v>46159.35416666666</v>
       </c>
       <c r="B228" s="4" t="n">
         <v>262</v>
@@ -11894,7 +11894,7 @@
     </row>
     <row r="229" ht="16" customHeight="1" s="5">
       <c r="A229" s="3" t="n">
-        <v>46158.36458333334</v>
+        <v>46159.36458333334</v>
       </c>
       <c r="B229" s="4" t="n">
         <v>445</v>
@@ -11941,7 +11941,7 @@
     </row>
     <row r="230" ht="16" customHeight="1" s="5">
       <c r="A230" s="3" t="n">
-        <v>46158.375</v>
+        <v>46159.375</v>
       </c>
       <c r="B230" s="4" t="n">
         <v>627</v>
@@ -11988,7 +11988,7 @@
     </row>
     <row r="231" ht="16" customHeight="1" s="5">
       <c r="A231" s="3" t="n">
-        <v>46158.38541666666</v>
+        <v>46159.38541666666</v>
       </c>
       <c r="B231" s="4" t="n">
         <v>623</v>
@@ -12035,7 +12035,7 @@
     </row>
     <row r="232" ht="16" customHeight="1" s="5">
       <c r="A232" s="3" t="n">
-        <v>46158.39583333334</v>
+        <v>46159.39583333334</v>
       </c>
       <c r="B232" s="4" t="n">
         <v>576</v>
@@ -12082,7 +12082,7 @@
     </row>
     <row r="233" ht="16" customHeight="1" s="5">
       <c r="A233" s="3" t="n">
-        <v>46158.40625</v>
+        <v>46159.40625</v>
       </c>
       <c r="B233" s="4" t="n">
         <v>542</v>
@@ -12129,7 +12129,7 @@
     </row>
     <row r="234" ht="16" customHeight="1" s="5">
       <c r="A234" s="3" t="n">
-        <v>46158.41666666666</v>
+        <v>46159.41666666666</v>
       </c>
       <c r="B234" s="4" t="n">
         <v>484</v>
@@ -12176,7 +12176,7 @@
     </row>
     <row r="235" ht="16" customHeight="1" s="5">
       <c r="A235" s="3" t="n">
-        <v>46158.42708333334</v>
+        <v>46159.42708333334</v>
       </c>
       <c r="B235" s="4" t="n">
         <v>377</v>
@@ -12223,7 +12223,7 @@
     </row>
     <row r="236" ht="16" customHeight="1" s="5">
       <c r="A236" s="3" t="n">
-        <v>46158.4375</v>
+        <v>46159.4375</v>
       </c>
       <c r="B236" s="4" t="n">
         <v>281</v>
@@ -12270,7 +12270,7 @@
     </row>
     <row r="237" ht="16" customHeight="1" s="5">
       <c r="A237" s="3" t="n">
-        <v>46158.44791666666</v>
+        <v>46159.44791666666</v>
       </c>
       <c r="B237" s="4" t="n">
         <v>386</v>
@@ -12317,7 +12317,7 @@
     </row>
     <row r="238" ht="16" customHeight="1" s="5">
       <c r="A238" s="3" t="n">
-        <v>46158.45833333334</v>
+        <v>46159.45833333334</v>
       </c>
       <c r="B238" s="4" t="n">
         <v>548</v>
@@ -12364,7 +12364,7 @@
     </row>
     <row r="239" ht="16" customHeight="1" s="5">
       <c r="A239" s="3" t="n">
-        <v>46158.46875</v>
+        <v>46159.46875</v>
       </c>
       <c r="B239" s="4" t="n">
         <v>620</v>
@@ -12411,7 +12411,7 @@
     </row>
     <row r="240" ht="16" customHeight="1" s="5">
       <c r="A240" s="3" t="n">
-        <v>46158.47916666666</v>
+        <v>46159.47916666666</v>
       </c>
       <c r="B240" s="4" t="n">
         <v>531</v>
@@ -12458,7 +12458,7 @@
     </row>
     <row r="241" ht="16" customHeight="1" s="5">
       <c r="A241" s="3" t="n">
-        <v>46158.48958333334</v>
+        <v>46159.48958333334</v>
       </c>
       <c r="B241" s="4" t="n">
         <v>491</v>
@@ -12505,7 +12505,7 @@
     </row>
     <row r="242" ht="16" customHeight="1" s="5">
       <c r="A242" s="3" t="n">
-        <v>46158.5</v>
+        <v>46159.5</v>
       </c>
       <c r="B242" s="4" t="n">
         <v>385</v>
@@ -12552,7 +12552,7 @@
     </row>
     <row r="243" ht="16" customHeight="1" s="5">
       <c r="A243" s="3" t="n">
-        <v>46158.51041666666</v>
+        <v>46159.51041666666</v>
       </c>
       <c r="B243" s="4" t="n">
         <v>397</v>
@@ -12599,7 +12599,7 @@
     </row>
     <row r="244" ht="16" customHeight="1" s="5">
       <c r="A244" s="3" t="n">
-        <v>46158.52083333334</v>
+        <v>46159.52083333334</v>
       </c>
       <c r="B244" s="4" t="n">
         <v>490</v>
@@ -12646,7 +12646,7 @@
     </row>
     <row r="245" ht="16" customHeight="1" s="5">
       <c r="A245" s="3" t="n">
-        <v>46158.53125</v>
+        <v>46159.53125</v>
       </c>
       <c r="B245" s="4" t="n">
         <v>547</v>
@@ -12693,7 +12693,7 @@
     </row>
     <row r="246" ht="16" customHeight="1" s="5">
       <c r="A246" s="3" t="n">
-        <v>46158.54166666666</v>
+        <v>46159.54166666666</v>
       </c>
       <c r="B246" s="4" t="n">
         <v>415</v>
@@ -12740,7 +12740,7 @@
     </row>
     <row r="247" ht="16" customHeight="1" s="5">
       <c r="A247" s="3" t="n">
-        <v>46158.55208333334</v>
+        <v>46159.55208333334</v>
       </c>
       <c r="B247" s="4" t="n">
         <v>228</v>
@@ -12787,7 +12787,7 @@
     </row>
     <row r="248" ht="16" customHeight="1" s="5">
       <c r="A248" s="3" t="n">
-        <v>46158.5625</v>
+        <v>46159.5625</v>
       </c>
       <c r="B248" s="4" t="n">
         <v>309</v>
@@ -12834,7 +12834,7 @@
     </row>
     <row r="249" ht="16" customHeight="1" s="5">
       <c r="A249" s="3" t="n">
-        <v>46158.57291666666</v>
+        <v>46159.57291666666</v>
       </c>
       <c r="B249" s="4" t="n">
         <v>411</v>
@@ -12881,7 +12881,7 @@
     </row>
     <row r="250" ht="16" customHeight="1" s="5">
       <c r="A250" s="3" t="n">
-        <v>46158.58333333334</v>
+        <v>46159.58333333334</v>
       </c>
       <c r="B250" s="4" t="n">
         <v>385</v>
@@ -12928,7 +12928,7 @@
     </row>
     <row r="251" ht="16" customHeight="1" s="5">
       <c r="A251" s="3" t="n">
-        <v>46158.59375</v>
+        <v>46159.59375</v>
       </c>
       <c r="B251" s="4" t="n">
         <v>436</v>
@@ -12975,7 +12975,7 @@
     </row>
     <row r="252" ht="16" customHeight="1" s="5">
       <c r="A252" s="3" t="n">
-        <v>46158.60416666666</v>
+        <v>46159.60416666666</v>
       </c>
       <c r="B252" s="4" t="n">
         <v>446</v>
@@ -13022,7 +13022,7 @@
     </row>
     <row r="253" ht="16" customHeight="1" s="5">
       <c r="A253" s="3" t="n">
-        <v>46158.61458333334</v>
+        <v>46159.61458333334</v>
       </c>
       <c r="B253" s="4" t="n">
         <v>426</v>
@@ -13069,7 +13069,7 @@
     </row>
     <row r="254" ht="16" customHeight="1" s="5">
       <c r="A254" s="3" t="n">
-        <v>46158.625</v>
+        <v>46159.625</v>
       </c>
       <c r="B254" s="4" t="n">
         <v>450</v>
@@ -13116,7 +13116,7 @@
     </row>
     <row r="255" ht="16" customHeight="1" s="5">
       <c r="A255" s="3" t="n">
-        <v>46158.63541666666</v>
+        <v>46159.63541666666</v>
       </c>
       <c r="B255" s="4" t="n">
         <v>322</v>
@@ -13163,7 +13163,7 @@
     </row>
     <row r="256" ht="16" customHeight="1" s="5">
       <c r="A256" s="3" t="n">
-        <v>46158.64583333334</v>
+        <v>46159.64583333334</v>
       </c>
       <c r="B256" s="4" t="n">
         <v>303</v>
@@ -13210,7 +13210,7 @@
     </row>
     <row r="257" ht="16" customHeight="1" s="5">
       <c r="A257" s="3" t="n">
-        <v>46158.65625</v>
+        <v>46159.65625</v>
       </c>
       <c r="B257" s="4" t="n">
         <v>496</v>
@@ -13257,7 +13257,7 @@
     </row>
     <row r="258" ht="16" customHeight="1" s="5">
       <c r="A258" s="3" t="n">
-        <v>46158.66666666666</v>
+        <v>46159.66666666666</v>
       </c>
       <c r="B258" s="4" t="n">
         <v>654</v>
@@ -13304,7 +13304,7 @@
     </row>
     <row r="259" ht="16" customHeight="1" s="5">
       <c r="A259" s="3" t="n">
-        <v>46158.67708333334</v>
+        <v>46159.67708333334</v>
       </c>
       <c r="B259" s="4" t="n">
         <v>781</v>
@@ -13351,7 +13351,7 @@
     </row>
     <row r="260" ht="16" customHeight="1" s="5">
       <c r="A260" s="3" t="n">
-        <v>46158.6875</v>
+        <v>46159.6875</v>
       </c>
       <c r="B260" s="4" t="n">
         <v>795</v>
@@ -13398,7 +13398,7 @@
     </row>
     <row r="261" ht="16" customHeight="1" s="5">
       <c r="A261" s="3" t="n">
-        <v>46158.69791666666</v>
+        <v>46159.69791666666</v>
       </c>
       <c r="B261" s="4" t="n">
         <v>569</v>
@@ -13445,7 +13445,7 @@
     </row>
     <row r="262" ht="16" customHeight="1" s="5">
       <c r="A262" s="3" t="n">
-        <v>46158.70833333334</v>
+        <v>46159.70833333334</v>
       </c>
       <c r="B262" s="4" t="n">
         <v>611</v>
@@ -13492,7 +13492,7 @@
     </row>
     <row r="263" ht="16" customHeight="1" s="5">
       <c r="A263" s="3" t="n">
-        <v>46158.71875</v>
+        <v>46159.71875</v>
       </c>
       <c r="B263" s="4" t="n">
         <v>794</v>
@@ -13539,7 +13539,7 @@
     </row>
     <row r="264" ht="16" customHeight="1" s="5">
       <c r="A264" s="3" t="n">
-        <v>46158.72916666666</v>
+        <v>46159.72916666666</v>
       </c>
       <c r="B264" s="4" t="n">
         <v>635</v>
@@ -13586,7 +13586,7 @@
     </row>
     <row r="265" ht="16" customHeight="1" s="5">
       <c r="A265" s="3" t="n">
-        <v>46158.73958333334</v>
+        <v>46159.73958333334</v>
       </c>
       <c r="B265" s="4" t="n">
         <v>642</v>
@@ -13633,7 +13633,7 @@
     </row>
     <row r="266" ht="16" customHeight="1" s="5">
       <c r="A266" s="3" t="n">
-        <v>46158.75</v>
+        <v>46159.75</v>
       </c>
       <c r="B266" s="4" t="n">
         <v>624</v>
@@ -13680,7 +13680,7 @@
     </row>
     <row r="267" ht="16" customHeight="1" s="5">
       <c r="A267" s="3" t="n">
-        <v>46158.76041666666</v>
+        <v>46159.76041666666</v>
       </c>
       <c r="B267" s="4" t="n">
         <v>608</v>
@@ -13727,7 +13727,7 @@
     </row>
     <row r="268" ht="16" customHeight="1" s="5">
       <c r="A268" s="3" t="n">
-        <v>46158.77083333334</v>
+        <v>46159.77083333334</v>
       </c>
       <c r="B268" s="4" t="n">
         <v>656</v>
@@ -13774,7 +13774,7 @@
     </row>
     <row r="269" ht="16" customHeight="1" s="5">
       <c r="A269" s="3" t="n">
-        <v>46158.78125</v>
+        <v>46159.78125</v>
       </c>
       <c r="B269" s="4" t="n">
         <v>512</v>
@@ -13821,7 +13821,7 @@
     </row>
     <row r="270" ht="16" customHeight="1" s="5">
       <c r="A270" s="3" t="n">
-        <v>46158.79166666666</v>
+        <v>46159.79166666666</v>
       </c>
       <c r="B270" s="4" t="n">
         <v>323</v>
@@ -13868,7 +13868,7 @@
     </row>
     <row r="271" ht="16" customHeight="1" s="5">
       <c r="A271" s="3" t="n">
-        <v>46158.80208333334</v>
+        <v>46159.80208333334</v>
       </c>
       <c r="B271" s="4" t="n">
         <v>438</v>
@@ -13915,7 +13915,7 @@
     </row>
     <row r="272" ht="16" customHeight="1" s="5">
       <c r="A272" s="3" t="n">
-        <v>46158.8125</v>
+        <v>46159.8125</v>
       </c>
       <c r="B272" s="4" t="n">
         <v>613</v>
@@ -13962,7 +13962,7 @@
     </row>
     <row r="273" ht="16" customHeight="1" s="5">
       <c r="A273" s="3" t="n">
-        <v>46158.82291666666</v>
+        <v>46159.82291666666</v>
       </c>
       <c r="B273" s="4" t="n">
         <v>547</v>
@@ -14009,7 +14009,7 @@
     </row>
     <row r="274" ht="16" customHeight="1" s="5">
       <c r="A274" s="3" t="n">
-        <v>46158.83333333334</v>
+        <v>46159.83333333334</v>
       </c>
       <c r="B274" s="4" t="n">
         <v>402</v>
@@ -14056,7 +14056,7 @@
     </row>
     <row r="275" ht="16" customHeight="1" s="5">
       <c r="A275" s="3" t="n">
-        <v>46158.84375</v>
+        <v>46159.84375</v>
       </c>
       <c r="B275" s="4" t="n">
         <v>341</v>
@@ -14103,7 +14103,7 @@
     </row>
     <row r="276" ht="16" customHeight="1" s="5">
       <c r="A276" s="3" t="n">
-        <v>46158.85416666666</v>
+        <v>46159.85416666666</v>
       </c>
       <c r="B276" s="4" t="n">
         <v>264</v>
@@ -14150,7 +14150,7 @@
     </row>
     <row r="277" ht="16" customHeight="1" s="5">
       <c r="A277" s="3" t="n">
-        <v>46158.86458333334</v>
+        <v>46159.86458333334</v>
       </c>
       <c r="B277" s="4" t="n">
         <v>116</v>
@@ -14197,7 +14197,7 @@
     </row>
     <row r="278" ht="16" customHeight="1" s="5">
       <c r="A278" s="3" t="n">
-        <v>46158.875</v>
+        <v>46159.875</v>
       </c>
       <c r="B278" s="4" t="n">
         <v>0</v>
@@ -14244,7 +14244,7 @@
     </row>
     <row r="279" ht="16" customHeight="1" s="5">
       <c r="A279" s="3" t="n">
-        <v>46158.88541666666</v>
+        <v>46159.88541666666</v>
       </c>
       <c r="B279" s="4" t="n">
         <v>10</v>
@@ -14291,7 +14291,7 @@
     </row>
     <row r="280" ht="16" customHeight="1" s="5">
       <c r="A280" s="3" t="n">
-        <v>46158.89583333334</v>
+        <v>46159.89583333334</v>
       </c>
       <c r="B280" s="4" t="n">
         <v>39</v>
@@ -14338,7 +14338,7 @@
     </row>
     <row r="281" ht="16" customHeight="1" s="5">
       <c r="A281" s="3" t="n">
-        <v>46158.90625</v>
+        <v>46159.90625</v>
       </c>
       <c r="B281" s="4" t="n">
         <v>109</v>
@@ -14385,7 +14385,7 @@
     </row>
     <row r="282" ht="16" customHeight="1" s="5">
       <c r="A282" s="3" t="n">
-        <v>46158.91666666666</v>
+        <v>46159.91666666666</v>
       </c>
       <c r="B282" s="4" t="n">
         <v>193</v>
@@ -14432,7 +14432,7 @@
     </row>
     <row r="283" ht="16" customHeight="1" s="5">
       <c r="A283" s="3" t="n">
-        <v>46158.92708333334</v>
+        <v>46159.92708333334</v>
       </c>
       <c r="B283" s="4" t="n">
         <v>217</v>
@@ -14479,7 +14479,7 @@
     </row>
     <row r="284" ht="16" customHeight="1" s="5">
       <c r="A284" s="3" t="n">
-        <v>46158.9375</v>
+        <v>46159.9375</v>
       </c>
       <c r="B284" s="4" t="n">
         <v>185</v>
@@ -14526,7 +14526,7 @@
     </row>
     <row r="285" ht="16" customHeight="1" s="5">
       <c r="A285" s="3" t="n">
-        <v>46158.94791666666</v>
+        <v>46159.94791666666</v>
       </c>
       <c r="B285" s="4" t="n">
         <v>27</v>
@@ -14573,7 +14573,7 @@
     </row>
     <row r="286" ht="16" customHeight="1" s="5">
       <c r="A286" s="3" t="n">
-        <v>46158.95833333334</v>
+        <v>46159.95833333334</v>
       </c>
       <c r="B286" s="4" t="n">
         <v>0</v>
@@ -14620,7 +14620,7 @@
     </row>
     <row r="287" ht="16" customHeight="1" s="5">
       <c r="A287" s="3" t="n">
-        <v>46158.96875</v>
+        <v>46159.96875</v>
       </c>
       <c r="B287" s="4" t="n">
         <v>0</v>
@@ -14667,7 +14667,7 @@
     </row>
     <row r="288" ht="16" customHeight="1" s="5">
       <c r="A288" s="3" t="n">
-        <v>46158.97916666666</v>
+        <v>46159.97916666666</v>
       </c>
       <c r="B288" s="4" t="n">
         <v>0</v>
@@ -14714,7 +14714,7 @@
     </row>
     <row r="289" ht="16" customHeight="1" s="5">
       <c r="A289" s="3" t="n">
-        <v>46158.98958333334</v>
+        <v>46159.98958333334</v>
       </c>
       <c r="B289" s="4" t="n">
         <v>0</v>
@@ -14761,7 +14761,7 @@
     </row>
     <row r="290" ht="16" customHeight="1" s="5">
       <c r="A290" s="3" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
       <c r="B290" s="4" t="n">
         <v>0</v>
@@ -14808,7 +14808,7 @@
     </row>
     <row r="291" ht="16" customHeight="1" s="5">
       <c r="A291" s="3" t="n">
-        <v>46159.01041666666</v>
+        <v>46160.01041666666</v>
       </c>
       <c r="B291" s="4" t="n">
         <v>10</v>
@@ -14855,7 +14855,7 @@
     </row>
     <row r="292" ht="16" customHeight="1" s="5">
       <c r="A292" s="3" t="n">
-        <v>46159.02083333334</v>
+        <v>46160.02083333334</v>
       </c>
       <c r="B292" s="4" t="n">
         <v>35</v>
@@ -14902,7 +14902,7 @@
     </row>
     <row r="293" ht="16" customHeight="1" s="5">
       <c r="A293" s="3" t="n">
-        <v>46159.03125</v>
+        <v>46160.03125</v>
       </c>
       <c r="B293" s="4" t="n">
         <v>62</v>
@@ -14949,7 +14949,7 @@
     </row>
     <row r="294" ht="16" customHeight="1" s="5">
       <c r="A294" s="3" t="n">
-        <v>46159.04166666666</v>
+        <v>46160.04166666666</v>
       </c>
       <c r="B294" s="4" t="n">
         <v>80</v>
@@ -14996,7 +14996,7 @@
     </row>
     <row r="295" ht="16" customHeight="1" s="5">
       <c r="A295" s="3" t="n">
-        <v>46159.05208333334</v>
+        <v>46160.05208333334</v>
       </c>
       <c r="B295" s="4" t="n">
         <v>27</v>
@@ -15043,7 +15043,7 @@
     </row>
     <row r="296" ht="16" customHeight="1" s="5">
       <c r="A296" s="3" t="n">
-        <v>46159.0625</v>
+        <v>46160.0625</v>
       </c>
       <c r="B296" s="4" t="n">
         <v>0</v>
@@ -15090,7 +15090,7 @@
     </row>
     <row r="297" ht="16" customHeight="1" s="5">
       <c r="A297" s="3" t="n">
-        <v>46159.07291666666</v>
+        <v>46160.07291666666</v>
       </c>
       <c r="B297" s="4" t="n">
         <v>4</v>
@@ -15137,7 +15137,7 @@
     </row>
     <row r="298" ht="16" customHeight="1" s="5">
       <c r="A298" s="3" t="n">
-        <v>46159.08333333334</v>
+        <v>46160.08333333334</v>
       </c>
       <c r="B298" s="4" t="n">
         <v>11</v>
@@ -15184,7 +15184,7 @@
     </row>
     <row r="299" ht="16" customHeight="1" s="5">
       <c r="A299" s="3" t="n">
-        <v>46159.09375</v>
+        <v>46160.09375</v>
       </c>
       <c r="B299" s="4" t="n">
         <v>20</v>
@@ -15231,7 +15231,7 @@
     </row>
     <row r="300" ht="16" customHeight="1" s="5">
       <c r="A300" s="3" t="n">
-        <v>46159.10416666666</v>
+        <v>46160.10416666666</v>
       </c>
       <c r="B300" s="4" t="n">
         <v>33</v>
@@ -15278,7 +15278,7 @@
     </row>
     <row r="301" ht="16" customHeight="1" s="5">
       <c r="A301" s="3" t="n">
-        <v>46159.11458333334</v>
+        <v>46160.11458333334</v>
       </c>
       <c r="B301" s="4" t="n">
         <v>17</v>
@@ -15325,7 +15325,7 @@
     </row>
     <row r="302" ht="16" customHeight="1" s="5">
       <c r="A302" s="3" t="n">
-        <v>46159.125</v>
+        <v>46160.125</v>
       </c>
       <c r="B302" s="4" t="n">
         <v>19</v>
@@ -15372,7 +15372,7 @@
     </row>
     <row r="303" ht="16" customHeight="1" s="5">
       <c r="A303" s="3" t="n">
-        <v>46159.13541666666</v>
+        <v>46160.13541666666</v>
       </c>
       <c r="B303" s="4" t="n">
         <v>26</v>
@@ -15419,7 +15419,7 @@
     </row>
     <row r="304" ht="16" customHeight="1" s="5">
       <c r="A304" s="3" t="n">
-        <v>46159.14583333334</v>
+        <v>46160.14583333334</v>
       </c>
       <c r="B304" s="4" t="n">
         <v>65</v>
@@ -15466,7 +15466,7 @@
     </row>
     <row r="305" ht="16" customHeight="1" s="5">
       <c r="A305" s="3" t="n">
-        <v>46159.15625</v>
+        <v>46160.15625</v>
       </c>
       <c r="B305" s="4" t="n">
         <v>256</v>
@@ -15513,7 +15513,7 @@
     </row>
     <row r="306" ht="16" customHeight="1" s="5">
       <c r="A306" s="3" t="n">
-        <v>46159.16666666666</v>
+        <v>46160.16666666666</v>
       </c>
       <c r="B306" s="4" t="n">
         <v>528</v>
@@ -15560,7 +15560,7 @@
     </row>
     <row r="307" ht="16" customHeight="1" s="5">
       <c r="A307" s="3" t="n">
-        <v>46159.17708333334</v>
+        <v>46160.17708333334</v>
       </c>
       <c r="B307" s="4" t="n">
         <v>850</v>
@@ -15607,7 +15607,7 @@
     </row>
     <row r="308" ht="16" customHeight="1" s="5">
       <c r="A308" s="3" t="n">
-        <v>46159.1875</v>
+        <v>46160.1875</v>
       </c>
       <c r="B308" s="4" t="n">
         <v>967</v>
@@ -15654,7 +15654,7 @@
     </row>
     <row r="309" ht="16" customHeight="1" s="5">
       <c r="A309" s="3" t="n">
-        <v>46159.19791666666</v>
+        <v>46160.19791666666</v>
       </c>
       <c r="B309" s="4" t="n">
         <v>755</v>
@@ -15701,7 +15701,7 @@
     </row>
     <row r="310" ht="16" customHeight="1" s="5">
       <c r="A310" s="3" t="n">
-        <v>46159.20833333334</v>
+        <v>46160.20833333334</v>
       </c>
       <c r="B310" s="4" t="n">
         <v>800</v>
@@ -15748,7 +15748,7 @@
     </row>
     <row r="311" ht="16" customHeight="1" s="5">
       <c r="A311" s="3" t="n">
-        <v>46159.21875</v>
+        <v>46160.21875</v>
       </c>
       <c r="B311" s="4" t="n">
         <v>656</v>
@@ -15795,7 +15795,7 @@
     </row>
     <row r="312" ht="16" customHeight="1" s="5">
       <c r="A312" s="3" t="n">
-        <v>46159.22916666666</v>
+        <v>46160.22916666666</v>
       </c>
       <c r="B312" s="4" t="n">
         <v>515</v>
@@ -15842,7 +15842,7 @@
     </row>
     <row r="313" ht="16" customHeight="1" s="5">
       <c r="A313" s="3" t="n">
-        <v>46159.23958333334</v>
+        <v>46160.23958333334</v>
       </c>
       <c r="B313" s="4" t="n">
         <v>474</v>
@@ -15889,7 +15889,7 @@
     </row>
     <row r="314" ht="16" customHeight="1" s="5">
       <c r="A314" s="3" t="n">
-        <v>46159.25</v>
+        <v>46160.25</v>
       </c>
       <c r="B314" s="4" t="n">
         <v>601</v>
@@ -15936,7 +15936,7 @@
     </row>
     <row r="315" ht="16" customHeight="1" s="5">
       <c r="A315" s="3" t="n">
-        <v>46159.26041666666</v>
+        <v>46160.26041666666</v>
       </c>
       <c r="B315" s="4" t="n">
         <v>632</v>
@@ -15983,7 +15983,7 @@
     </row>
     <row r="316" ht="16" customHeight="1" s="5">
       <c r="A316" s="3" t="n">
-        <v>46159.27083333334</v>
+        <v>46160.27083333334</v>
       </c>
       <c r="B316" s="4" t="n">
         <v>592</v>
@@ -16030,7 +16030,7 @@
     </row>
     <row r="317" ht="16" customHeight="1" s="5">
       <c r="A317" s="3" t="n">
-        <v>46159.28125</v>
+        <v>46160.28125</v>
       </c>
       <c r="B317" s="4" t="n">
         <v>493</v>
@@ -16077,7 +16077,7 @@
     </row>
     <row r="318" ht="16" customHeight="1" s="5">
       <c r="A318" s="3" t="n">
-        <v>46159.29166666666</v>
+        <v>46160.29166666666</v>
       </c>
       <c r="B318" s="4" t="n">
         <v>448</v>
@@ -16124,7 +16124,7 @@
     </row>
     <row r="319" ht="16" customHeight="1" s="5">
       <c r="A319" s="3" t="n">
-        <v>46159.30208333334</v>
+        <v>46160.30208333334</v>
       </c>
       <c r="B319" s="4" t="n">
         <v>459</v>
@@ -16171,7 +16171,7 @@
     </row>
     <row r="320" ht="16" customHeight="1" s="5">
       <c r="A320" s="3" t="n">
-        <v>46159.3125</v>
+        <v>46160.3125</v>
       </c>
       <c r="B320" s="4" t="n">
         <v>432</v>
@@ -16218,7 +16218,7 @@
     </row>
     <row r="321" ht="16" customHeight="1" s="5">
       <c r="A321" s="3" t="n">
-        <v>46159.32291666666</v>
+        <v>46160.32291666666</v>
       </c>
       <c r="B321" s="4" t="n">
         <v>368</v>
@@ -16265,7 +16265,7 @@
     </row>
     <row r="322" ht="16" customHeight="1" s="5">
       <c r="A322" s="3" t="n">
-        <v>46159.33333333334</v>
+        <v>46160.33333333334</v>
       </c>
       <c r="B322" s="4" t="n">
         <v>320</v>
@@ -16312,7 +16312,7 @@
     </row>
     <row r="323" ht="16" customHeight="1" s="5">
       <c r="A323" s="3" t="n">
-        <v>46159.34375</v>
+        <v>46160.34375</v>
       </c>
       <c r="B323" s="4" t="n">
         <v>237</v>
@@ -16359,7 +16359,7 @@
     </row>
     <row r="324" ht="16" customHeight="1" s="5">
       <c r="A324" s="3" t="n">
-        <v>46159.35416666666</v>
+        <v>46160.35416666666</v>
       </c>
       <c r="B324" s="4" t="n">
         <v>262</v>
@@ -16406,7 +16406,7 @@
     </row>
     <row r="325" ht="16" customHeight="1" s="5">
       <c r="A325" s="3" t="n">
-        <v>46159.36458333334</v>
+        <v>46160.36458333334</v>
       </c>
       <c r="B325" s="4" t="n">
         <v>445</v>
@@ -16453,7 +16453,7 @@
     </row>
     <row r="326" ht="16" customHeight="1" s="5">
       <c r="A326" s="3" t="n">
-        <v>46159.375</v>
+        <v>46160.375</v>
       </c>
       <c r="B326" s="4" t="n">
         <v>627</v>
@@ -16500,7 +16500,7 @@
     </row>
     <row r="327" ht="16" customHeight="1" s="5">
       <c r="A327" s="3" t="n">
-        <v>46159.38541666666</v>
+        <v>46160.38541666666</v>
       </c>
       <c r="B327" s="4" t="n">
         <v>623</v>
@@ -16547,7 +16547,7 @@
     </row>
     <row r="328" ht="16" customHeight="1" s="5">
       <c r="A328" s="3" t="n">
-        <v>46159.39583333334</v>
+        <v>46160.39583333334</v>
       </c>
       <c r="B328" s="4" t="n">
         <v>576</v>
@@ -16594,7 +16594,7 @@
     </row>
     <row r="329" ht="16" customHeight="1" s="5">
       <c r="A329" s="3" t="n">
-        <v>46159.40625</v>
+        <v>46160.40625</v>
       </c>
       <c r="B329" s="4" t="n">
         <v>542</v>
@@ -16641,7 +16641,7 @@
     </row>
     <row r="330" ht="16" customHeight="1" s="5">
       <c r="A330" s="3" t="n">
-        <v>46159.41666666666</v>
+        <v>46160.41666666666</v>
       </c>
       <c r="B330" s="4" t="n">
         <v>484</v>
@@ -16688,7 +16688,7 @@
     </row>
     <row r="331" ht="16" customHeight="1" s="5">
       <c r="A331" s="3" t="n">
-        <v>46159.42708333334</v>
+        <v>46160.42708333334</v>
       </c>
       <c r="B331" s="4" t="n">
         <v>377</v>
@@ -16735,7 +16735,7 @@
     </row>
     <row r="332" ht="16" customHeight="1" s="5">
       <c r="A332" s="3" t="n">
-        <v>46159.4375</v>
+        <v>46160.4375</v>
       </c>
       <c r="B332" s="4" t="n">
         <v>281</v>
@@ -16782,7 +16782,7 @@
     </row>
     <row r="333" ht="16" customHeight="1" s="5">
       <c r="A333" s="3" t="n">
-        <v>46159.44791666666</v>
+        <v>46160.44791666666</v>
       </c>
       <c r="B333" s="4" t="n">
         <v>386</v>
@@ -16829,7 +16829,7 @@
     </row>
     <row r="334" ht="16" customHeight="1" s="5">
       <c r="A334" s="3" t="n">
-        <v>46159.45833333334</v>
+        <v>46160.45833333334</v>
       </c>
       <c r="B334" s="4" t="n">
         <v>548</v>
@@ -16876,7 +16876,7 @@
     </row>
     <row r="335" ht="16" customHeight="1" s="5">
       <c r="A335" s="3" t="n">
-        <v>46159.46875</v>
+        <v>46160.46875</v>
       </c>
       <c r="B335" s="4" t="n">
         <v>620</v>
@@ -16923,7 +16923,7 @@
     </row>
     <row r="336" ht="16" customHeight="1" s="5">
       <c r="A336" s="3" t="n">
-        <v>46159.47916666666</v>
+        <v>46160.47916666666</v>
       </c>
       <c r="B336" s="4" t="n">
         <v>531</v>
@@ -16970,7 +16970,7 @@
     </row>
     <row r="337" ht="16" customHeight="1" s="5">
       <c r="A337" s="3" t="n">
-        <v>46159.48958333334</v>
+        <v>46160.48958333334</v>
       </c>
       <c r="B337" s="4" t="n">
         <v>491</v>
@@ -17017,7 +17017,7 @@
     </row>
     <row r="338" ht="16" customHeight="1" s="5">
       <c r="A338" s="3" t="n">
-        <v>46159.5</v>
+        <v>46160.5</v>
       </c>
       <c r="B338" s="4" t="n">
         <v>385</v>
@@ -17064,7 +17064,7 @@
     </row>
     <row r="339" ht="16" customHeight="1" s="5">
       <c r="A339" s="3" t="n">
-        <v>46159.51041666666</v>
+        <v>46160.51041666666</v>
       </c>
       <c r="B339" s="4" t="n">
         <v>397</v>
@@ -17111,7 +17111,7 @@
     </row>
     <row r="340" ht="16" customHeight="1" s="5">
       <c r="A340" s="3" t="n">
-        <v>46159.52083333334</v>
+        <v>46160.52083333334</v>
       </c>
       <c r="B340" s="4" t="n">
         <v>490</v>
@@ -17158,7 +17158,7 @@
     </row>
     <row r="341" ht="16" customHeight="1" s="5">
       <c r="A341" s="3" t="n">
-        <v>46159.53125</v>
+        <v>46160.53125</v>
       </c>
       <c r="B341" s="4" t="n">
         <v>547</v>
@@ -17205,7 +17205,7 @@
     </row>
     <row r="342" ht="16" customHeight="1" s="5">
       <c r="A342" s="3" t="n">
-        <v>46159.54166666666</v>
+        <v>46160.54166666666</v>
       </c>
       <c r="B342" s="4" t="n">
         <v>415</v>
@@ -17252,7 +17252,7 @@
     </row>
     <row r="343" ht="16" customHeight="1" s="5">
       <c r="A343" s="3" t="n">
-        <v>46159.55208333334</v>
+        <v>46160.55208333334</v>
       </c>
       <c r="B343" s="4" t="n">
         <v>228</v>
@@ -17299,7 +17299,7 @@
     </row>
     <row r="344" ht="16" customHeight="1" s="5">
       <c r="A344" s="3" t="n">
-        <v>46159.5625</v>
+        <v>46160.5625</v>
       </c>
       <c r="B344" s="4" t="n">
         <v>309</v>
@@ -17346,7 +17346,7 @@
     </row>
     <row r="345" ht="16" customHeight="1" s="5">
       <c r="A345" s="3" t="n">
-        <v>46159.57291666666</v>
+        <v>46160.57291666666</v>
       </c>
       <c r="B345" s="4" t="n">
         <v>411</v>
@@ -17393,7 +17393,7 @@
     </row>
     <row r="346" ht="16" customHeight="1" s="5">
       <c r="A346" s="3" t="n">
-        <v>46159.58333333334</v>
+        <v>46160.58333333334</v>
       </c>
       <c r="B346" s="4" t="n">
         <v>385</v>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="347" ht="16" customHeight="1" s="5">
       <c r="A347" s="3" t="n">
-        <v>46159.59375</v>
+        <v>46160.59375</v>
       </c>
       <c r="B347" s="4" t="n">
         <v>436</v>
@@ -17487,7 +17487,7 @@
     </row>
     <row r="348" ht="16" customHeight="1" s="5">
       <c r="A348" s="3" t="n">
-        <v>46159.60416666666</v>
+        <v>46160.60416666666</v>
       </c>
       <c r="B348" s="4" t="n">
         <v>446</v>
@@ -17534,7 +17534,7 @@
     </row>
     <row r="349" ht="16" customHeight="1" s="5">
       <c r="A349" s="3" t="n">
-        <v>46159.61458333334</v>
+        <v>46160.61458333334</v>
       </c>
       <c r="B349" s="4" t="n">
         <v>426</v>
@@ -17581,7 +17581,7 @@
     </row>
     <row r="350" ht="16" customHeight="1" s="5">
       <c r="A350" s="3" t="n">
-        <v>46159.625</v>
+        <v>46160.625</v>
       </c>
       <c r="B350" s="4" t="n">
         <v>450</v>
@@ -17628,7 +17628,7 @@
     </row>
     <row r="351" ht="16" customHeight="1" s="5">
       <c r="A351" s="3" t="n">
-        <v>46159.63541666666</v>
+        <v>46160.63541666666</v>
       </c>
       <c r="B351" s="4" t="n">
         <v>322</v>
@@ -17675,7 +17675,7 @@
     </row>
     <row r="352" ht="16" customHeight="1" s="5">
       <c r="A352" s="3" t="n">
-        <v>46159.64583333334</v>
+        <v>46160.64583333334</v>
       </c>
       <c r="B352" s="4" t="n">
         <v>303</v>
@@ -17722,7 +17722,7 @@
     </row>
     <row r="353" ht="16" customHeight="1" s="5">
       <c r="A353" s="3" t="n">
-        <v>46159.65625</v>
+        <v>46160.65625</v>
       </c>
       <c r="B353" s="4" t="n">
         <v>496</v>
@@ -17769,7 +17769,7 @@
     </row>
     <row r="354" ht="16" customHeight="1" s="5">
       <c r="A354" s="3" t="n">
-        <v>46159.66666666666</v>
+        <v>46160.66666666666</v>
       </c>
       <c r="B354" s="4" t="n">
         <v>654</v>
@@ -17816,7 +17816,7 @@
     </row>
     <row r="355" ht="16" customHeight="1" s="5">
       <c r="A355" s="3" t="n">
-        <v>46159.67708333334</v>
+        <v>46160.67708333334</v>
       </c>
       <c r="B355" s="4" t="n">
         <v>781</v>
@@ -17863,7 +17863,7 @@
     </row>
     <row r="356" ht="16" customHeight="1" s="5">
       <c r="A356" s="3" t="n">
-        <v>46159.6875</v>
+        <v>46160.6875</v>
       </c>
       <c r="B356" s="4" t="n">
         <v>795</v>
@@ -17910,7 +17910,7 @@
     </row>
     <row r="357" ht="16" customHeight="1" s="5">
       <c r="A357" s="3" t="n">
-        <v>46159.69791666666</v>
+        <v>46160.69791666666</v>
       </c>
       <c r="B357" s="4" t="n">
         <v>569</v>
@@ -17957,7 +17957,7 @@
     </row>
     <row r="358" ht="16" customHeight="1" s="5">
       <c r="A358" s="3" t="n">
-        <v>46159.70833333334</v>
+        <v>46160.70833333334</v>
       </c>
       <c r="B358" s="4" t="n">
         <v>611</v>
@@ -18004,7 +18004,7 @@
     </row>
     <row r="359" ht="16" customHeight="1" s="5">
       <c r="A359" s="3" t="n">
-        <v>46159.71875</v>
+        <v>46160.71875</v>
       </c>
       <c r="B359" s="4" t="n">
         <v>794</v>
@@ -18051,7 +18051,7 @@
     </row>
     <row r="360" ht="16" customHeight="1" s="5">
       <c r="A360" s="3" t="n">
-        <v>46159.72916666666</v>
+        <v>46160.72916666666</v>
       </c>
       <c r="B360" s="4" t="n">
         <v>635</v>
@@ -18098,7 +18098,7 @@
     </row>
     <row r="361" ht="16" customHeight="1" s="5">
       <c r="A361" s="3" t="n">
-        <v>46159.73958333334</v>
+        <v>46160.73958333334</v>
       </c>
       <c r="B361" s="4" t="n">
         <v>642</v>
@@ -18145,7 +18145,7 @@
     </row>
     <row r="362" ht="16" customHeight="1" s="5">
       <c r="A362" s="3" t="n">
-        <v>46159.75</v>
+        <v>46160.75</v>
       </c>
       <c r="B362" s="4" t="n">
         <v>624</v>
@@ -18192,7 +18192,7 @@
     </row>
     <row r="363" ht="16" customHeight="1" s="5">
       <c r="A363" s="3" t="n">
-        <v>46159.76041666666</v>
+        <v>46160.76041666666</v>
       </c>
       <c r="B363" s="4" t="n">
         <v>608</v>
@@ -18239,7 +18239,7 @@
     </row>
     <row r="364" ht="16" customHeight="1" s="5">
       <c r="A364" s="3" t="n">
-        <v>46159.77083333334</v>
+        <v>46160.77083333334</v>
       </c>
       <c r="B364" s="4" t="n">
         <v>656</v>
@@ -18286,7 +18286,7 @@
     </row>
     <row r="365" ht="16" customHeight="1" s="5">
       <c r="A365" s="3" t="n">
-        <v>46159.78125</v>
+        <v>46160.78125</v>
       </c>
       <c r="B365" s="4" t="n">
         <v>512</v>
@@ -18333,7 +18333,7 @@
     </row>
     <row r="366" ht="16" customHeight="1" s="5">
       <c r="A366" s="3" t="n">
-        <v>46159.79166666666</v>
+        <v>46160.79166666666</v>
       </c>
       <c r="B366" s="4" t="n">
         <v>323</v>
@@ -18380,7 +18380,7 @@
     </row>
     <row r="367" ht="16" customHeight="1" s="5">
       <c r="A367" s="3" t="n">
-        <v>46159.80208333334</v>
+        <v>46160.80208333334</v>
       </c>
       <c r="B367" s="4" t="n">
         <v>438</v>
@@ -18427,7 +18427,7 @@
     </row>
     <row r="368" ht="16" customHeight="1" s="5">
       <c r="A368" s="3" t="n">
-        <v>46159.8125</v>
+        <v>46160.8125</v>
       </c>
       <c r="B368" s="4" t="n">
         <v>613</v>
@@ -18474,7 +18474,7 @@
     </row>
     <row r="369" ht="16" customHeight="1" s="5">
       <c r="A369" s="3" t="n">
-        <v>46159.82291666666</v>
+        <v>46160.82291666666</v>
       </c>
       <c r="B369" s="4" t="n">
         <v>547</v>
@@ -18521,7 +18521,7 @@
     </row>
     <row r="370" ht="16" customHeight="1" s="5">
       <c r="A370" s="3" t="n">
-        <v>46159.83333333334</v>
+        <v>46160.83333333334</v>
       </c>
       <c r="B370" s="4" t="n">
         <v>402</v>
@@ -18568,7 +18568,7 @@
     </row>
     <row r="371" ht="16" customHeight="1" s="5">
       <c r="A371" s="3" t="n">
-        <v>46159.84375</v>
+        <v>46160.84375</v>
       </c>
       <c r="B371" s="4" t="n">
         <v>341</v>
@@ -18615,7 +18615,7 @@
     </row>
     <row r="372" ht="16" customHeight="1" s="5">
       <c r="A372" s="3" t="n">
-        <v>46159.85416666666</v>
+        <v>46160.85416666666</v>
       </c>
       <c r="B372" s="4" t="n">
         <v>264</v>
@@ -18662,7 +18662,7 @@
     </row>
     <row r="373" ht="16" customHeight="1" s="5">
       <c r="A373" s="3" t="n">
-        <v>46159.86458333334</v>
+        <v>46160.86458333334</v>
       </c>
       <c r="B373" s="4" t="n">
         <v>116</v>
@@ -18709,7 +18709,7 @@
     </row>
     <row r="374" ht="16" customHeight="1" s="5">
       <c r="A374" s="3" t="n">
-        <v>46159.875</v>
+        <v>46160.875</v>
       </c>
       <c r="B374" s="4" t="n">
         <v>0</v>
@@ -18756,7 +18756,7 @@
     </row>
     <row r="375" ht="16" customHeight="1" s="5">
       <c r="A375" s="3" t="n">
-        <v>46159.88541666666</v>
+        <v>46160.88541666666</v>
       </c>
       <c r="B375" s="4" t="n">
         <v>10</v>
@@ -18803,7 +18803,7 @@
     </row>
     <row r="376" ht="16" customHeight="1" s="5">
       <c r="A376" s="3" t="n">
-        <v>46159.89583333334</v>
+        <v>46160.89583333334</v>
       </c>
       <c r="B376" s="4" t="n">
         <v>39</v>
@@ -18850,7 +18850,7 @@
     </row>
     <row r="377" ht="16" customHeight="1" s="5">
       <c r="A377" s="3" t="n">
-        <v>46159.90625</v>
+        <v>46160.90625</v>
       </c>
       <c r="B377" s="4" t="n">
         <v>109</v>
@@ -18897,7 +18897,7 @@
     </row>
     <row r="378" ht="16" customHeight="1" s="5">
       <c r="A378" s="3" t="n">
-        <v>46159.91666666666</v>
+        <v>46160.91666666666</v>
       </c>
       <c r="B378" s="4" t="n">
         <v>193</v>
@@ -18944,7 +18944,7 @@
     </row>
     <row r="379" ht="16" customHeight="1" s="5">
       <c r="A379" s="3" t="n">
-        <v>46159.92708333334</v>
+        <v>46160.92708333334</v>
       </c>
       <c r="B379" s="4" t="n">
         <v>217</v>
@@ -18991,7 +18991,7 @@
     </row>
     <row r="380" ht="16" customHeight="1" s="5">
       <c r="A380" s="3" t="n">
-        <v>46159.9375</v>
+        <v>46160.9375</v>
       </c>
       <c r="B380" s="4" t="n">
         <v>185</v>
@@ -19038,7 +19038,7 @@
     </row>
     <row r="381" ht="16" customHeight="1" s="5">
       <c r="A381" s="3" t="n">
-        <v>46159.94791666666</v>
+        <v>46160.94791666666</v>
       </c>
       <c r="B381" s="4" t="n">
         <v>27</v>
@@ -19085,7 +19085,7 @@
     </row>
     <row r="382" ht="16" customHeight="1" s="5">
       <c r="A382" s="3" t="n">
-        <v>46159.95833333334</v>
+        <v>46160.95833333334</v>
       </c>
       <c r="B382" s="4" t="n">
         <v>0</v>
@@ -19132,7 +19132,7 @@
     </row>
     <row r="383" ht="16" customHeight="1" s="5">
       <c r="A383" s="3" t="n">
-        <v>46159.96875</v>
+        <v>46160.96875</v>
       </c>
       <c r="B383" s="4" t="n">
         <v>0</v>
@@ -19179,7 +19179,7 @@
     </row>
     <row r="384" ht="16" customHeight="1" s="5">
       <c r="A384" s="3" t="n">
-        <v>46159.97916666666</v>
+        <v>46160.97916666666</v>
       </c>
       <c r="B384" s="4" t="n">
         <v>0</v>
@@ -19226,7 +19226,7 @@
     </row>
     <row r="385" ht="16" customHeight="1" s="5">
       <c r="A385" s="3" t="n">
-        <v>46159.98958333334</v>
+        <v>46160.98958333334</v>
       </c>
       <c r="B385" s="4" t="n">
         <v>0</v>

</xml_diff>